<commit_message>
Sync from vault 2026-05-26 09:10:12
</commit_message>
<xml_diff>
--- a/content/Archief/0. PDFs & docs/Obol docs & forms/Irmijn Inc/Irma backup log.xlsx
+++ b/content/Archief/0. PDFs & docs/Obol docs & forms/Irmijn Inc/Irma backup log.xlsx
@@ -15,9 +15,10 @@
   </sheets>
   <definedNames>
     <definedName function="false" hidden="true" localSheetId="3" name="_xlnm._FilterDatabase" vbProcedure="false">Tatdata!$A$1:$B$13</definedName>
-    <definedName function="false" hidden="true" localSheetId="2" name="_xlnm._FilterDatabase" vbProcedure="false">Tatjes!$A$1:$F$91</definedName>
-    <definedName function="false" hidden="false" localSheetId="2" name="_xlnm._FilterDatabase" vbProcedure="false">Tatjes!$A$1:$F$90</definedName>
-    <definedName function="false" hidden="false" localSheetId="2" name="_xlnm._FilterDatabase_0" vbProcedure="false">Tatjes!$A$1:$F$88</definedName>
+    <definedName function="false" hidden="true" localSheetId="2" name="_xlnm._FilterDatabase" vbProcedure="false">Tatjes!$A$1:$F$92</definedName>
+    <definedName function="false" hidden="false" localSheetId="2" name="_xlnm._FilterDatabase" vbProcedure="false">Tatjes!$A$1:$F$91</definedName>
+    <definedName function="false" hidden="false" localSheetId="2" name="_xlnm._FilterDatabase_0" vbProcedure="false">Tatjes!$A$1:$F$90</definedName>
+    <definedName function="false" hidden="false" localSheetId="2" name="_xlnm._FilterDatabase_0_0" vbProcedure="false">Tatjes!$A$1:$F$88</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.001"/>
   <extLst>
@@ -29,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="484" uniqueCount="100">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="490" uniqueCount="101">
   <si>
     <t xml:space="preserve">Pagina</t>
   </si>
@@ -157,6 +158,9 @@
     <t xml:space="preserve">Blaadje</t>
   </si>
   <si>
+    <t xml:space="preserve">Zwarte kubus</t>
+  </si>
+  <si>
     <t xml:space="preserve">Jaar</t>
   </si>
   <si>
@@ -277,10 +281,10 @@
     <t xml:space="preserve">Oranje</t>
   </si>
   <si>
-    <t xml:space="preserve">Groen</t>
+    <t xml:space="preserve">Gras</t>
   </si>
   <si>
-    <t xml:space="preserve">Gras</t>
+    <t xml:space="preserve">Groen</t>
   </si>
   <si>
     <t xml:space="preserve">Wit</t>
@@ -473,14 +477,14 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF00A933"/>
-        <bgColor rgb="FF008080"/>
+        <fgColor rgb="FFBBE33D"/>
+        <bgColor rgb="FFACB20C"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFBBE33D"/>
-        <bgColor rgb="FFACB20C"/>
+        <fgColor rgb="FF00A933"/>
+        <bgColor rgb="FF008080"/>
       </patternFill>
     </fill>
     <fill>
@@ -639,11 +643,11 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="14" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="14" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="15" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="15" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -844,7 +848,7 @@
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>Omschrijving Kaft Zonnebloem Koperen ei Ruitje Pimpelmees Mijnvogel in Mineur Vlinderbeest Scheepswiel Vondst Tala Vlinder Wolkendroom Kanarie Kopernest Klaver Irmijn Inc logo Obol Boyz Vuurmot Vrijer dan wij Lege kooi In de urn Apenweegschaal Puzzel Groene steen Libel Gift van de Moeders Heks met klauw Bijtje Hoeders Lieveheersbeestje Diep. Diep. Diep. Paal etc Blaadje</c:v>
+                  <c:v>Omschrijving Kaft Zonnebloem Koperen ei Ruitje Pimpelmees Mijnvogel in Mineur Vlinderbeest Scheepswiel Vondst Tala Vlinder Wolkendroom Kanarie Kopernest Klaver Irmijn Inc logo Obol Boyz Vuurmot Vrijer dan wij Lege kooi In de urn Apenweegschaal Puzzel Groene steen Libel Gift van de Moeders Heks met klauw Bijtje Hoeders Lieveheersbeestje Diep. Diep. Diep. Paal etc Blaadje Zwarte kubus</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -1473,13 +1477,13 @@
                   <c:v>123</c:v>
                 </c:pt>
                 <c:pt idx="78">
-                  <c:v>127</c:v>
+                  <c:v>126</c:v>
                 </c:pt>
                 <c:pt idx="79">
-                  <c:v/>
+                  <c:v>130</c:v>
                 </c:pt>
                 <c:pt idx="80">
-                  <c:v/>
+                  <c:v>131</c:v>
                 </c:pt>
                 <c:pt idx="81">
                   <c:v/>
@@ -1593,11 +1597,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="75096402"/>
-        <c:axId val="22154157"/>
+        <c:axId val="70902698"/>
+        <c:axId val="31228987"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="75096402"/>
+        <c:axId val="70902698"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1653,14 +1657,14 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="22154157"/>
+        <c:crossAx val="31228987"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
         <c:lblOffset val="100"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="22154157"/>
+        <c:axId val="31228987"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1725,7 +1729,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="75096402"/>
+        <c:crossAx val="70902698"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -2428,10 +2432,10 @@
                   <c:v>46</c:v>
                 </c:pt>
                 <c:pt idx="78">
-                  <c:v/>
+                  <c:v>47</c:v>
                 </c:pt>
                 <c:pt idx="79">
-                  <c:v/>
+                  <c:v>47</c:v>
                 </c:pt>
                 <c:pt idx="80">
                   <c:v/>
@@ -3175,10 +3179,10 @@
                   <c:v>17</c:v>
                 </c:pt>
                 <c:pt idx="78">
-                  <c:v/>
+                  <c:v>17</c:v>
                 </c:pt>
                 <c:pt idx="79">
-                  <c:v/>
+                  <c:v>18</c:v>
                 </c:pt>
                 <c:pt idx="80">
                   <c:v/>
@@ -3922,10 +3926,10 @@
                   <c:v>11</c:v>
                 </c:pt>
                 <c:pt idx="78">
-                  <c:v/>
+                  <c:v>11</c:v>
                 </c:pt>
                 <c:pt idx="79">
-                  <c:v/>
+                  <c:v>11</c:v>
                 </c:pt>
                 <c:pt idx="80">
                   <c:v/>
@@ -4669,10 +4673,10 @@
                   <c:v>4</c:v>
                 </c:pt>
                 <c:pt idx="78">
-                  <c:v/>
+                  <c:v>4</c:v>
                 </c:pt>
                 <c:pt idx="79">
-                  <c:v/>
+                  <c:v>4</c:v>
                 </c:pt>
                 <c:pt idx="80">
                   <c:v/>
@@ -4786,11 +4790,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="88581778"/>
-        <c:axId val="12737401"/>
+        <c:axId val="23335886"/>
+        <c:axId val="49722141"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="88581778"/>
+        <c:axId val="23335886"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -4846,14 +4850,14 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="12737401"/>
+        <c:crossAx val="49722141"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
         <c:lblOffset val="100"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="12737401"/>
+        <c:axId val="49722141"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -4918,7 +4922,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="88581778"/>
+        <c:crossAx val="23335886"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -5006,10 +5010,10 @@
           <c:layoutTarget val="inner"/>
           <c:xMode val="edge"/>
           <c:yMode val="edge"/>
-          <c:x val="0.0889541789085454"/>
-          <c:y val="0.110925864176948"/>
-          <c:w val="0.846158654747765"/>
-          <c:h val="0.793709014115816"/>
+          <c:x val="0.0889597399349837"/>
+          <c:y val="0.110938194753224"/>
+          <c:w val="0.846086521630408"/>
+          <c:h val="0.793574922187639"/>
         </c:manualLayout>
       </c:layout>
       <c:lineChart>
@@ -5141,11 +5145,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="58617047"/>
-        <c:axId val="25462843"/>
+        <c:axId val="35082363"/>
+        <c:axId val="87082147"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="58617047"/>
+        <c:axId val="35082363"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -5173,14 +5177,14 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="25462843"/>
+        <c:crossAx val="87082147"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
         <c:lblOffset val="100"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="25462843"/>
+        <c:axId val="87082147"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -5245,7 +5249,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="58617047"/>
+        <c:crossAx val="35082363"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -5283,9 +5287,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>179640</xdr:colOff>
+      <xdr:colOff>179280</xdr:colOff>
       <xdr:row>23</xdr:row>
-      <xdr:rowOff>43200</xdr:rowOff>
+      <xdr:rowOff>42840</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -5294,7 +5298,7 @@
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
         <a:off x="6578280" y="543600"/>
-        <a:ext cx="5758200" cy="3238200"/>
+        <a:ext cx="5757840" cy="3237840"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -5313,9 +5317,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>343440</xdr:colOff>
+      <xdr:colOff>343080</xdr:colOff>
       <xdr:row>52</xdr:row>
-      <xdr:rowOff>91440</xdr:rowOff>
+      <xdr:rowOff>91080</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -5324,7 +5328,7 @@
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
         <a:off x="6741360" y="5305320"/>
-        <a:ext cx="5758920" cy="3238920"/>
+        <a:ext cx="5758560" cy="3238560"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -5348,9 +5352,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>12</xdr:col>
-      <xdr:colOff>462960</xdr:colOff>
+      <xdr:colOff>462600</xdr:colOff>
       <xdr:row>21</xdr:row>
-      <xdr:rowOff>71640</xdr:rowOff>
+      <xdr:rowOff>71280</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -5359,7 +5363,7 @@
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
         <a:off x="2646720" y="246600"/>
-        <a:ext cx="5758560" cy="3238560"/>
+        <a:ext cx="5758200" cy="3238200"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -6154,11 +6158,11 @@
       </c>
       <c r="K27" s="0" t="n">
         <f aca="false">COUNTIF($D$1:$D$121,$J27)</f>
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="L27" s="6" t="n">
         <f aca="false">$K27/$K$31</f>
-        <v>0.582278481012658</v>
+        <v>0.580246913580247</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6192,11 +6196,11 @@
       </c>
       <c r="K28" s="0" t="n">
         <f aca="false">COUNTIF($D$1:$D$121,$J28)</f>
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="L28" s="6" t="n">
         <f aca="false">$K28/$K$31</f>
-        <v>0.215189873417721</v>
+        <v>0.222222222222222</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6238,7 +6242,7 @@
       </c>
       <c r="L29" s="6" t="n">
         <f aca="false">$K29/$K$31</f>
-        <v>0.139240506329114</v>
+        <v>0.135802469135802</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6280,7 +6284,7 @@
       </c>
       <c r="L30" s="6" t="n">
         <f aca="false">$K30/$K$31</f>
-        <v>0.0506329113924051</v>
+        <v>0.0493827160493827</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6318,7 +6322,7 @@
       </c>
       <c r="K31" s="0" t="n">
         <f aca="false">COUNTA($D$1:$D$121)</f>
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="L31" s="6" t="n">
         <f aca="false">$K31/$K$31</f>
@@ -7669,7 +7673,8 @@
         <v>77</v>
       </c>
       <c r="B79" s="1" t="n">
-        <v>127</v>
+        <f aca="false">ROUNDDOWN((B80+B78)/2,0)</f>
+        <v>126</v>
       </c>
       <c r="C79" s="2" t="s">
         <v>41</v>
@@ -7698,21 +7703,59 @@
       <c r="A80" s="1" t="n">
         <v>78</v>
       </c>
-      <c r="D80" s="5"/>
-      <c r="E80" s="5"/>
-      <c r="F80" s="5"/>
-      <c r="G80" s="5"/>
-      <c r="H80" s="5"/>
+      <c r="B80" s="1" t="n">
+        <v>130</v>
+      </c>
+      <c r="D80" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="E80" s="5" t="n">
+        <f aca="false">COUNTIF($D$2:$D80,E$1)</f>
+        <v>17</v>
+      </c>
+      <c r="F80" s="5" t="n">
+        <f aca="false">COUNTIF($D$2:$D80,F$1)</f>
+        <v>47</v>
+      </c>
+      <c r="G80" s="5" t="n">
+        <f aca="false">COUNTIF($D$2:$D80,G$1)</f>
+        <v>11</v>
+      </c>
+      <c r="H80" s="5" t="n">
+        <f aca="false">COUNTIF($D$2:$D80,H$1)</f>
+        <v>4</v>
+      </c>
     </row>
     <row r="81" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A81" s="1" t="n">
         <v>79</v>
       </c>
-      <c r="D81" s="5"/>
-      <c r="E81" s="5"/>
-      <c r="F81" s="5"/>
-      <c r="G81" s="5"/>
-      <c r="H81" s="5"/>
+      <c r="B81" s="1" t="n">
+        <f aca="false">IF(COUNTA(B82)&gt;0,ROUNDDOWN((B82+B80)/2,0),B80+1)</f>
+        <v>131</v>
+      </c>
+      <c r="C81" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="D81" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="E81" s="5" t="n">
+        <f aca="false">COUNTIF($D$2:$D81,E$1)</f>
+        <v>18</v>
+      </c>
+      <c r="F81" s="5" t="n">
+        <f aca="false">COUNTIF($D$2:$D81,F$1)</f>
+        <v>47</v>
+      </c>
+      <c r="G81" s="5" t="n">
+        <f aca="false">COUNTIF($D$2:$D81,G$1)</f>
+        <v>11</v>
+      </c>
+      <c r="H81" s="5" t="n">
+        <f aca="false">COUNTIF($D$2:$D81,H$1)</f>
+        <v>4</v>
+      </c>
     </row>
     <row r="82" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A82" s="1" t="n">
@@ -8136,13 +8179,13 @@
   <sheetData>
     <row r="1" s="4" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="4" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="E1" s="4" t="s">
         <v>2</v>
@@ -8164,7 +8207,7 @@
         <v>429.419178082192</v>
       </c>
       <c r="E2" s="0" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8183,7 +8226,7 @@
         <v>429.419178082192</v>
       </c>
       <c r="E3" s="0" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8202,7 +8245,7 @@
         <v>432.419178082192</v>
       </c>
       <c r="E4" s="0" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8221,7 +8264,7 @@
         <v>433.419178082192</v>
       </c>
       <c r="E5" s="8" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8240,7 +8283,7 @@
         <v>436.419178082192</v>
       </c>
       <c r="E6" s="0" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8259,7 +8302,7 @@
         <v>436.419178082192</v>
       </c>
       <c r="E7" s="0" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8278,7 +8321,7 @@
         <v>437.419178082192</v>
       </c>
       <c r="E8" s="0" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8297,7 +8340,7 @@
         <v>439.419178082192</v>
       </c>
       <c r="E9" s="0" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8316,7 +8359,7 @@
         <v>440.419178082192</v>
       </c>
       <c r="E10" s="0" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8335,7 +8378,7 @@
         <v>443.419178082192</v>
       </c>
       <c r="E11" s="0" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8354,7 +8397,7 @@
         <v>446.419178082192</v>
       </c>
       <c r="E12" s="0" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8373,7 +8416,7 @@
         <v>447.419178082192</v>
       </c>
       <c r="E13" s="0" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8392,7 +8435,7 @@
         <v>447.419178082192</v>
       </c>
       <c r="E14" s="8" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8411,7 +8454,7 @@
         <v>448.419178082192</v>
       </c>
       <c r="E15" s="0" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8430,7 +8473,7 @@
         <v>449.419178082192</v>
       </c>
       <c r="E16" s="8" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8449,7 +8492,7 @@
         <v>449.419178082192</v>
       </c>
       <c r="E17" s="0" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8468,7 +8511,7 @@
         <v>450.419178082192</v>
       </c>
       <c r="E18" s="0" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8487,7 +8530,7 @@
         <v>450.419178082192</v>
       </c>
       <c r="E19" s="0" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
     </row>
   </sheetData>
@@ -8507,7 +8550,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F91"/>
+  <dimension ref="A1:F92"/>
   <sheetFormatPr defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="9.63"/>
@@ -8519,33 +8562,33 @@
   <sheetData>
     <row r="1" s="9" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="9" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B1" s="9" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="C1" s="9" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D1" s="9" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="E1" s="9" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="F1" s="9" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="10" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="B2" s="11" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C2" s="8" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="D2" s="0" t="n">
         <f aca="false">IF(ISBLANK(A2),"",COUNTIF(A:A,A2))</f>
@@ -8562,13 +8605,13 @@
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="10" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="B3" s="11" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C3" s="12" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="D3" s="0" t="n">
         <f aca="false">IF(ISBLANK(A3),"",COUNTIF(A:A,A3))</f>
@@ -8585,13 +8628,13 @@
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="10" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="B4" s="11" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C4" s="13" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="D4" s="0" t="n">
         <f aca="false">IF(ISBLANK(A4),"",COUNTIF(A:A,A4))</f>
@@ -8608,13 +8651,13 @@
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="10" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="B5" s="14" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="C5" s="15" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="D5" s="0" t="n">
         <f aca="false">IF(ISBLANK(A5),"",COUNTIF(A:A,A5))</f>
@@ -8631,13 +8674,13 @@
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="10" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="B6" s="14" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="C6" s="15" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="D6" s="0" t="n">
         <f aca="false">IF(ISBLANK(A6),"",COUNTIF(A:A,A6))</f>
@@ -8654,13 +8697,13 @@
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="10" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="B7" s="14" t="s">
+        <v>75</v>
+      </c>
+      <c r="C7" s="13" t="s">
         <v>74</v>
-      </c>
-      <c r="C7" s="13" t="s">
-        <v>73</v>
       </c>
       <c r="D7" s="0" t="n">
         <f aca="false">IF(ISBLANK(A7),"",COUNTIF(A:A,A7))</f>
@@ -8677,13 +8720,13 @@
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="10" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="B8" s="16" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="C8" s="17" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="D8" s="0" t="n">
         <f aca="false">IF(ISBLANK(A8),"",COUNTIF(A:A,A8))</f>
@@ -8695,18 +8738,18 @@
       </c>
       <c r="F8" s="0" t="n">
         <f aca="false">IF(ISBLANK(C8),"",COUNTIF(C:C,C8))</f>
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="10" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="B9" s="16" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="C9" s="10" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="D9" s="0" t="n">
         <f aca="false">IF(ISBLANK(A9),"",COUNTIF(A:A,A9))</f>
@@ -8723,13 +8766,13 @@
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="10" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="B10" s="15" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C10" s="10" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="D10" s="0" t="n">
         <f aca="false">IF(ISBLANK(A10),"",COUNTIF(A:A,A10))</f>
@@ -8746,13 +8789,13 @@
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="10" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="B11" s="18" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="C11" s="14" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="D11" s="0" t="n">
         <f aca="false">IF(ISBLANK(A11),"",COUNTIF(A:A,A11))</f>
@@ -8769,13 +8812,13 @@
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="10" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="B12" s="19" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="C12" s="8" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="D12" s="0" t="n">
         <f aca="false">IF(ISBLANK(A12),"",COUNTIF(A:A,A12))</f>
@@ -8792,13 +8835,13 @@
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="10" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="B13" s="19" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="C13" s="10" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="D13" s="0" t="n">
         <f aca="false">IF(ISBLANK(A13),"",COUNTIF(A:A,A13))</f>
@@ -8815,13 +8858,13 @@
     </row>
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="10" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="B14" s="20" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="C14" s="8" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="D14" s="0" t="n">
         <f aca="false">IF(ISBLANK(A14),"",COUNTIF(A:A,A14))</f>
@@ -8838,13 +8881,13 @@
     </row>
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="10" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="B15" s="20" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="C15" s="8" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="D15" s="0" t="n">
         <f aca="false">IF(ISBLANK(A15),"",COUNTIF(A:A,A15))</f>
@@ -8861,13 +8904,13 @@
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="10" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="B16" s="13" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="C16" s="11" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="D16" s="0" t="n">
         <f aca="false">IF(ISBLANK(A16),"",COUNTIF(A:A,A16))</f>
@@ -8884,13 +8927,13 @@
     </row>
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="10" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="B17" s="13" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="C17" s="11" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="D17" s="0" t="n">
         <f aca="false">IF(ISBLANK(A17),"",COUNTIF(A:A,A17))</f>
@@ -8910,10 +8953,10 @@
         <v>33</v>
       </c>
       <c r="B18" s="11" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C18" s="12" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="D18" s="0" t="n">
         <f aca="false">IF(ISBLANK(A18),"",COUNTIF(A:A,A18))</f>
@@ -8933,10 +8976,10 @@
         <v>33</v>
       </c>
       <c r="B19" s="11" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C19" s="12" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="D19" s="0" t="n">
         <f aca="false">IF(ISBLANK(A19),"",COUNTIF(A:A,A19))</f>
@@ -8956,10 +8999,10 @@
         <v>33</v>
       </c>
       <c r="B20" s="11" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C20" s="12" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="D20" s="0" t="n">
         <f aca="false">IF(ISBLANK(A20),"",COUNTIF(A:A,A20))</f>
@@ -8979,10 +9022,10 @@
         <v>33</v>
       </c>
       <c r="B21" s="8" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C21" s="17" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="D21" s="0" t="n">
         <f aca="false">IF(ISBLANK(A21),"",COUNTIF(A:A,A21))</f>
@@ -8994,7 +9037,7 @@
       </c>
       <c r="F21" s="0" t="n">
         <f aca="false">IF(ISBLANK(C21),"",COUNTIF(C:C,C21))</f>
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9002,9 +9045,9 @@
         <v>33</v>
       </c>
       <c r="B22" s="21" t="s">
-        <v>82</v>
-      </c>
-      <c r="C22" s="12" t="s">
+        <v>83</v>
+      </c>
+      <c r="C22" s="8" t="s">
         <v>72</v>
       </c>
       <c r="D22" s="0" t="n">
@@ -9017,7 +9060,7 @@
       </c>
       <c r="F22" s="0" t="n">
         <f aca="false">IF(ISBLANK(C22),"",COUNTIF(C:C,C22))</f>
-        <v>11</v>
+        <v>18</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9025,10 +9068,10 @@
         <v>33</v>
       </c>
       <c r="B23" s="21" t="s">
-        <v>82</v>
-      </c>
-      <c r="C23" s="11" t="s">
-        <v>70</v>
+        <v>83</v>
+      </c>
+      <c r="C23" s="12" t="s">
+        <v>73</v>
       </c>
       <c r="D23" s="0" t="n">
         <f aca="false">IF(ISBLANK(A23),"",COUNTIF(A:A,A23))</f>
@@ -9040,18 +9083,18 @@
       </c>
       <c r="F23" s="0" t="n">
         <f aca="false">IF(ISBLANK(C23),"",COUNTIF(C:C,C23))</f>
-        <v>6</v>
+        <v>11</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="11" t="s">
         <v>33</v>
       </c>
-      <c r="B24" s="21" t="s">
-        <v>82</v>
-      </c>
-      <c r="C24" s="22" t="s">
-        <v>83</v>
+      <c r="B24" s="22" t="s">
+        <v>84</v>
+      </c>
+      <c r="C24" s="12" t="s">
+        <v>73</v>
       </c>
       <c r="D24" s="0" t="n">
         <f aca="false">IF(ISBLANK(A24),"",COUNTIF(A:A,A24))</f>
@@ -9063,7 +9106,7 @@
       </c>
       <c r="F24" s="0" t="n">
         <f aca="false">IF(ISBLANK(C24),"",COUNTIF(C:C,C24))</f>
-        <v>3</v>
+        <v>11</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9071,9 +9114,9 @@
         <v>33</v>
       </c>
       <c r="B25" s="22" t="s">
-        <v>83</v>
-      </c>
-      <c r="C25" s="8" t="s">
+        <v>84</v>
+      </c>
+      <c r="C25" s="11" t="s">
         <v>71</v>
       </c>
       <c r="D25" s="0" t="n">
@@ -9082,11 +9125,11 @@
       </c>
       <c r="E25" s="0" t="n">
         <f aca="false">IF(ISBLANK(B25),"",COUNTIF(B:B,B25))</f>
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F25" s="0" t="n">
         <f aca="false">IF(ISBLANK(C25),"",COUNTIF(C:C,C25))</f>
-        <v>18</v>
+        <v>6</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9094,10 +9137,10 @@
         <v>33</v>
       </c>
       <c r="B26" s="22" t="s">
+        <v>84</v>
+      </c>
+      <c r="C26" s="21" t="s">
         <v>83</v>
-      </c>
-      <c r="C26" s="12" t="s">
-        <v>72</v>
       </c>
       <c r="D26" s="0" t="n">
         <f aca="false">IF(ISBLANK(A26),"",COUNTIF(A:A,A26))</f>
@@ -9105,11 +9148,11 @@
       </c>
       <c r="E26" s="0" t="n">
         <f aca="false">IF(ISBLANK(B26),"",COUNTIF(B:B,B26))</f>
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F26" s="0" t="n">
         <f aca="false">IF(ISBLANK(C26),"",COUNTIF(C:C,C26))</f>
-        <v>11</v>
+        <v>3</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9117,10 +9160,10 @@
         <v>33</v>
       </c>
       <c r="B27" s="16" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="C27" s="12" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="D27" s="0" t="n">
         <f aca="false">IF(ISBLANK(A27),"",COUNTIF(A:A,A27))</f>
@@ -9140,10 +9183,10 @@
         <v>33</v>
       </c>
       <c r="B28" s="16" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="C28" s="23" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="D28" s="0" t="n">
         <f aca="false">IF(ISBLANK(A28),"",COUNTIF(A:A,A28))</f>
@@ -9163,10 +9206,10 @@
         <v>33</v>
       </c>
       <c r="B29" s="15" t="s">
+        <v>76</v>
+      </c>
+      <c r="C29" s="14" t="s">
         <v>75</v>
-      </c>
-      <c r="C29" s="14" t="s">
-        <v>74</v>
       </c>
       <c r="D29" s="0" t="n">
         <f aca="false">IF(ISBLANK(A29),"",COUNTIF(A:A,A29))</f>
@@ -9186,10 +9229,10 @@
         <v>33</v>
       </c>
       <c r="B30" s="15" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C30" s="16" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="D30" s="0" t="n">
         <f aca="false">IF(ISBLANK(A30),"",COUNTIF(A:A,A30))</f>
@@ -9209,10 +9252,10 @@
         <v>33</v>
       </c>
       <c r="B31" s="20" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="C31" s="8" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="D31" s="0" t="n">
         <f aca="false">IF(ISBLANK(A31),"",COUNTIF(A:A,A31))</f>
@@ -9232,10 +9275,10 @@
         <v>33</v>
       </c>
       <c r="B32" s="12" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="C32" s="17" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="D32" s="0" t="n">
         <f aca="false">IF(ISBLANK(A32),"",COUNTIF(A:A,A32))</f>
@@ -9247,15 +9290,15 @@
       </c>
       <c r="F32" s="0" t="n">
         <f aca="false">IF(ISBLANK(C32),"",COUNTIF(C:C,C32))</f>
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="21" t="s">
-        <v>85</v>
+      <c r="A33" s="22" t="s">
+        <v>86</v>
       </c>
       <c r="B33" s="8" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="D33" s="0" t="n">
         <f aca="false">IF(ISBLANK(A33),"",COUNTIF(A:A,A33))</f>
@@ -9271,11 +9314,11 @@
       </c>
     </row>
     <row r="34" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="21" t="s">
-        <v>85</v>
+      <c r="A34" s="22" t="s">
+        <v>86</v>
       </c>
       <c r="B34" s="8" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="D34" s="0" t="n">
         <f aca="false">IF(ISBLANK(A34),"",COUNTIF(A:A,A34))</f>
@@ -9291,11 +9334,11 @@
       </c>
     </row>
     <row r="35" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="21" t="s">
-        <v>85</v>
+      <c r="A35" s="22" t="s">
+        <v>86</v>
       </c>
       <c r="B35" s="8" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="D35" s="0" t="n">
         <f aca="false">IF(ISBLANK(A35),"",COUNTIF(A:A,A35))</f>
@@ -9311,11 +9354,11 @@
       </c>
     </row>
     <row r="36" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="21" t="s">
-        <v>85</v>
+      <c r="A36" s="22" t="s">
+        <v>86</v>
       </c>
       <c r="B36" s="8" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="D36" s="0" t="n">
         <f aca="false">IF(ISBLANK(A36),"",COUNTIF(A:A,A36))</f>
@@ -9331,11 +9374,11 @@
       </c>
     </row>
     <row r="37" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="21" t="s">
-        <v>85</v>
+      <c r="A37" s="22" t="s">
+        <v>86</v>
       </c>
       <c r="B37" s="21" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="D37" s="0" t="n">
         <f aca="false">IF(ISBLANK(A37),"",COUNTIF(A:A,A37))</f>
@@ -9351,10 +9394,10 @@
       </c>
     </row>
     <row r="38" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="21" t="s">
-        <v>85</v>
-      </c>
-      <c r="B38" s="22" t="s">
+      <c r="A38" s="22" t="s">
+        <v>86</v>
+      </c>
+      <c r="B38" s="21" t="s">
         <v>83</v>
       </c>
       <c r="D38" s="0" t="n">
@@ -9363,7 +9406,7 @@
       </c>
       <c r="E38" s="0" t="n">
         <f aca="false">IF(ISBLANK(B38),"",COUNTIF(B:B,B38))</f>
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F38" s="0" t="str">
         <f aca="false">IF(ISBLANK(C38),"",COUNTIF(C:C,C38))</f>
@@ -9371,11 +9414,11 @@
       </c>
     </row>
     <row r="39" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="21" t="s">
-        <v>85</v>
+      <c r="A39" s="22" t="s">
+        <v>86</v>
       </c>
       <c r="B39" s="22" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="D39" s="0" t="n">
         <f aca="false">IF(ISBLANK(A39),"",COUNTIF(A:A,A39))</f>
@@ -9383,7 +9426,7 @@
       </c>
       <c r="E39" s="0" t="n">
         <f aca="false">IF(ISBLANK(B39),"",COUNTIF(B:B,B39))</f>
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F39" s="0" t="str">
         <f aca="false">IF(ISBLANK(C39),"",COUNTIF(C:C,C39))</f>
@@ -9391,11 +9434,11 @@
       </c>
     </row>
     <row r="40" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="21" t="s">
-        <v>85</v>
+      <c r="A40" s="22" t="s">
+        <v>86</v>
       </c>
       <c r="B40" s="17" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="D40" s="0" t="n">
         <f aca="false">IF(ISBLANK(A40),"",COUNTIF(A:A,A40))</f>
@@ -9411,11 +9454,11 @@
       </c>
     </row>
     <row r="41" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="21" t="s">
-        <v>85</v>
+      <c r="A41" s="22" t="s">
+        <v>86</v>
       </c>
       <c r="B41" s="17" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="D41" s="0" t="n">
         <f aca="false">IF(ISBLANK(A41),"",COUNTIF(A:A,A41))</f>
@@ -9431,11 +9474,11 @@
       </c>
     </row>
     <row r="42" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A42" s="21" t="s">
-        <v>85</v>
+      <c r="A42" s="22" t="s">
+        <v>86</v>
       </c>
       <c r="B42" s="17" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="D42" s="0" t="n">
         <f aca="false">IF(ISBLANK(A42),"",COUNTIF(A:A,A42))</f>
@@ -9451,11 +9494,11 @@
       </c>
     </row>
     <row r="43" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A43" s="21" t="s">
-        <v>85</v>
+      <c r="A43" s="22" t="s">
+        <v>86</v>
       </c>
       <c r="B43" s="24" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="D43" s="0" t="n">
         <f aca="false">IF(ISBLANK(A43),"",COUNTIF(A:A,A43))</f>
@@ -9471,11 +9514,11 @@
       </c>
     </row>
     <row r="44" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A44" s="21" t="s">
-        <v>85</v>
+      <c r="A44" s="22" t="s">
+        <v>86</v>
       </c>
       <c r="B44" s="24" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="D44" s="0" t="n">
         <f aca="false">IF(ISBLANK(A44),"",COUNTIF(A:A,A44))</f>
@@ -9495,10 +9538,10 @@
         <v>19</v>
       </c>
       <c r="B45" s="11" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C45" s="12" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="D45" s="0" t="n">
         <f aca="false">IF(ISBLANK(A45),"",COUNTIF(A:A,A45))</f>
@@ -9518,10 +9561,10 @@
         <v>19</v>
       </c>
       <c r="B46" s="11" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C46" s="12" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="D46" s="0" t="n">
         <f aca="false">IF(ISBLANK(A46),"",COUNTIF(A:A,A46))</f>
@@ -9541,9 +9584,9 @@
         <v>19</v>
       </c>
       <c r="B47" s="11" t="s">
-        <v>70</v>
-      </c>
-      <c r="C47" s="22" t="s">
+        <v>71</v>
+      </c>
+      <c r="C47" s="21" t="s">
         <v>83</v>
       </c>
       <c r="D47" s="0" t="n">
@@ -9564,10 +9607,10 @@
         <v>19</v>
       </c>
       <c r="B48" s="8" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C48" s="20" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="D48" s="0" t="n">
         <f aca="false">IF(ISBLANK(A48),"",COUNTIF(A:A,A48))</f>
@@ -9586,11 +9629,11 @@
       <c r="A49" s="20" t="s">
         <v>19</v>
       </c>
-      <c r="B49" s="22" t="s">
+      <c r="B49" s="21" t="s">
         <v>83</v>
       </c>
       <c r="C49" s="11" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="D49" s="0" t="n">
         <f aca="false">IF(ISBLANK(A49),"",COUNTIF(A:A,A49))</f>
@@ -9598,7 +9641,7 @@
       </c>
       <c r="E49" s="0" t="n">
         <f aca="false">IF(ISBLANK(B49),"",COUNTIF(B:B,B49))</f>
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F49" s="0" t="n">
         <f aca="false">IF(ISBLANK(C49),"",COUNTIF(C:C,C49))</f>
@@ -9609,11 +9652,11 @@
       <c r="A50" s="20" t="s">
         <v>19</v>
       </c>
-      <c r="B50" s="22" t="s">
+      <c r="B50" s="21" t="s">
         <v>83</v>
       </c>
       <c r="C50" s="11" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="D50" s="0" t="n">
         <f aca="false">IF(ISBLANK(A50),"",COUNTIF(A:A,A50))</f>
@@ -9621,7 +9664,7 @@
       </c>
       <c r="E50" s="0" t="n">
         <f aca="false">IF(ISBLANK(B50),"",COUNTIF(B:B,B50))</f>
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F50" s="0" t="n">
         <f aca="false">IF(ISBLANK(C50),"",COUNTIF(C:C,C50))</f>
@@ -9633,10 +9676,10 @@
         <v>19</v>
       </c>
       <c r="B51" s="16" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="C51" s="12" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="D51" s="0" t="n">
         <f aca="false">IF(ISBLANK(A51),"",COUNTIF(A:A,A51))</f>
@@ -9656,10 +9699,10 @@
         <v>19</v>
       </c>
       <c r="B52" s="16" t="s">
+        <v>77</v>
+      </c>
+      <c r="C52" s="15" t="s">
         <v>76</v>
-      </c>
-      <c r="C52" s="15" t="s">
-        <v>75</v>
       </c>
       <c r="D52" s="0" t="n">
         <f aca="false">IF(ISBLANK(A52),"",COUNTIF(A:A,A52))</f>
@@ -9679,10 +9722,10 @@
         <v>19</v>
       </c>
       <c r="B53" s="15" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C53" s="19" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="D53" s="0" t="n">
         <f aca="false">IF(ISBLANK(A53),"",COUNTIF(A:A,A53))</f>
@@ -9702,10 +9745,10 @@
         <v>19</v>
       </c>
       <c r="B54" s="20" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="C54" s="8" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="D54" s="0" t="n">
         <f aca="false">IF(ISBLANK(A54),"",COUNTIF(A:A,A54))</f>
@@ -9725,10 +9768,10 @@
         <v>19</v>
       </c>
       <c r="B55" s="25" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="C55" s="8" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="D55" s="0" t="n">
         <f aca="false">IF(ISBLANK(A55),"",COUNTIF(A:A,A55))</f>
@@ -9745,13 +9788,13 @@
     </row>
     <row r="56" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="15" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="B56" s="14" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="C56" s="15" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="D56" s="0" t="n">
         <f aca="false">IF(ISBLANK(A56),"",COUNTIF(A:A,A56))</f>
@@ -9768,13 +9811,13 @@
     </row>
     <row r="57" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="15" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="B57" s="14" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="C57" s="15" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="D57" s="0" t="n">
         <f aca="false">IF(ISBLANK(A57),"",COUNTIF(A:A,A57))</f>
@@ -9791,13 +9834,13 @@
     </row>
     <row r="58" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="15" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="B58" s="14" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="C58" s="15" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="D58" s="0" t="n">
         <f aca="false">IF(ISBLANK(A58),"",COUNTIF(A:A,A58))</f>
@@ -9814,13 +9857,13 @@
     </row>
     <row r="59" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="15" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="B59" s="14" t="s">
+        <v>75</v>
+      </c>
+      <c r="C59" s="13" t="s">
         <v>74</v>
-      </c>
-      <c r="C59" s="13" t="s">
-        <v>73</v>
       </c>
       <c r="D59" s="0" t="n">
         <f aca="false">IF(ISBLANK(A59),"",COUNTIF(A:A,A59))</f>
@@ -9837,13 +9880,13 @@
     </row>
     <row r="60" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="15" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="B60" s="16" t="s">
+        <v>77</v>
+      </c>
+      <c r="C60" s="15" t="s">
         <v>76</v>
-      </c>
-      <c r="C60" s="15" t="s">
-        <v>75</v>
       </c>
       <c r="D60" s="0" t="n">
         <f aca="false">IF(ISBLANK(A60),"",COUNTIF(A:A,A60))</f>
@@ -9860,13 +9903,13 @@
     </row>
     <row r="61" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="15" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="B61" s="15" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C61" s="19" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="D61" s="0" t="n">
         <f aca="false">IF(ISBLANK(A61),"",COUNTIF(A:A,A61))</f>
@@ -9883,13 +9926,13 @@
     </row>
     <row r="62" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="15" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="B62" s="19" t="s">
+        <v>81</v>
+      </c>
+      <c r="C62" s="18" t="s">
         <v>80</v>
-      </c>
-      <c r="C62" s="18" t="s">
-        <v>79</v>
       </c>
       <c r="D62" s="0" t="n">
         <f aca="false">IF(ISBLANK(A62),"",COUNTIF(A:A,A62))</f>
@@ -9906,13 +9949,13 @@
     </row>
     <row r="63" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="15" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="B63" s="19" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="C63" s="10" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="D63" s="0" t="n">
         <f aca="false">IF(ISBLANK(A63),"",COUNTIF(A:A,A63))</f>
@@ -9929,13 +9972,13 @@
     </row>
     <row r="64" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="15" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="B64" s="17" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="C64" s="8" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="D64" s="0" t="n">
         <f aca="false">IF(ISBLANK(A64),"",COUNTIF(A:A,A64))</f>
@@ -9952,13 +9995,13 @@
     </row>
     <row r="65" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="15" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="B65" s="12" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="C65" s="11" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="D65" s="0" t="n">
         <f aca="false">IF(ISBLANK(A65),"",COUNTIF(A:A,A65))</f>
@@ -9974,68 +10017,68 @@
       </c>
     </row>
     <row r="66" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A66" s="8" t="s">
-        <v>36</v>
-      </c>
-      <c r="B66" s="18" t="s">
-        <v>79</v>
-      </c>
-      <c r="C66" s="8" t="s">
+      <c r="A66" s="21" t="s">
+        <v>90</v>
+      </c>
+      <c r="B66" s="11" t="s">
         <v>71</v>
+      </c>
+      <c r="C66" s="12" t="s">
+        <v>73</v>
       </c>
       <c r="D66" s="0" t="n">
         <f aca="false">IF(ISBLANK(A66),"",COUNTIF(A:A,A66))</f>
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E66" s="0" t="n">
         <f aca="false">IF(ISBLANK(B66),"",COUNTIF(B:B,B66))</f>
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="F66" s="0" t="n">
         <f aca="false">IF(ISBLANK(C66),"",COUNTIF(C:C,C66))</f>
-        <v>18</v>
+        <v>11</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A67" s="8" t="s">
-        <v>36</v>
-      </c>
-      <c r="B67" s="18" t="s">
-        <v>79</v>
-      </c>
-      <c r="C67" s="8" t="s">
-        <v>71</v>
+      <c r="A67" s="21" t="s">
+        <v>90</v>
+      </c>
+      <c r="B67" s="8" t="s">
+        <v>72</v>
+      </c>
+      <c r="C67" s="17" t="s">
+        <v>78</v>
       </c>
       <c r="D67" s="0" t="n">
         <f aca="false">IF(ISBLANK(A67),"",COUNTIF(A:A,A67))</f>
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E67" s="0" t="n">
         <f aca="false">IF(ISBLANK(B67),"",COUNTIF(B:B,B67))</f>
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="F67" s="0" t="n">
         <f aca="false">IF(ISBLANK(C67),"",COUNTIF(C:C,C67))</f>
-        <v>18</v>
+        <v>5</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A68" s="8" t="s">
-        <v>36</v>
-      </c>
-      <c r="B68" s="18" t="s">
-        <v>79</v>
+      <c r="A68" s="21" t="s">
+        <v>90</v>
+      </c>
+      <c r="B68" s="21" t="s">
+        <v>83</v>
       </c>
       <c r="C68" s="8" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="D68" s="0" t="n">
         <f aca="false">IF(ISBLANK(A68),"",COUNTIF(A:A,A68))</f>
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E68" s="0" t="n">
         <f aca="false">IF(ISBLANK(B68),"",COUNTIF(B:B,B68))</f>
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F68" s="0" t="n">
         <f aca="false">IF(ISBLANK(C68),"",COUNTIF(C:C,C68))</f>
@@ -10043,45 +10086,45 @@
       </c>
     </row>
     <row r="69" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A69" s="8" t="s">
-        <v>36</v>
-      </c>
-      <c r="B69" s="18" t="s">
-        <v>79</v>
-      </c>
-      <c r="C69" s="8" t="s">
-        <v>71</v>
+      <c r="A69" s="21" t="s">
+        <v>90</v>
+      </c>
+      <c r="B69" s="21" t="s">
+        <v>83</v>
+      </c>
+      <c r="C69" s="17" t="s">
+        <v>78</v>
       </c>
       <c r="D69" s="0" t="n">
         <f aca="false">IF(ISBLANK(A69),"",COUNTIF(A:A,A69))</f>
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E69" s="0" t="n">
         <f aca="false">IF(ISBLANK(B69),"",COUNTIF(B:B,B69))</f>
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F69" s="0" t="n">
         <f aca="false">IF(ISBLANK(C69),"",COUNTIF(C:C,C69))</f>
-        <v>18</v>
+        <v>5</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A70" s="8" t="s">
-        <v>36</v>
-      </c>
-      <c r="B70" s="18" t="s">
-        <v>79</v>
+      <c r="A70" s="21" t="s">
+        <v>90</v>
+      </c>
+      <c r="B70" s="22" t="s">
+        <v>84</v>
       </c>
       <c r="C70" s="8" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="D70" s="0" t="n">
         <f aca="false">IF(ISBLANK(A70),"",COUNTIF(A:A,A70))</f>
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E70" s="0" t="n">
         <f aca="false">IF(ISBLANK(B70),"",COUNTIF(B:B,B70))</f>
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F70" s="0" t="n">
         <f aca="false">IF(ISBLANK(C70),"",COUNTIF(C:C,C70))</f>
@@ -10089,60 +10132,60 @@
       </c>
     </row>
     <row r="71" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A71" s="8" t="s">
-        <v>36</v>
-      </c>
-      <c r="B71" s="18" t="s">
-        <v>79</v>
-      </c>
-      <c r="C71" s="8" t="s">
-        <v>71</v>
+      <c r="A71" s="21" t="s">
+        <v>90</v>
+      </c>
+      <c r="B71" s="22" t="s">
+        <v>84</v>
+      </c>
+      <c r="C71" s="21" t="s">
+        <v>83</v>
       </c>
       <c r="D71" s="0" t="n">
         <f aca="false">IF(ISBLANK(A71),"",COUNTIF(A:A,A71))</f>
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E71" s="0" t="n">
         <f aca="false">IF(ISBLANK(B71),"",COUNTIF(B:B,B71))</f>
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F71" s="0" t="n">
         <f aca="false">IF(ISBLANK(C71),"",COUNTIF(C:C,C71))</f>
-        <v>18</v>
+        <v>3</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A72" s="22" t="s">
-        <v>89</v>
-      </c>
-      <c r="B72" s="11" t="s">
-        <v>70</v>
-      </c>
-      <c r="C72" s="12" t="s">
+      <c r="A72" s="21" t="s">
+        <v>90</v>
+      </c>
+      <c r="B72" s="26" t="s">
+        <v>91</v>
+      </c>
+      <c r="C72" s="8" t="s">
         <v>72</v>
       </c>
       <c r="D72" s="0" t="n">
         <f aca="false">IF(ISBLANK(A72),"",COUNTIF(A:A,A72))</f>
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E72" s="0" t="n">
         <f aca="false">IF(ISBLANK(B72),"",COUNTIF(B:B,B72))</f>
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="F72" s="0" t="n">
         <f aca="false">IF(ISBLANK(C72),"",COUNTIF(C:C,C72))</f>
-        <v>11</v>
+        <v>18</v>
       </c>
     </row>
     <row r="73" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A73" s="22" t="s">
-        <v>89</v>
-      </c>
-      <c r="B73" s="8" t="s">
-        <v>71</v>
-      </c>
-      <c r="C73" s="17" t="s">
-        <v>77</v>
+      <c r="A73" s="8" t="s">
+        <v>36</v>
+      </c>
+      <c r="B73" s="18" t="s">
+        <v>80</v>
+      </c>
+      <c r="C73" s="8" t="s">
+        <v>72</v>
       </c>
       <c r="D73" s="0" t="n">
         <f aca="false">IF(ISBLANK(A73),"",COUNTIF(A:A,A73))</f>
@@ -10150,22 +10193,22 @@
       </c>
       <c r="E73" s="0" t="n">
         <f aca="false">IF(ISBLANK(B73),"",COUNTIF(B:B,B73))</f>
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="F73" s="0" t="n">
         <f aca="false">IF(ISBLANK(C73),"",COUNTIF(C:C,C73))</f>
-        <v>4</v>
+        <v>18</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A74" s="22" t="s">
-        <v>89</v>
-      </c>
-      <c r="B74" s="21" t="s">
-        <v>82</v>
+      <c r="A74" s="8" t="s">
+        <v>36</v>
+      </c>
+      <c r="B74" s="18" t="s">
+        <v>80</v>
       </c>
       <c r="C74" s="8" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="D74" s="0" t="n">
         <f aca="false">IF(ISBLANK(A74),"",COUNTIF(A:A,A74))</f>
@@ -10173,7 +10216,7 @@
       </c>
       <c r="E74" s="0" t="n">
         <f aca="false">IF(ISBLANK(B74),"",COUNTIF(B:B,B74))</f>
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F74" s="0" t="n">
         <f aca="false">IF(ISBLANK(C74),"",COUNTIF(C:C,C74))</f>
@@ -10181,14 +10224,14 @@
       </c>
     </row>
     <row r="75" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A75" s="22" t="s">
-        <v>89</v>
-      </c>
-      <c r="B75" s="21" t="s">
-        <v>82</v>
-      </c>
-      <c r="C75" s="22" t="s">
-        <v>83</v>
+      <c r="A75" s="8" t="s">
+        <v>36</v>
+      </c>
+      <c r="B75" s="18" t="s">
+        <v>80</v>
+      </c>
+      <c r="C75" s="8" t="s">
+        <v>72</v>
       </c>
       <c r="D75" s="0" t="n">
         <f aca="false">IF(ISBLANK(A75),"",COUNTIF(A:A,A75))</f>
@@ -10196,22 +10239,22 @@
       </c>
       <c r="E75" s="0" t="n">
         <f aca="false">IF(ISBLANK(B75),"",COUNTIF(B:B,B75))</f>
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F75" s="0" t="n">
         <f aca="false">IF(ISBLANK(C75),"",COUNTIF(C:C,C75))</f>
-        <v>3</v>
+        <v>18</v>
       </c>
     </row>
     <row r="76" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A76" s="22" t="s">
-        <v>89</v>
-      </c>
-      <c r="B76" s="22" t="s">
-        <v>83</v>
+      <c r="A76" s="8" t="s">
+        <v>36</v>
+      </c>
+      <c r="B76" s="18" t="s">
+        <v>80</v>
       </c>
       <c r="C76" s="8" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="D76" s="0" t="n">
         <f aca="false">IF(ISBLANK(A76),"",COUNTIF(A:A,A76))</f>
@@ -10227,14 +10270,14 @@
       </c>
     </row>
     <row r="77" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A77" s="22" t="s">
-        <v>89</v>
-      </c>
-      <c r="B77" s="26" t="s">
-        <v>90</v>
+      <c r="A77" s="8" t="s">
+        <v>36</v>
+      </c>
+      <c r="B77" s="18" t="s">
+        <v>80</v>
       </c>
       <c r="C77" s="8" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="D77" s="0" t="n">
         <f aca="false">IF(ISBLANK(A77),"",COUNTIF(A:A,A77))</f>
@@ -10242,7 +10285,7 @@
       </c>
       <c r="E77" s="0" t="n">
         <f aca="false">IF(ISBLANK(B77),"",COUNTIF(B:B,B77))</f>
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="F77" s="0" t="n">
         <f aca="false">IF(ISBLANK(C77),"",COUNTIF(C:C,C77))</f>
@@ -10250,31 +10293,34 @@
       </c>
     </row>
     <row r="78" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A78" s="21" t="s">
-        <v>91</v>
-      </c>
-      <c r="B78" s="8" t="s">
-        <v>71</v>
+      <c r="A78" s="8" t="s">
+        <v>36</v>
+      </c>
+      <c r="B78" s="18" t="s">
+        <v>80</v>
+      </c>
+      <c r="C78" s="8" t="s">
+        <v>72</v>
       </c>
       <c r="D78" s="0" t="n">
         <f aca="false">IF(ISBLANK(A78),"",COUNTIF(A:A,A78))</f>
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="E78" s="0" t="n">
         <f aca="false">IF(ISBLANK(B78),"",COUNTIF(B:B,B78))</f>
-        <v>9</v>
-      </c>
-      <c r="F78" s="0" t="str">
+        <v>7</v>
+      </c>
+      <c r="F78" s="0" t="n">
         <f aca="false">IF(ISBLANK(C78),"",COUNTIF(C:C,C78))</f>
-        <v/>
+        <v>18</v>
       </c>
     </row>
     <row r="79" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A79" s="21" t="s">
-        <v>91</v>
-      </c>
-      <c r="B79" s="21" t="s">
-        <v>82</v>
+      <c r="A79" s="22" t="s">
+        <v>92</v>
+      </c>
+      <c r="B79" s="8" t="s">
+        <v>72</v>
       </c>
       <c r="D79" s="0" t="n">
         <f aca="false">IF(ISBLANK(A79),"",COUNTIF(A:A,A79))</f>
@@ -10282,7 +10328,7 @@
       </c>
       <c r="E79" s="0" t="n">
         <f aca="false">IF(ISBLANK(B79),"",COUNTIF(B:B,B79))</f>
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="F79" s="0" t="str">
         <f aca="false">IF(ISBLANK(C79),"",COUNTIF(C:C,C79))</f>
@@ -10290,11 +10336,11 @@
       </c>
     </row>
     <row r="80" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A80" s="21" t="s">
-        <v>91</v>
-      </c>
-      <c r="B80" s="21" t="s">
-        <v>82</v>
+      <c r="A80" s="22" t="s">
+        <v>92</v>
+      </c>
+      <c r="B80" s="22" t="s">
+        <v>84</v>
       </c>
       <c r="D80" s="0" t="n">
         <f aca="false">IF(ISBLANK(A80),"",COUNTIF(A:A,A80))</f>
@@ -10310,11 +10356,11 @@
       </c>
     </row>
     <row r="81" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A81" s="21" t="s">
-        <v>91</v>
-      </c>
-      <c r="B81" s="17" t="s">
-        <v>77</v>
+      <c r="A81" s="22" t="s">
+        <v>92</v>
+      </c>
+      <c r="B81" s="22" t="s">
+        <v>84</v>
       </c>
       <c r="D81" s="0" t="n">
         <f aca="false">IF(ISBLANK(A81),"",COUNTIF(A:A,A81))</f>
@@ -10322,7 +10368,7 @@
       </c>
       <c r="E81" s="0" t="n">
         <f aca="false">IF(ISBLANK(B81),"",COUNTIF(B:B,B81))</f>
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="F81" s="0" t="str">
         <f aca="false">IF(ISBLANK(C81),"",COUNTIF(C:C,C81))</f>
@@ -10330,37 +10376,34 @@
       </c>
     </row>
     <row r="82" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A82" s="25" t="s">
+      <c r="A82" s="22" t="s">
         <v>92</v>
       </c>
-      <c r="B82" s="8" t="s">
-        <v>71</v>
-      </c>
-      <c r="C82" s="18" t="s">
-        <v>79</v>
+      <c r="B82" s="17" t="s">
+        <v>78</v>
       </c>
       <c r="D82" s="0" t="n">
         <f aca="false">IF(ISBLANK(A82),"",COUNTIF(A:A,A82))</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E82" s="0" t="n">
         <f aca="false">IF(ISBLANK(B82),"",COUNTIF(B:B,B82))</f>
-        <v>9</v>
-      </c>
-      <c r="F82" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="F82" s="0" t="str">
         <f aca="false">IF(ISBLANK(C82),"",COUNTIF(C:C,C82))</f>
-        <v>5</v>
+        <v/>
       </c>
     </row>
     <row r="83" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A83" s="25" t="s">
-        <v>92</v>
-      </c>
-      <c r="B83" s="20" t="s">
-        <v>81</v>
+        <v>93</v>
+      </c>
+      <c r="B83" s="8" t="s">
+        <v>72</v>
       </c>
       <c r="C83" s="18" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="D83" s="0" t="n">
         <f aca="false">IF(ISBLANK(A83),"",COUNTIF(A:A,A83))</f>
@@ -10368,7 +10411,7 @@
       </c>
       <c r="E83" s="0" t="n">
         <f aca="false">IF(ISBLANK(B83),"",COUNTIF(B:B,B83))</f>
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="F83" s="0" t="n">
         <f aca="false">IF(ISBLANK(C83),"",COUNTIF(C:C,C83))</f>
@@ -10377,13 +10420,13 @@
     </row>
     <row r="84" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A84" s="25" t="s">
-        <v>92</v>
-      </c>
-      <c r="B84" s="25" t="s">
-        <v>87</v>
+        <v>93</v>
+      </c>
+      <c r="B84" s="20" t="s">
+        <v>82</v>
       </c>
       <c r="C84" s="18" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="D84" s="0" t="n">
         <f aca="false">IF(ISBLANK(A84),"",COUNTIF(A:A,A84))</f>
@@ -10391,7 +10434,7 @@
       </c>
       <c r="E84" s="0" t="n">
         <f aca="false">IF(ISBLANK(B84),"",COUNTIF(B:B,B84))</f>
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="F84" s="0" t="n">
         <f aca="false">IF(ISBLANK(C84),"",COUNTIF(C:C,C84))</f>
@@ -10399,14 +10442,14 @@
       </c>
     </row>
     <row r="85" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A85" s="19" t="s">
+      <c r="A85" s="25" t="s">
         <v>93</v>
       </c>
-      <c r="B85" s="14" t="s">
-        <v>74</v>
+      <c r="B85" s="25" t="s">
+        <v>88</v>
       </c>
       <c r="C85" s="18" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="D85" s="0" t="n">
         <f aca="false">IF(ISBLANK(A85),"",COUNTIF(A:A,A85))</f>
@@ -10414,7 +10457,7 @@
       </c>
       <c r="E85" s="0" t="n">
         <f aca="false">IF(ISBLANK(B85),"",COUNTIF(B:B,B85))</f>
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="F85" s="0" t="n">
         <f aca="false">IF(ISBLANK(C85),"",COUNTIF(C:C,C85))</f>
@@ -10423,13 +10466,13 @@
     </row>
     <row r="86" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A86" s="19" t="s">
-        <v>93</v>
-      </c>
-      <c r="B86" s="15" t="s">
+        <v>94</v>
+      </c>
+      <c r="B86" s="14" t="s">
         <v>75</v>
       </c>
-      <c r="C86" s="14" t="s">
-        <v>74</v>
+      <c r="C86" s="18" t="s">
+        <v>80</v>
       </c>
       <c r="D86" s="0" t="n">
         <f aca="false">IF(ISBLANK(A86),"",COUNTIF(A:A,A86))</f>
@@ -10437,22 +10480,22 @@
       </c>
       <c r="E86" s="0" t="n">
         <f aca="false">IF(ISBLANK(B86),"",COUNTIF(B:B,B86))</f>
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="F86" s="0" t="n">
         <f aca="false">IF(ISBLANK(C86),"",COUNTIF(C:C,C86))</f>
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="87" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A87" s="19" t="s">
-        <v>93</v>
-      </c>
-      <c r="B87" s="19" t="s">
-        <v>80</v>
-      </c>
-      <c r="C87" s="19" t="s">
-        <v>80</v>
+        <v>94</v>
+      </c>
+      <c r="B87" s="15" t="s">
+        <v>76</v>
+      </c>
+      <c r="C87" s="14" t="s">
+        <v>75</v>
       </c>
       <c r="D87" s="0" t="n">
         <f aca="false">IF(ISBLANK(A87),"",COUNTIF(A:A,A87))</f>
@@ -10460,7 +10503,7 @@
       </c>
       <c r="E87" s="0" t="n">
         <f aca="false">IF(ISBLANK(B87),"",COUNTIF(B:B,B87))</f>
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="F87" s="0" t="n">
         <f aca="false">IF(ISBLANK(C87),"",COUNTIF(C:C,C87))</f>
@@ -10468,14 +10511,14 @@
       </c>
     </row>
     <row r="88" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A88" s="27" t="s">
+      <c r="A88" s="19" t="s">
         <v>94</v>
       </c>
-      <c r="B88" s="14" t="s">
-        <v>74</v>
-      </c>
-      <c r="C88" s="15" t="s">
-        <v>75</v>
+      <c r="B88" s="19" t="s">
+        <v>81</v>
+      </c>
+      <c r="C88" s="19" t="s">
+        <v>81</v>
       </c>
       <c r="D88" s="0" t="n">
         <f aca="false">IF(ISBLANK(A88),"",COUNTIF(A:A,A88))</f>
@@ -10483,22 +10526,22 @@
       </c>
       <c r="E88" s="0" t="n">
         <f aca="false">IF(ISBLANK(B88),"",COUNTIF(B:B,B88))</f>
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="F88" s="0" t="n">
         <f aca="false">IF(ISBLANK(C88),"",COUNTIF(C:C,C88))</f>
-        <v>8</v>
+        <v>3</v>
       </c>
     </row>
     <row r="89" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A89" s="27" t="s">
-        <v>94</v>
-      </c>
-      <c r="B89" s="27" t="s">
         <v>95</v>
       </c>
-      <c r="C89" s="28" t="s">
-        <v>96</v>
+      <c r="B89" s="14" t="s">
+        <v>75</v>
+      </c>
+      <c r="C89" s="15" t="s">
+        <v>76</v>
       </c>
       <c r="D89" s="0" t="n">
         <f aca="false">IF(ISBLANK(A89),"",COUNTIF(A:A,A89))</f>
@@ -10506,22 +10549,22 @@
       </c>
       <c r="E89" s="0" t="n">
         <f aca="false">IF(ISBLANK(B89),"",COUNTIF(B:B,B89))</f>
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="F89" s="0" t="n">
         <f aca="false">IF(ISBLANK(C89),"",COUNTIF(C:C,C89))</f>
-        <v>2</v>
+        <v>8</v>
       </c>
     </row>
     <row r="90" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A90" s="27" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="B90" s="27" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="C90" s="28" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="D90" s="0" t="n">
         <f aca="false">IF(ISBLANK(A90),"",COUNTIF(A:A,A90))</f>
@@ -10537,30 +10580,53 @@
       </c>
     </row>
     <row r="91" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A91" s="16" t="s">
+      <c r="A91" s="27" t="s">
+        <v>95</v>
+      </c>
+      <c r="B91" s="27" t="s">
+        <v>96</v>
+      </c>
+      <c r="C91" s="28" t="s">
         <v>97</v>
-      </c>
-      <c r="B91" s="15" t="s">
-        <v>75</v>
-      </c>
-      <c r="C91" s="16" t="s">
-        <v>76</v>
       </c>
       <c r="D91" s="0" t="n">
         <f aca="false">IF(ISBLANK(A91),"",COUNTIF(A:A,A91))</f>
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E91" s="0" t="n">
         <f aca="false">IF(ISBLANK(B91),"",COUNTIF(B:B,B91))</f>
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="F91" s="0" t="n">
         <f aca="false">IF(ISBLANK(C91),"",COUNTIF(C:C,C91))</f>
         <v>2</v>
       </c>
     </row>
+    <row r="92" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A92" s="16" t="s">
+        <v>98</v>
+      </c>
+      <c r="B92" s="15" t="s">
+        <v>76</v>
+      </c>
+      <c r="C92" s="16" t="s">
+        <v>77</v>
+      </c>
+      <c r="D92" s="0" t="n">
+        <f aca="false">IF(ISBLANK(A92),"",COUNTIF(A:A,A92))</f>
+        <v>1</v>
+      </c>
+      <c r="E92" s="0" t="n">
+        <f aca="false">IF(ISBLANK(B92),"",COUNTIF(B:B,B92))</f>
+        <v>7</v>
+      </c>
+      <c r="F92" s="0" t="n">
+        <f aca="false">IF(ISBLANK(C92),"",COUNTIF(C:C,C92))</f>
+        <v>2</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:F91"/>
+  <autoFilter ref="A1:F92"/>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
   <pageSetup paperSize="9" scale="100" firstPageNumber="0" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" useFirstPageNumber="false" horizontalDpi="300" verticalDpi="300" copies="1"/>
@@ -10595,54 +10661,54 @@
   <sheetData>
     <row r="1" s="9" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="9" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="D1" s="9" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="G1" s="9" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="H1" s="3" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="J1" s="9" t="s">
+        <v>100</v>
+      </c>
+      <c r="K1" s="3" t="s">
         <v>99</v>
-      </c>
-      <c r="K1" s="3" t="s">
-        <v>98</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="10" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="B2" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!A:A,A2)</f>
         <v>16</v>
       </c>
       <c r="D2" s="11" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E2" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!B:B,D2)</f>
         <v>10</v>
       </c>
       <c r="G2" s="8" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="H2" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!C:C,G2)</f>
         <v>18</v>
       </c>
       <c r="J2" s="8" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="K2" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!B:B,J2)*2+COUNTIF(Tatjes!C:C,J2)</f>
@@ -10658,21 +10724,21 @@
         <v>15</v>
       </c>
       <c r="D3" s="8" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="E3" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!B:B,D3)</f>
         <v>9</v>
       </c>
       <c r="G3" s="12" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="H3" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!C:C,G3)</f>
         <v>11</v>
       </c>
       <c r="J3" s="11" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="K3" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!B:B,J3)*2+COUNTIF(Tatjes!C:C,J3)</f>
@@ -10680,29 +10746,29 @@
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="21" t="s">
-        <v>85</v>
+      <c r="A4" s="22" t="s">
+        <v>86</v>
       </c>
       <c r="B4" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!A:A,A4)</f>
         <v>12</v>
       </c>
       <c r="D4" s="14" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="E4" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!B:B,D4)</f>
         <v>9</v>
       </c>
       <c r="G4" s="15" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="H4" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!C:C,G4)</f>
         <v>8</v>
       </c>
       <c r="J4" s="15" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="K4" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!B:B,J4)*2+COUNTIF(Tatjes!C:C,J4)</f>
@@ -10718,21 +10784,21 @@
         <v>11</v>
       </c>
       <c r="D5" s="21" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="E5" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!B:B,D5)</f>
         <v>8</v>
       </c>
       <c r="G5" s="11" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="H5" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!C:C,G5)</f>
         <v>6</v>
       </c>
       <c r="J5" s="14" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="K5" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!B:B,J5)*2+COUNTIF(Tatjes!C:C,J5)</f>
@@ -10741,28 +10807,28 @@
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="15" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="B6" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!A:A,A6)</f>
         <v>10</v>
       </c>
       <c r="D6" s="22" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="E6" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!B:B,D6)</f>
-        <v>7</v>
-      </c>
-      <c r="G6" s="18" t="s">
-        <v>79</v>
+        <v>8</v>
+      </c>
+      <c r="G6" s="17" t="s">
+        <v>78</v>
       </c>
       <c r="H6" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!C:C,G6)</f>
         <v>5</v>
       </c>
-      <c r="J6" s="18" t="s">
-        <v>79</v>
+      <c r="J6" s="21" t="s">
+        <v>83</v>
       </c>
       <c r="K6" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!B:B,J6)*2+COUNTIF(Tatjes!C:C,J6)</f>
@@ -10770,59 +10836,59 @@
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="8" t="s">
-        <v>36</v>
+      <c r="A7" s="21" t="s">
+        <v>90</v>
       </c>
       <c r="B7" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!A:A,A7)</f>
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D7" s="16" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="E7" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!B:B,D7)</f>
         <v>7</v>
       </c>
-      <c r="G7" s="17" t="s">
-        <v>77</v>
+      <c r="G7" s="18" t="s">
+        <v>80</v>
       </c>
       <c r="H7" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!C:C,G7)</f>
-        <v>4</v>
-      </c>
-      <c r="J7" s="22" t="s">
-        <v>83</v>
+        <v>5</v>
+      </c>
+      <c r="J7" s="18" t="s">
+        <v>80</v>
       </c>
       <c r="K7" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!B:B,J7)*2+COUNTIF(Tatjes!C:C,J7)</f>
-        <v>17</v>
+        <v>19</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="22" t="s">
-        <v>89</v>
+      <c r="A8" s="8" t="s">
+        <v>36</v>
       </c>
       <c r="B8" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!A:A,A8)</f>
         <v>6</v>
       </c>
       <c r="D8" s="15" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="E8" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!B:B,D8)</f>
         <v>7</v>
       </c>
       <c r="G8" s="19" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="H8" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!C:C,G8)</f>
         <v>3</v>
       </c>
-      <c r="J8" s="21" t="s">
-        <v>82</v>
+      <c r="J8" s="22" t="s">
+        <v>84</v>
       </c>
       <c r="K8" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!B:B,J8)*2+COUNTIF(Tatjes!C:C,J8)</f>
@@ -10830,21 +10896,21 @@
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="21" t="s">
-        <v>91</v>
+      <c r="A9" s="22" t="s">
+        <v>92</v>
       </c>
       <c r="B9" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!A:A,A9)</f>
         <v>4</v>
       </c>
       <c r="D9" s="18" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="E9" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!B:B,D9)</f>
         <v>7</v>
       </c>
-      <c r="G9" s="22" t="s">
+      <c r="G9" s="21" t="s">
         <v>83</v>
       </c>
       <c r="H9" s="1" t="n">
@@ -10852,7 +10918,7 @@
         <v>3</v>
       </c>
       <c r="J9" s="16" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="K9" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!B:B,J9)*2+COUNTIF(Tatjes!C:C,J9)</f>
@@ -10861,28 +10927,28 @@
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="25" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="B10" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!A:A,A10)</f>
         <v>3</v>
       </c>
       <c r="D10" s="19" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="E10" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!B:B,D10)</f>
         <v>5</v>
       </c>
       <c r="G10" s="13" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="H10" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!C:C,G10)</f>
         <v>3</v>
       </c>
       <c r="J10" s="12" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="K10" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!B:B,J10)*2+COUNTIF(Tatjes!C:C,J10)</f>
@@ -10891,58 +10957,58 @@
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="19" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="B11" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!A:A,A11)</f>
         <v>3</v>
       </c>
       <c r="D11" s="17" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="E11" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!B:B,D11)</f>
         <v>5</v>
       </c>
       <c r="G11" s="14" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="H11" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!C:C,G11)</f>
         <v>3</v>
       </c>
       <c r="J11" s="17" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="K11" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!B:B,J11)*2+COUNTIF(Tatjes!C:C,J11)</f>
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="27" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="B12" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!A:A,A12)</f>
         <v>3</v>
       </c>
       <c r="D12" s="20" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="E12" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!B:B,D12)</f>
         <v>5</v>
       </c>
       <c r="G12" s="28" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="H12" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!C:C,G12)</f>
         <v>2</v>
       </c>
       <c r="J12" s="19" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="K12" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!B:B,J12)*2+COUNTIF(Tatjes!C:C,J12)</f>
@@ -10951,28 +11017,28 @@
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="16" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="B13" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!A:A,A13)</f>
         <v>1</v>
       </c>
       <c r="D13" s="12" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="E13" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!B:B,D13)</f>
         <v>2</v>
       </c>
       <c r="G13" s="16" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="H13" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!C:C,G13)</f>
         <v>2</v>
       </c>
       <c r="J13" s="20" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="K13" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!B:B,J13)*2+COUNTIF(Tatjes!C:C,J13)</f>
@@ -10981,21 +11047,21 @@
     </row>
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D14" s="27" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="E14" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!B:B,D14)</f>
         <v>2</v>
       </c>
       <c r="G14" s="20" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="H14" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!C:C,G14)</f>
         <v>1</v>
       </c>
       <c r="J14" s="13" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="K14" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!B:B,J14)*2+COUNTIF(Tatjes!C:C,J14)</f>
@@ -11008,24 +11074,24 @@
       </c>
       <c r="B15" s="3" t="n">
         <f aca="false">COUNTA(Tatjes!A:A)-1</f>
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="D15" s="13" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="E15" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!B:B,D15)</f>
         <v>2</v>
       </c>
       <c r="G15" s="23" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="H15" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!C:C,G15)</f>
         <v>1</v>
       </c>
       <c r="J15" s="27" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="K15" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!B:B,J15)*2+COUNTIF(Tatjes!C:C,J15)</f>
@@ -11034,21 +11100,21 @@
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D16" s="24" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="E16" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!B:B,D16)</f>
         <v>2</v>
       </c>
       <c r="G16" s="27" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="H16" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!C:C,G16)</f>
         <v>0</v>
       </c>
       <c r="J16" s="24" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="K16" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!B:B,J16)*2+COUNTIF(Tatjes!C:C,J16)</f>
@@ -11057,21 +11123,21 @@
     </row>
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D17" s="25" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="E17" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!B:B,D17)</f>
         <v>2</v>
       </c>
-      <c r="G17" s="21" t="s">
-        <v>82</v>
+      <c r="G17" s="22" t="s">
+        <v>84</v>
       </c>
       <c r="H17" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!C:C,G17)</f>
         <v>0</v>
       </c>
       <c r="J17" s="25" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="K17" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!B:B,J17)*2+COUNTIF(Tatjes!C:C,J17)</f>
@@ -11080,21 +11146,21 @@
     </row>
     <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D18" s="26" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="E18" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!B:B,D18)</f>
         <v>1</v>
       </c>
       <c r="G18" s="24" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="H18" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!C:C,G18)</f>
         <v>0</v>
       </c>
       <c r="J18" s="28" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="K18" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!B:B,J18)*2+COUNTIF(Tatjes!C:C,J18)</f>
@@ -11103,21 +11169,21 @@
     </row>
     <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D19" s="28" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="E19" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!B:B,D19)</f>
         <v>0</v>
       </c>
       <c r="G19" s="26" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="H19" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!C:C,G19)</f>
         <v>0</v>
       </c>
       <c r="J19" s="26" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="K19" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!B:B,J19)*2+COUNTIF(Tatjes!C:C,J19)</f>
@@ -11126,21 +11192,21 @@
     </row>
     <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D20" s="23" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="E20" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!B:B,D20)</f>
         <v>0</v>
       </c>
       <c r="G20" s="25" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="H20" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!C:C,G20)</f>
         <v>0</v>
       </c>
       <c r="J20" s="23" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="K20" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!B:B,J20)*2+COUNTIF(Tatjes!C:C,J20)</f>

</xml_diff>

<commit_message>
Sync from vault 2026-06-03 09:55:22
</commit_message>
<xml_diff>
--- a/content/Archief/0. PDFs & docs/Obol docs & forms/Irmijn Inc/Irma backup log.xlsx
+++ b/content/Archief/0. PDFs & docs/Obol docs & forms/Irmijn Inc/Irma backup log.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="3"/>
   </bookViews>
   <sheets>
     <sheet name="Logboek" sheetId="1" state="visible" r:id="rId2"/>
@@ -15,10 +15,11 @@
   </sheets>
   <definedNames>
     <definedName function="false" hidden="true" localSheetId="3" name="_xlnm._FilterDatabase" vbProcedure="false">Tatdata!$A$1:$B$13</definedName>
-    <definedName function="false" hidden="true" localSheetId="2" name="_xlnm._FilterDatabase" vbProcedure="false">Tatjes!$A$1:$F$92</definedName>
-    <definedName function="false" hidden="false" localSheetId="2" name="_xlnm._FilterDatabase" vbProcedure="false">Tatjes!$A$1:$F$91</definedName>
-    <definedName function="false" hidden="false" localSheetId="2" name="_xlnm._FilterDatabase_0" vbProcedure="false">Tatjes!$A$1:$F$90</definedName>
-    <definedName function="false" hidden="false" localSheetId="2" name="_xlnm._FilterDatabase_0_0" vbProcedure="false">Tatjes!$A$1:$F$88</definedName>
+    <definedName function="false" hidden="true" localSheetId="2" name="_xlnm._FilterDatabase" vbProcedure="false">Tatjes!$A$1:$F$93</definedName>
+    <definedName function="false" hidden="false" localSheetId="2" name="_xlnm._FilterDatabase" vbProcedure="false">Tatjes!$A$1:$F$92</definedName>
+    <definedName function="false" hidden="false" localSheetId="2" name="_xlnm._FilterDatabase_0" vbProcedure="false">Tatjes!$A$1:$F$91</definedName>
+    <definedName function="false" hidden="false" localSheetId="2" name="_xlnm._FilterDatabase_0_0" vbProcedure="false">Tatjes!$A$1:$F$90</definedName>
+    <definedName function="false" hidden="false" localSheetId="2" name="_xlnm._FilterDatabase_0_0_0" vbProcedure="false">Tatjes!$A$1:$F$88</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.001"/>
   <extLst>
@@ -30,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="490" uniqueCount="101">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="493" uniqueCount="101">
   <si>
     <t xml:space="preserve">Pagina</t>
   </si>
@@ -1597,11 +1598,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="70902698"/>
-        <c:axId val="31228987"/>
+        <c:axId val="60225116"/>
+        <c:axId val="23597406"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="70902698"/>
+        <c:axId val="60225116"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1657,14 +1658,14 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="31228987"/>
+        <c:crossAx val="23597406"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
         <c:lblOffset val="100"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="31228987"/>
+        <c:axId val="23597406"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1729,7 +1730,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="70902698"/>
+        <c:crossAx val="60225116"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -4790,11 +4791,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="23335886"/>
-        <c:axId val="49722141"/>
+        <c:axId val="37232827"/>
+        <c:axId val="6225379"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="23335886"/>
+        <c:axId val="37232827"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -4850,14 +4851,14 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="49722141"/>
+        <c:crossAx val="6225379"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
         <c:lblOffset val="100"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="49722141"/>
+        <c:axId val="6225379"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -4922,7 +4923,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="23335886"/>
+        <c:crossAx val="37232827"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -5010,10 +5011,10 @@
           <c:layoutTarget val="inner"/>
           <c:xMode val="edge"/>
           <c:yMode val="edge"/>
-          <c:x val="0.0889597399349837"/>
-          <c:y val="0.110938194753224"/>
-          <c:w val="0.846086521630408"/>
-          <c:h val="0.793574922187639"/>
+          <c:x val="0.0889653016567677"/>
+          <c:y val="0.110950528071151"/>
+          <c:w val="0.846014379493592"/>
+          <c:h val="0.793440800444691"/>
         </c:manualLayout>
       </c:layout>
       <c:lineChart>
@@ -5145,11 +5146,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="35082363"/>
-        <c:axId val="87082147"/>
+        <c:axId val="48539564"/>
+        <c:axId val="1579423"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="35082363"/>
+        <c:axId val="48539564"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -5177,14 +5178,14 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="87082147"/>
+        <c:crossAx val="1579423"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
         <c:lblOffset val="100"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="87082147"/>
+        <c:axId val="1579423"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -5249,7 +5250,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="35082363"/>
+        <c:crossAx val="48539564"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -5287,9 +5288,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>179280</xdr:colOff>
+      <xdr:colOff>178920</xdr:colOff>
       <xdr:row>23</xdr:row>
-      <xdr:rowOff>42840</xdr:rowOff>
+      <xdr:rowOff>42480</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -5298,7 +5299,7 @@
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
         <a:off x="6578280" y="543600"/>
-        <a:ext cx="5757840" cy="3237840"/>
+        <a:ext cx="5757480" cy="3237480"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -5317,9 +5318,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>343080</xdr:colOff>
+      <xdr:colOff>342720</xdr:colOff>
       <xdr:row>52</xdr:row>
-      <xdr:rowOff>91080</xdr:rowOff>
+      <xdr:rowOff>90720</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -5328,7 +5329,7 @@
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
         <a:off x="6741360" y="5305320"/>
-        <a:ext cx="5758560" cy="3238560"/>
+        <a:ext cx="5758200" cy="3238200"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -5352,9 +5353,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>12</xdr:col>
-      <xdr:colOff>462600</xdr:colOff>
+      <xdr:colOff>462240</xdr:colOff>
       <xdr:row>21</xdr:row>
-      <xdr:rowOff>71280</xdr:rowOff>
+      <xdr:rowOff>70920</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -5363,7 +5364,7 @@
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
         <a:off x="2646720" y="246600"/>
-        <a:ext cx="5758200" cy="3238200"/>
+        <a:ext cx="5757840" cy="3237840"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -8550,7 +8551,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F92"/>
+  <dimension ref="A1:F93"/>
   <sheetFormatPr defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="9.63"/>
@@ -8738,7 +8739,7 @@
       </c>
       <c r="F8" s="0" t="n">
         <f aca="false">IF(ISBLANK(C8),"",COUNTIF(C:C,C8))</f>
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8960,7 +8961,7 @@
       </c>
       <c r="D18" s="0" t="n">
         <f aca="false">IF(ISBLANK(A18),"",COUNTIF(A:A,A18))</f>
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="E18" s="0" t="n">
         <f aca="false">IF(ISBLANK(B18),"",COUNTIF(B:B,B18))</f>
@@ -8983,7 +8984,7 @@
       </c>
       <c r="D19" s="0" t="n">
         <f aca="false">IF(ISBLANK(A19),"",COUNTIF(A:A,A19))</f>
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="E19" s="0" t="n">
         <f aca="false">IF(ISBLANK(B19),"",COUNTIF(B:B,B19))</f>
@@ -9006,7 +9007,7 @@
       </c>
       <c r="D20" s="0" t="n">
         <f aca="false">IF(ISBLANK(A20),"",COUNTIF(A:A,A20))</f>
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="E20" s="0" t="n">
         <f aca="false">IF(ISBLANK(B20),"",COUNTIF(B:B,B20))</f>
@@ -9029,7 +9030,7 @@
       </c>
       <c r="D21" s="0" t="n">
         <f aca="false">IF(ISBLANK(A21),"",COUNTIF(A:A,A21))</f>
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="E21" s="0" t="n">
         <f aca="false">IF(ISBLANK(B21),"",COUNTIF(B:B,B21))</f>
@@ -9037,7 +9038,7 @@
       </c>
       <c r="F21" s="0" t="n">
         <f aca="false">IF(ISBLANK(C21),"",COUNTIF(C:C,C21))</f>
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9052,11 +9053,11 @@
       </c>
       <c r="D22" s="0" t="n">
         <f aca="false">IF(ISBLANK(A22),"",COUNTIF(A:A,A22))</f>
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="E22" s="0" t="n">
         <f aca="false">IF(ISBLANK(B22),"",COUNTIF(B:B,B22))</f>
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="F22" s="0" t="n">
         <f aca="false">IF(ISBLANK(C22),"",COUNTIF(C:C,C22))</f>
@@ -9075,11 +9076,11 @@
       </c>
       <c r="D23" s="0" t="n">
         <f aca="false">IF(ISBLANK(A23),"",COUNTIF(A:A,A23))</f>
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="E23" s="0" t="n">
         <f aca="false">IF(ISBLANK(B23),"",COUNTIF(B:B,B23))</f>
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="F23" s="0" t="n">
         <f aca="false">IF(ISBLANK(C23),"",COUNTIF(C:C,C23))</f>
@@ -9090,23 +9091,23 @@
       <c r="A24" s="11" t="s">
         <v>33</v>
       </c>
-      <c r="B24" s="22" t="s">
-        <v>84</v>
-      </c>
-      <c r="C24" s="12" t="s">
-        <v>73</v>
+      <c r="B24" s="21" t="s">
+        <v>83</v>
+      </c>
+      <c r="C24" s="17" t="s">
+        <v>78</v>
       </c>
       <c r="D24" s="0" t="n">
         <f aca="false">IF(ISBLANK(A24),"",COUNTIF(A:A,A24))</f>
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="E24" s="0" t="n">
         <f aca="false">IF(ISBLANK(B24),"",COUNTIF(B:B,B24))</f>
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="F24" s="0" t="n">
         <f aca="false">IF(ISBLANK(C24),"",COUNTIF(C:C,C24))</f>
-        <v>11</v>
+        <v>6</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9116,12 +9117,12 @@
       <c r="B25" s="22" t="s">
         <v>84</v>
       </c>
-      <c r="C25" s="11" t="s">
-        <v>71</v>
+      <c r="C25" s="12" t="s">
+        <v>73</v>
       </c>
       <c r="D25" s="0" t="n">
         <f aca="false">IF(ISBLANK(A25),"",COUNTIF(A:A,A25))</f>
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="E25" s="0" t="n">
         <f aca="false">IF(ISBLANK(B25),"",COUNTIF(B:B,B25))</f>
@@ -9129,7 +9130,7 @@
       </c>
       <c r="F25" s="0" t="n">
         <f aca="false">IF(ISBLANK(C25),"",COUNTIF(C:C,C25))</f>
-        <v>6</v>
+        <v>11</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9139,12 +9140,12 @@
       <c r="B26" s="22" t="s">
         <v>84</v>
       </c>
-      <c r="C26" s="21" t="s">
-        <v>83</v>
+      <c r="C26" s="11" t="s">
+        <v>71</v>
       </c>
       <c r="D26" s="0" t="n">
         <f aca="false">IF(ISBLANK(A26),"",COUNTIF(A:A,A26))</f>
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="E26" s="0" t="n">
         <f aca="false">IF(ISBLANK(B26),"",COUNTIF(B:B,B26))</f>
@@ -9152,30 +9153,30 @@
       </c>
       <c r="F26" s="0" t="n">
         <f aca="false">IF(ISBLANK(C26),"",COUNTIF(C:C,C26))</f>
-        <v>3</v>
+        <v>6</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="11" t="s">
         <v>33</v>
       </c>
-      <c r="B27" s="16" t="s">
-        <v>77</v>
-      </c>
-      <c r="C27" s="12" t="s">
-        <v>73</v>
+      <c r="B27" s="22" t="s">
+        <v>84</v>
+      </c>
+      <c r="C27" s="21" t="s">
+        <v>83</v>
       </c>
       <c r="D27" s="0" t="n">
         <f aca="false">IF(ISBLANK(A27),"",COUNTIF(A:A,A27))</f>
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="E27" s="0" t="n">
         <f aca="false">IF(ISBLANK(B27),"",COUNTIF(B:B,B27))</f>
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F27" s="0" t="n">
         <f aca="false">IF(ISBLANK(C27),"",COUNTIF(C:C,C27))</f>
-        <v>11</v>
+        <v>3</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9185,12 +9186,12 @@
       <c r="B28" s="16" t="s">
         <v>77</v>
       </c>
-      <c r="C28" s="23" t="s">
-        <v>85</v>
+      <c r="C28" s="12" t="s">
+        <v>73</v>
       </c>
       <c r="D28" s="0" t="n">
         <f aca="false">IF(ISBLANK(A28),"",COUNTIF(A:A,A28))</f>
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="E28" s="0" t="n">
         <f aca="false">IF(ISBLANK(B28),"",COUNTIF(B:B,B28))</f>
@@ -9198,22 +9199,22 @@
       </c>
       <c r="F28" s="0" t="n">
         <f aca="false">IF(ISBLANK(C28),"",COUNTIF(C:C,C28))</f>
-        <v>1</v>
+        <v>11</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="11" t="s">
         <v>33</v>
       </c>
-      <c r="B29" s="15" t="s">
-        <v>76</v>
-      </c>
-      <c r="C29" s="14" t="s">
-        <v>75</v>
+      <c r="B29" s="16" t="s">
+        <v>77</v>
+      </c>
+      <c r="C29" s="23" t="s">
+        <v>85</v>
       </c>
       <c r="D29" s="0" t="n">
         <f aca="false">IF(ISBLANK(A29),"",COUNTIF(A:A,A29))</f>
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="E29" s="0" t="n">
         <f aca="false">IF(ISBLANK(B29),"",COUNTIF(B:B,B29))</f>
@@ -9221,7 +9222,7 @@
       </c>
       <c r="F29" s="0" t="n">
         <f aca="false">IF(ISBLANK(C29),"",COUNTIF(C:C,C29))</f>
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9231,12 +9232,12 @@
       <c r="B30" s="15" t="s">
         <v>76</v>
       </c>
-      <c r="C30" s="16" t="s">
-        <v>77</v>
+      <c r="C30" s="14" t="s">
+        <v>75</v>
       </c>
       <c r="D30" s="0" t="n">
         <f aca="false">IF(ISBLANK(A30),"",COUNTIF(A:A,A30))</f>
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="E30" s="0" t="n">
         <f aca="false">IF(ISBLANK(B30),"",COUNTIF(B:B,B30))</f>
@@ -9244,73 +9245,76 @@
       </c>
       <c r="F30" s="0" t="n">
         <f aca="false">IF(ISBLANK(C30),"",COUNTIF(C:C,C30))</f>
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="11" t="s">
         <v>33</v>
       </c>
-      <c r="B31" s="20" t="s">
-        <v>82</v>
-      </c>
-      <c r="C31" s="8" t="s">
-        <v>72</v>
+      <c r="B31" s="15" t="s">
+        <v>76</v>
+      </c>
+      <c r="C31" s="16" t="s">
+        <v>77</v>
       </c>
       <c r="D31" s="0" t="n">
         <f aca="false">IF(ISBLANK(A31),"",COUNTIF(A:A,A31))</f>
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="E31" s="0" t="n">
         <f aca="false">IF(ISBLANK(B31),"",COUNTIF(B:B,B31))</f>
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="F31" s="0" t="n">
         <f aca="false">IF(ISBLANK(C31),"",COUNTIF(C:C,C31))</f>
-        <v>18</v>
+        <v>2</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="11" t="s">
         <v>33</v>
       </c>
-      <c r="B32" s="12" t="s">
-        <v>73</v>
-      </c>
-      <c r="C32" s="17" t="s">
-        <v>78</v>
+      <c r="B32" s="20" t="s">
+        <v>82</v>
+      </c>
+      <c r="C32" s="8" t="s">
+        <v>72</v>
       </c>
       <c r="D32" s="0" t="n">
         <f aca="false">IF(ISBLANK(A32),"",COUNTIF(A:A,A32))</f>
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="E32" s="0" t="n">
         <f aca="false">IF(ISBLANK(B32),"",COUNTIF(B:B,B32))</f>
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="F32" s="0" t="n">
         <f aca="false">IF(ISBLANK(C32),"",COUNTIF(C:C,C32))</f>
-        <v>5</v>
+        <v>18</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="22" t="s">
-        <v>86</v>
-      </c>
-      <c r="B33" s="8" t="s">
-        <v>72</v>
+      <c r="A33" s="11" t="s">
+        <v>33</v>
+      </c>
+      <c r="B33" s="12" t="s">
+        <v>73</v>
+      </c>
+      <c r="C33" s="17" t="s">
+        <v>78</v>
       </c>
       <c r="D33" s="0" t="n">
         <f aca="false">IF(ISBLANK(A33),"",COUNTIF(A:A,A33))</f>
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="E33" s="0" t="n">
         <f aca="false">IF(ISBLANK(B33),"",COUNTIF(B:B,B33))</f>
-        <v>9</v>
-      </c>
-      <c r="F33" s="0" t="str">
+        <v>2</v>
+      </c>
+      <c r="F33" s="0" t="n">
         <f aca="false">IF(ISBLANK(C33),"",COUNTIF(C:C,C33))</f>
-        <v/>
+        <v>6</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9377,8 +9381,8 @@
       <c r="A37" s="22" t="s">
         <v>86</v>
       </c>
-      <c r="B37" s="21" t="s">
-        <v>83</v>
+      <c r="B37" s="8" t="s">
+        <v>72</v>
       </c>
       <c r="D37" s="0" t="n">
         <f aca="false">IF(ISBLANK(A37),"",COUNTIF(A:A,A37))</f>
@@ -9386,7 +9390,7 @@
       </c>
       <c r="E37" s="0" t="n">
         <f aca="false">IF(ISBLANK(B37),"",COUNTIF(B:B,B37))</f>
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="F37" s="0" t="str">
         <f aca="false">IF(ISBLANK(C37),"",COUNTIF(C:C,C37))</f>
@@ -9406,7 +9410,7 @@
       </c>
       <c r="E38" s="0" t="n">
         <f aca="false">IF(ISBLANK(B38),"",COUNTIF(B:B,B38))</f>
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="F38" s="0" t="str">
         <f aca="false">IF(ISBLANK(C38),"",COUNTIF(C:C,C38))</f>
@@ -9417,8 +9421,8 @@
       <c r="A39" s="22" t="s">
         <v>86</v>
       </c>
-      <c r="B39" s="22" t="s">
-        <v>84</v>
+      <c r="B39" s="21" t="s">
+        <v>83</v>
       </c>
       <c r="D39" s="0" t="n">
         <f aca="false">IF(ISBLANK(A39),"",COUNTIF(A:A,A39))</f>
@@ -9426,7 +9430,7 @@
       </c>
       <c r="E39" s="0" t="n">
         <f aca="false">IF(ISBLANK(B39),"",COUNTIF(B:B,B39))</f>
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="F39" s="0" t="str">
         <f aca="false">IF(ISBLANK(C39),"",COUNTIF(C:C,C39))</f>
@@ -9437,8 +9441,8 @@
       <c r="A40" s="22" t="s">
         <v>86</v>
       </c>
-      <c r="B40" s="17" t="s">
-        <v>78</v>
+      <c r="B40" s="22" t="s">
+        <v>84</v>
       </c>
       <c r="D40" s="0" t="n">
         <f aca="false">IF(ISBLANK(A40),"",COUNTIF(A:A,A40))</f>
@@ -9446,7 +9450,7 @@
       </c>
       <c r="E40" s="0" t="n">
         <f aca="false">IF(ISBLANK(B40),"",COUNTIF(B:B,B40))</f>
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="F40" s="0" t="str">
         <f aca="false">IF(ISBLANK(C40),"",COUNTIF(C:C,C40))</f>
@@ -9497,8 +9501,8 @@
       <c r="A43" s="22" t="s">
         <v>86</v>
       </c>
-      <c r="B43" s="24" t="s">
-        <v>87</v>
+      <c r="B43" s="17" t="s">
+        <v>78</v>
       </c>
       <c r="D43" s="0" t="n">
         <f aca="false">IF(ISBLANK(A43),"",COUNTIF(A:A,A43))</f>
@@ -9506,7 +9510,7 @@
       </c>
       <c r="E43" s="0" t="n">
         <f aca="false">IF(ISBLANK(B43),"",COUNTIF(B:B,B43))</f>
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="F43" s="0" t="str">
         <f aca="false">IF(ISBLANK(C43),"",COUNTIF(C:C,C43))</f>
@@ -9534,26 +9538,23 @@
       </c>
     </row>
     <row r="45" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A45" s="20" t="s">
-        <v>19</v>
-      </c>
-      <c r="B45" s="11" t="s">
-        <v>71</v>
-      </c>
-      <c r="C45" s="12" t="s">
-        <v>73</v>
+      <c r="A45" s="22" t="s">
+        <v>86</v>
+      </c>
+      <c r="B45" s="24" t="s">
+        <v>87</v>
       </c>
       <c r="D45" s="0" t="n">
         <f aca="false">IF(ISBLANK(A45),"",COUNTIF(A:A,A45))</f>
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E45" s="0" t="n">
         <f aca="false">IF(ISBLANK(B45),"",COUNTIF(B:B,B45))</f>
-        <v>10</v>
-      </c>
-      <c r="F45" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="F45" s="0" t="str">
         <f aca="false">IF(ISBLANK(C45),"",COUNTIF(C:C,C45))</f>
-        <v>11</v>
+        <v/>
       </c>
     </row>
     <row r="46" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9586,8 +9587,8 @@
       <c r="B47" s="11" t="s">
         <v>71</v>
       </c>
-      <c r="C47" s="21" t="s">
-        <v>83</v>
+      <c r="C47" s="12" t="s">
+        <v>73</v>
       </c>
       <c r="D47" s="0" t="n">
         <f aca="false">IF(ISBLANK(A47),"",COUNTIF(A:A,A47))</f>
@@ -9599,18 +9600,18 @@
       </c>
       <c r="F47" s="0" t="n">
         <f aca="false">IF(ISBLANK(C47),"",COUNTIF(C:C,C47))</f>
-        <v>3</v>
+        <v>11</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="20" t="s">
         <v>19</v>
       </c>
-      <c r="B48" s="8" t="s">
-        <v>72</v>
-      </c>
-      <c r="C48" s="20" t="s">
-        <v>82</v>
+      <c r="B48" s="11" t="s">
+        <v>71</v>
+      </c>
+      <c r="C48" s="21" t="s">
+        <v>83</v>
       </c>
       <c r="D48" s="0" t="n">
         <f aca="false">IF(ISBLANK(A48),"",COUNTIF(A:A,A48))</f>
@@ -9618,22 +9619,22 @@
       </c>
       <c r="E48" s="0" t="n">
         <f aca="false">IF(ISBLANK(B48),"",COUNTIF(B:B,B48))</f>
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F48" s="0" t="n">
         <f aca="false">IF(ISBLANK(C48),"",COUNTIF(C:C,C48))</f>
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="20" t="s">
         <v>19</v>
       </c>
-      <c r="B49" s="21" t="s">
-        <v>83</v>
-      </c>
-      <c r="C49" s="11" t="s">
-        <v>71</v>
+      <c r="B49" s="8" t="s">
+        <v>72</v>
+      </c>
+      <c r="C49" s="20" t="s">
+        <v>82</v>
       </c>
       <c r="D49" s="0" t="n">
         <f aca="false">IF(ISBLANK(A49),"",COUNTIF(A:A,A49))</f>
@@ -9641,11 +9642,11 @@
       </c>
       <c r="E49" s="0" t="n">
         <f aca="false">IF(ISBLANK(B49),"",COUNTIF(B:B,B49))</f>
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="F49" s="0" t="n">
         <f aca="false">IF(ISBLANK(C49),"",COUNTIF(C:C,C49))</f>
-        <v>6</v>
+        <v>1</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9664,7 +9665,7 @@
       </c>
       <c r="E50" s="0" t="n">
         <f aca="false">IF(ISBLANK(B50),"",COUNTIF(B:B,B50))</f>
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="F50" s="0" t="n">
         <f aca="false">IF(ISBLANK(C50),"",COUNTIF(C:C,C50))</f>
@@ -9675,11 +9676,11 @@
       <c r="A51" s="20" t="s">
         <v>19</v>
       </c>
-      <c r="B51" s="16" t="s">
-        <v>77</v>
-      </c>
-      <c r="C51" s="12" t="s">
-        <v>73</v>
+      <c r="B51" s="21" t="s">
+        <v>83</v>
+      </c>
+      <c r="C51" s="11" t="s">
+        <v>71</v>
       </c>
       <c r="D51" s="0" t="n">
         <f aca="false">IF(ISBLANK(A51),"",COUNTIF(A:A,A51))</f>
@@ -9687,11 +9688,11 @@
       </c>
       <c r="E51" s="0" t="n">
         <f aca="false">IF(ISBLANK(B51),"",COUNTIF(B:B,B51))</f>
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="F51" s="0" t="n">
         <f aca="false">IF(ISBLANK(C51),"",COUNTIF(C:C,C51))</f>
-        <v>11</v>
+        <v>6</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9701,8 +9702,8 @@
       <c r="B52" s="16" t="s">
         <v>77</v>
       </c>
-      <c r="C52" s="15" t="s">
-        <v>76</v>
+      <c r="C52" s="12" t="s">
+        <v>73</v>
       </c>
       <c r="D52" s="0" t="n">
         <f aca="false">IF(ISBLANK(A52),"",COUNTIF(A:A,A52))</f>
@@ -9714,18 +9715,18 @@
       </c>
       <c r="F52" s="0" t="n">
         <f aca="false">IF(ISBLANK(C52),"",COUNTIF(C:C,C52))</f>
-        <v>8</v>
+        <v>11</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="20" t="s">
         <v>19</v>
       </c>
-      <c r="B53" s="15" t="s">
+      <c r="B53" s="16" t="s">
+        <v>77</v>
+      </c>
+      <c r="C53" s="15" t="s">
         <v>76</v>
-      </c>
-      <c r="C53" s="19" t="s">
-        <v>81</v>
       </c>
       <c r="D53" s="0" t="n">
         <f aca="false">IF(ISBLANK(A53),"",COUNTIF(A:A,A53))</f>
@@ -9737,18 +9738,18 @@
       </c>
       <c r="F53" s="0" t="n">
         <f aca="false">IF(ISBLANK(C53),"",COUNTIF(C:C,C53))</f>
-        <v>3</v>
+        <v>8</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="20" t="s">
         <v>19</v>
       </c>
-      <c r="B54" s="20" t="s">
-        <v>82</v>
-      </c>
-      <c r="C54" s="8" t="s">
-        <v>72</v>
+      <c r="B54" s="15" t="s">
+        <v>76</v>
+      </c>
+      <c r="C54" s="19" t="s">
+        <v>81</v>
       </c>
       <c r="D54" s="0" t="n">
         <f aca="false">IF(ISBLANK(A54),"",COUNTIF(A:A,A54))</f>
@@ -9756,19 +9757,19 @@
       </c>
       <c r="E54" s="0" t="n">
         <f aca="false">IF(ISBLANK(B54),"",COUNTIF(B:B,B54))</f>
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="F54" s="0" t="n">
         <f aca="false">IF(ISBLANK(C54),"",COUNTIF(C:C,C54))</f>
-        <v>18</v>
+        <v>3</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="20" t="s">
         <v>19</v>
       </c>
-      <c r="B55" s="25" t="s">
-        <v>88</v>
+      <c r="B55" s="20" t="s">
+        <v>82</v>
       </c>
       <c r="C55" s="8" t="s">
         <v>72</v>
@@ -9779,7 +9780,7 @@
       </c>
       <c r="E55" s="0" t="n">
         <f aca="false">IF(ISBLANK(B55),"",COUNTIF(B:B,B55))</f>
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="F55" s="0" t="n">
         <f aca="false">IF(ISBLANK(C55),"",COUNTIF(C:C,C55))</f>
@@ -9787,26 +9788,26 @@
       </c>
     </row>
     <row r="56" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A56" s="15" t="s">
-        <v>89</v>
-      </c>
-      <c r="B56" s="14" t="s">
-        <v>75</v>
-      </c>
-      <c r="C56" s="15" t="s">
-        <v>76</v>
+      <c r="A56" s="20" t="s">
+        <v>19</v>
+      </c>
+      <c r="B56" s="25" t="s">
+        <v>88</v>
+      </c>
+      <c r="C56" s="8" t="s">
+        <v>72</v>
       </c>
       <c r="D56" s="0" t="n">
         <f aca="false">IF(ISBLANK(A56),"",COUNTIF(A:A,A56))</f>
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="E56" s="0" t="n">
         <f aca="false">IF(ISBLANK(B56),"",COUNTIF(B:B,B56))</f>
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="F56" s="0" t="n">
         <f aca="false">IF(ISBLANK(C56),"",COUNTIF(C:C,C56))</f>
-        <v>8</v>
+        <v>18</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9862,8 +9863,8 @@
       <c r="B59" s="14" t="s">
         <v>75</v>
       </c>
-      <c r="C59" s="13" t="s">
-        <v>74</v>
+      <c r="C59" s="15" t="s">
+        <v>76</v>
       </c>
       <c r="D59" s="0" t="n">
         <f aca="false">IF(ISBLANK(A59),"",COUNTIF(A:A,A59))</f>
@@ -9875,18 +9876,18 @@
       </c>
       <c r="F59" s="0" t="n">
         <f aca="false">IF(ISBLANK(C59),"",COUNTIF(C:C,C59))</f>
-        <v>3</v>
+        <v>8</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="15" t="s">
         <v>89</v>
       </c>
-      <c r="B60" s="16" t="s">
-        <v>77</v>
-      </c>
-      <c r="C60" s="15" t="s">
-        <v>76</v>
+      <c r="B60" s="14" t="s">
+        <v>75</v>
+      </c>
+      <c r="C60" s="13" t="s">
+        <v>74</v>
       </c>
       <c r="D60" s="0" t="n">
         <f aca="false">IF(ISBLANK(A60),"",COUNTIF(A:A,A60))</f>
@@ -9894,22 +9895,22 @@
       </c>
       <c r="E60" s="0" t="n">
         <f aca="false">IF(ISBLANK(B60),"",COUNTIF(B:B,B60))</f>
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="F60" s="0" t="n">
         <f aca="false">IF(ISBLANK(C60),"",COUNTIF(C:C,C60))</f>
-        <v>8</v>
+        <v>3</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="15" t="s">
         <v>89</v>
       </c>
-      <c r="B61" s="15" t="s">
+      <c r="B61" s="16" t="s">
+        <v>77</v>
+      </c>
+      <c r="C61" s="15" t="s">
         <v>76</v>
-      </c>
-      <c r="C61" s="19" t="s">
-        <v>81</v>
       </c>
       <c r="D61" s="0" t="n">
         <f aca="false">IF(ISBLANK(A61),"",COUNTIF(A:A,A61))</f>
@@ -9921,18 +9922,18 @@
       </c>
       <c r="F61" s="0" t="n">
         <f aca="false">IF(ISBLANK(C61),"",COUNTIF(C:C,C61))</f>
-        <v>3</v>
+        <v>8</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="15" t="s">
         <v>89</v>
       </c>
-      <c r="B62" s="19" t="s">
+      <c r="B62" s="15" t="s">
+        <v>76</v>
+      </c>
+      <c r="C62" s="19" t="s">
         <v>81</v>
-      </c>
-      <c r="C62" s="18" t="s">
-        <v>80</v>
       </c>
       <c r="D62" s="0" t="n">
         <f aca="false">IF(ISBLANK(A62),"",COUNTIF(A:A,A62))</f>
@@ -9940,11 +9941,11 @@
       </c>
       <c r="E62" s="0" t="n">
         <f aca="false">IF(ISBLANK(B62),"",COUNTIF(B:B,B62))</f>
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="F62" s="0" t="n">
         <f aca="false">IF(ISBLANK(C62),"",COUNTIF(C:C,C62))</f>
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9954,8 +9955,8 @@
       <c r="B63" s="19" t="s">
         <v>81</v>
       </c>
-      <c r="C63" s="10" t="s">
-        <v>79</v>
+      <c r="C63" s="18" t="s">
+        <v>80</v>
       </c>
       <c r="D63" s="0" t="n">
         <f aca="false">IF(ISBLANK(A63),"",COUNTIF(A:A,A63))</f>
@@ -9967,18 +9968,18 @@
       </c>
       <c r="F63" s="0" t="n">
         <f aca="false">IF(ISBLANK(C63),"",COUNTIF(C:C,C63))</f>
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="15" t="s">
         <v>89</v>
       </c>
-      <c r="B64" s="17" t="s">
-        <v>78</v>
-      </c>
-      <c r="C64" s="8" t="s">
-        <v>72</v>
+      <c r="B64" s="19" t="s">
+        <v>81</v>
+      </c>
+      <c r="C64" s="10" t="s">
+        <v>79</v>
       </c>
       <c r="D64" s="0" t="n">
         <f aca="false">IF(ISBLANK(A64),"",COUNTIF(A:A,A64))</f>
@@ -9990,18 +9991,18 @@
       </c>
       <c r="F64" s="0" t="n">
         <f aca="false">IF(ISBLANK(C64),"",COUNTIF(C:C,C64))</f>
-        <v>18</v>
+        <v>4</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="15" t="s">
         <v>89</v>
       </c>
-      <c r="B65" s="12" t="s">
-        <v>73</v>
-      </c>
-      <c r="C65" s="11" t="s">
-        <v>71</v>
+      <c r="B65" s="17" t="s">
+        <v>78</v>
+      </c>
+      <c r="C65" s="8" t="s">
+        <v>72</v>
       </c>
       <c r="D65" s="0" t="n">
         <f aca="false">IF(ISBLANK(A65),"",COUNTIF(A:A,A65))</f>
@@ -10009,45 +10010,45 @@
       </c>
       <c r="E65" s="0" t="n">
         <f aca="false">IF(ISBLANK(B65),"",COUNTIF(B:B,B65))</f>
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="F65" s="0" t="n">
         <f aca="false">IF(ISBLANK(C65),"",COUNTIF(C:C,C65))</f>
-        <v>6</v>
+        <v>18</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A66" s="21" t="s">
-        <v>90</v>
-      </c>
-      <c r="B66" s="11" t="s">
+      <c r="A66" s="15" t="s">
+        <v>89</v>
+      </c>
+      <c r="B66" s="12" t="s">
+        <v>73</v>
+      </c>
+      <c r="C66" s="11" t="s">
         <v>71</v>
-      </c>
-      <c r="C66" s="12" t="s">
-        <v>73</v>
       </c>
       <c r="D66" s="0" t="n">
         <f aca="false">IF(ISBLANK(A66),"",COUNTIF(A:A,A66))</f>
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="E66" s="0" t="n">
         <f aca="false">IF(ISBLANK(B66),"",COUNTIF(B:B,B66))</f>
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="F66" s="0" t="n">
         <f aca="false">IF(ISBLANK(C66),"",COUNTIF(C:C,C66))</f>
-        <v>11</v>
+        <v>6</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="21" t="s">
         <v>90</v>
       </c>
-      <c r="B67" s="8" t="s">
-        <v>72</v>
-      </c>
-      <c r="C67" s="17" t="s">
-        <v>78</v>
+      <c r="B67" s="11" t="s">
+        <v>71</v>
+      </c>
+      <c r="C67" s="12" t="s">
+        <v>73</v>
       </c>
       <c r="D67" s="0" t="n">
         <f aca="false">IF(ISBLANK(A67),"",COUNTIF(A:A,A67))</f>
@@ -10055,22 +10056,22 @@
       </c>
       <c r="E67" s="0" t="n">
         <f aca="false">IF(ISBLANK(B67),"",COUNTIF(B:B,B67))</f>
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F67" s="0" t="n">
         <f aca="false">IF(ISBLANK(C67),"",COUNTIF(C:C,C67))</f>
-        <v>5</v>
+        <v>11</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="21" t="s">
         <v>90</v>
       </c>
-      <c r="B68" s="21" t="s">
-        <v>83</v>
-      </c>
-      <c r="C68" s="8" t="s">
+      <c r="B68" s="8" t="s">
         <v>72</v>
+      </c>
+      <c r="C68" s="17" t="s">
+        <v>78</v>
       </c>
       <c r="D68" s="0" t="n">
         <f aca="false">IF(ISBLANK(A68),"",COUNTIF(A:A,A68))</f>
@@ -10078,11 +10079,11 @@
       </c>
       <c r="E68" s="0" t="n">
         <f aca="false">IF(ISBLANK(B68),"",COUNTIF(B:B,B68))</f>
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="F68" s="0" t="n">
         <f aca="false">IF(ISBLANK(C68),"",COUNTIF(C:C,C68))</f>
-        <v>18</v>
+        <v>6</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10092,8 +10093,8 @@
       <c r="B69" s="21" t="s">
         <v>83</v>
       </c>
-      <c r="C69" s="17" t="s">
-        <v>78</v>
+      <c r="C69" s="8" t="s">
+        <v>72</v>
       </c>
       <c r="D69" s="0" t="n">
         <f aca="false">IF(ISBLANK(A69),"",COUNTIF(A:A,A69))</f>
@@ -10101,22 +10102,22 @@
       </c>
       <c r="E69" s="0" t="n">
         <f aca="false">IF(ISBLANK(B69),"",COUNTIF(B:B,B69))</f>
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="F69" s="0" t="n">
         <f aca="false">IF(ISBLANK(C69),"",COUNTIF(C:C,C69))</f>
-        <v>5</v>
+        <v>18</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A70" s="21" t="s">
         <v>90</v>
       </c>
-      <c r="B70" s="22" t="s">
-        <v>84</v>
-      </c>
-      <c r="C70" s="8" t="s">
-        <v>72</v>
+      <c r="B70" s="21" t="s">
+        <v>83</v>
+      </c>
+      <c r="C70" s="17" t="s">
+        <v>78</v>
       </c>
       <c r="D70" s="0" t="n">
         <f aca="false">IF(ISBLANK(A70),"",COUNTIF(A:A,A70))</f>
@@ -10124,11 +10125,11 @@
       </c>
       <c r="E70" s="0" t="n">
         <f aca="false">IF(ISBLANK(B70),"",COUNTIF(B:B,B70))</f>
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="F70" s="0" t="n">
         <f aca="false">IF(ISBLANK(C70),"",COUNTIF(C:C,C70))</f>
-        <v>18</v>
+        <v>6</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10138,8 +10139,8 @@
       <c r="B71" s="22" t="s">
         <v>84</v>
       </c>
-      <c r="C71" s="21" t="s">
-        <v>83</v>
+      <c r="C71" s="8" t="s">
+        <v>72</v>
       </c>
       <c r="D71" s="0" t="n">
         <f aca="false">IF(ISBLANK(A71),"",COUNTIF(A:A,A71))</f>
@@ -10151,18 +10152,18 @@
       </c>
       <c r="F71" s="0" t="n">
         <f aca="false">IF(ISBLANK(C71),"",COUNTIF(C:C,C71))</f>
-        <v>3</v>
+        <v>18</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A72" s="21" t="s">
         <v>90</v>
       </c>
-      <c r="B72" s="26" t="s">
-        <v>91</v>
-      </c>
-      <c r="C72" s="8" t="s">
-        <v>72</v>
+      <c r="B72" s="22" t="s">
+        <v>84</v>
+      </c>
+      <c r="C72" s="21" t="s">
+        <v>83</v>
       </c>
       <c r="D72" s="0" t="n">
         <f aca="false">IF(ISBLANK(A72),"",COUNTIF(A:A,A72))</f>
@@ -10170,30 +10171,30 @@
       </c>
       <c r="E72" s="0" t="n">
         <f aca="false">IF(ISBLANK(B72),"",COUNTIF(B:B,B72))</f>
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="F72" s="0" t="n">
         <f aca="false">IF(ISBLANK(C72),"",COUNTIF(C:C,C72))</f>
-        <v>18</v>
+        <v>3</v>
       </c>
     </row>
     <row r="73" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A73" s="8" t="s">
-        <v>36</v>
-      </c>
-      <c r="B73" s="18" t="s">
-        <v>80</v>
+      <c r="A73" s="21" t="s">
+        <v>90</v>
+      </c>
+      <c r="B73" s="26" t="s">
+        <v>91</v>
       </c>
       <c r="C73" s="8" t="s">
         <v>72</v>
       </c>
       <c r="D73" s="0" t="n">
         <f aca="false">IF(ISBLANK(A73),"",COUNTIF(A:A,A73))</f>
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E73" s="0" t="n">
         <f aca="false">IF(ISBLANK(B73),"",COUNTIF(B:B,B73))</f>
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="F73" s="0" t="n">
         <f aca="false">IF(ISBLANK(C73),"",COUNTIF(C:C,C73))</f>
@@ -10316,31 +10317,34 @@
       </c>
     </row>
     <row r="79" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A79" s="22" t="s">
-        <v>92</v>
-      </c>
-      <c r="B79" s="8" t="s">
+      <c r="A79" s="8" t="s">
+        <v>36</v>
+      </c>
+      <c r="B79" s="18" t="s">
+        <v>80</v>
+      </c>
+      <c r="C79" s="8" t="s">
         <v>72</v>
       </c>
       <c r="D79" s="0" t="n">
         <f aca="false">IF(ISBLANK(A79),"",COUNTIF(A:A,A79))</f>
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="E79" s="0" t="n">
         <f aca="false">IF(ISBLANK(B79),"",COUNTIF(B:B,B79))</f>
-        <v>9</v>
-      </c>
-      <c r="F79" s="0" t="str">
+        <v>7</v>
+      </c>
+      <c r="F79" s="0" t="n">
         <f aca="false">IF(ISBLANK(C79),"",COUNTIF(C:C,C79))</f>
-        <v/>
+        <v>18</v>
       </c>
     </row>
     <row r="80" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A80" s="22" t="s">
         <v>92</v>
       </c>
-      <c r="B80" s="22" t="s">
-        <v>84</v>
+      <c r="B80" s="8" t="s">
+        <v>72</v>
       </c>
       <c r="D80" s="0" t="n">
         <f aca="false">IF(ISBLANK(A80),"",COUNTIF(A:A,A80))</f>
@@ -10348,7 +10352,7 @@
       </c>
       <c r="E80" s="0" t="n">
         <f aca="false">IF(ISBLANK(B80),"",COUNTIF(B:B,B80))</f>
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="F80" s="0" t="str">
         <f aca="false">IF(ISBLANK(C80),"",COUNTIF(C:C,C80))</f>
@@ -10379,8 +10383,8 @@
       <c r="A82" s="22" t="s">
         <v>92</v>
       </c>
-      <c r="B82" s="17" t="s">
-        <v>78</v>
+      <c r="B82" s="22" t="s">
+        <v>84</v>
       </c>
       <c r="D82" s="0" t="n">
         <f aca="false">IF(ISBLANK(A82),"",COUNTIF(A:A,A82))</f>
@@ -10388,7 +10392,7 @@
       </c>
       <c r="E82" s="0" t="n">
         <f aca="false">IF(ISBLANK(B82),"",COUNTIF(B:B,B82))</f>
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="F82" s="0" t="str">
         <f aca="false">IF(ISBLANK(C82),"",COUNTIF(C:C,C82))</f>
@@ -10396,34 +10400,31 @@
       </c>
     </row>
     <row r="83" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A83" s="25" t="s">
-        <v>93</v>
-      </c>
-      <c r="B83" s="8" t="s">
-        <v>72</v>
-      </c>
-      <c r="C83" s="18" t="s">
-        <v>80</v>
+      <c r="A83" s="22" t="s">
+        <v>92</v>
+      </c>
+      <c r="B83" s="17" t="s">
+        <v>78</v>
       </c>
       <c r="D83" s="0" t="n">
         <f aca="false">IF(ISBLANK(A83),"",COUNTIF(A:A,A83))</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E83" s="0" t="n">
         <f aca="false">IF(ISBLANK(B83),"",COUNTIF(B:B,B83))</f>
-        <v>9</v>
-      </c>
-      <c r="F83" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="F83" s="0" t="str">
         <f aca="false">IF(ISBLANK(C83),"",COUNTIF(C:C,C83))</f>
-        <v>5</v>
+        <v/>
       </c>
     </row>
     <row r="84" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A84" s="25" t="s">
         <v>93</v>
       </c>
-      <c r="B84" s="20" t="s">
-        <v>82</v>
+      <c r="B84" s="8" t="s">
+        <v>72</v>
       </c>
       <c r="C84" s="18" t="s">
         <v>80</v>
@@ -10434,7 +10435,7 @@
       </c>
       <c r="E84" s="0" t="n">
         <f aca="false">IF(ISBLANK(B84),"",COUNTIF(B:B,B84))</f>
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="F84" s="0" t="n">
         <f aca="false">IF(ISBLANK(C84),"",COUNTIF(C:C,C84))</f>
@@ -10445,8 +10446,8 @@
       <c r="A85" s="25" t="s">
         <v>93</v>
       </c>
-      <c r="B85" s="25" t="s">
-        <v>88</v>
+      <c r="B85" s="20" t="s">
+        <v>82</v>
       </c>
       <c r="C85" s="18" t="s">
         <v>80</v>
@@ -10457,7 +10458,7 @@
       </c>
       <c r="E85" s="0" t="n">
         <f aca="false">IF(ISBLANK(B85),"",COUNTIF(B:B,B85))</f>
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="F85" s="0" t="n">
         <f aca="false">IF(ISBLANK(C85),"",COUNTIF(C:C,C85))</f>
@@ -10465,11 +10466,11 @@
       </c>
     </row>
     <row r="86" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A86" s="19" t="s">
-        <v>94</v>
-      </c>
-      <c r="B86" s="14" t="s">
-        <v>75</v>
+      <c r="A86" s="25" t="s">
+        <v>93</v>
+      </c>
+      <c r="B86" s="25" t="s">
+        <v>88</v>
       </c>
       <c r="C86" s="18" t="s">
         <v>80</v>
@@ -10480,7 +10481,7 @@
       </c>
       <c r="E86" s="0" t="n">
         <f aca="false">IF(ISBLANK(B86),"",COUNTIF(B:B,B86))</f>
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="F86" s="0" t="n">
         <f aca="false">IF(ISBLANK(C86),"",COUNTIF(C:C,C86))</f>
@@ -10491,11 +10492,11 @@
       <c r="A87" s="19" t="s">
         <v>94</v>
       </c>
-      <c r="B87" s="15" t="s">
-        <v>76</v>
-      </c>
-      <c r="C87" s="14" t="s">
+      <c r="B87" s="14" t="s">
         <v>75</v>
+      </c>
+      <c r="C87" s="18" t="s">
+        <v>80</v>
       </c>
       <c r="D87" s="0" t="n">
         <f aca="false">IF(ISBLANK(A87),"",COUNTIF(A:A,A87))</f>
@@ -10503,22 +10504,22 @@
       </c>
       <c r="E87" s="0" t="n">
         <f aca="false">IF(ISBLANK(B87),"",COUNTIF(B:B,B87))</f>
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="F87" s="0" t="n">
         <f aca="false">IF(ISBLANK(C87),"",COUNTIF(C:C,C87))</f>
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="88" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A88" s="19" t="s">
         <v>94</v>
       </c>
-      <c r="B88" s="19" t="s">
-        <v>81</v>
-      </c>
-      <c r="C88" s="19" t="s">
-        <v>81</v>
+      <c r="B88" s="15" t="s">
+        <v>76</v>
+      </c>
+      <c r="C88" s="14" t="s">
+        <v>75</v>
       </c>
       <c r="D88" s="0" t="n">
         <f aca="false">IF(ISBLANK(A88),"",COUNTIF(A:A,A88))</f>
@@ -10526,7 +10527,7 @@
       </c>
       <c r="E88" s="0" t="n">
         <f aca="false">IF(ISBLANK(B88),"",COUNTIF(B:B,B88))</f>
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="F88" s="0" t="n">
         <f aca="false">IF(ISBLANK(C88),"",COUNTIF(C:C,C88))</f>
@@ -10534,14 +10535,14 @@
       </c>
     </row>
     <row r="89" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A89" s="27" t="s">
-        <v>95</v>
-      </c>
-      <c r="B89" s="14" t="s">
-        <v>75</v>
-      </c>
-      <c r="C89" s="15" t="s">
-        <v>76</v>
+      <c r="A89" s="19" t="s">
+        <v>94</v>
+      </c>
+      <c r="B89" s="19" t="s">
+        <v>81</v>
+      </c>
+      <c r="C89" s="19" t="s">
+        <v>81</v>
       </c>
       <c r="D89" s="0" t="n">
         <f aca="false">IF(ISBLANK(A89),"",COUNTIF(A:A,A89))</f>
@@ -10549,22 +10550,22 @@
       </c>
       <c r="E89" s="0" t="n">
         <f aca="false">IF(ISBLANK(B89),"",COUNTIF(B:B,B89))</f>
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="F89" s="0" t="n">
         <f aca="false">IF(ISBLANK(C89),"",COUNTIF(C:C,C89))</f>
-        <v>8</v>
+        <v>3</v>
       </c>
     </row>
     <row r="90" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A90" s="27" t="s">
         <v>95</v>
       </c>
-      <c r="B90" s="27" t="s">
-        <v>96</v>
-      </c>
-      <c r="C90" s="28" t="s">
-        <v>97</v>
+      <c r="B90" s="14" t="s">
+        <v>75</v>
+      </c>
+      <c r="C90" s="15" t="s">
+        <v>76</v>
       </c>
       <c r="D90" s="0" t="n">
         <f aca="false">IF(ISBLANK(A90),"",COUNTIF(A:A,A90))</f>
@@ -10572,11 +10573,11 @@
       </c>
       <c r="E90" s="0" t="n">
         <f aca="false">IF(ISBLANK(B90),"",COUNTIF(B:B,B90))</f>
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="F90" s="0" t="n">
         <f aca="false">IF(ISBLANK(C90),"",COUNTIF(C:C,C90))</f>
-        <v>2</v>
+        <v>8</v>
       </c>
     </row>
     <row r="91" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10603,30 +10604,53 @@
       </c>
     </row>
     <row r="92" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A92" s="16" t="s">
-        <v>98</v>
-      </c>
-      <c r="B92" s="15" t="s">
-        <v>76</v>
-      </c>
-      <c r="C92" s="16" t="s">
-        <v>77</v>
+      <c r="A92" s="27" t="s">
+        <v>95</v>
+      </c>
+      <c r="B92" s="27" t="s">
+        <v>96</v>
+      </c>
+      <c r="C92" s="28" t="s">
+        <v>97</v>
       </c>
       <c r="D92" s="0" t="n">
         <f aca="false">IF(ISBLANK(A92),"",COUNTIF(A:A,A92))</f>
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E92" s="0" t="n">
         <f aca="false">IF(ISBLANK(B92),"",COUNTIF(B:B,B92))</f>
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="F92" s="0" t="n">
         <f aca="false">IF(ISBLANK(C92),"",COUNTIF(C:C,C92))</f>
         <v>2</v>
       </c>
     </row>
+    <row r="93" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A93" s="16" t="s">
+        <v>98</v>
+      </c>
+      <c r="B93" s="15" t="s">
+        <v>76</v>
+      </c>
+      <c r="C93" s="16" t="s">
+        <v>77</v>
+      </c>
+      <c r="D93" s="0" t="n">
+        <f aca="false">IF(ISBLANK(A93),"",COUNTIF(A:A,A93))</f>
+        <v>1</v>
+      </c>
+      <c r="E93" s="0" t="n">
+        <f aca="false">IF(ISBLANK(B93),"",COUNTIF(B:B,B93))</f>
+        <v>7</v>
+      </c>
+      <c r="F93" s="0" t="n">
+        <f aca="false">IF(ISBLANK(C93),"",COUNTIF(C:C,C93))</f>
+        <v>2</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:F92"/>
+  <autoFilter ref="A1:F93"/>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
   <pageSetup paperSize="9" scale="100" firstPageNumber="0" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" useFirstPageNumber="false" horizontalDpi="300" verticalDpi="300" copies="1"/>
@@ -10721,7 +10745,7 @@
       </c>
       <c r="B3" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!A:A,A3)</f>
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="D3" s="8" t="s">
         <v>72</v>
@@ -10753,8 +10777,8 @@
         <f aca="false">COUNTIF(Tatjes!A:A,A4)</f>
         <v>12</v>
       </c>
-      <c r="D4" s="14" t="s">
-        <v>75</v>
+      <c r="D4" s="21" t="s">
+        <v>83</v>
       </c>
       <c r="E4" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!B:B,D4)</f>
@@ -10783,12 +10807,12 @@
         <f aca="false">COUNTIF(Tatjes!A:A,A5)</f>
         <v>11</v>
       </c>
-      <c r="D5" s="21" t="s">
-        <v>83</v>
+      <c r="D5" s="14" t="s">
+        <v>75</v>
       </c>
       <c r="E5" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!B:B,D5)</f>
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="G5" s="11" t="s">
         <v>71</v>
@@ -10797,8 +10821,8 @@
         <f aca="false">COUNTIF(Tatjes!C:C,G5)</f>
         <v>6</v>
       </c>
-      <c r="J5" s="14" t="s">
-        <v>75</v>
+      <c r="J5" s="21" t="s">
+        <v>83</v>
       </c>
       <c r="K5" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!B:B,J5)*2+COUNTIF(Tatjes!C:C,J5)</f>
@@ -10825,14 +10849,14 @@
       </c>
       <c r="H6" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!C:C,G6)</f>
-        <v>5</v>
-      </c>
-      <c r="J6" s="21" t="s">
-        <v>83</v>
+        <v>6</v>
+      </c>
+      <c r="J6" s="14" t="s">
+        <v>75</v>
       </c>
       <c r="K6" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!B:B,J6)*2+COUNTIF(Tatjes!C:C,J6)</f>
-        <v>19</v>
+        <v>21</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10917,8 +10941,8 @@
         <f aca="false">COUNTIF(Tatjes!C:C,G9)</f>
         <v>3</v>
       </c>
-      <c r="J9" s="16" t="s">
-        <v>77</v>
+      <c r="J9" s="17" t="s">
+        <v>78</v>
       </c>
       <c r="K9" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!B:B,J9)*2+COUNTIF(Tatjes!C:C,J9)</f>
@@ -10947,12 +10971,12 @@
         <f aca="false">COUNTIF(Tatjes!C:C,G10)</f>
         <v>3</v>
       </c>
-      <c r="J10" s="12" t="s">
-        <v>73</v>
+      <c r="J10" s="16" t="s">
+        <v>77</v>
       </c>
       <c r="K10" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!B:B,J10)*2+COUNTIF(Tatjes!C:C,J10)</f>
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10977,8 +11001,8 @@
         <f aca="false">COUNTIF(Tatjes!C:C,G11)</f>
         <v>3</v>
       </c>
-      <c r="J11" s="17" t="s">
-        <v>78</v>
+      <c r="J11" s="12" t="s">
+        <v>73</v>
       </c>
       <c r="K11" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!B:B,J11)*2+COUNTIF(Tatjes!C:C,J11)</f>
@@ -11074,7 +11098,7 @@
       </c>
       <c r="B15" s="3" t="n">
         <f aca="false">COUNTA(Tatjes!A:A)-1</f>
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="D15" s="13" t="s">
         <v>74</v>

</xml_diff>

<commit_message>
Sync from vault 2026-06-03 10:07:58
</commit_message>
<xml_diff>
--- a/content/Archief/0. PDFs & docs/Obol docs & forms/Irmijn Inc/Irma backup log.xlsx
+++ b/content/Archief/0. PDFs & docs/Obol docs & forms/Irmijn Inc/Irma backup log.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="3"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="Logboek" sheetId="1" state="visible" r:id="rId2"/>
@@ -802,7 +802,7 @@
 </styleSheet>
 </file>
 
-<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <c:lang val="en-US"/>
   <c:roundedCorners val="0"/>
@@ -1598,11 +1598,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="60225116"/>
-        <c:axId val="23597406"/>
+        <c:axId val="68735520"/>
+        <c:axId val="59746143"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="60225116"/>
+        <c:axId val="68735520"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1658,14 +1658,14 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="23597406"/>
+        <c:crossAx val="59746143"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
         <c:lblOffset val="100"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="23597406"/>
+        <c:axId val="59746143"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1730,7 +1730,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="60225116"/>
+        <c:crossAx val="68735520"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -1757,7 +1757,7 @@
 </c:chartSpace>
 </file>
 
-<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/charts/chart5.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <c:lang val="en-US"/>
   <c:roundedCorners val="0"/>
@@ -4791,11 +4791,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="37232827"/>
-        <c:axId val="6225379"/>
+        <c:axId val="24737048"/>
+        <c:axId val="80774908"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="37232827"/>
+        <c:axId val="24737048"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -4851,14 +4851,14 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="6225379"/>
+        <c:crossAx val="80774908"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
         <c:lblOffset val="100"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="6225379"/>
+        <c:axId val="80774908"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -4923,7 +4923,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="37232827"/>
+        <c:crossAx val="24737048"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -4957,7 +4957,7 @@
         </a:p>
       </c:txPr>
     </c:legend>
-    <c:plotVisOnly val="1"/>
+    <c:plotVisOnly val="0"/>
     <c:dispBlanksAs val="gap"/>
   </c:chart>
   <c:spPr>
@@ -4971,7 +4971,7 @@
 </c:chartSpace>
 </file>
 
-<file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/charts/chart6.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <c:lang val="en-US"/>
   <c:roundedCorners val="0"/>
@@ -5146,11 +5146,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="48539564"/>
-        <c:axId val="1579423"/>
+        <c:axId val="62636774"/>
+        <c:axId val="54095425"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="48539564"/>
+        <c:axId val="62636774"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -5178,14 +5178,14 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1579423"/>
+        <c:crossAx val="54095425"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
         <c:lblOffset val="100"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="1579423"/>
+        <c:axId val="54095425"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -5250,7 +5250,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="48539564"/>
+        <c:crossAx val="62636774"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -5390,7 +5390,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:AMJ120"/>
+  <dimension ref="A1:AMJ200"/>
   <sheetFormatPr defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="7.54"/>
@@ -7742,19 +7742,19 @@
         <v>4</v>
       </c>
       <c r="E81" s="5" t="n">
-        <f aca="false">COUNTIF($D$2:$D81,E$1)</f>
+        <f aca="false">IF(COUNTA($D81)&gt;0,COUNTIF($D$2:$D81,E$1),"")</f>
         <v>18</v>
       </c>
       <c r="F81" s="5" t="n">
-        <f aca="false">COUNTIF($D$2:$D81,F$1)</f>
+        <f aca="false">IF(COUNTA($D81)&gt;0,COUNTIF($D$2:$D81,F$1),"")</f>
         <v>47</v>
       </c>
       <c r="G81" s="5" t="n">
-        <f aca="false">COUNTIF($D$2:$D81,G$1)</f>
+        <f aca="false">IF(COUNTA($D81)&gt;0,COUNTIF($D$2:$D81,G$1),"")</f>
         <v>11</v>
       </c>
       <c r="H81" s="5" t="n">
-        <f aca="false">COUNTIF($D$2:$D81,H$1)</f>
+        <f aca="false">IF(COUNTA($D81)&gt;0,COUNTIF($D$2:$D81,H$1),"")</f>
         <v>4</v>
       </c>
     </row>
@@ -7763,390 +7763,2298 @@
         <v>80</v>
       </c>
       <c r="D82" s="5"/>
-      <c r="E82" s="5"/>
-      <c r="F82" s="5"/>
-      <c r="G82" s="5"/>
-      <c r="H82" s="5"/>
+      <c r="E82" s="5" t="str">
+        <f aca="false">IF(COUNTA($D82)&gt;0,COUNTIF($D$2:$D82,E$1),"")</f>
+        <v/>
+      </c>
+      <c r="F82" s="5" t="str">
+        <f aca="false">IF(COUNTA($D82)&gt;0,COUNTIF($D$2:$D82,F$1),"")</f>
+        <v/>
+      </c>
+      <c r="G82" s="5" t="str">
+        <f aca="false">IF(COUNTA($D82)&gt;0,COUNTIF($D$2:$D82,G$1),"")</f>
+        <v/>
+      </c>
+      <c r="H82" s="5" t="str">
+        <f aca="false">IF(COUNTA($D82)&gt;0,COUNTIF($D$2:$D82,H$1),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="83" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A83" s="1" t="n">
         <v>81</v>
       </c>
       <c r="D83" s="5"/>
-      <c r="E83" s="5"/>
-      <c r="F83" s="5"/>
-      <c r="G83" s="5"/>
-      <c r="H83" s="5"/>
+      <c r="E83" s="5" t="str">
+        <f aca="false">IF(COUNTA($D83)&gt;0,COUNTIF($D$2:$D83,E$1),"")</f>
+        <v/>
+      </c>
+      <c r="F83" s="5" t="str">
+        <f aca="false">IF(COUNTA($D83)&gt;0,COUNTIF($D$2:$D83,F$1),"")</f>
+        <v/>
+      </c>
+      <c r="G83" s="5" t="str">
+        <f aca="false">IF(COUNTA($D83)&gt;0,COUNTIF($D$2:$D83,G$1),"")</f>
+        <v/>
+      </c>
+      <c r="H83" s="5" t="str">
+        <f aca="false">IF(COUNTA($D83)&gt;0,COUNTIF($D$2:$D83,H$1),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="84" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A84" s="1" t="n">
         <v>82</v>
       </c>
       <c r="D84" s="5"/>
-      <c r="E84" s="5"/>
-      <c r="F84" s="5"/>
-      <c r="G84" s="5"/>
-      <c r="H84" s="5"/>
+      <c r="E84" s="5" t="str">
+        <f aca="false">IF(COUNTA($D84)&gt;0,COUNTIF($D$2:$D84,E$1),"")</f>
+        <v/>
+      </c>
+      <c r="F84" s="5" t="str">
+        <f aca="false">IF(COUNTA($D84)&gt;0,COUNTIF($D$2:$D84,F$1),"")</f>
+        <v/>
+      </c>
+      <c r="G84" s="5" t="str">
+        <f aca="false">IF(COUNTA($D84)&gt;0,COUNTIF($D$2:$D84,G$1),"")</f>
+        <v/>
+      </c>
+      <c r="H84" s="5" t="str">
+        <f aca="false">IF(COUNTA($D84)&gt;0,COUNTIF($D$2:$D84,H$1),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="85" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A85" s="1" t="n">
         <v>83</v>
       </c>
       <c r="D85" s="5"/>
-      <c r="E85" s="5"/>
-      <c r="F85" s="5"/>
-      <c r="G85" s="5"/>
-      <c r="H85" s="5"/>
+      <c r="E85" s="5" t="str">
+        <f aca="false">IF(COUNTA($D85)&gt;0,COUNTIF($D$2:$D85,E$1),"")</f>
+        <v/>
+      </c>
+      <c r="F85" s="5" t="str">
+        <f aca="false">IF(COUNTA($D85)&gt;0,COUNTIF($D$2:$D85,F$1),"")</f>
+        <v/>
+      </c>
+      <c r="G85" s="5" t="str">
+        <f aca="false">IF(COUNTA($D85)&gt;0,COUNTIF($D$2:$D85,G$1),"")</f>
+        <v/>
+      </c>
+      <c r="H85" s="5" t="str">
+        <f aca="false">IF(COUNTA($D85)&gt;0,COUNTIF($D$2:$D85,H$1),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="86" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A86" s="1" t="n">
         <v>84</v>
       </c>
       <c r="D86" s="5"/>
-      <c r="E86" s="5"/>
-      <c r="F86" s="5"/>
-      <c r="G86" s="5"/>
-      <c r="H86" s="5"/>
+      <c r="E86" s="5" t="str">
+        <f aca="false">IF(COUNTA($D86)&gt;0,COUNTIF($D$2:$D86,E$1),"")</f>
+        <v/>
+      </c>
+      <c r="F86" s="5" t="str">
+        <f aca="false">IF(COUNTA($D86)&gt;0,COUNTIF($D$2:$D86,F$1),"")</f>
+        <v/>
+      </c>
+      <c r="G86" s="5" t="str">
+        <f aca="false">IF(COUNTA($D86)&gt;0,COUNTIF($D$2:$D86,G$1),"")</f>
+        <v/>
+      </c>
+      <c r="H86" s="5" t="str">
+        <f aca="false">IF(COUNTA($D86)&gt;0,COUNTIF($D$2:$D86,H$1),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="87" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A87" s="1" t="n">
         <v>85</v>
       </c>
       <c r="D87" s="5"/>
-      <c r="E87" s="5"/>
-      <c r="F87" s="5"/>
-      <c r="G87" s="5"/>
-      <c r="H87" s="5"/>
+      <c r="E87" s="5" t="str">
+        <f aca="false">IF(COUNTA($D87)&gt;0,COUNTIF($D$2:$D87,E$1),"")</f>
+        <v/>
+      </c>
+      <c r="F87" s="5" t="str">
+        <f aca="false">IF(COUNTA($D87)&gt;0,COUNTIF($D$2:$D87,F$1),"")</f>
+        <v/>
+      </c>
+      <c r="G87" s="5" t="str">
+        <f aca="false">IF(COUNTA($D87)&gt;0,COUNTIF($D$2:$D87,G$1),"")</f>
+        <v/>
+      </c>
+      <c r="H87" s="5" t="str">
+        <f aca="false">IF(COUNTA($D87)&gt;0,COUNTIF($D$2:$D87,H$1),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="88" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A88" s="1" t="n">
         <v>86</v>
       </c>
       <c r="D88" s="5"/>
-      <c r="E88" s="5"/>
-      <c r="F88" s="5"/>
-      <c r="G88" s="5"/>
-      <c r="H88" s="5"/>
+      <c r="E88" s="5" t="str">
+        <f aca="false">IF(COUNTA($D88)&gt;0,COUNTIF($D$2:$D88,E$1),"")</f>
+        <v/>
+      </c>
+      <c r="F88" s="5" t="str">
+        <f aca="false">IF(COUNTA($D88)&gt;0,COUNTIF($D$2:$D88,F$1),"")</f>
+        <v/>
+      </c>
+      <c r="G88" s="5" t="str">
+        <f aca="false">IF(COUNTA($D88)&gt;0,COUNTIF($D$2:$D88,G$1),"")</f>
+        <v/>
+      </c>
+      <c r="H88" s="5" t="str">
+        <f aca="false">IF(COUNTA($D88)&gt;0,COUNTIF($D$2:$D88,H$1),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="89" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A89" s="1" t="n">
         <v>87</v>
       </c>
       <c r="D89" s="5"/>
-      <c r="E89" s="5"/>
-      <c r="F89" s="5"/>
-      <c r="G89" s="5"/>
-      <c r="H89" s="5"/>
+      <c r="E89" s="5" t="str">
+        <f aca="false">IF(COUNTA($D89)&gt;0,COUNTIF($D$2:$D89,E$1),"")</f>
+        <v/>
+      </c>
+      <c r="F89" s="5" t="str">
+        <f aca="false">IF(COUNTA($D89)&gt;0,COUNTIF($D$2:$D89,F$1),"")</f>
+        <v/>
+      </c>
+      <c r="G89" s="5" t="str">
+        <f aca="false">IF(COUNTA($D89)&gt;0,COUNTIF($D$2:$D89,G$1),"")</f>
+        <v/>
+      </c>
+      <c r="H89" s="5" t="str">
+        <f aca="false">IF(COUNTA($D89)&gt;0,COUNTIF($D$2:$D89,H$1),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="90" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A90" s="1" t="n">
         <v>88</v>
       </c>
       <c r="D90" s="5"/>
-      <c r="E90" s="5"/>
-      <c r="F90" s="5"/>
-      <c r="G90" s="5"/>
-      <c r="H90" s="5"/>
+      <c r="E90" s="5" t="str">
+        <f aca="false">IF(COUNTA($D90)&gt;0,COUNTIF($D$2:$D90,E$1),"")</f>
+        <v/>
+      </c>
+      <c r="F90" s="5" t="str">
+        <f aca="false">IF(COUNTA($D90)&gt;0,COUNTIF($D$2:$D90,F$1),"")</f>
+        <v/>
+      </c>
+      <c r="G90" s="5" t="str">
+        <f aca="false">IF(COUNTA($D90)&gt;0,COUNTIF($D$2:$D90,G$1),"")</f>
+        <v/>
+      </c>
+      <c r="H90" s="5" t="str">
+        <f aca="false">IF(COUNTA($D90)&gt;0,COUNTIF($D$2:$D90,H$1),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="91" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A91" s="1" t="n">
         <v>89</v>
       </c>
       <c r="D91" s="5"/>
-      <c r="E91" s="5"/>
-      <c r="F91" s="5"/>
-      <c r="G91" s="5"/>
-      <c r="H91" s="5"/>
+      <c r="E91" s="5" t="str">
+        <f aca="false">IF(COUNTA($D91)&gt;0,COUNTIF($D$2:$D91,E$1),"")</f>
+        <v/>
+      </c>
+      <c r="F91" s="5" t="str">
+        <f aca="false">IF(COUNTA($D91)&gt;0,COUNTIF($D$2:$D91,F$1),"")</f>
+        <v/>
+      </c>
+      <c r="G91" s="5" t="str">
+        <f aca="false">IF(COUNTA($D91)&gt;0,COUNTIF($D$2:$D91,G$1),"")</f>
+        <v/>
+      </c>
+      <c r="H91" s="5" t="str">
+        <f aca="false">IF(COUNTA($D91)&gt;0,COUNTIF($D$2:$D91,H$1),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="92" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A92" s="1" t="n">
         <v>90</v>
       </c>
       <c r="D92" s="5"/>
-      <c r="E92" s="5"/>
-      <c r="F92" s="5"/>
-      <c r="G92" s="5"/>
-      <c r="H92" s="5"/>
+      <c r="E92" s="5" t="str">
+        <f aca="false">IF(COUNTA($D92)&gt;0,COUNTIF($D$2:$D92,E$1),"")</f>
+        <v/>
+      </c>
+      <c r="F92" s="5" t="str">
+        <f aca="false">IF(COUNTA($D92)&gt;0,COUNTIF($D$2:$D92,F$1),"")</f>
+        <v/>
+      </c>
+      <c r="G92" s="5" t="str">
+        <f aca="false">IF(COUNTA($D92)&gt;0,COUNTIF($D$2:$D92,G$1),"")</f>
+        <v/>
+      </c>
+      <c r="H92" s="5" t="str">
+        <f aca="false">IF(COUNTA($D92)&gt;0,COUNTIF($D$2:$D92,H$1),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="93" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A93" s="1" t="n">
         <v>91</v>
       </c>
       <c r="D93" s="5"/>
-      <c r="E93" s="5"/>
-      <c r="F93" s="5"/>
-      <c r="G93" s="5"/>
-      <c r="H93" s="5"/>
+      <c r="E93" s="5" t="str">
+        <f aca="false">IF(COUNTA($D93)&gt;0,COUNTIF($D$2:$D93,E$1),"")</f>
+        <v/>
+      </c>
+      <c r="F93" s="5" t="str">
+        <f aca="false">IF(COUNTA($D93)&gt;0,COUNTIF($D$2:$D93,F$1),"")</f>
+        <v/>
+      </c>
+      <c r="G93" s="5" t="str">
+        <f aca="false">IF(COUNTA($D93)&gt;0,COUNTIF($D$2:$D93,G$1),"")</f>
+        <v/>
+      </c>
+      <c r="H93" s="5" t="str">
+        <f aca="false">IF(COUNTA($D93)&gt;0,COUNTIF($D$2:$D93,H$1),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="94" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A94" s="1" t="n">
         <v>92</v>
       </c>
       <c r="D94" s="5"/>
-      <c r="E94" s="5"/>
-      <c r="F94" s="5"/>
-      <c r="G94" s="5"/>
-      <c r="H94" s="5"/>
+      <c r="E94" s="5" t="str">
+        <f aca="false">IF(COUNTA($D94)&gt;0,COUNTIF($D$2:$D94,E$1),"")</f>
+        <v/>
+      </c>
+      <c r="F94" s="5" t="str">
+        <f aca="false">IF(COUNTA($D94)&gt;0,COUNTIF($D$2:$D94,F$1),"")</f>
+        <v/>
+      </c>
+      <c r="G94" s="5" t="str">
+        <f aca="false">IF(COUNTA($D94)&gt;0,COUNTIF($D$2:$D94,G$1),"")</f>
+        <v/>
+      </c>
+      <c r="H94" s="5" t="str">
+        <f aca="false">IF(COUNTA($D94)&gt;0,COUNTIF($D$2:$D94,H$1),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="95" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A95" s="1" t="n">
         <v>93</v>
       </c>
       <c r="D95" s="5"/>
-      <c r="E95" s="5"/>
-      <c r="F95" s="5"/>
-      <c r="G95" s="5"/>
-      <c r="H95" s="5"/>
+      <c r="E95" s="5" t="str">
+        <f aca="false">IF(COUNTA($D95)&gt;0,COUNTIF($D$2:$D95,E$1),"")</f>
+        <v/>
+      </c>
+      <c r="F95" s="5" t="str">
+        <f aca="false">IF(COUNTA($D95)&gt;0,COUNTIF($D$2:$D95,F$1),"")</f>
+        <v/>
+      </c>
+      <c r="G95" s="5" t="str">
+        <f aca="false">IF(COUNTA($D95)&gt;0,COUNTIF($D$2:$D95,G$1),"")</f>
+        <v/>
+      </c>
+      <c r="H95" s="5" t="str">
+        <f aca="false">IF(COUNTA($D95)&gt;0,COUNTIF($D$2:$D95,H$1),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="96" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A96" s="1" t="n">
         <v>94</v>
       </c>
       <c r="D96" s="5"/>
-      <c r="E96" s="5"/>
-      <c r="F96" s="5"/>
-      <c r="G96" s="5"/>
-      <c r="H96" s="5"/>
+      <c r="E96" s="5" t="str">
+        <f aca="false">IF(COUNTA($D96)&gt;0,COUNTIF($D$2:$D96,E$1),"")</f>
+        <v/>
+      </c>
+      <c r="F96" s="5" t="str">
+        <f aca="false">IF(COUNTA($D96)&gt;0,COUNTIF($D$2:$D96,F$1),"")</f>
+        <v/>
+      </c>
+      <c r="G96" s="5" t="str">
+        <f aca="false">IF(COUNTA($D96)&gt;0,COUNTIF($D$2:$D96,G$1),"")</f>
+        <v/>
+      </c>
+      <c r="H96" s="5" t="str">
+        <f aca="false">IF(COUNTA($D96)&gt;0,COUNTIF($D$2:$D96,H$1),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="97" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A97" s="1" t="n">
         <v>95</v>
       </c>
       <c r="D97" s="5"/>
-      <c r="E97" s="5"/>
-      <c r="F97" s="5"/>
-      <c r="G97" s="5"/>
-      <c r="H97" s="5"/>
+      <c r="E97" s="5" t="str">
+        <f aca="false">IF(COUNTA($D97)&gt;0,COUNTIF($D$2:$D97,E$1),"")</f>
+        <v/>
+      </c>
+      <c r="F97" s="5" t="str">
+        <f aca="false">IF(COUNTA($D97)&gt;0,COUNTIF($D$2:$D97,F$1),"")</f>
+        <v/>
+      </c>
+      <c r="G97" s="5" t="str">
+        <f aca="false">IF(COUNTA($D97)&gt;0,COUNTIF($D$2:$D97,G$1),"")</f>
+        <v/>
+      </c>
+      <c r="H97" s="5" t="str">
+        <f aca="false">IF(COUNTA($D97)&gt;0,COUNTIF($D$2:$D97,H$1),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="98" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A98" s="1" t="n">
         <v>96</v>
       </c>
       <c r="D98" s="5"/>
-      <c r="E98" s="5"/>
-      <c r="F98" s="5"/>
-      <c r="G98" s="5"/>
-      <c r="H98" s="5"/>
+      <c r="E98" s="5" t="str">
+        <f aca="false">IF(COUNTA($D98)&gt;0,COUNTIF($D$2:$D98,E$1),"")</f>
+        <v/>
+      </c>
+      <c r="F98" s="5" t="str">
+        <f aca="false">IF(COUNTA($D98)&gt;0,COUNTIF($D$2:$D98,F$1),"")</f>
+        <v/>
+      </c>
+      <c r="G98" s="5" t="str">
+        <f aca="false">IF(COUNTA($D98)&gt;0,COUNTIF($D$2:$D98,G$1),"")</f>
+        <v/>
+      </c>
+      <c r="H98" s="5" t="str">
+        <f aca="false">IF(COUNTA($D98)&gt;0,COUNTIF($D$2:$D98,H$1),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="99" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A99" s="1" t="n">
         <v>97</v>
       </c>
       <c r="D99" s="5"/>
-      <c r="E99" s="5"/>
-      <c r="F99" s="5"/>
-      <c r="G99" s="5"/>
-      <c r="H99" s="5"/>
+      <c r="E99" s="5" t="str">
+        <f aca="false">IF(COUNTA($D99)&gt;0,COUNTIF($D$2:$D99,E$1),"")</f>
+        <v/>
+      </c>
+      <c r="F99" s="5" t="str">
+        <f aca="false">IF(COUNTA($D99)&gt;0,COUNTIF($D$2:$D99,F$1),"")</f>
+        <v/>
+      </c>
+      <c r="G99" s="5" t="str">
+        <f aca="false">IF(COUNTA($D99)&gt;0,COUNTIF($D$2:$D99,G$1),"")</f>
+        <v/>
+      </c>
+      <c r="H99" s="5" t="str">
+        <f aca="false">IF(COUNTA($D99)&gt;0,COUNTIF($D$2:$D99,H$1),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="100" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A100" s="1" t="n">
         <v>98</v>
       </c>
       <c r="D100" s="5"/>
-      <c r="E100" s="5"/>
-      <c r="F100" s="5"/>
-      <c r="G100" s="5"/>
-      <c r="H100" s="5"/>
+      <c r="E100" s="5" t="str">
+        <f aca="false">IF(COUNTA($D100)&gt;0,COUNTIF($D$2:$D100,E$1),"")</f>
+        <v/>
+      </c>
+      <c r="F100" s="5" t="str">
+        <f aca="false">IF(COUNTA($D100)&gt;0,COUNTIF($D$2:$D100,F$1),"")</f>
+        <v/>
+      </c>
+      <c r="G100" s="5" t="str">
+        <f aca="false">IF(COUNTA($D100)&gt;0,COUNTIF($D$2:$D100,G$1),"")</f>
+        <v/>
+      </c>
+      <c r="H100" s="5" t="str">
+        <f aca="false">IF(COUNTA($D100)&gt;0,COUNTIF($D$2:$D100,H$1),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="101" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A101" s="1" t="n">
         <v>99</v>
       </c>
       <c r="D101" s="5"/>
-      <c r="E101" s="5"/>
-      <c r="F101" s="5"/>
-      <c r="G101" s="5"/>
-      <c r="H101" s="5"/>
+      <c r="E101" s="5" t="str">
+        <f aca="false">IF(COUNTA($D101)&gt;0,COUNTIF($D$2:$D101,E$1),"")</f>
+        <v/>
+      </c>
+      <c r="F101" s="5" t="str">
+        <f aca="false">IF(COUNTA($D101)&gt;0,COUNTIF($D$2:$D101,F$1),"")</f>
+        <v/>
+      </c>
+      <c r="G101" s="5" t="str">
+        <f aca="false">IF(COUNTA($D101)&gt;0,COUNTIF($D$2:$D101,G$1),"")</f>
+        <v/>
+      </c>
+      <c r="H101" s="5" t="str">
+        <f aca="false">IF(COUNTA($D101)&gt;0,COUNTIF($D$2:$D101,H$1),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="102" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A102" s="1" t="n">
         <v>100</v>
       </c>
       <c r="D102" s="5"/>
-      <c r="E102" s="5"/>
-      <c r="F102" s="5"/>
-      <c r="G102" s="5"/>
-      <c r="H102" s="5"/>
+      <c r="E102" s="5" t="str">
+        <f aca="false">IF(COUNTA($D102)&gt;0,COUNTIF($D$2:$D102,E$1),"")</f>
+        <v/>
+      </c>
+      <c r="F102" s="5" t="str">
+        <f aca="false">IF(COUNTA($D102)&gt;0,COUNTIF($D$2:$D102,F$1),"")</f>
+        <v/>
+      </c>
+      <c r="G102" s="5" t="str">
+        <f aca="false">IF(COUNTA($D102)&gt;0,COUNTIF($D$2:$D102,G$1),"")</f>
+        <v/>
+      </c>
+      <c r="H102" s="5" t="str">
+        <f aca="false">IF(COUNTA($D102)&gt;0,COUNTIF($D$2:$D102,H$1),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="103" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A103" s="1" t="n">
         <v>101</v>
       </c>
       <c r="D103" s="5"/>
-      <c r="E103" s="5"/>
-      <c r="F103" s="5"/>
-      <c r="G103" s="5"/>
-      <c r="H103" s="5"/>
+      <c r="E103" s="5" t="str">
+        <f aca="false">IF(COUNTA($D103)&gt;0,COUNTIF($D$2:$D103,E$1),"")</f>
+        <v/>
+      </c>
+      <c r="F103" s="5" t="str">
+        <f aca="false">IF(COUNTA($D103)&gt;0,COUNTIF($D$2:$D103,F$1),"")</f>
+        <v/>
+      </c>
+      <c r="G103" s="5" t="str">
+        <f aca="false">IF(COUNTA($D103)&gt;0,COUNTIF($D$2:$D103,G$1),"")</f>
+        <v/>
+      </c>
+      <c r="H103" s="5" t="str">
+        <f aca="false">IF(COUNTA($D103)&gt;0,COUNTIF($D$2:$D103,H$1),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="104" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A104" s="1" t="n">
         <v>102</v>
       </c>
       <c r="D104" s="5"/>
-      <c r="E104" s="5"/>
-      <c r="F104" s="5"/>
-      <c r="G104" s="5"/>
-      <c r="H104" s="5"/>
+      <c r="E104" s="5" t="str">
+        <f aca="false">IF(COUNTA($D104)&gt;0,COUNTIF($D$2:$D104,E$1),"")</f>
+        <v/>
+      </c>
+      <c r="F104" s="5" t="str">
+        <f aca="false">IF(COUNTA($D104)&gt;0,COUNTIF($D$2:$D104,F$1),"")</f>
+        <v/>
+      </c>
+      <c r="G104" s="5" t="str">
+        <f aca="false">IF(COUNTA($D104)&gt;0,COUNTIF($D$2:$D104,G$1),"")</f>
+        <v/>
+      </c>
+      <c r="H104" s="5" t="str">
+        <f aca="false">IF(COUNTA($D104)&gt;0,COUNTIF($D$2:$D104,H$1),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="105" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A105" s="1" t="n">
         <v>103</v>
       </c>
       <c r="D105" s="5"/>
-      <c r="E105" s="5"/>
-      <c r="F105" s="5"/>
-      <c r="G105" s="5"/>
-      <c r="H105" s="5"/>
+      <c r="E105" s="5" t="str">
+        <f aca="false">IF(COUNTA($D105)&gt;0,COUNTIF($D$2:$D105,E$1),"")</f>
+        <v/>
+      </c>
+      <c r="F105" s="5" t="str">
+        <f aca="false">IF(COUNTA($D105)&gt;0,COUNTIF($D$2:$D105,F$1),"")</f>
+        <v/>
+      </c>
+      <c r="G105" s="5" t="str">
+        <f aca="false">IF(COUNTA($D105)&gt;0,COUNTIF($D$2:$D105,G$1),"")</f>
+        <v/>
+      </c>
+      <c r="H105" s="5" t="str">
+        <f aca="false">IF(COUNTA($D105)&gt;0,COUNTIF($D$2:$D105,H$1),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="106" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A106" s="1" t="n">
         <v>104</v>
       </c>
       <c r="D106" s="5"/>
-      <c r="E106" s="5"/>
-      <c r="F106" s="5"/>
-      <c r="G106" s="5"/>
-      <c r="H106" s="5"/>
+      <c r="E106" s="5" t="str">
+        <f aca="false">IF(COUNTA($D106)&gt;0,COUNTIF($D$2:$D106,E$1),"")</f>
+        <v/>
+      </c>
+      <c r="F106" s="5" t="str">
+        <f aca="false">IF(COUNTA($D106)&gt;0,COUNTIF($D$2:$D106,F$1),"")</f>
+        <v/>
+      </c>
+      <c r="G106" s="5" t="str">
+        <f aca="false">IF(COUNTA($D106)&gt;0,COUNTIF($D$2:$D106,G$1),"")</f>
+        <v/>
+      </c>
+      <c r="H106" s="5" t="str">
+        <f aca="false">IF(COUNTA($D106)&gt;0,COUNTIF($D$2:$D106,H$1),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="107" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A107" s="1" t="n">
         <v>105</v>
       </c>
       <c r="D107" s="5"/>
-      <c r="E107" s="5"/>
-      <c r="F107" s="5"/>
-      <c r="G107" s="5"/>
-      <c r="H107" s="5"/>
+      <c r="E107" s="5" t="str">
+        <f aca="false">IF(COUNTA($D107)&gt;0,COUNTIF($D$2:$D107,E$1),"")</f>
+        <v/>
+      </c>
+      <c r="F107" s="5" t="str">
+        <f aca="false">IF(COUNTA($D107)&gt;0,COUNTIF($D$2:$D107,F$1),"")</f>
+        <v/>
+      </c>
+      <c r="G107" s="5" t="str">
+        <f aca="false">IF(COUNTA($D107)&gt;0,COUNTIF($D$2:$D107,G$1),"")</f>
+        <v/>
+      </c>
+      <c r="H107" s="5" t="str">
+        <f aca="false">IF(COUNTA($D107)&gt;0,COUNTIF($D$2:$D107,H$1),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="108" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A108" s="1" t="n">
         <v>106</v>
       </c>
       <c r="D108" s="5"/>
-      <c r="E108" s="5"/>
-      <c r="F108" s="5"/>
-      <c r="G108" s="5"/>
-      <c r="H108" s="5"/>
+      <c r="E108" s="5" t="str">
+        <f aca="false">IF(COUNTA($D108)&gt;0,COUNTIF($D$2:$D108,E$1),"")</f>
+        <v/>
+      </c>
+      <c r="F108" s="5" t="str">
+        <f aca="false">IF(COUNTA($D108)&gt;0,COUNTIF($D$2:$D108,F$1),"")</f>
+        <v/>
+      </c>
+      <c r="G108" s="5" t="str">
+        <f aca="false">IF(COUNTA($D108)&gt;0,COUNTIF($D$2:$D108,G$1),"")</f>
+        <v/>
+      </c>
+      <c r="H108" s="5" t="str">
+        <f aca="false">IF(COUNTA($D108)&gt;0,COUNTIF($D$2:$D108,H$1),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="109" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A109" s="1" t="n">
         <v>107</v>
       </c>
       <c r="D109" s="5"/>
-      <c r="E109" s="5"/>
-      <c r="F109" s="5"/>
-      <c r="G109" s="5"/>
-      <c r="H109" s="5"/>
+      <c r="E109" s="5" t="str">
+        <f aca="false">IF(COUNTA($D109)&gt;0,COUNTIF($D$2:$D109,E$1),"")</f>
+        <v/>
+      </c>
+      <c r="F109" s="5" t="str">
+        <f aca="false">IF(COUNTA($D109)&gt;0,COUNTIF($D$2:$D109,F$1),"")</f>
+        <v/>
+      </c>
+      <c r="G109" s="5" t="str">
+        <f aca="false">IF(COUNTA($D109)&gt;0,COUNTIF($D$2:$D109,G$1),"")</f>
+        <v/>
+      </c>
+      <c r="H109" s="5" t="str">
+        <f aca="false">IF(COUNTA($D109)&gt;0,COUNTIF($D$2:$D109,H$1),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="110" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A110" s="1" t="n">
         <v>108</v>
       </c>
       <c r="D110" s="5"/>
-      <c r="E110" s="5"/>
-      <c r="F110" s="5"/>
-      <c r="G110" s="5"/>
-      <c r="H110" s="5"/>
+      <c r="E110" s="5" t="str">
+        <f aca="false">IF(COUNTA($D110)&gt;0,COUNTIF($D$2:$D110,E$1),"")</f>
+        <v/>
+      </c>
+      <c r="F110" s="5" t="str">
+        <f aca="false">IF(COUNTA($D110)&gt;0,COUNTIF($D$2:$D110,F$1),"")</f>
+        <v/>
+      </c>
+      <c r="G110" s="5" t="str">
+        <f aca="false">IF(COUNTA($D110)&gt;0,COUNTIF($D$2:$D110,G$1),"")</f>
+        <v/>
+      </c>
+      <c r="H110" s="5" t="str">
+        <f aca="false">IF(COUNTA($D110)&gt;0,COUNTIF($D$2:$D110,H$1),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="111" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A111" s="1" t="n">
         <v>109</v>
       </c>
       <c r="D111" s="5"/>
-      <c r="E111" s="5"/>
-      <c r="F111" s="5"/>
-      <c r="G111" s="5"/>
-      <c r="H111" s="5"/>
+      <c r="E111" s="5" t="str">
+        <f aca="false">IF(COUNTA($D111)&gt;0,COUNTIF($D$2:$D111,E$1),"")</f>
+        <v/>
+      </c>
+      <c r="F111" s="5" t="str">
+        <f aca="false">IF(COUNTA($D111)&gt;0,COUNTIF($D$2:$D111,F$1),"")</f>
+        <v/>
+      </c>
+      <c r="G111" s="5" t="str">
+        <f aca="false">IF(COUNTA($D111)&gt;0,COUNTIF($D$2:$D111,G$1),"")</f>
+        <v/>
+      </c>
+      <c r="H111" s="5" t="str">
+        <f aca="false">IF(COUNTA($D111)&gt;0,COUNTIF($D$2:$D111,H$1),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="112" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A112" s="1" t="n">
         <v>110</v>
       </c>
       <c r="D112" s="5"/>
-      <c r="E112" s="5"/>
-      <c r="F112" s="5"/>
-      <c r="G112" s="5"/>
-      <c r="H112" s="5"/>
+      <c r="E112" s="5" t="str">
+        <f aca="false">IF(COUNTA($D112)&gt;0,COUNTIF($D$2:$D112,E$1),"")</f>
+        <v/>
+      </c>
+      <c r="F112" s="5" t="str">
+        <f aca="false">IF(COUNTA($D112)&gt;0,COUNTIF($D$2:$D112,F$1),"")</f>
+        <v/>
+      </c>
+      <c r="G112" s="5" t="str">
+        <f aca="false">IF(COUNTA($D112)&gt;0,COUNTIF($D$2:$D112,G$1),"")</f>
+        <v/>
+      </c>
+      <c r="H112" s="5" t="str">
+        <f aca="false">IF(COUNTA($D112)&gt;0,COUNTIF($D$2:$D112,H$1),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="113" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A113" s="1" t="n">
         <v>111</v>
       </c>
       <c r="D113" s="5"/>
-      <c r="E113" s="5"/>
-      <c r="F113" s="5"/>
-      <c r="G113" s="5"/>
-      <c r="H113" s="5"/>
+      <c r="E113" s="5" t="str">
+        <f aca="false">IF(COUNTA($D113)&gt;0,COUNTIF($D$2:$D113,E$1),"")</f>
+        <v/>
+      </c>
+      <c r="F113" s="5" t="str">
+        <f aca="false">IF(COUNTA($D113)&gt;0,COUNTIF($D$2:$D113,F$1),"")</f>
+        <v/>
+      </c>
+      <c r="G113" s="5" t="str">
+        <f aca="false">IF(COUNTA($D113)&gt;0,COUNTIF($D$2:$D113,G$1),"")</f>
+        <v/>
+      </c>
+      <c r="H113" s="5" t="str">
+        <f aca="false">IF(COUNTA($D113)&gt;0,COUNTIF($D$2:$D113,H$1),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="114" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A114" s="1" t="n">
         <v>112</v>
       </c>
       <c r="D114" s="5"/>
-      <c r="E114" s="5"/>
-      <c r="F114" s="5"/>
-      <c r="G114" s="5"/>
-      <c r="H114" s="5"/>
+      <c r="E114" s="5" t="str">
+        <f aca="false">IF(COUNTA($D114)&gt;0,COUNTIF($D$2:$D114,E$1),"")</f>
+        <v/>
+      </c>
+      <c r="F114" s="5" t="str">
+        <f aca="false">IF(COUNTA($D114)&gt;0,COUNTIF($D$2:$D114,F$1),"")</f>
+        <v/>
+      </c>
+      <c r="G114" s="5" t="str">
+        <f aca="false">IF(COUNTA($D114)&gt;0,COUNTIF($D$2:$D114,G$1),"")</f>
+        <v/>
+      </c>
+      <c r="H114" s="5" t="str">
+        <f aca="false">IF(COUNTA($D114)&gt;0,COUNTIF($D$2:$D114,H$1),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="115" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D115" s="5"/>
-      <c r="E115" s="5"/>
-      <c r="F115" s="5"/>
-      <c r="G115" s="5"/>
-      <c r="H115" s="5"/>
+      <c r="E115" s="5" t="str">
+        <f aca="false">IF(COUNTA($D115)&gt;0,COUNTIF($D$2:$D115,E$1),"")</f>
+        <v/>
+      </c>
+      <c r="F115" s="5" t="str">
+        <f aca="false">IF(COUNTA($D115)&gt;0,COUNTIF($D$2:$D115,F$1),"")</f>
+        <v/>
+      </c>
+      <c r="G115" s="5" t="str">
+        <f aca="false">IF(COUNTA($D115)&gt;0,COUNTIF($D$2:$D115,G$1),"")</f>
+        <v/>
+      </c>
+      <c r="H115" s="5" t="str">
+        <f aca="false">IF(COUNTA($D115)&gt;0,COUNTIF($D$2:$D115,H$1),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="116" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D116" s="5"/>
-      <c r="E116" s="5"/>
-      <c r="F116" s="5"/>
-      <c r="G116" s="5"/>
-      <c r="H116" s="5"/>
+      <c r="E116" s="5" t="str">
+        <f aca="false">IF(COUNTA($D116)&gt;0,COUNTIF($D$2:$D116,E$1),"")</f>
+        <v/>
+      </c>
+      <c r="F116" s="5" t="str">
+        <f aca="false">IF(COUNTA($D116)&gt;0,COUNTIF($D$2:$D116,F$1),"")</f>
+        <v/>
+      </c>
+      <c r="G116" s="5" t="str">
+        <f aca="false">IF(COUNTA($D116)&gt;0,COUNTIF($D$2:$D116,G$1),"")</f>
+        <v/>
+      </c>
+      <c r="H116" s="5" t="str">
+        <f aca="false">IF(COUNTA($D116)&gt;0,COUNTIF($D$2:$D116,H$1),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="117" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D117" s="5"/>
-      <c r="E117" s="5"/>
-      <c r="F117" s="5"/>
-      <c r="G117" s="5"/>
-      <c r="H117" s="5"/>
+      <c r="E117" s="5" t="str">
+        <f aca="false">IF(COUNTA($D117)&gt;0,COUNTIF($D$2:$D117,E$1),"")</f>
+        <v/>
+      </c>
+      <c r="F117" s="5" t="str">
+        <f aca="false">IF(COUNTA($D117)&gt;0,COUNTIF($D$2:$D117,F$1),"")</f>
+        <v/>
+      </c>
+      <c r="G117" s="5" t="str">
+        <f aca="false">IF(COUNTA($D117)&gt;0,COUNTIF($D$2:$D117,G$1),"")</f>
+        <v/>
+      </c>
+      <c r="H117" s="5" t="str">
+        <f aca="false">IF(COUNTA($D117)&gt;0,COUNTIF($D$2:$D117,H$1),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="118" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D118" s="5"/>
-      <c r="E118" s="5"/>
-      <c r="F118" s="5"/>
-      <c r="G118" s="5"/>
-      <c r="H118" s="5"/>
+      <c r="E118" s="5" t="str">
+        <f aca="false">IF(COUNTA($D118)&gt;0,COUNTIF($D$2:$D118,E$1),"")</f>
+        <v/>
+      </c>
+      <c r="F118" s="5" t="str">
+        <f aca="false">IF(COUNTA($D118)&gt;0,COUNTIF($D$2:$D118,F$1),"")</f>
+        <v/>
+      </c>
+      <c r="G118" s="5" t="str">
+        <f aca="false">IF(COUNTA($D118)&gt;0,COUNTIF($D$2:$D118,G$1),"")</f>
+        <v/>
+      </c>
+      <c r="H118" s="5" t="str">
+        <f aca="false">IF(COUNTA($D118)&gt;0,COUNTIF($D$2:$D118,H$1),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="119" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D119" s="5"/>
-      <c r="E119" s="5"/>
-      <c r="F119" s="5"/>
-      <c r="G119" s="5"/>
-      <c r="H119" s="5"/>
+      <c r="E119" s="5" t="str">
+        <f aca="false">IF(COUNTA($D119)&gt;0,COUNTIF($D$2:$D119,E$1),"")</f>
+        <v/>
+      </c>
+      <c r="F119" s="5" t="str">
+        <f aca="false">IF(COUNTA($D119)&gt;0,COUNTIF($D$2:$D119,F$1),"")</f>
+        <v/>
+      </c>
+      <c r="G119" s="5" t="str">
+        <f aca="false">IF(COUNTA($D119)&gt;0,COUNTIF($D$2:$D119,G$1),"")</f>
+        <v/>
+      </c>
+      <c r="H119" s="5" t="str">
+        <f aca="false">IF(COUNTA($D119)&gt;0,COUNTIF($D$2:$D119,H$1),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="120" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D120" s="5"/>
-      <c r="E120" s="5"/>
-      <c r="F120" s="5"/>
-      <c r="G120" s="5"/>
-      <c r="H120" s="5"/>
+      <c r="E120" s="5" t="str">
+        <f aca="false">IF(COUNTA($D120)&gt;0,COUNTIF($D$2:$D120,E$1),"")</f>
+        <v/>
+      </c>
+      <c r="F120" s="5" t="str">
+        <f aca="false">IF(COUNTA($D120)&gt;0,COUNTIF($D$2:$D120,F$1),"")</f>
+        <v/>
+      </c>
+      <c r="G120" s="5" t="str">
+        <f aca="false">IF(COUNTA($D120)&gt;0,COUNTIF($D$2:$D120,G$1),"")</f>
+        <v/>
+      </c>
+      <c r="H120" s="5" t="str">
+        <f aca="false">IF(COUNTA($D120)&gt;0,COUNTIF($D$2:$D120,H$1),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="121" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E121" s="5" t="str">
+        <f aca="false">IF(COUNTA($D121)&gt;0,COUNTIF($D$2:$D121,E$1),"")</f>
+        <v/>
+      </c>
+      <c r="F121" s="5" t="str">
+        <f aca="false">IF(COUNTA($D121)&gt;0,COUNTIF($D$2:$D121,F$1),"")</f>
+        <v/>
+      </c>
+      <c r="G121" s="5" t="str">
+        <f aca="false">IF(COUNTA($D121)&gt;0,COUNTIF($D$2:$D121,G$1),"")</f>
+        <v/>
+      </c>
+      <c r="H121" s="5" t="str">
+        <f aca="false">IF(COUNTA($D121)&gt;0,COUNTIF($D$2:$D121,H$1),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="122" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E122" s="5" t="str">
+        <f aca="false">IF(COUNTA($D122)&gt;0,COUNTIF($D$2:$D122,E$1),"")</f>
+        <v/>
+      </c>
+      <c r="F122" s="5" t="str">
+        <f aca="false">IF(COUNTA($D122)&gt;0,COUNTIF($D$2:$D122,F$1),"")</f>
+        <v/>
+      </c>
+      <c r="G122" s="5" t="str">
+        <f aca="false">IF(COUNTA($D122)&gt;0,COUNTIF($D$2:$D122,G$1),"")</f>
+        <v/>
+      </c>
+      <c r="H122" s="5" t="str">
+        <f aca="false">IF(COUNTA($D122)&gt;0,COUNTIF($D$2:$D122,H$1),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="123" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E123" s="5" t="str">
+        <f aca="false">IF(COUNTA($D123)&gt;0,COUNTIF($D$2:$D123,E$1),"")</f>
+        <v/>
+      </c>
+      <c r="F123" s="5" t="str">
+        <f aca="false">IF(COUNTA($D123)&gt;0,COUNTIF($D$2:$D123,F$1),"")</f>
+        <v/>
+      </c>
+      <c r="G123" s="5" t="str">
+        <f aca="false">IF(COUNTA($D123)&gt;0,COUNTIF($D$2:$D123,G$1),"")</f>
+        <v/>
+      </c>
+      <c r="H123" s="5" t="str">
+        <f aca="false">IF(COUNTA($D123)&gt;0,COUNTIF($D$2:$D123,H$1),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="124" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E124" s="5" t="str">
+        <f aca="false">IF(COUNTA($D124)&gt;0,COUNTIF($D$2:$D124,E$1),"")</f>
+        <v/>
+      </c>
+      <c r="F124" s="5" t="str">
+        <f aca="false">IF(COUNTA($D124)&gt;0,COUNTIF($D$2:$D124,F$1),"")</f>
+        <v/>
+      </c>
+      <c r="G124" s="5" t="str">
+        <f aca="false">IF(COUNTA($D124)&gt;0,COUNTIF($D$2:$D124,G$1),"")</f>
+        <v/>
+      </c>
+      <c r="H124" s="5" t="str">
+        <f aca="false">IF(COUNTA($D124)&gt;0,COUNTIF($D$2:$D124,H$1),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="125" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E125" s="5" t="str">
+        <f aca="false">IF(COUNTA($D125)&gt;0,COUNTIF($D$2:$D125,E$1),"")</f>
+        <v/>
+      </c>
+      <c r="F125" s="5" t="str">
+        <f aca="false">IF(COUNTA($D125)&gt;0,COUNTIF($D$2:$D125,F$1),"")</f>
+        <v/>
+      </c>
+      <c r="G125" s="5" t="str">
+        <f aca="false">IF(COUNTA($D125)&gt;0,COUNTIF($D$2:$D125,G$1),"")</f>
+        <v/>
+      </c>
+      <c r="H125" s="5" t="str">
+        <f aca="false">IF(COUNTA($D125)&gt;0,COUNTIF($D$2:$D125,H$1),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="126" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E126" s="5" t="str">
+        <f aca="false">IF(COUNTA($D126)&gt;0,COUNTIF($D$2:$D126,E$1),"")</f>
+        <v/>
+      </c>
+      <c r="F126" s="5" t="str">
+        <f aca="false">IF(COUNTA($D126)&gt;0,COUNTIF($D$2:$D126,F$1),"")</f>
+        <v/>
+      </c>
+      <c r="G126" s="5" t="str">
+        <f aca="false">IF(COUNTA($D126)&gt;0,COUNTIF($D$2:$D126,G$1),"")</f>
+        <v/>
+      </c>
+      <c r="H126" s="5" t="str">
+        <f aca="false">IF(COUNTA($D126)&gt;0,COUNTIF($D$2:$D126,H$1),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="127" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E127" s="5" t="str">
+        <f aca="false">IF(COUNTA($D127)&gt;0,COUNTIF($D$2:$D127,E$1),"")</f>
+        <v/>
+      </c>
+      <c r="F127" s="5" t="str">
+        <f aca="false">IF(COUNTA($D127)&gt;0,COUNTIF($D$2:$D127,F$1),"")</f>
+        <v/>
+      </c>
+      <c r="G127" s="5" t="str">
+        <f aca="false">IF(COUNTA($D127)&gt;0,COUNTIF($D$2:$D127,G$1),"")</f>
+        <v/>
+      </c>
+      <c r="H127" s="5" t="str">
+        <f aca="false">IF(COUNTA($D127)&gt;0,COUNTIF($D$2:$D127,H$1),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="128" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E128" s="5" t="str">
+        <f aca="false">IF(COUNTA($D128)&gt;0,COUNTIF($D$2:$D128,E$1),"")</f>
+        <v/>
+      </c>
+      <c r="F128" s="5" t="str">
+        <f aca="false">IF(COUNTA($D128)&gt;0,COUNTIF($D$2:$D128,F$1),"")</f>
+        <v/>
+      </c>
+      <c r="G128" s="5" t="str">
+        <f aca="false">IF(COUNTA($D128)&gt;0,COUNTIF($D$2:$D128,G$1),"")</f>
+        <v/>
+      </c>
+      <c r="H128" s="5" t="str">
+        <f aca="false">IF(COUNTA($D128)&gt;0,COUNTIF($D$2:$D128,H$1),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="129" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E129" s="5" t="str">
+        <f aca="false">IF(COUNTA($D129)&gt;0,COUNTIF($D$2:$D129,E$1),"")</f>
+        <v/>
+      </c>
+      <c r="F129" s="5" t="str">
+        <f aca="false">IF(COUNTA($D129)&gt;0,COUNTIF($D$2:$D129,F$1),"")</f>
+        <v/>
+      </c>
+      <c r="G129" s="5" t="str">
+        <f aca="false">IF(COUNTA($D129)&gt;0,COUNTIF($D$2:$D129,G$1),"")</f>
+        <v/>
+      </c>
+      <c r="H129" s="5" t="str">
+        <f aca="false">IF(COUNTA($D129)&gt;0,COUNTIF($D$2:$D129,H$1),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="130" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E130" s="5" t="str">
+        <f aca="false">IF(COUNTA($D130)&gt;0,COUNTIF($D$2:$D130,E$1),"")</f>
+        <v/>
+      </c>
+      <c r="F130" s="5" t="str">
+        <f aca="false">IF(COUNTA($D130)&gt;0,COUNTIF($D$2:$D130,F$1),"")</f>
+        <v/>
+      </c>
+      <c r="G130" s="5" t="str">
+        <f aca="false">IF(COUNTA($D130)&gt;0,COUNTIF($D$2:$D130,G$1),"")</f>
+        <v/>
+      </c>
+      <c r="H130" s="5" t="str">
+        <f aca="false">IF(COUNTA($D130)&gt;0,COUNTIF($D$2:$D130,H$1),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="131" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E131" s="5" t="str">
+        <f aca="false">IF(COUNTA($D131)&gt;0,COUNTIF($D$2:$D131,E$1),"")</f>
+        <v/>
+      </c>
+      <c r="F131" s="5" t="str">
+        <f aca="false">IF(COUNTA($D131)&gt;0,COUNTIF($D$2:$D131,F$1),"")</f>
+        <v/>
+      </c>
+      <c r="G131" s="5" t="str">
+        <f aca="false">IF(COUNTA($D131)&gt;0,COUNTIF($D$2:$D131,G$1),"")</f>
+        <v/>
+      </c>
+      <c r="H131" s="5" t="str">
+        <f aca="false">IF(COUNTA($D131)&gt;0,COUNTIF($D$2:$D131,H$1),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="132" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E132" s="5" t="str">
+        <f aca="false">IF(COUNTA($D132)&gt;0,COUNTIF($D$2:$D132,E$1),"")</f>
+        <v/>
+      </c>
+      <c r="F132" s="5" t="str">
+        <f aca="false">IF(COUNTA($D132)&gt;0,COUNTIF($D$2:$D132,F$1),"")</f>
+        <v/>
+      </c>
+      <c r="G132" s="5" t="str">
+        <f aca="false">IF(COUNTA($D132)&gt;0,COUNTIF($D$2:$D132,G$1),"")</f>
+        <v/>
+      </c>
+      <c r="H132" s="5" t="str">
+        <f aca="false">IF(COUNTA($D132)&gt;0,COUNTIF($D$2:$D132,H$1),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="133" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E133" s="5" t="str">
+        <f aca="false">IF(COUNTA($D133)&gt;0,COUNTIF($D$2:$D133,E$1),"")</f>
+        <v/>
+      </c>
+      <c r="F133" s="5" t="str">
+        <f aca="false">IF(COUNTA($D133)&gt;0,COUNTIF($D$2:$D133,F$1),"")</f>
+        <v/>
+      </c>
+      <c r="G133" s="5" t="str">
+        <f aca="false">IF(COUNTA($D133)&gt;0,COUNTIF($D$2:$D133,G$1),"")</f>
+        <v/>
+      </c>
+      <c r="H133" s="5" t="str">
+        <f aca="false">IF(COUNTA($D133)&gt;0,COUNTIF($D$2:$D133,H$1),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="134" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E134" s="5" t="str">
+        <f aca="false">IF(COUNTA($D134)&gt;0,COUNTIF($D$2:$D134,E$1),"")</f>
+        <v/>
+      </c>
+      <c r="F134" s="5" t="str">
+        <f aca="false">IF(COUNTA($D134)&gt;0,COUNTIF($D$2:$D134,F$1),"")</f>
+        <v/>
+      </c>
+      <c r="G134" s="5" t="str">
+        <f aca="false">IF(COUNTA($D134)&gt;0,COUNTIF($D$2:$D134,G$1),"")</f>
+        <v/>
+      </c>
+      <c r="H134" s="5" t="str">
+        <f aca="false">IF(COUNTA($D134)&gt;0,COUNTIF($D$2:$D134,H$1),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="135" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E135" s="5" t="str">
+        <f aca="false">IF(COUNTA($D135)&gt;0,COUNTIF($D$2:$D135,E$1),"")</f>
+        <v/>
+      </c>
+      <c r="F135" s="5" t="str">
+        <f aca="false">IF(COUNTA($D135)&gt;0,COUNTIF($D$2:$D135,F$1),"")</f>
+        <v/>
+      </c>
+      <c r="G135" s="5" t="str">
+        <f aca="false">IF(COUNTA($D135)&gt;0,COUNTIF($D$2:$D135,G$1),"")</f>
+        <v/>
+      </c>
+      <c r="H135" s="5" t="str">
+        <f aca="false">IF(COUNTA($D135)&gt;0,COUNTIF($D$2:$D135,H$1),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="136" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E136" s="5" t="str">
+        <f aca="false">IF(COUNTA($D136)&gt;0,COUNTIF($D$2:$D136,E$1),"")</f>
+        <v/>
+      </c>
+      <c r="F136" s="5" t="str">
+        <f aca="false">IF(COUNTA($D136)&gt;0,COUNTIF($D$2:$D136,F$1),"")</f>
+        <v/>
+      </c>
+      <c r="G136" s="5" t="str">
+        <f aca="false">IF(COUNTA($D136)&gt;0,COUNTIF($D$2:$D136,G$1),"")</f>
+        <v/>
+      </c>
+      <c r="H136" s="5" t="str">
+        <f aca="false">IF(COUNTA($D136)&gt;0,COUNTIF($D$2:$D136,H$1),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="137" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E137" s="5" t="str">
+        <f aca="false">IF(COUNTA($D137)&gt;0,COUNTIF($D$2:$D137,E$1),"")</f>
+        <v/>
+      </c>
+      <c r="F137" s="5" t="str">
+        <f aca="false">IF(COUNTA($D137)&gt;0,COUNTIF($D$2:$D137,F$1),"")</f>
+        <v/>
+      </c>
+      <c r="G137" s="5" t="str">
+        <f aca="false">IF(COUNTA($D137)&gt;0,COUNTIF($D$2:$D137,G$1),"")</f>
+        <v/>
+      </c>
+      <c r="H137" s="5" t="str">
+        <f aca="false">IF(COUNTA($D137)&gt;0,COUNTIF($D$2:$D137,H$1),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="138" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E138" s="5" t="str">
+        <f aca="false">IF(COUNTA($D138)&gt;0,COUNTIF($D$2:$D138,E$1),"")</f>
+        <v/>
+      </c>
+      <c r="F138" s="5" t="str">
+        <f aca="false">IF(COUNTA($D138)&gt;0,COUNTIF($D$2:$D138,F$1),"")</f>
+        <v/>
+      </c>
+      <c r="G138" s="5" t="str">
+        <f aca="false">IF(COUNTA($D138)&gt;0,COUNTIF($D$2:$D138,G$1),"")</f>
+        <v/>
+      </c>
+      <c r="H138" s="5" t="str">
+        <f aca="false">IF(COUNTA($D138)&gt;0,COUNTIF($D$2:$D138,H$1),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="139" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E139" s="5" t="str">
+        <f aca="false">IF(COUNTA($D139)&gt;0,COUNTIF($D$2:$D139,E$1),"")</f>
+        <v/>
+      </c>
+      <c r="F139" s="5" t="str">
+        <f aca="false">IF(COUNTA($D139)&gt;0,COUNTIF($D$2:$D139,F$1),"")</f>
+        <v/>
+      </c>
+      <c r="G139" s="5" t="str">
+        <f aca="false">IF(COUNTA($D139)&gt;0,COUNTIF($D$2:$D139,G$1),"")</f>
+        <v/>
+      </c>
+      <c r="H139" s="5" t="str">
+        <f aca="false">IF(COUNTA($D139)&gt;0,COUNTIF($D$2:$D139,H$1),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="140" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E140" s="5" t="str">
+        <f aca="false">IF(COUNTA($D140)&gt;0,COUNTIF($D$2:$D140,E$1),"")</f>
+        <v/>
+      </c>
+      <c r="F140" s="5" t="str">
+        <f aca="false">IF(COUNTA($D140)&gt;0,COUNTIF($D$2:$D140,F$1),"")</f>
+        <v/>
+      </c>
+      <c r="G140" s="5" t="str">
+        <f aca="false">IF(COUNTA($D140)&gt;0,COUNTIF($D$2:$D140,G$1),"")</f>
+        <v/>
+      </c>
+      <c r="H140" s="5" t="str">
+        <f aca="false">IF(COUNTA($D140)&gt;0,COUNTIF($D$2:$D140,H$1),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="141" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E141" s="5" t="str">
+        <f aca="false">IF(COUNTA($D141)&gt;0,COUNTIF($D$2:$D141,E$1),"")</f>
+        <v/>
+      </c>
+      <c r="F141" s="5" t="str">
+        <f aca="false">IF(COUNTA($D141)&gt;0,COUNTIF($D$2:$D141,F$1),"")</f>
+        <v/>
+      </c>
+      <c r="G141" s="5" t="str">
+        <f aca="false">IF(COUNTA($D141)&gt;0,COUNTIF($D$2:$D141,G$1),"")</f>
+        <v/>
+      </c>
+      <c r="H141" s="5" t="str">
+        <f aca="false">IF(COUNTA($D141)&gt;0,COUNTIF($D$2:$D141,H$1),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="142" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E142" s="5" t="str">
+        <f aca="false">IF(COUNTA($D142)&gt;0,COUNTIF($D$2:$D142,E$1),"")</f>
+        <v/>
+      </c>
+      <c r="F142" s="5" t="str">
+        <f aca="false">IF(COUNTA($D142)&gt;0,COUNTIF($D$2:$D142,F$1),"")</f>
+        <v/>
+      </c>
+      <c r="G142" s="5" t="str">
+        <f aca="false">IF(COUNTA($D142)&gt;0,COUNTIF($D$2:$D142,G$1),"")</f>
+        <v/>
+      </c>
+      <c r="H142" s="5" t="str">
+        <f aca="false">IF(COUNTA($D142)&gt;0,COUNTIF($D$2:$D142,H$1),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="143" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E143" s="5" t="str">
+        <f aca="false">IF(COUNTA($D143)&gt;0,COUNTIF($D$2:$D143,E$1),"")</f>
+        <v/>
+      </c>
+      <c r="F143" s="5" t="str">
+        <f aca="false">IF(COUNTA($D143)&gt;0,COUNTIF($D$2:$D143,F$1),"")</f>
+        <v/>
+      </c>
+      <c r="G143" s="5" t="str">
+        <f aca="false">IF(COUNTA($D143)&gt;0,COUNTIF($D$2:$D143,G$1),"")</f>
+        <v/>
+      </c>
+      <c r="H143" s="5" t="str">
+        <f aca="false">IF(COUNTA($D143)&gt;0,COUNTIF($D$2:$D143,H$1),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="144" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E144" s="5" t="str">
+        <f aca="false">IF(COUNTA($D144)&gt;0,COUNTIF($D$2:$D144,E$1),"")</f>
+        <v/>
+      </c>
+      <c r="F144" s="5" t="str">
+        <f aca="false">IF(COUNTA($D144)&gt;0,COUNTIF($D$2:$D144,F$1),"")</f>
+        <v/>
+      </c>
+      <c r="G144" s="5" t="str">
+        <f aca="false">IF(COUNTA($D144)&gt;0,COUNTIF($D$2:$D144,G$1),"")</f>
+        <v/>
+      </c>
+      <c r="H144" s="5" t="str">
+        <f aca="false">IF(COUNTA($D144)&gt;0,COUNTIF($D$2:$D144,H$1),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="145" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E145" s="5" t="str">
+        <f aca="false">IF(COUNTA($D145)&gt;0,COUNTIF($D$2:$D145,E$1),"")</f>
+        <v/>
+      </c>
+      <c r="F145" s="5" t="str">
+        <f aca="false">IF(COUNTA($D145)&gt;0,COUNTIF($D$2:$D145,F$1),"")</f>
+        <v/>
+      </c>
+      <c r="G145" s="5" t="str">
+        <f aca="false">IF(COUNTA($D145)&gt;0,COUNTIF($D$2:$D145,G$1),"")</f>
+        <v/>
+      </c>
+      <c r="H145" s="5" t="str">
+        <f aca="false">IF(COUNTA($D145)&gt;0,COUNTIF($D$2:$D145,H$1),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="146" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E146" s="5" t="str">
+        <f aca="false">IF(COUNTA($D146)&gt;0,COUNTIF($D$2:$D146,E$1),"")</f>
+        <v/>
+      </c>
+      <c r="F146" s="5" t="str">
+        <f aca="false">IF(COUNTA($D146)&gt;0,COUNTIF($D$2:$D146,F$1),"")</f>
+        <v/>
+      </c>
+      <c r="G146" s="5" t="str">
+        <f aca="false">IF(COUNTA($D146)&gt;0,COUNTIF($D$2:$D146,G$1),"")</f>
+        <v/>
+      </c>
+      <c r="H146" s="5" t="str">
+        <f aca="false">IF(COUNTA($D146)&gt;0,COUNTIF($D$2:$D146,H$1),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="147" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E147" s="5" t="str">
+        <f aca="false">IF(COUNTA($D147)&gt;0,COUNTIF($D$2:$D147,E$1),"")</f>
+        <v/>
+      </c>
+      <c r="F147" s="5" t="str">
+        <f aca="false">IF(COUNTA($D147)&gt;0,COUNTIF($D$2:$D147,F$1),"")</f>
+        <v/>
+      </c>
+      <c r="G147" s="5" t="str">
+        <f aca="false">IF(COUNTA($D147)&gt;0,COUNTIF($D$2:$D147,G$1),"")</f>
+        <v/>
+      </c>
+      <c r="H147" s="5" t="str">
+        <f aca="false">IF(COUNTA($D147)&gt;0,COUNTIF($D$2:$D147,H$1),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="148" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E148" s="5" t="str">
+        <f aca="false">IF(COUNTA($D148)&gt;0,COUNTIF($D$2:$D148,E$1),"")</f>
+        <v/>
+      </c>
+      <c r="F148" s="5" t="str">
+        <f aca="false">IF(COUNTA($D148)&gt;0,COUNTIF($D$2:$D148,F$1),"")</f>
+        <v/>
+      </c>
+      <c r="G148" s="5" t="str">
+        <f aca="false">IF(COUNTA($D148)&gt;0,COUNTIF($D$2:$D148,G$1),"")</f>
+        <v/>
+      </c>
+      <c r="H148" s="5" t="str">
+        <f aca="false">IF(COUNTA($D148)&gt;0,COUNTIF($D$2:$D148,H$1),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="149" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E149" s="5" t="str">
+        <f aca="false">IF(COUNTA($D149)&gt;0,COUNTIF($D$2:$D149,E$1),"")</f>
+        <v/>
+      </c>
+      <c r="F149" s="5" t="str">
+        <f aca="false">IF(COUNTA($D149)&gt;0,COUNTIF($D$2:$D149,F$1),"")</f>
+        <v/>
+      </c>
+      <c r="G149" s="5" t="str">
+        <f aca="false">IF(COUNTA($D149)&gt;0,COUNTIF($D$2:$D149,G$1),"")</f>
+        <v/>
+      </c>
+      <c r="H149" s="5" t="str">
+        <f aca="false">IF(COUNTA($D149)&gt;0,COUNTIF($D$2:$D149,H$1),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="150" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E150" s="5" t="str">
+        <f aca="false">IF(COUNTA($D150)&gt;0,COUNTIF($D$2:$D150,E$1),"")</f>
+        <v/>
+      </c>
+      <c r="F150" s="5" t="str">
+        <f aca="false">IF(COUNTA($D150)&gt;0,COUNTIF($D$2:$D150,F$1),"")</f>
+        <v/>
+      </c>
+      <c r="G150" s="5" t="str">
+        <f aca="false">IF(COUNTA($D150)&gt;0,COUNTIF($D$2:$D150,G$1),"")</f>
+        <v/>
+      </c>
+      <c r="H150" s="5" t="str">
+        <f aca="false">IF(COUNTA($D150)&gt;0,COUNTIF($D$2:$D150,H$1),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="151" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E151" s="5" t="str">
+        <f aca="false">IF(COUNTA($D151)&gt;0,COUNTIF($D$2:$D151,E$1),"")</f>
+        <v/>
+      </c>
+      <c r="F151" s="5" t="str">
+        <f aca="false">IF(COUNTA($D151)&gt;0,COUNTIF($D$2:$D151,F$1),"")</f>
+        <v/>
+      </c>
+      <c r="G151" s="5" t="str">
+        <f aca="false">IF(COUNTA($D151)&gt;0,COUNTIF($D$2:$D151,G$1),"")</f>
+        <v/>
+      </c>
+      <c r="H151" s="5" t="str">
+        <f aca="false">IF(COUNTA($D151)&gt;0,COUNTIF($D$2:$D151,H$1),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="152" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E152" s="5" t="str">
+        <f aca="false">IF(COUNTA($D152)&gt;0,COUNTIF($D$2:$D152,E$1),"")</f>
+        <v/>
+      </c>
+      <c r="F152" s="5" t="str">
+        <f aca="false">IF(COUNTA($D152)&gt;0,COUNTIF($D$2:$D152,F$1),"")</f>
+        <v/>
+      </c>
+      <c r="G152" s="5" t="str">
+        <f aca="false">IF(COUNTA($D152)&gt;0,COUNTIF($D$2:$D152,G$1),"")</f>
+        <v/>
+      </c>
+      <c r="H152" s="5" t="str">
+        <f aca="false">IF(COUNTA($D152)&gt;0,COUNTIF($D$2:$D152,H$1),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="153" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E153" s="5" t="str">
+        <f aca="false">IF(COUNTA($D153)&gt;0,COUNTIF($D$2:$D153,E$1),"")</f>
+        <v/>
+      </c>
+      <c r="F153" s="5" t="str">
+        <f aca="false">IF(COUNTA($D153)&gt;0,COUNTIF($D$2:$D153,F$1),"")</f>
+        <v/>
+      </c>
+      <c r="G153" s="5" t="str">
+        <f aca="false">IF(COUNTA($D153)&gt;0,COUNTIF($D$2:$D153,G$1),"")</f>
+        <v/>
+      </c>
+      <c r="H153" s="5" t="str">
+        <f aca="false">IF(COUNTA($D153)&gt;0,COUNTIF($D$2:$D153,H$1),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="154" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E154" s="5" t="str">
+        <f aca="false">IF(COUNTA($D154)&gt;0,COUNTIF($D$2:$D154,E$1),"")</f>
+        <v/>
+      </c>
+      <c r="F154" s="5" t="str">
+        <f aca="false">IF(COUNTA($D154)&gt;0,COUNTIF($D$2:$D154,F$1),"")</f>
+        <v/>
+      </c>
+      <c r="G154" s="5" t="str">
+        <f aca="false">IF(COUNTA($D154)&gt;0,COUNTIF($D$2:$D154,G$1),"")</f>
+        <v/>
+      </c>
+      <c r="H154" s="5" t="str">
+        <f aca="false">IF(COUNTA($D154)&gt;0,COUNTIF($D$2:$D154,H$1),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="155" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E155" s="5" t="str">
+        <f aca="false">IF(COUNTA($D155)&gt;0,COUNTIF($D$2:$D155,E$1),"")</f>
+        <v/>
+      </c>
+      <c r="F155" s="5" t="str">
+        <f aca="false">IF(COUNTA($D155)&gt;0,COUNTIF($D$2:$D155,F$1),"")</f>
+        <v/>
+      </c>
+      <c r="G155" s="5" t="str">
+        <f aca="false">IF(COUNTA($D155)&gt;0,COUNTIF($D$2:$D155,G$1),"")</f>
+        <v/>
+      </c>
+      <c r="H155" s="5" t="str">
+        <f aca="false">IF(COUNTA($D155)&gt;0,COUNTIF($D$2:$D155,H$1),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="156" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E156" s="5" t="str">
+        <f aca="false">IF(COUNTA($D156)&gt;0,COUNTIF($D$2:$D156,E$1),"")</f>
+        <v/>
+      </c>
+      <c r="F156" s="5" t="str">
+        <f aca="false">IF(COUNTA($D156)&gt;0,COUNTIF($D$2:$D156,F$1),"")</f>
+        <v/>
+      </c>
+      <c r="G156" s="5" t="str">
+        <f aca="false">IF(COUNTA($D156)&gt;0,COUNTIF($D$2:$D156,G$1),"")</f>
+        <v/>
+      </c>
+      <c r="H156" s="5" t="str">
+        <f aca="false">IF(COUNTA($D156)&gt;0,COUNTIF($D$2:$D156,H$1),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="157" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E157" s="5" t="str">
+        <f aca="false">IF(COUNTA($D157)&gt;0,COUNTIF($D$2:$D157,E$1),"")</f>
+        <v/>
+      </c>
+      <c r="F157" s="5" t="str">
+        <f aca="false">IF(COUNTA($D157)&gt;0,COUNTIF($D$2:$D157,F$1),"")</f>
+        <v/>
+      </c>
+      <c r="G157" s="5" t="str">
+        <f aca="false">IF(COUNTA($D157)&gt;0,COUNTIF($D$2:$D157,G$1),"")</f>
+        <v/>
+      </c>
+      <c r="H157" s="5" t="str">
+        <f aca="false">IF(COUNTA($D157)&gt;0,COUNTIF($D$2:$D157,H$1),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="158" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E158" s="5" t="str">
+        <f aca="false">IF(COUNTA($D158)&gt;0,COUNTIF($D$2:$D158,E$1),"")</f>
+        <v/>
+      </c>
+      <c r="F158" s="5" t="str">
+        <f aca="false">IF(COUNTA($D158)&gt;0,COUNTIF($D$2:$D158,F$1),"")</f>
+        <v/>
+      </c>
+      <c r="G158" s="5" t="str">
+        <f aca="false">IF(COUNTA($D158)&gt;0,COUNTIF($D$2:$D158,G$1),"")</f>
+        <v/>
+      </c>
+      <c r="H158" s="5" t="str">
+        <f aca="false">IF(COUNTA($D158)&gt;0,COUNTIF($D$2:$D158,H$1),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="159" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E159" s="5" t="str">
+        <f aca="false">IF(COUNTA($D159)&gt;0,COUNTIF($D$2:$D159,E$1),"")</f>
+        <v/>
+      </c>
+      <c r="F159" s="5" t="str">
+        <f aca="false">IF(COUNTA($D159)&gt;0,COUNTIF($D$2:$D159,F$1),"")</f>
+        <v/>
+      </c>
+      <c r="G159" s="5" t="str">
+        <f aca="false">IF(COUNTA($D159)&gt;0,COUNTIF($D$2:$D159,G$1),"")</f>
+        <v/>
+      </c>
+      <c r="H159" s="5" t="str">
+        <f aca="false">IF(COUNTA($D159)&gt;0,COUNTIF($D$2:$D159,H$1),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="160" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E160" s="5" t="str">
+        <f aca="false">IF(COUNTA($D160)&gt;0,COUNTIF($D$2:$D160,E$1),"")</f>
+        <v/>
+      </c>
+      <c r="F160" s="5" t="str">
+        <f aca="false">IF(COUNTA($D160)&gt;0,COUNTIF($D$2:$D160,F$1),"")</f>
+        <v/>
+      </c>
+      <c r="G160" s="5" t="str">
+        <f aca="false">IF(COUNTA($D160)&gt;0,COUNTIF($D$2:$D160,G$1),"")</f>
+        <v/>
+      </c>
+      <c r="H160" s="5" t="str">
+        <f aca="false">IF(COUNTA($D160)&gt;0,COUNTIF($D$2:$D160,H$1),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="161" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E161" s="5" t="str">
+        <f aca="false">IF(COUNTA($D161)&gt;0,COUNTIF($D$2:$D161,E$1),"")</f>
+        <v/>
+      </c>
+      <c r="F161" s="5" t="str">
+        <f aca="false">IF(COUNTA($D161)&gt;0,COUNTIF($D$2:$D161,F$1),"")</f>
+        <v/>
+      </c>
+      <c r="G161" s="5" t="str">
+        <f aca="false">IF(COUNTA($D161)&gt;0,COUNTIF($D$2:$D161,G$1),"")</f>
+        <v/>
+      </c>
+      <c r="H161" s="5" t="str">
+        <f aca="false">IF(COUNTA($D161)&gt;0,COUNTIF($D$2:$D161,H$1),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="162" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E162" s="5" t="str">
+        <f aca="false">IF(COUNTA($D162)&gt;0,COUNTIF($D$2:$D162,E$1),"")</f>
+        <v/>
+      </c>
+      <c r="F162" s="5" t="str">
+        <f aca="false">IF(COUNTA($D162)&gt;0,COUNTIF($D$2:$D162,F$1),"")</f>
+        <v/>
+      </c>
+      <c r="G162" s="5" t="str">
+        <f aca="false">IF(COUNTA($D162)&gt;0,COUNTIF($D$2:$D162,G$1),"")</f>
+        <v/>
+      </c>
+      <c r="H162" s="5" t="str">
+        <f aca="false">IF(COUNTA($D162)&gt;0,COUNTIF($D$2:$D162,H$1),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="163" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E163" s="5" t="str">
+        <f aca="false">IF(COUNTA($D163)&gt;0,COUNTIF($D$2:$D163,E$1),"")</f>
+        <v/>
+      </c>
+      <c r="F163" s="5" t="str">
+        <f aca="false">IF(COUNTA($D163)&gt;0,COUNTIF($D$2:$D163,F$1),"")</f>
+        <v/>
+      </c>
+      <c r="G163" s="5" t="str">
+        <f aca="false">IF(COUNTA($D163)&gt;0,COUNTIF($D$2:$D163,G$1),"")</f>
+        <v/>
+      </c>
+      <c r="H163" s="5" t="str">
+        <f aca="false">IF(COUNTA($D163)&gt;0,COUNTIF($D$2:$D163,H$1),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="164" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E164" s="5" t="str">
+        <f aca="false">IF(COUNTA($D164)&gt;0,COUNTIF($D$2:$D164,E$1),"")</f>
+        <v/>
+      </c>
+      <c r="F164" s="5" t="str">
+        <f aca="false">IF(COUNTA($D164)&gt;0,COUNTIF($D$2:$D164,F$1),"")</f>
+        <v/>
+      </c>
+      <c r="G164" s="5" t="str">
+        <f aca="false">IF(COUNTA($D164)&gt;0,COUNTIF($D$2:$D164,G$1),"")</f>
+        <v/>
+      </c>
+      <c r="H164" s="5" t="str">
+        <f aca="false">IF(COUNTA($D164)&gt;0,COUNTIF($D$2:$D164,H$1),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="165" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E165" s="5" t="str">
+        <f aca="false">IF(COUNTA($D165)&gt;0,COUNTIF($D$2:$D165,E$1),"")</f>
+        <v/>
+      </c>
+      <c r="F165" s="5" t="str">
+        <f aca="false">IF(COUNTA($D165)&gt;0,COUNTIF($D$2:$D165,F$1),"")</f>
+        <v/>
+      </c>
+      <c r="G165" s="5" t="str">
+        <f aca="false">IF(COUNTA($D165)&gt;0,COUNTIF($D$2:$D165,G$1),"")</f>
+        <v/>
+      </c>
+      <c r="H165" s="5" t="str">
+        <f aca="false">IF(COUNTA($D165)&gt;0,COUNTIF($D$2:$D165,H$1),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="166" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E166" s="5" t="str">
+        <f aca="false">IF(COUNTA($D166)&gt;0,COUNTIF($D$2:$D166,E$1),"")</f>
+        <v/>
+      </c>
+      <c r="F166" s="5" t="str">
+        <f aca="false">IF(COUNTA($D166)&gt;0,COUNTIF($D$2:$D166,F$1),"")</f>
+        <v/>
+      </c>
+      <c r="G166" s="5" t="str">
+        <f aca="false">IF(COUNTA($D166)&gt;0,COUNTIF($D$2:$D166,G$1),"")</f>
+        <v/>
+      </c>
+      <c r="H166" s="5" t="str">
+        <f aca="false">IF(COUNTA($D166)&gt;0,COUNTIF($D$2:$D166,H$1),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="167" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E167" s="5" t="str">
+        <f aca="false">IF(COUNTA($D167)&gt;0,COUNTIF($D$2:$D167,E$1),"")</f>
+        <v/>
+      </c>
+      <c r="F167" s="5" t="str">
+        <f aca="false">IF(COUNTA($D167)&gt;0,COUNTIF($D$2:$D167,F$1),"")</f>
+        <v/>
+      </c>
+      <c r="G167" s="5" t="str">
+        <f aca="false">IF(COUNTA($D167)&gt;0,COUNTIF($D$2:$D167,G$1),"")</f>
+        <v/>
+      </c>
+      <c r="H167" s="5" t="str">
+        <f aca="false">IF(COUNTA($D167)&gt;0,COUNTIF($D$2:$D167,H$1),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="168" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E168" s="5" t="str">
+        <f aca="false">IF(COUNTA($D168)&gt;0,COUNTIF($D$2:$D168,E$1),"")</f>
+        <v/>
+      </c>
+      <c r="F168" s="5" t="str">
+        <f aca="false">IF(COUNTA($D168)&gt;0,COUNTIF($D$2:$D168,F$1),"")</f>
+        <v/>
+      </c>
+      <c r="G168" s="5" t="str">
+        <f aca="false">IF(COUNTA($D168)&gt;0,COUNTIF($D$2:$D168,G$1),"")</f>
+        <v/>
+      </c>
+      <c r="H168" s="5" t="str">
+        <f aca="false">IF(COUNTA($D168)&gt;0,COUNTIF($D$2:$D168,H$1),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="169" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E169" s="5" t="str">
+        <f aca="false">IF(COUNTA($D169)&gt;0,COUNTIF($D$2:$D169,E$1),"")</f>
+        <v/>
+      </c>
+      <c r="F169" s="5" t="str">
+        <f aca="false">IF(COUNTA($D169)&gt;0,COUNTIF($D$2:$D169,F$1),"")</f>
+        <v/>
+      </c>
+      <c r="G169" s="5" t="str">
+        <f aca="false">IF(COUNTA($D169)&gt;0,COUNTIF($D$2:$D169,G$1),"")</f>
+        <v/>
+      </c>
+      <c r="H169" s="5" t="str">
+        <f aca="false">IF(COUNTA($D169)&gt;0,COUNTIF($D$2:$D169,H$1),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="170" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E170" s="5" t="str">
+        <f aca="false">IF(COUNTA($D170)&gt;0,COUNTIF($D$2:$D170,E$1),"")</f>
+        <v/>
+      </c>
+      <c r="F170" s="5" t="str">
+        <f aca="false">IF(COUNTA($D170)&gt;0,COUNTIF($D$2:$D170,F$1),"")</f>
+        <v/>
+      </c>
+      <c r="G170" s="5" t="str">
+        <f aca="false">IF(COUNTA($D170)&gt;0,COUNTIF($D$2:$D170,G$1),"")</f>
+        <v/>
+      </c>
+      <c r="H170" s="5" t="str">
+        <f aca="false">IF(COUNTA($D170)&gt;0,COUNTIF($D$2:$D170,H$1),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="171" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E171" s="5" t="str">
+        <f aca="false">IF(COUNTA($D171)&gt;0,COUNTIF($D$2:$D171,E$1),"")</f>
+        <v/>
+      </c>
+      <c r="F171" s="5" t="str">
+        <f aca="false">IF(COUNTA($D171)&gt;0,COUNTIF($D$2:$D171,F$1),"")</f>
+        <v/>
+      </c>
+      <c r="G171" s="5" t="str">
+        <f aca="false">IF(COUNTA($D171)&gt;0,COUNTIF($D$2:$D171,G$1),"")</f>
+        <v/>
+      </c>
+      <c r="H171" s="5" t="str">
+        <f aca="false">IF(COUNTA($D171)&gt;0,COUNTIF($D$2:$D171,H$1),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="172" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E172" s="5" t="str">
+        <f aca="false">IF(COUNTA($D172)&gt;0,COUNTIF($D$2:$D172,E$1),"")</f>
+        <v/>
+      </c>
+      <c r="F172" s="5" t="str">
+        <f aca="false">IF(COUNTA($D172)&gt;0,COUNTIF($D$2:$D172,F$1),"")</f>
+        <v/>
+      </c>
+      <c r="G172" s="5" t="str">
+        <f aca="false">IF(COUNTA($D172)&gt;0,COUNTIF($D$2:$D172,G$1),"")</f>
+        <v/>
+      </c>
+      <c r="H172" s="5" t="str">
+        <f aca="false">IF(COUNTA($D172)&gt;0,COUNTIF($D$2:$D172,H$1),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="173" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E173" s="5" t="str">
+        <f aca="false">IF(COUNTA($D173)&gt;0,COUNTIF($D$2:$D173,E$1),"")</f>
+        <v/>
+      </c>
+      <c r="F173" s="5" t="str">
+        <f aca="false">IF(COUNTA($D173)&gt;0,COUNTIF($D$2:$D173,F$1),"")</f>
+        <v/>
+      </c>
+      <c r="G173" s="5" t="str">
+        <f aca="false">IF(COUNTA($D173)&gt;0,COUNTIF($D$2:$D173,G$1),"")</f>
+        <v/>
+      </c>
+      <c r="H173" s="5" t="str">
+        <f aca="false">IF(COUNTA($D173)&gt;0,COUNTIF($D$2:$D173,H$1),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="174" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E174" s="5" t="str">
+        <f aca="false">IF(COUNTA($D174)&gt;0,COUNTIF($D$2:$D174,E$1),"")</f>
+        <v/>
+      </c>
+      <c r="F174" s="5" t="str">
+        <f aca="false">IF(COUNTA($D174)&gt;0,COUNTIF($D$2:$D174,F$1),"")</f>
+        <v/>
+      </c>
+      <c r="G174" s="5" t="str">
+        <f aca="false">IF(COUNTA($D174)&gt;0,COUNTIF($D$2:$D174,G$1),"")</f>
+        <v/>
+      </c>
+      <c r="H174" s="5" t="str">
+        <f aca="false">IF(COUNTA($D174)&gt;0,COUNTIF($D$2:$D174,H$1),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="175" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E175" s="5" t="str">
+        <f aca="false">IF(COUNTA($D175)&gt;0,COUNTIF($D$2:$D175,E$1),"")</f>
+        <v/>
+      </c>
+      <c r="F175" s="5" t="str">
+        <f aca="false">IF(COUNTA($D175)&gt;0,COUNTIF($D$2:$D175,F$1),"")</f>
+        <v/>
+      </c>
+      <c r="G175" s="5" t="str">
+        <f aca="false">IF(COUNTA($D175)&gt;0,COUNTIF($D$2:$D175,G$1),"")</f>
+        <v/>
+      </c>
+      <c r="H175" s="5" t="str">
+        <f aca="false">IF(COUNTA($D175)&gt;0,COUNTIF($D$2:$D175,H$1),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="176" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E176" s="5" t="str">
+        <f aca="false">IF(COUNTA($D176)&gt;0,COUNTIF($D$2:$D176,E$1),"")</f>
+        <v/>
+      </c>
+      <c r="F176" s="5" t="str">
+        <f aca="false">IF(COUNTA($D176)&gt;0,COUNTIF($D$2:$D176,F$1),"")</f>
+        <v/>
+      </c>
+      <c r="G176" s="5" t="str">
+        <f aca="false">IF(COUNTA($D176)&gt;0,COUNTIF($D$2:$D176,G$1),"")</f>
+        <v/>
+      </c>
+      <c r="H176" s="5" t="str">
+        <f aca="false">IF(COUNTA($D176)&gt;0,COUNTIF($D$2:$D176,H$1),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="177" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E177" s="5" t="str">
+        <f aca="false">IF(COUNTA($D177)&gt;0,COUNTIF($D$2:$D177,E$1),"")</f>
+        <v/>
+      </c>
+      <c r="F177" s="5" t="str">
+        <f aca="false">IF(COUNTA($D177)&gt;0,COUNTIF($D$2:$D177,F$1),"")</f>
+        <v/>
+      </c>
+      <c r="G177" s="5" t="str">
+        <f aca="false">IF(COUNTA($D177)&gt;0,COUNTIF($D$2:$D177,G$1),"")</f>
+        <v/>
+      </c>
+      <c r="H177" s="5" t="str">
+        <f aca="false">IF(COUNTA($D177)&gt;0,COUNTIF($D$2:$D177,H$1),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="178" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E178" s="5" t="str">
+        <f aca="false">IF(COUNTA($D178)&gt;0,COUNTIF($D$2:$D178,E$1),"")</f>
+        <v/>
+      </c>
+      <c r="F178" s="5" t="str">
+        <f aca="false">IF(COUNTA($D178)&gt;0,COUNTIF($D$2:$D178,F$1),"")</f>
+        <v/>
+      </c>
+      <c r="G178" s="5" t="str">
+        <f aca="false">IF(COUNTA($D178)&gt;0,COUNTIF($D$2:$D178,G$1),"")</f>
+        <v/>
+      </c>
+      <c r="H178" s="5" t="str">
+        <f aca="false">IF(COUNTA($D178)&gt;0,COUNTIF($D$2:$D178,H$1),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="179" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E179" s="5" t="str">
+        <f aca="false">IF(COUNTA($D179)&gt;0,COUNTIF($D$2:$D179,E$1),"")</f>
+        <v/>
+      </c>
+      <c r="F179" s="5" t="str">
+        <f aca="false">IF(COUNTA($D179)&gt;0,COUNTIF($D$2:$D179,F$1),"")</f>
+        <v/>
+      </c>
+      <c r="G179" s="5" t="str">
+        <f aca="false">IF(COUNTA($D179)&gt;0,COUNTIF($D$2:$D179,G$1),"")</f>
+        <v/>
+      </c>
+      <c r="H179" s="5" t="str">
+        <f aca="false">IF(COUNTA($D179)&gt;0,COUNTIF($D$2:$D179,H$1),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="180" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E180" s="5" t="str">
+        <f aca="false">IF(COUNTA($D180)&gt;0,COUNTIF($D$2:$D180,E$1),"")</f>
+        <v/>
+      </c>
+      <c r="F180" s="5" t="str">
+        <f aca="false">IF(COUNTA($D180)&gt;0,COUNTIF($D$2:$D180,F$1),"")</f>
+        <v/>
+      </c>
+      <c r="G180" s="5" t="str">
+        <f aca="false">IF(COUNTA($D180)&gt;0,COUNTIF($D$2:$D180,G$1),"")</f>
+        <v/>
+      </c>
+      <c r="H180" s="5" t="str">
+        <f aca="false">IF(COUNTA($D180)&gt;0,COUNTIF($D$2:$D180,H$1),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="181" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E181" s="5" t="str">
+        <f aca="false">IF(COUNTA($D181)&gt;0,COUNTIF($D$2:$D181,E$1),"")</f>
+        <v/>
+      </c>
+      <c r="F181" s="5" t="str">
+        <f aca="false">IF(COUNTA($D181)&gt;0,COUNTIF($D$2:$D181,F$1),"")</f>
+        <v/>
+      </c>
+      <c r="G181" s="5" t="str">
+        <f aca="false">IF(COUNTA($D181)&gt;0,COUNTIF($D$2:$D181,G$1),"")</f>
+        <v/>
+      </c>
+      <c r="H181" s="5" t="str">
+        <f aca="false">IF(COUNTA($D181)&gt;0,COUNTIF($D$2:$D181,H$1),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="182" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E182" s="5" t="str">
+        <f aca="false">IF(COUNTA($D182)&gt;0,COUNTIF($D$2:$D182,E$1),"")</f>
+        <v/>
+      </c>
+      <c r="F182" s="5" t="str">
+        <f aca="false">IF(COUNTA($D182)&gt;0,COUNTIF($D$2:$D182,F$1),"")</f>
+        <v/>
+      </c>
+      <c r="G182" s="5" t="str">
+        <f aca="false">IF(COUNTA($D182)&gt;0,COUNTIF($D$2:$D182,G$1),"")</f>
+        <v/>
+      </c>
+      <c r="H182" s="5" t="str">
+        <f aca="false">IF(COUNTA($D182)&gt;0,COUNTIF($D$2:$D182,H$1),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="183" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E183" s="5" t="str">
+        <f aca="false">IF(COUNTA($D183)&gt;0,COUNTIF($D$2:$D183,E$1),"")</f>
+        <v/>
+      </c>
+      <c r="F183" s="5" t="str">
+        <f aca="false">IF(COUNTA($D183)&gt;0,COUNTIF($D$2:$D183,F$1),"")</f>
+        <v/>
+      </c>
+      <c r="G183" s="5" t="str">
+        <f aca="false">IF(COUNTA($D183)&gt;0,COUNTIF($D$2:$D183,G$1),"")</f>
+        <v/>
+      </c>
+      <c r="H183" s="5" t="str">
+        <f aca="false">IF(COUNTA($D183)&gt;0,COUNTIF($D$2:$D183,H$1),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="184" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E184" s="5" t="str">
+        <f aca="false">IF(COUNTA($D184)&gt;0,COUNTIF($D$2:$D184,E$1),"")</f>
+        <v/>
+      </c>
+      <c r="F184" s="5" t="str">
+        <f aca="false">IF(COUNTA($D184)&gt;0,COUNTIF($D$2:$D184,F$1),"")</f>
+        <v/>
+      </c>
+      <c r="G184" s="5" t="str">
+        <f aca="false">IF(COUNTA($D184)&gt;0,COUNTIF($D$2:$D184,G$1),"")</f>
+        <v/>
+      </c>
+      <c r="H184" s="5" t="str">
+        <f aca="false">IF(COUNTA($D184)&gt;0,COUNTIF($D$2:$D184,H$1),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="185" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E185" s="5" t="str">
+        <f aca="false">IF(COUNTA($D185)&gt;0,COUNTIF($D$2:$D185,E$1),"")</f>
+        <v/>
+      </c>
+      <c r="F185" s="5" t="str">
+        <f aca="false">IF(COUNTA($D185)&gt;0,COUNTIF($D$2:$D185,F$1),"")</f>
+        <v/>
+      </c>
+      <c r="G185" s="5" t="str">
+        <f aca="false">IF(COUNTA($D185)&gt;0,COUNTIF($D$2:$D185,G$1),"")</f>
+        <v/>
+      </c>
+      <c r="H185" s="5" t="str">
+        <f aca="false">IF(COUNTA($D185)&gt;0,COUNTIF($D$2:$D185,H$1),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="186" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E186" s="5" t="str">
+        <f aca="false">IF(COUNTA($D186)&gt;0,COUNTIF($D$2:$D186,E$1),"")</f>
+        <v/>
+      </c>
+      <c r="F186" s="5" t="str">
+        <f aca="false">IF(COUNTA($D186)&gt;0,COUNTIF($D$2:$D186,F$1),"")</f>
+        <v/>
+      </c>
+      <c r="G186" s="5" t="str">
+        <f aca="false">IF(COUNTA($D186)&gt;0,COUNTIF($D$2:$D186,G$1),"")</f>
+        <v/>
+      </c>
+      <c r="H186" s="5" t="str">
+        <f aca="false">IF(COUNTA($D186)&gt;0,COUNTIF($D$2:$D186,H$1),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="187" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E187" s="5" t="str">
+        <f aca="false">IF(COUNTA($D187)&gt;0,COUNTIF($D$2:$D187,E$1),"")</f>
+        <v/>
+      </c>
+      <c r="F187" s="5" t="str">
+        <f aca="false">IF(COUNTA($D187)&gt;0,COUNTIF($D$2:$D187,F$1),"")</f>
+        <v/>
+      </c>
+      <c r="G187" s="5" t="str">
+        <f aca="false">IF(COUNTA($D187)&gt;0,COUNTIF($D$2:$D187,G$1),"")</f>
+        <v/>
+      </c>
+      <c r="H187" s="5" t="str">
+        <f aca="false">IF(COUNTA($D187)&gt;0,COUNTIF($D$2:$D187,H$1),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="188" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E188" s="5" t="str">
+        <f aca="false">IF(COUNTA($D188)&gt;0,COUNTIF($D$2:$D188,E$1),"")</f>
+        <v/>
+      </c>
+      <c r="F188" s="5" t="str">
+        <f aca="false">IF(COUNTA($D188)&gt;0,COUNTIF($D$2:$D188,F$1),"")</f>
+        <v/>
+      </c>
+      <c r="G188" s="5" t="str">
+        <f aca="false">IF(COUNTA($D188)&gt;0,COUNTIF($D$2:$D188,G$1),"")</f>
+        <v/>
+      </c>
+      <c r="H188" s="5" t="str">
+        <f aca="false">IF(COUNTA($D188)&gt;0,COUNTIF($D$2:$D188,H$1),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="189" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E189" s="5" t="str">
+        <f aca="false">IF(COUNTA($D189)&gt;0,COUNTIF($D$2:$D189,E$1),"")</f>
+        <v/>
+      </c>
+      <c r="F189" s="5" t="str">
+        <f aca="false">IF(COUNTA($D189)&gt;0,COUNTIF($D$2:$D189,F$1),"")</f>
+        <v/>
+      </c>
+      <c r="G189" s="5" t="str">
+        <f aca="false">IF(COUNTA($D189)&gt;0,COUNTIF($D$2:$D189,G$1),"")</f>
+        <v/>
+      </c>
+      <c r="H189" s="5" t="str">
+        <f aca="false">IF(COUNTA($D189)&gt;0,COUNTIF($D$2:$D189,H$1),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="190" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E190" s="5" t="str">
+        <f aca="false">IF(COUNTA($D190)&gt;0,COUNTIF($D$2:$D190,E$1),"")</f>
+        <v/>
+      </c>
+      <c r="F190" s="5" t="str">
+        <f aca="false">IF(COUNTA($D190)&gt;0,COUNTIF($D$2:$D190,F$1),"")</f>
+        <v/>
+      </c>
+      <c r="G190" s="5" t="str">
+        <f aca="false">IF(COUNTA($D190)&gt;0,COUNTIF($D$2:$D190,G$1),"")</f>
+        <v/>
+      </c>
+      <c r="H190" s="5" t="str">
+        <f aca="false">IF(COUNTA($D190)&gt;0,COUNTIF($D$2:$D190,H$1),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="191" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E191" s="5" t="str">
+        <f aca="false">IF(COUNTA($D191)&gt;0,COUNTIF($D$2:$D191,E$1),"")</f>
+        <v/>
+      </c>
+      <c r="F191" s="5" t="str">
+        <f aca="false">IF(COUNTA($D191)&gt;0,COUNTIF($D$2:$D191,F$1),"")</f>
+        <v/>
+      </c>
+      <c r="G191" s="5" t="str">
+        <f aca="false">IF(COUNTA($D191)&gt;0,COUNTIF($D$2:$D191,G$1),"")</f>
+        <v/>
+      </c>
+      <c r="H191" s="5" t="str">
+        <f aca="false">IF(COUNTA($D191)&gt;0,COUNTIF($D$2:$D191,H$1),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="192" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E192" s="5" t="str">
+        <f aca="false">IF(COUNTA($D192)&gt;0,COUNTIF($D$2:$D192,E$1),"")</f>
+        <v/>
+      </c>
+      <c r="F192" s="5" t="str">
+        <f aca="false">IF(COUNTA($D192)&gt;0,COUNTIF($D$2:$D192,F$1),"")</f>
+        <v/>
+      </c>
+      <c r="G192" s="5" t="str">
+        <f aca="false">IF(COUNTA($D192)&gt;0,COUNTIF($D$2:$D192,G$1),"")</f>
+        <v/>
+      </c>
+      <c r="H192" s="5" t="str">
+        <f aca="false">IF(COUNTA($D192)&gt;0,COUNTIF($D$2:$D192,H$1),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="193" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E193" s="5" t="str">
+        <f aca="false">IF(COUNTA($D193)&gt;0,COUNTIF($D$2:$D193,E$1),"")</f>
+        <v/>
+      </c>
+      <c r="F193" s="5" t="str">
+        <f aca="false">IF(COUNTA($D193)&gt;0,COUNTIF($D$2:$D193,F$1),"")</f>
+        <v/>
+      </c>
+      <c r="G193" s="5" t="str">
+        <f aca="false">IF(COUNTA($D193)&gt;0,COUNTIF($D$2:$D193,G$1),"")</f>
+        <v/>
+      </c>
+      <c r="H193" s="5" t="str">
+        <f aca="false">IF(COUNTA($D193)&gt;0,COUNTIF($D$2:$D193,H$1),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="194" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E194" s="5" t="str">
+        <f aca="false">IF(COUNTA($D194)&gt;0,COUNTIF($D$2:$D194,E$1),"")</f>
+        <v/>
+      </c>
+      <c r="F194" s="5" t="str">
+        <f aca="false">IF(COUNTA($D194)&gt;0,COUNTIF($D$2:$D194,F$1),"")</f>
+        <v/>
+      </c>
+      <c r="G194" s="5" t="str">
+        <f aca="false">IF(COUNTA($D194)&gt;0,COUNTIF($D$2:$D194,G$1),"")</f>
+        <v/>
+      </c>
+      <c r="H194" s="5" t="str">
+        <f aca="false">IF(COUNTA($D194)&gt;0,COUNTIF($D$2:$D194,H$1),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="195" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E195" s="5" t="str">
+        <f aca="false">IF(COUNTA($D195)&gt;0,COUNTIF($D$2:$D195,E$1),"")</f>
+        <v/>
+      </c>
+      <c r="F195" s="5" t="str">
+        <f aca="false">IF(COUNTA($D195)&gt;0,COUNTIF($D$2:$D195,F$1),"")</f>
+        <v/>
+      </c>
+      <c r="G195" s="5" t="str">
+        <f aca="false">IF(COUNTA($D195)&gt;0,COUNTIF($D$2:$D195,G$1),"")</f>
+        <v/>
+      </c>
+      <c r="H195" s="5" t="str">
+        <f aca="false">IF(COUNTA($D195)&gt;0,COUNTIF($D$2:$D195,H$1),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="196" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E196" s="5" t="str">
+        <f aca="false">IF(COUNTA($D196)&gt;0,COUNTIF($D$2:$D196,E$1),"")</f>
+        <v/>
+      </c>
+      <c r="F196" s="5" t="str">
+        <f aca="false">IF(COUNTA($D196)&gt;0,COUNTIF($D$2:$D196,F$1),"")</f>
+        <v/>
+      </c>
+      <c r="G196" s="5" t="str">
+        <f aca="false">IF(COUNTA($D196)&gt;0,COUNTIF($D$2:$D196,G$1),"")</f>
+        <v/>
+      </c>
+      <c r="H196" s="5" t="str">
+        <f aca="false">IF(COUNTA($D196)&gt;0,COUNTIF($D$2:$D196,H$1),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="197" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E197" s="5" t="str">
+        <f aca="false">IF(COUNTA($D197)&gt;0,COUNTIF($D$2:$D197,E$1),"")</f>
+        <v/>
+      </c>
+      <c r="F197" s="5" t="str">
+        <f aca="false">IF(COUNTA($D197)&gt;0,COUNTIF($D$2:$D197,F$1),"")</f>
+        <v/>
+      </c>
+      <c r="G197" s="5" t="str">
+        <f aca="false">IF(COUNTA($D197)&gt;0,COUNTIF($D$2:$D197,G$1),"")</f>
+        <v/>
+      </c>
+      <c r="H197" s="5" t="str">
+        <f aca="false">IF(COUNTA($D197)&gt;0,COUNTIF($D$2:$D197,H$1),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="198" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E198" s="5" t="str">
+        <f aca="false">IF(COUNTA($D198)&gt;0,COUNTIF($D$2:$D198,E$1),"")</f>
+        <v/>
+      </c>
+      <c r="F198" s="5" t="str">
+        <f aca="false">IF(COUNTA($D198)&gt;0,COUNTIF($D$2:$D198,F$1),"")</f>
+        <v/>
+      </c>
+      <c r="G198" s="5" t="str">
+        <f aca="false">IF(COUNTA($D198)&gt;0,COUNTIF($D$2:$D198,G$1),"")</f>
+        <v/>
+      </c>
+      <c r="H198" s="5" t="str">
+        <f aca="false">IF(COUNTA($D198)&gt;0,COUNTIF($D$2:$D198,H$1),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="199" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E199" s="5" t="str">
+        <f aca="false">IF(COUNTA($D199)&gt;0,COUNTIF($D$2:$D199,E$1),"")</f>
+        <v/>
+      </c>
+      <c r="F199" s="5" t="str">
+        <f aca="false">IF(COUNTA($D199)&gt;0,COUNTIF($D$2:$D199,F$1),"")</f>
+        <v/>
+      </c>
+      <c r="G199" s="5" t="str">
+        <f aca="false">IF(COUNTA($D199)&gt;0,COUNTIF($D$2:$D199,G$1),"")</f>
+        <v/>
+      </c>
+      <c r="H199" s="5" t="str">
+        <f aca="false">IF(COUNTA($D199)&gt;0,COUNTIF($D$2:$D199,H$1),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="200" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E200" s="5" t="str">
+        <f aca="false">IF(COUNTA($D200)&gt;0,COUNTIF($D$2:$D200,E$1),"")</f>
+        <v/>
+      </c>
+      <c r="F200" s="5" t="str">
+        <f aca="false">IF(COUNTA($D200)&gt;0,COUNTIF($D$2:$D200,F$1),"")</f>
+        <v/>
+      </c>
+      <c r="G200" s="5" t="str">
+        <f aca="false">IF(COUNTA($D200)&gt;0,COUNTIF($D$2:$D200,G$1),"")</f>
+        <v/>
+      </c>
+      <c r="H200" s="5" t="str">
+        <f aca="false">IF(COUNTA($D200)&gt;0,COUNTIF($D$2:$D200,H$1),"")</f>
+        <v/>
+      </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="D1:H120">
+  <conditionalFormatting sqref="D1:H81 D82:D120 E82:H200">
     <cfRule type="cellIs" priority="2" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
       <formula>"Log"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D1:H120">
+  <conditionalFormatting sqref="D1:H81 D82:D120 E82:H200">
     <cfRule type="cellIs" priority="3" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="1">
       <formula>"Patroon"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D1:H120">
+  <conditionalFormatting sqref="D1:H81 D82:D120 E82:H200">
     <cfRule type="cellIs" priority="4" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="2">
       <formula>"Gedicht"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D1:H120">
+  <conditionalFormatting sqref="D1:H81 D82:D120 E82:H200">
     <cfRule type="cellIs" priority="5" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="3">
       <formula>"Schets"</formula>
     </cfRule>

</xml_diff>

<commit_message>
Sync from vault 2026-06-05 10:36:53
</commit_message>
<xml_diff>
--- a/content/Archief/0. PDFs & docs/Obol docs & forms/Irmijn Inc/Irma backup log.xlsx
+++ b/content/Archief/0. PDFs & docs/Obol docs & forms/Irmijn Inc/Irma backup log.xlsx
@@ -14,12 +14,14 @@
     <sheet name="Tatdata" sheetId="4" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="true" localSheetId="3" name="_xlnm._FilterDatabase" vbProcedure="false">Tatdata!$A$1:$B$13</definedName>
-    <definedName function="false" hidden="true" localSheetId="2" name="_xlnm._FilterDatabase" vbProcedure="false">Tatjes!$A$1:$F$93</definedName>
-    <definedName function="false" hidden="false" localSheetId="2" name="_xlnm._FilterDatabase" vbProcedure="false">Tatjes!$A$1:$F$92</definedName>
-    <definedName function="false" hidden="false" localSheetId="2" name="_xlnm._FilterDatabase_0" vbProcedure="false">Tatjes!$A$1:$F$91</definedName>
-    <definedName function="false" hidden="false" localSheetId="2" name="_xlnm._FilterDatabase_0_0" vbProcedure="false">Tatjes!$A$1:$F$90</definedName>
-    <definedName function="false" hidden="false" localSheetId="2" name="_xlnm._FilterDatabase_0_0_0" vbProcedure="false">Tatjes!$A$1:$F$88</definedName>
+    <definedName function="false" hidden="true" localSheetId="3" name="_xlnm._FilterDatabase" vbProcedure="false">Tatdata!$A$1:$B$14</definedName>
+    <definedName function="false" hidden="true" localSheetId="2" name="_xlnm._FilterDatabase" vbProcedure="false">Tatjes!$A$1:$F$94</definedName>
+    <definedName function="false" hidden="false" localSheetId="2" name="_xlnm._FilterDatabase" vbProcedure="false">Tatjes!$A$1:$F$93</definedName>
+    <definedName function="false" hidden="false" localSheetId="2" name="_xlnm._FilterDatabase_0" vbProcedure="false">Tatjes!$A$1:$F$92</definedName>
+    <definedName function="false" hidden="false" localSheetId="2" name="_xlnm._FilterDatabase_0_0" vbProcedure="false">Tatjes!$A$1:$F$91</definedName>
+    <definedName function="false" hidden="false" localSheetId="2" name="_xlnm._FilterDatabase_0_0_0" vbProcedure="false">Tatjes!$A$1:$F$90</definedName>
+    <definedName function="false" hidden="false" localSheetId="2" name="_xlnm._FilterDatabase_0_0_0_0" vbProcedure="false">Tatjes!$A$1:$F$88</definedName>
+    <definedName function="false" hidden="false" localSheetId="3" name="_xlnm._FilterDatabase" vbProcedure="false">Tatdata!$A$1:$B$13</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.001"/>
   <extLst>
@@ -31,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="493" uniqueCount="101">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="496" uniqueCount="102">
   <si>
     <t xml:space="preserve">Pagina</t>
   </si>
@@ -246,6 +248,15 @@
     <t xml:space="preserve">Bloem</t>
   </si>
   <si>
+    <t xml:space="preserve">Zilver</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Paars</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Marine</t>
+  </si>
+  <si>
     <t xml:space="preserve">Blauw</t>
   </si>
   <si>
@@ -253,15 +264,6 @@
   </si>
   <si>
     <t xml:space="preserve">Aqua</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Marine</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Zilver</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Paars</t>
   </si>
   <si>
     <t xml:space="preserve">Lila</t>
@@ -325,6 +327,9 @@
   </si>
   <si>
     <t xml:space="preserve">Grijs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mier</t>
   </si>
   <si>
     <t xml:space="preserve">Molentje</t>
@@ -418,14 +423,14 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF00CAFF"/>
-        <bgColor rgb="FF33CCCC"/>
+        <fgColor rgb="FFDDDDDD"/>
+        <bgColor rgb="FFFFCCCC"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF9BE2F6"/>
-        <bgColor rgb="FFCCFFFF"/>
+        <fgColor rgb="FF800080"/>
+        <bgColor rgb="FF800080"/>
       </patternFill>
     </fill>
     <fill>
@@ -436,14 +441,14 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFDDDDDD"/>
-        <bgColor rgb="FFFFCCCC"/>
+        <fgColor rgb="FF00CAFF"/>
+        <bgColor rgb="FF33CCCC"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF800080"/>
-        <bgColor rgb="FF800080"/>
+        <fgColor rgb="FF9BE2F6"/>
+        <bgColor rgb="FFCCFFFF"/>
       </patternFill>
     </fill>
     <fill>
@@ -608,7 +613,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -620,7 +625,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="8" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="8" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1598,11 +1603,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="68735520"/>
-        <c:axId val="59746143"/>
+        <c:axId val="74773951"/>
+        <c:axId val="78633205"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="68735520"/>
+        <c:axId val="74773951"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1658,14 +1663,14 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="59746143"/>
+        <c:crossAx val="78633205"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
         <c:lblOffset val="100"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="59746143"/>
+        <c:axId val="78633205"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1730,7 +1735,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="68735520"/>
+        <c:crossAx val="74773951"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -4791,11 +4796,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="24737048"/>
-        <c:axId val="80774908"/>
+        <c:axId val="94870094"/>
+        <c:axId val="9340594"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="24737048"/>
+        <c:axId val="94870094"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -4851,14 +4856,14 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="80774908"/>
+        <c:crossAx val="9340594"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
         <c:lblOffset val="100"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="80774908"/>
+        <c:axId val="9340594"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -4923,7 +4928,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="24737048"/>
+        <c:crossAx val="94870094"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -5011,10 +5016,10 @@
           <c:layoutTarget val="inner"/>
           <c:xMode val="edge"/>
           <c:yMode val="edge"/>
-          <c:x val="0.0889653016567677"/>
-          <c:y val="0.110950528071151"/>
-          <c:w val="0.846014379493592"/>
-          <c:h val="0.793440800444691"/>
+          <c:x val="0.0889708640740278"/>
+          <c:y val="0.110962864131643"/>
+          <c:w val="0.845942228335626"/>
+          <c:h val="0.793306648877029"/>
         </c:manualLayout>
       </c:layout>
       <c:lineChart>
@@ -5146,11 +5151,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="62636774"/>
-        <c:axId val="54095425"/>
+        <c:axId val="88120819"/>
+        <c:axId val="38893722"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="62636774"/>
+        <c:axId val="88120819"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -5178,14 +5183,14 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="54095425"/>
+        <c:crossAx val="38893722"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
         <c:lblOffset val="100"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="54095425"/>
+        <c:axId val="38893722"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -5250,7 +5255,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="62636774"/>
+        <c:crossAx val="88120819"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -5288,9 +5293,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>178920</xdr:colOff>
+      <xdr:colOff>178560</xdr:colOff>
       <xdr:row>23</xdr:row>
-      <xdr:rowOff>42480</xdr:rowOff>
+      <xdr:rowOff>42120</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -5299,7 +5304,7 @@
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
         <a:off x="6578280" y="543600"/>
-        <a:ext cx="5757480" cy="3237480"/>
+        <a:ext cx="5757120" cy="3237120"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -5318,9 +5323,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>342720</xdr:colOff>
+      <xdr:colOff>342360</xdr:colOff>
       <xdr:row>52</xdr:row>
-      <xdr:rowOff>90720</xdr:rowOff>
+      <xdr:rowOff>90360</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -5329,7 +5334,7 @@
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
         <a:off x="6741360" y="5305320"/>
-        <a:ext cx="5758200" cy="3238200"/>
+        <a:ext cx="5757840" cy="3237840"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -5353,9 +5358,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>12</xdr:col>
-      <xdr:colOff>462240</xdr:colOff>
+      <xdr:colOff>461880</xdr:colOff>
       <xdr:row>21</xdr:row>
-      <xdr:rowOff>70920</xdr:rowOff>
+      <xdr:rowOff>70560</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -5364,7 +5369,7 @@
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
         <a:off x="2646720" y="246600"/>
-        <a:ext cx="5757840" cy="3237840"/>
+        <a:ext cx="5757480" cy="3237480"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -10459,7 +10464,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F93"/>
+  <dimension ref="A1:F94"/>
   <sheetFormatPr defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="9.63"/>
@@ -10496,7 +10501,7 @@
       <c r="B2" s="11" t="s">
         <v>71</v>
       </c>
-      <c r="C2" s="8" t="s">
+      <c r="C2" s="12" t="s">
         <v>72</v>
       </c>
       <c r="D2" s="0" t="n">
@@ -10505,11 +10510,11 @@
       </c>
       <c r="E2" s="0" t="n">
         <f aca="false">IF(ISBLANK(B2),"",COUNTIF(B:B,B2))</f>
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F2" s="0" t="n">
         <f aca="false">IF(ISBLANK(C2),"",COUNTIF(C:C,C2))</f>
-        <v>18</v>
+        <v>8</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10520,7 +10525,7 @@
         <v>71</v>
       </c>
       <c r="C3" s="12" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="D3" s="0" t="n">
         <f aca="false">IF(ISBLANK(A3),"",COUNTIF(A:A,A3))</f>
@@ -10528,11 +10533,11 @@
       </c>
       <c r="E3" s="0" t="n">
         <f aca="false">IF(ISBLANK(B3),"",COUNTIF(B:B,B3))</f>
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F3" s="0" t="n">
         <f aca="false">IF(ISBLANK(C3),"",COUNTIF(C:C,C3))</f>
-        <v>11</v>
+        <v>8</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10543,7 +10548,7 @@
         <v>71</v>
       </c>
       <c r="C4" s="13" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="D4" s="0" t="n">
         <f aca="false">IF(ISBLANK(A4),"",COUNTIF(A:A,A4))</f>
@@ -10551,11 +10556,11 @@
       </c>
       <c r="E4" s="0" t="n">
         <f aca="false">IF(ISBLANK(B4),"",COUNTIF(B:B,B4))</f>
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F4" s="0" t="n">
         <f aca="false">IF(ISBLANK(C4),"",COUNTIF(C:C,C4))</f>
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10563,10 +10568,10 @@
         <v>70</v>
       </c>
       <c r="B5" s="14" t="s">
+        <v>74</v>
+      </c>
+      <c r="C5" s="8" t="s">
         <v>75</v>
-      </c>
-      <c r="C5" s="15" t="s">
-        <v>76</v>
       </c>
       <c r="D5" s="0" t="n">
         <f aca="false">IF(ISBLANK(A5),"",COUNTIF(A:A,A5))</f>
@@ -10574,11 +10579,11 @@
       </c>
       <c r="E5" s="0" t="n">
         <f aca="false">IF(ISBLANK(B5),"",COUNTIF(B:B,B5))</f>
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F5" s="0" t="n">
         <f aca="false">IF(ISBLANK(C5),"",COUNTIF(C:C,C5))</f>
-        <v>8</v>
+        <v>18</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10586,7 +10591,7 @@
         <v>70</v>
       </c>
       <c r="B6" s="14" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C6" s="15" t="s">
         <v>76</v>
@@ -10597,11 +10602,11 @@
       </c>
       <c r="E6" s="0" t="n">
         <f aca="false">IF(ISBLANK(B6),"",COUNTIF(B:B,B6))</f>
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F6" s="0" t="n">
         <f aca="false">IF(ISBLANK(C6),"",COUNTIF(C:C,C6))</f>
-        <v>8</v>
+        <v>11</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10609,10 +10614,10 @@
         <v>70</v>
       </c>
       <c r="B7" s="14" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C7" s="13" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="D7" s="0" t="n">
         <f aca="false">IF(ISBLANK(A7),"",COUNTIF(A:A,A7))</f>
@@ -10620,11 +10625,11 @@
       </c>
       <c r="E7" s="0" t="n">
         <f aca="false">IF(ISBLANK(B7),"",COUNTIF(B:B,B7))</f>
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F7" s="0" t="n">
         <f aca="false">IF(ISBLANK(C7),"",COUNTIF(C:C,C7))</f>
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10677,8 +10682,8 @@
       <c r="A10" s="10" t="s">
         <v>70</v>
       </c>
-      <c r="B10" s="15" t="s">
-        <v>76</v>
+      <c r="B10" s="12" t="s">
+        <v>72</v>
       </c>
       <c r="C10" s="10" t="s">
         <v>79</v>
@@ -10703,8 +10708,8 @@
       <c r="B11" s="18" t="s">
         <v>80</v>
       </c>
-      <c r="C11" s="14" t="s">
-        <v>75</v>
+      <c r="C11" s="11" t="s">
+        <v>71</v>
       </c>
       <c r="D11" s="0" t="n">
         <f aca="false">IF(ISBLANK(A11),"",COUNTIF(A:A,A11))</f>
@@ -10727,7 +10732,7 @@
         <v>81</v>
       </c>
       <c r="C12" s="8" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="D12" s="0" t="n">
         <f aca="false">IF(ISBLANK(A12),"",COUNTIF(A:A,A12))</f>
@@ -10773,7 +10778,7 @@
         <v>82</v>
       </c>
       <c r="C14" s="8" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="D14" s="0" t="n">
         <f aca="false">IF(ISBLANK(A14),"",COUNTIF(A:A,A14))</f>
@@ -10796,7 +10801,7 @@
         <v>82</v>
       </c>
       <c r="C15" s="8" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="D15" s="0" t="n">
         <f aca="false">IF(ISBLANK(A15),"",COUNTIF(A:A,A15))</f>
@@ -10816,10 +10821,10 @@
         <v>70</v>
       </c>
       <c r="B16" s="13" t="s">
+        <v>73</v>
+      </c>
+      <c r="C16" s="14" t="s">
         <v>74</v>
-      </c>
-      <c r="C16" s="11" t="s">
-        <v>71</v>
       </c>
       <c r="D16" s="0" t="n">
         <f aca="false">IF(ISBLANK(A16),"",COUNTIF(A:A,A16))</f>
@@ -10827,11 +10832,11 @@
       </c>
       <c r="E16" s="0" t="n">
         <f aca="false">IF(ISBLANK(B16),"",COUNTIF(B:B,B16))</f>
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F16" s="0" t="n">
         <f aca="false">IF(ISBLANK(C16),"",COUNTIF(C:C,C16))</f>
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10839,10 +10844,10 @@
         <v>70</v>
       </c>
       <c r="B17" s="13" t="s">
+        <v>73</v>
+      </c>
+      <c r="C17" s="14" t="s">
         <v>74</v>
-      </c>
-      <c r="C17" s="11" t="s">
-        <v>71</v>
       </c>
       <c r="D17" s="0" t="n">
         <f aca="false">IF(ISBLANK(A17),"",COUNTIF(A:A,A17))</f>
@@ -10850,22 +10855,22 @@
       </c>
       <c r="E17" s="0" t="n">
         <f aca="false">IF(ISBLANK(B17),"",COUNTIF(B:B,B17))</f>
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F17" s="0" t="n">
         <f aca="false">IF(ISBLANK(C17),"",COUNTIF(C:C,C17))</f>
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="11" t="s">
+      <c r="A18" s="14" t="s">
         <v>33</v>
       </c>
-      <c r="B18" s="11" t="s">
-        <v>71</v>
-      </c>
-      <c r="C18" s="12" t="s">
-        <v>73</v>
+      <c r="B18" s="21" t="s">
+        <v>83</v>
+      </c>
+      <c r="C18" s="8" t="s">
+        <v>75</v>
       </c>
       <c r="D18" s="0" t="n">
         <f aca="false">IF(ISBLANK(A18),"",COUNTIF(A:A,A18))</f>
@@ -10877,18 +10882,18 @@
       </c>
       <c r="F18" s="0" t="n">
         <f aca="false">IF(ISBLANK(C18),"",COUNTIF(C:C,C18))</f>
-        <v>11</v>
+        <v>18</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="11" t="s">
+      <c r="A19" s="14" t="s">
         <v>33</v>
       </c>
-      <c r="B19" s="11" t="s">
-        <v>71</v>
-      </c>
-      <c r="C19" s="12" t="s">
-        <v>73</v>
+      <c r="B19" s="21" t="s">
+        <v>83</v>
+      </c>
+      <c r="C19" s="15" t="s">
+        <v>76</v>
       </c>
       <c r="D19" s="0" t="n">
         <f aca="false">IF(ISBLANK(A19),"",COUNTIF(A:A,A19))</f>
@@ -10904,14 +10909,14 @@
       </c>
     </row>
     <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="11" t="s">
+      <c r="A20" s="14" t="s">
         <v>33</v>
       </c>
-      <c r="B20" s="11" t="s">
-        <v>71</v>
-      </c>
-      <c r="C20" s="12" t="s">
-        <v>73</v>
+      <c r="B20" s="21" t="s">
+        <v>83</v>
+      </c>
+      <c r="C20" s="17" t="s">
+        <v>78</v>
       </c>
       <c r="D20" s="0" t="n">
         <f aca="false">IF(ISBLANK(A20),"",COUNTIF(A:A,A20))</f>
@@ -10923,15 +10928,15 @@
       </c>
       <c r="F20" s="0" t="n">
         <f aca="false">IF(ISBLANK(C20),"",COUNTIF(C:C,C20))</f>
-        <v>11</v>
+        <v>6</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="11" t="s">
+      <c r="A21" s="14" t="s">
         <v>33</v>
       </c>
       <c r="B21" s="8" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="C21" s="17" t="s">
         <v>78</v>
@@ -10950,14 +10955,14 @@
       </c>
     </row>
     <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="11" t="s">
+      <c r="A22" s="14" t="s">
         <v>33</v>
       </c>
-      <c r="B22" s="21" t="s">
-        <v>83</v>
-      </c>
-      <c r="C22" s="8" t="s">
-        <v>72</v>
+      <c r="B22" s="14" t="s">
+        <v>74</v>
+      </c>
+      <c r="C22" s="15" t="s">
+        <v>76</v>
       </c>
       <c r="D22" s="0" t="n">
         <f aca="false">IF(ISBLANK(A22),"",COUNTIF(A:A,A22))</f>
@@ -10965,22 +10970,22 @@
       </c>
       <c r="E22" s="0" t="n">
         <f aca="false">IF(ISBLANK(B22),"",COUNTIF(B:B,B22))</f>
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F22" s="0" t="n">
         <f aca="false">IF(ISBLANK(C22),"",COUNTIF(C:C,C22))</f>
-        <v>18</v>
+        <v>11</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="11" t="s">
+      <c r="A23" s="14" t="s">
         <v>33</v>
       </c>
-      <c r="B23" s="21" t="s">
-        <v>83</v>
-      </c>
-      <c r="C23" s="12" t="s">
-        <v>73</v>
+      <c r="B23" s="14" t="s">
+        <v>74</v>
+      </c>
+      <c r="C23" s="15" t="s">
+        <v>76</v>
       </c>
       <c r="D23" s="0" t="n">
         <f aca="false">IF(ISBLANK(A23),"",COUNTIF(A:A,A23))</f>
@@ -10988,7 +10993,7 @@
       </c>
       <c r="E23" s="0" t="n">
         <f aca="false">IF(ISBLANK(B23),"",COUNTIF(B:B,B23))</f>
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F23" s="0" t="n">
         <f aca="false">IF(ISBLANK(C23),"",COUNTIF(C:C,C23))</f>
@@ -10996,14 +11001,14 @@
       </c>
     </row>
     <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="11" t="s">
+      <c r="A24" s="14" t="s">
         <v>33</v>
       </c>
-      <c r="B24" s="21" t="s">
-        <v>83</v>
-      </c>
-      <c r="C24" s="17" t="s">
-        <v>78</v>
+      <c r="B24" s="14" t="s">
+        <v>74</v>
+      </c>
+      <c r="C24" s="15" t="s">
+        <v>76</v>
       </c>
       <c r="D24" s="0" t="n">
         <f aca="false">IF(ISBLANK(A24),"",COUNTIF(A:A,A24))</f>
@@ -11011,22 +11016,22 @@
       </c>
       <c r="E24" s="0" t="n">
         <f aca="false">IF(ISBLANK(B24),"",COUNTIF(B:B,B24))</f>
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F24" s="0" t="n">
         <f aca="false">IF(ISBLANK(C24),"",COUNTIF(C:C,C24))</f>
-        <v>6</v>
+        <v>11</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="11" t="s">
+      <c r="A25" s="14" t="s">
         <v>33</v>
       </c>
       <c r="B25" s="22" t="s">
         <v>84</v>
       </c>
-      <c r="C25" s="12" t="s">
-        <v>73</v>
+      <c r="C25" s="15" t="s">
+        <v>76</v>
       </c>
       <c r="D25" s="0" t="n">
         <f aca="false">IF(ISBLANK(A25),"",COUNTIF(A:A,A25))</f>
@@ -11042,14 +11047,14 @@
       </c>
     </row>
     <row r="26" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="11" t="s">
+      <c r="A26" s="14" t="s">
         <v>33</v>
       </c>
       <c r="B26" s="22" t="s">
         <v>84</v>
       </c>
-      <c r="C26" s="11" t="s">
-        <v>71</v>
+      <c r="C26" s="14" t="s">
+        <v>74</v>
       </c>
       <c r="D26" s="0" t="n">
         <f aca="false">IF(ISBLANK(A26),"",COUNTIF(A:A,A26))</f>
@@ -11061,11 +11066,11 @@
       </c>
       <c r="F26" s="0" t="n">
         <f aca="false">IF(ISBLANK(C26),"",COUNTIF(C:C,C26))</f>
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="11" t="s">
+      <c r="A27" s="14" t="s">
         <v>33</v>
       </c>
       <c r="B27" s="22" t="s">
@@ -11088,14 +11093,14 @@
       </c>
     </row>
     <row r="28" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="11" t="s">
+      <c r="A28" s="14" t="s">
         <v>33</v>
       </c>
       <c r="B28" s="16" t="s">
         <v>77</v>
       </c>
-      <c r="C28" s="12" t="s">
-        <v>73</v>
+      <c r="C28" s="15" t="s">
+        <v>76</v>
       </c>
       <c r="D28" s="0" t="n">
         <f aca="false">IF(ISBLANK(A28),"",COUNTIF(A:A,A28))</f>
@@ -11111,7 +11116,7 @@
       </c>
     </row>
     <row r="29" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="11" t="s">
+      <c r="A29" s="14" t="s">
         <v>33</v>
       </c>
       <c r="B29" s="16" t="s">
@@ -11134,14 +11139,14 @@
       </c>
     </row>
     <row r="30" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="11" t="s">
+      <c r="A30" s="14" t="s">
         <v>33</v>
       </c>
-      <c r="B30" s="15" t="s">
-        <v>76</v>
-      </c>
-      <c r="C30" s="14" t="s">
-        <v>75</v>
+      <c r="B30" s="12" t="s">
+        <v>72</v>
+      </c>
+      <c r="C30" s="11" t="s">
+        <v>71</v>
       </c>
       <c r="D30" s="0" t="n">
         <f aca="false">IF(ISBLANK(A30),"",COUNTIF(A:A,A30))</f>
@@ -11157,11 +11162,11 @@
       </c>
     </row>
     <row r="31" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="11" t="s">
+      <c r="A31" s="14" t="s">
         <v>33</v>
       </c>
-      <c r="B31" s="15" t="s">
-        <v>76</v>
+      <c r="B31" s="12" t="s">
+        <v>72</v>
       </c>
       <c r="C31" s="16" t="s">
         <v>77</v>
@@ -11180,14 +11185,14 @@
       </c>
     </row>
     <row r="32" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="11" t="s">
+      <c r="A32" s="14" t="s">
         <v>33</v>
       </c>
       <c r="B32" s="20" t="s">
         <v>82</v>
       </c>
       <c r="C32" s="8" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="D32" s="0" t="n">
         <f aca="false">IF(ISBLANK(A32),"",COUNTIF(A:A,A32))</f>
@@ -11203,11 +11208,11 @@
       </c>
     </row>
     <row r="33" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="11" t="s">
+      <c r="A33" s="14" t="s">
         <v>33</v>
       </c>
-      <c r="B33" s="12" t="s">
-        <v>73</v>
+      <c r="B33" s="15" t="s">
+        <v>76</v>
       </c>
       <c r="C33" s="17" t="s">
         <v>78</v>
@@ -11229,8 +11234,8 @@
       <c r="A34" s="22" t="s">
         <v>86</v>
       </c>
-      <c r="B34" s="8" t="s">
-        <v>72</v>
+      <c r="B34" s="21" t="s">
+        <v>83</v>
       </c>
       <c r="D34" s="0" t="n">
         <f aca="false">IF(ISBLANK(A34),"",COUNTIF(A:A,A34))</f>
@@ -11238,7 +11243,7 @@
       </c>
       <c r="E34" s="0" t="n">
         <f aca="false">IF(ISBLANK(B34),"",COUNTIF(B:B,B34))</f>
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F34" s="0" t="str">
         <f aca="false">IF(ISBLANK(C34),"",COUNTIF(C:C,C34))</f>
@@ -11249,8 +11254,8 @@
       <c r="A35" s="22" t="s">
         <v>86</v>
       </c>
-      <c r="B35" s="8" t="s">
-        <v>72</v>
+      <c r="B35" s="21" t="s">
+        <v>83</v>
       </c>
       <c r="D35" s="0" t="n">
         <f aca="false">IF(ISBLANK(A35),"",COUNTIF(A:A,A35))</f>
@@ -11258,7 +11263,7 @@
       </c>
       <c r="E35" s="0" t="n">
         <f aca="false">IF(ISBLANK(B35),"",COUNTIF(B:B,B35))</f>
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F35" s="0" t="str">
         <f aca="false">IF(ISBLANK(C35),"",COUNTIF(C:C,C35))</f>
@@ -11270,7 +11275,7 @@
         <v>86</v>
       </c>
       <c r="B36" s="8" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="D36" s="0" t="n">
         <f aca="false">IF(ISBLANK(A36),"",COUNTIF(A:A,A36))</f>
@@ -11290,7 +11295,7 @@
         <v>86</v>
       </c>
       <c r="B37" s="8" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="D37" s="0" t="n">
         <f aca="false">IF(ISBLANK(A37),"",COUNTIF(A:A,A37))</f>
@@ -11309,8 +11314,8 @@
       <c r="A38" s="22" t="s">
         <v>86</v>
       </c>
-      <c r="B38" s="21" t="s">
-        <v>83</v>
+      <c r="B38" s="8" t="s">
+        <v>75</v>
       </c>
       <c r="D38" s="0" t="n">
         <f aca="false">IF(ISBLANK(A38),"",COUNTIF(A:A,A38))</f>
@@ -11329,8 +11334,8 @@
       <c r="A39" s="22" t="s">
         <v>86</v>
       </c>
-      <c r="B39" s="21" t="s">
-        <v>83</v>
+      <c r="B39" s="8" t="s">
+        <v>75</v>
       </c>
       <c r="D39" s="0" t="n">
         <f aca="false">IF(ISBLANK(A39),"",COUNTIF(A:A,A39))</f>
@@ -11469,10 +11474,10 @@
       <c r="A46" s="20" t="s">
         <v>19</v>
       </c>
-      <c r="B46" s="11" t="s">
-        <v>71</v>
-      </c>
-      <c r="C46" s="12" t="s">
+      <c r="B46" s="21" t="s">
+        <v>83</v>
+      </c>
+      <c r="C46" s="13" t="s">
         <v>73</v>
       </c>
       <c r="D46" s="0" t="n">
@@ -11485,17 +11490,17 @@
       </c>
       <c r="F46" s="0" t="n">
         <f aca="false">IF(ISBLANK(C46),"",COUNTIF(C:C,C46))</f>
-        <v>11</v>
+        <v>5</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="20" t="s">
         <v>19</v>
       </c>
-      <c r="B47" s="11" t="s">
-        <v>71</v>
-      </c>
-      <c r="C47" s="12" t="s">
+      <c r="B47" s="21" t="s">
+        <v>83</v>
+      </c>
+      <c r="C47" s="13" t="s">
         <v>73</v>
       </c>
       <c r="D47" s="0" t="n">
@@ -11508,18 +11513,18 @@
       </c>
       <c r="F47" s="0" t="n">
         <f aca="false">IF(ISBLANK(C47),"",COUNTIF(C:C,C47))</f>
-        <v>11</v>
+        <v>5</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="20" t="s">
         <v>19</v>
       </c>
-      <c r="B48" s="11" t="s">
-        <v>71</v>
-      </c>
-      <c r="C48" s="21" t="s">
-        <v>83</v>
+      <c r="B48" s="8" t="s">
+        <v>75</v>
+      </c>
+      <c r="C48" s="20" t="s">
+        <v>82</v>
       </c>
       <c r="D48" s="0" t="n">
         <f aca="false">IF(ISBLANK(A48),"",COUNTIF(A:A,A48))</f>
@@ -11527,22 +11532,22 @@
       </c>
       <c r="E48" s="0" t="n">
         <f aca="false">IF(ISBLANK(B48),"",COUNTIF(B:B,B48))</f>
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F48" s="0" t="n">
         <f aca="false">IF(ISBLANK(C48),"",COUNTIF(C:C,C48))</f>
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="20" t="s">
         <v>19</v>
       </c>
-      <c r="B49" s="8" t="s">
-        <v>72</v>
-      </c>
-      <c r="C49" s="20" t="s">
-        <v>82</v>
+      <c r="B49" s="14" t="s">
+        <v>74</v>
+      </c>
+      <c r="C49" s="15" t="s">
+        <v>76</v>
       </c>
       <c r="D49" s="0" t="n">
         <f aca="false">IF(ISBLANK(A49),"",COUNTIF(A:A,A49))</f>
@@ -11550,22 +11555,22 @@
       </c>
       <c r="E49" s="0" t="n">
         <f aca="false">IF(ISBLANK(B49),"",COUNTIF(B:B,B49))</f>
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F49" s="0" t="n">
         <f aca="false">IF(ISBLANK(C49),"",COUNTIF(C:C,C49))</f>
-        <v>1</v>
+        <v>11</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="20" t="s">
         <v>19</v>
       </c>
-      <c r="B50" s="21" t="s">
-        <v>83</v>
-      </c>
-      <c r="C50" s="11" t="s">
-        <v>71</v>
+      <c r="B50" s="16" t="s">
+        <v>77</v>
+      </c>
+      <c r="C50" s="15" t="s">
+        <v>76</v>
       </c>
       <c r="D50" s="0" t="n">
         <f aca="false">IF(ISBLANK(A50),"",COUNTIF(A:A,A50))</f>
@@ -11573,22 +11578,22 @@
       </c>
       <c r="E50" s="0" t="n">
         <f aca="false">IF(ISBLANK(B50),"",COUNTIF(B:B,B50))</f>
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="F50" s="0" t="n">
         <f aca="false">IF(ISBLANK(C50),"",COUNTIF(C:C,C50))</f>
-        <v>6</v>
+        <v>11</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="20" t="s">
         <v>19</v>
       </c>
-      <c r="B51" s="21" t="s">
-        <v>83</v>
-      </c>
-      <c r="C51" s="11" t="s">
-        <v>71</v>
+      <c r="B51" s="16" t="s">
+        <v>77</v>
+      </c>
+      <c r="C51" s="12" t="s">
+        <v>72</v>
       </c>
       <c r="D51" s="0" t="n">
         <f aca="false">IF(ISBLANK(A51),"",COUNTIF(A:A,A51))</f>
@@ -11596,22 +11601,22 @@
       </c>
       <c r="E51" s="0" t="n">
         <f aca="false">IF(ISBLANK(B51),"",COUNTIF(B:B,B51))</f>
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="F51" s="0" t="n">
         <f aca="false">IF(ISBLANK(C51),"",COUNTIF(C:C,C51))</f>
-        <v>6</v>
+        <v>8</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="20" t="s">
         <v>19</v>
       </c>
-      <c r="B52" s="16" t="s">
-        <v>77</v>
-      </c>
-      <c r="C52" s="12" t="s">
-        <v>73</v>
+      <c r="B52" s="12" t="s">
+        <v>72</v>
+      </c>
+      <c r="C52" s="19" t="s">
+        <v>81</v>
       </c>
       <c r="D52" s="0" t="n">
         <f aca="false">IF(ISBLANK(A52),"",COUNTIF(A:A,A52))</f>
@@ -11623,18 +11628,18 @@
       </c>
       <c r="F52" s="0" t="n">
         <f aca="false">IF(ISBLANK(C52),"",COUNTIF(C:C,C52))</f>
-        <v>11</v>
+        <v>3</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="20" t="s">
         <v>19</v>
       </c>
-      <c r="B53" s="16" t="s">
-        <v>77</v>
-      </c>
-      <c r="C53" s="15" t="s">
-        <v>76</v>
+      <c r="B53" s="20" t="s">
+        <v>82</v>
+      </c>
+      <c r="C53" s="8" t="s">
+        <v>75</v>
       </c>
       <c r="D53" s="0" t="n">
         <f aca="false">IF(ISBLANK(A53),"",COUNTIF(A:A,A53))</f>
@@ -11642,22 +11647,22 @@
       </c>
       <c r="E53" s="0" t="n">
         <f aca="false">IF(ISBLANK(B53),"",COUNTIF(B:B,B53))</f>
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="F53" s="0" t="n">
         <f aca="false">IF(ISBLANK(C53),"",COUNTIF(C:C,C53))</f>
-        <v>8</v>
+        <v>18</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="20" t="s">
         <v>19</v>
       </c>
-      <c r="B54" s="15" t="s">
+      <c r="B54" s="13" t="s">
+        <v>73</v>
+      </c>
+      <c r="C54" s="15" t="s">
         <v>76</v>
-      </c>
-      <c r="C54" s="19" t="s">
-        <v>81</v>
       </c>
       <c r="D54" s="0" t="n">
         <f aca="false">IF(ISBLANK(A54),"",COUNTIF(A:A,A54))</f>
@@ -11665,22 +11670,22 @@
       </c>
       <c r="E54" s="0" t="n">
         <f aca="false">IF(ISBLANK(B54),"",COUNTIF(B:B,B54))</f>
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="F54" s="0" t="n">
         <f aca="false">IF(ISBLANK(C54),"",COUNTIF(C:C,C54))</f>
-        <v>3</v>
+        <v>11</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="20" t="s">
         <v>19</v>
       </c>
-      <c r="B55" s="20" t="s">
-        <v>82</v>
-      </c>
-      <c r="C55" s="8" t="s">
-        <v>72</v>
+      <c r="B55" s="13" t="s">
+        <v>73</v>
+      </c>
+      <c r="C55" s="21" t="s">
+        <v>83</v>
       </c>
       <c r="D55" s="0" t="n">
         <f aca="false">IF(ISBLANK(A55),"",COUNTIF(A:A,A55))</f>
@@ -11688,11 +11693,11 @@
       </c>
       <c r="E55" s="0" t="n">
         <f aca="false">IF(ISBLANK(B55),"",COUNTIF(B:B,B55))</f>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F55" s="0" t="n">
         <f aca="false">IF(ISBLANK(C55),"",COUNTIF(C:C,C55))</f>
-        <v>18</v>
+        <v>3</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11703,7 +11708,7 @@
         <v>88</v>
       </c>
       <c r="C56" s="8" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="D56" s="0" t="n">
         <f aca="false">IF(ISBLANK(A56),"",COUNTIF(A:A,A56))</f>
@@ -11719,14 +11724,14 @@
       </c>
     </row>
     <row r="57" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A57" s="15" t="s">
+      <c r="A57" s="12" t="s">
         <v>89</v>
       </c>
-      <c r="B57" s="14" t="s">
-        <v>75</v>
-      </c>
-      <c r="C57" s="15" t="s">
-        <v>76</v>
+      <c r="B57" s="11" t="s">
+        <v>71</v>
+      </c>
+      <c r="C57" s="12" t="s">
+        <v>72</v>
       </c>
       <c r="D57" s="0" t="n">
         <f aca="false">IF(ISBLANK(A57),"",COUNTIF(A:A,A57))</f>
@@ -11742,14 +11747,14 @@
       </c>
     </row>
     <row r="58" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A58" s="15" t="s">
+      <c r="A58" s="12" t="s">
         <v>89</v>
       </c>
-      <c r="B58" s="14" t="s">
-        <v>75</v>
-      </c>
-      <c r="C58" s="15" t="s">
-        <v>76</v>
+      <c r="B58" s="11" t="s">
+        <v>71</v>
+      </c>
+      <c r="C58" s="12" t="s">
+        <v>72</v>
       </c>
       <c r="D58" s="0" t="n">
         <f aca="false">IF(ISBLANK(A58),"",COUNTIF(A:A,A58))</f>
@@ -11765,14 +11770,14 @@
       </c>
     </row>
     <row r="59" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A59" s="15" t="s">
+      <c r="A59" s="12" t="s">
         <v>89</v>
       </c>
-      <c r="B59" s="14" t="s">
-        <v>75</v>
-      </c>
-      <c r="C59" s="15" t="s">
-        <v>76</v>
+      <c r="B59" s="11" t="s">
+        <v>71</v>
+      </c>
+      <c r="C59" s="12" t="s">
+        <v>72</v>
       </c>
       <c r="D59" s="0" t="n">
         <f aca="false">IF(ISBLANK(A59),"",COUNTIF(A:A,A59))</f>
@@ -11788,14 +11793,14 @@
       </c>
     </row>
     <row r="60" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A60" s="15" t="s">
+      <c r="A60" s="12" t="s">
         <v>89</v>
       </c>
-      <c r="B60" s="14" t="s">
-        <v>75</v>
+      <c r="B60" s="11" t="s">
+        <v>71</v>
       </c>
       <c r="C60" s="13" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="D60" s="0" t="n">
         <f aca="false">IF(ISBLANK(A60),"",COUNTIF(A:A,A60))</f>
@@ -11807,18 +11812,18 @@
       </c>
       <c r="F60" s="0" t="n">
         <f aca="false">IF(ISBLANK(C60),"",COUNTIF(C:C,C60))</f>
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A61" s="15" t="s">
+      <c r="A61" s="12" t="s">
         <v>89</v>
       </c>
       <c r="B61" s="16" t="s">
         <v>77</v>
       </c>
-      <c r="C61" s="15" t="s">
-        <v>76</v>
+      <c r="C61" s="12" t="s">
+        <v>72</v>
       </c>
       <c r="D61" s="0" t="n">
         <f aca="false">IF(ISBLANK(A61),"",COUNTIF(A:A,A61))</f>
@@ -11834,11 +11839,11 @@
       </c>
     </row>
     <row r="62" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A62" s="15" t="s">
+      <c r="A62" s="12" t="s">
         <v>89</v>
       </c>
-      <c r="B62" s="15" t="s">
-        <v>76</v>
+      <c r="B62" s="12" t="s">
+        <v>72</v>
       </c>
       <c r="C62" s="19" t="s">
         <v>81</v>
@@ -11857,7 +11862,7 @@
       </c>
     </row>
     <row r="63" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A63" s="15" t="s">
+      <c r="A63" s="12" t="s">
         <v>89</v>
       </c>
       <c r="B63" s="19" t="s">
@@ -11880,7 +11885,7 @@
       </c>
     </row>
     <row r="64" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A64" s="15" t="s">
+      <c r="A64" s="12" t="s">
         <v>89</v>
       </c>
       <c r="B64" s="19" t="s">
@@ -11903,14 +11908,14 @@
       </c>
     </row>
     <row r="65" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A65" s="15" t="s">
+      <c r="A65" s="12" t="s">
         <v>89</v>
       </c>
       <c r="B65" s="17" t="s">
         <v>78</v>
       </c>
       <c r="C65" s="8" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="D65" s="0" t="n">
         <f aca="false">IF(ISBLANK(A65),"",COUNTIF(A:A,A65))</f>
@@ -11926,14 +11931,14 @@
       </c>
     </row>
     <row r="66" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A66" s="15" t="s">
+      <c r="A66" s="12" t="s">
         <v>89</v>
       </c>
-      <c r="B66" s="12" t="s">
-        <v>73</v>
-      </c>
-      <c r="C66" s="11" t="s">
-        <v>71</v>
+      <c r="B66" s="15" t="s">
+        <v>76</v>
+      </c>
+      <c r="C66" s="14" t="s">
+        <v>74</v>
       </c>
       <c r="D66" s="0" t="n">
         <f aca="false">IF(ISBLANK(A66),"",COUNTIF(A:A,A66))</f>
@@ -11945,18 +11950,18 @@
       </c>
       <c r="F66" s="0" t="n">
         <f aca="false">IF(ISBLANK(C66),"",COUNTIF(C:C,C66))</f>
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="21" t="s">
         <v>90</v>
       </c>
-      <c r="B67" s="11" t="s">
-        <v>71</v>
-      </c>
-      <c r="C67" s="12" t="s">
-        <v>73</v>
+      <c r="B67" s="21" t="s">
+        <v>83</v>
+      </c>
+      <c r="C67" s="8" t="s">
+        <v>75</v>
       </c>
       <c r="D67" s="0" t="n">
         <f aca="false">IF(ISBLANK(A67),"",COUNTIF(A:A,A67))</f>
@@ -11968,15 +11973,15 @@
       </c>
       <c r="F67" s="0" t="n">
         <f aca="false">IF(ISBLANK(C67),"",COUNTIF(C:C,C67))</f>
-        <v>11</v>
+        <v>18</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="21" t="s">
         <v>90</v>
       </c>
-      <c r="B68" s="8" t="s">
-        <v>72</v>
+      <c r="B68" s="21" t="s">
+        <v>83</v>
       </c>
       <c r="C68" s="17" t="s">
         <v>78</v>
@@ -11987,7 +11992,7 @@
       </c>
       <c r="E68" s="0" t="n">
         <f aca="false">IF(ISBLANK(B68),"",COUNTIF(B:B,B68))</f>
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F68" s="0" t="n">
         <f aca="false">IF(ISBLANK(C68),"",COUNTIF(C:C,C68))</f>
@@ -11998,11 +12003,11 @@
       <c r="A69" s="21" t="s">
         <v>90</v>
       </c>
-      <c r="B69" s="21" t="s">
-        <v>83</v>
-      </c>
-      <c r="C69" s="8" t="s">
-        <v>72</v>
+      <c r="B69" s="8" t="s">
+        <v>75</v>
+      </c>
+      <c r="C69" s="17" t="s">
+        <v>78</v>
       </c>
       <c r="D69" s="0" t="n">
         <f aca="false">IF(ISBLANK(A69),"",COUNTIF(A:A,A69))</f>
@@ -12014,18 +12019,18 @@
       </c>
       <c r="F69" s="0" t="n">
         <f aca="false">IF(ISBLANK(C69),"",COUNTIF(C:C,C69))</f>
-        <v>18</v>
+        <v>6</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A70" s="21" t="s">
         <v>90</v>
       </c>
-      <c r="B70" s="21" t="s">
-        <v>83</v>
-      </c>
-      <c r="C70" s="17" t="s">
-        <v>78</v>
+      <c r="B70" s="14" t="s">
+        <v>74</v>
+      </c>
+      <c r="C70" s="15" t="s">
+        <v>76</v>
       </c>
       <c r="D70" s="0" t="n">
         <f aca="false">IF(ISBLANK(A70),"",COUNTIF(A:A,A70))</f>
@@ -12033,11 +12038,11 @@
       </c>
       <c r="E70" s="0" t="n">
         <f aca="false">IF(ISBLANK(B70),"",COUNTIF(B:B,B70))</f>
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F70" s="0" t="n">
         <f aca="false">IF(ISBLANK(C70),"",COUNTIF(C:C,C70))</f>
-        <v>6</v>
+        <v>11</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12048,7 +12053,7 @@
         <v>84</v>
       </c>
       <c r="C71" s="8" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="D71" s="0" t="n">
         <f aca="false">IF(ISBLANK(A71),"",COUNTIF(A:A,A71))</f>
@@ -12094,7 +12099,7 @@
         <v>91</v>
       </c>
       <c r="C73" s="8" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="D73" s="0" t="n">
         <f aca="false">IF(ISBLANK(A73),"",COUNTIF(A:A,A73))</f>
@@ -12117,7 +12122,7 @@
         <v>80</v>
       </c>
       <c r="C74" s="8" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="D74" s="0" t="n">
         <f aca="false">IF(ISBLANK(A74),"",COUNTIF(A:A,A74))</f>
@@ -12140,7 +12145,7 @@
         <v>80</v>
       </c>
       <c r="C75" s="8" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="D75" s="0" t="n">
         <f aca="false">IF(ISBLANK(A75),"",COUNTIF(A:A,A75))</f>
@@ -12163,7 +12168,7 @@
         <v>80</v>
       </c>
       <c r="C76" s="8" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="D76" s="0" t="n">
         <f aca="false">IF(ISBLANK(A76),"",COUNTIF(A:A,A76))</f>
@@ -12186,7 +12191,7 @@
         <v>80</v>
       </c>
       <c r="C77" s="8" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="D77" s="0" t="n">
         <f aca="false">IF(ISBLANK(A77),"",COUNTIF(A:A,A77))</f>
@@ -12209,7 +12214,7 @@
         <v>80</v>
       </c>
       <c r="C78" s="8" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="D78" s="0" t="n">
         <f aca="false">IF(ISBLANK(A78),"",COUNTIF(A:A,A78))</f>
@@ -12232,7 +12237,7 @@
         <v>80</v>
       </c>
       <c r="C79" s="8" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="D79" s="0" t="n">
         <f aca="false">IF(ISBLANK(A79),"",COUNTIF(A:A,A79))</f>
@@ -12252,7 +12257,7 @@
         <v>92</v>
       </c>
       <c r="B80" s="8" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="D80" s="0" t="n">
         <f aca="false">IF(ISBLANK(A80),"",COUNTIF(A:A,A80))</f>
@@ -12332,7 +12337,7 @@
         <v>93</v>
       </c>
       <c r="B84" s="8" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="C84" s="18" t="s">
         <v>80</v>
@@ -12400,8 +12405,8 @@
       <c r="A87" s="19" t="s">
         <v>94</v>
       </c>
-      <c r="B87" s="14" t="s">
-        <v>75</v>
+      <c r="B87" s="11" t="s">
+        <v>71</v>
       </c>
       <c r="C87" s="18" t="s">
         <v>80</v>
@@ -12423,11 +12428,11 @@
       <c r="A88" s="19" t="s">
         <v>94</v>
       </c>
-      <c r="B88" s="15" t="s">
-        <v>76</v>
-      </c>
-      <c r="C88" s="14" t="s">
-        <v>75</v>
+      <c r="B88" s="12" t="s">
+        <v>72</v>
+      </c>
+      <c r="C88" s="11" t="s">
+        <v>71</v>
       </c>
       <c r="D88" s="0" t="n">
         <f aca="false">IF(ISBLANK(A88),"",COUNTIF(A:A,A88))</f>
@@ -12469,11 +12474,11 @@
       <c r="A90" s="27" t="s">
         <v>95</v>
       </c>
-      <c r="B90" s="14" t="s">
-        <v>75</v>
-      </c>
-      <c r="C90" s="15" t="s">
-        <v>76</v>
+      <c r="B90" s="11" t="s">
+        <v>71</v>
+      </c>
+      <c r="C90" s="12" t="s">
+        <v>72</v>
       </c>
       <c r="D90" s="0" t="n">
         <f aca="false">IF(ISBLANK(A90),"",COUNTIF(A:A,A90))</f>
@@ -12535,14 +12540,11 @@
       </c>
     </row>
     <row r="93" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A93" s="16" t="s">
+      <c r="A93" s="18" t="s">
         <v>98</v>
       </c>
-      <c r="B93" s="15" t="s">
-        <v>76</v>
-      </c>
-      <c r="C93" s="16" t="s">
-        <v>77</v>
+      <c r="B93" s="21" t="s">
+        <v>83</v>
       </c>
       <c r="D93" s="0" t="n">
         <f aca="false">IF(ISBLANK(A93),"",COUNTIF(A:A,A93))</f>
@@ -12550,15 +12552,38 @@
       </c>
       <c r="E93" s="0" t="n">
         <f aca="false">IF(ISBLANK(B93),"",COUNTIF(B:B,B93))</f>
+        <v>10</v>
+      </c>
+      <c r="F93" s="0" t="str">
+        <f aca="false">IF(ISBLANK(C93),"",COUNTIF(C:C,C93))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="94" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A94" s="16" t="s">
+        <v>99</v>
+      </c>
+      <c r="B94" s="12" t="s">
+        <v>72</v>
+      </c>
+      <c r="C94" s="16" t="s">
+        <v>77</v>
+      </c>
+      <c r="D94" s="0" t="n">
+        <f aca="false">IF(ISBLANK(A94),"",COUNTIF(A:A,A94))</f>
+        <v>1</v>
+      </c>
+      <c r="E94" s="0" t="n">
+        <f aca="false">IF(ISBLANK(B94),"",COUNTIF(B:B,B94))</f>
         <v>7</v>
       </c>
-      <c r="F93" s="0" t="n">
-        <f aca="false">IF(ISBLANK(C93),"",COUNTIF(C:C,C93))</f>
+      <c r="F94" s="0" t="n">
+        <f aca="false">IF(ISBLANK(C94),"",COUNTIF(C:C,C94))</f>
         <v>2</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F93"/>
+  <autoFilter ref="A1:F94"/>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
   <pageSetup paperSize="9" scale="100" firstPageNumber="0" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" useFirstPageNumber="false" horizontalDpi="300" verticalDpi="300" copies="1"/>
@@ -12596,25 +12621,25 @@
         <v>64</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="D1" s="9" t="s">
         <v>65</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="G1" s="9" t="s">
         <v>66</v>
       </c>
       <c r="H1" s="3" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="J1" s="9" t="s">
+        <v>101</v>
+      </c>
+      <c r="K1" s="3" t="s">
         <v>100</v>
-      </c>
-      <c r="K1" s="3" t="s">
-        <v>99</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12625,22 +12650,22 @@
         <f aca="false">COUNTIF(Tatjes!A:A,A2)</f>
         <v>16</v>
       </c>
-      <c r="D2" s="11" t="s">
-        <v>71</v>
+      <c r="D2" s="21" t="s">
+        <v>83</v>
       </c>
       <c r="E2" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!B:B,D2)</f>
         <v>10</v>
       </c>
       <c r="G2" s="8" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="H2" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!C:C,G2)</f>
         <v>18</v>
       </c>
       <c r="J2" s="8" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="K2" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!B:B,J2)*2+COUNTIF(Tatjes!C:C,J2)</f>
@@ -12648,7 +12673,7 @@
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="11" t="s">
+      <c r="A3" s="14" t="s">
         <v>33</v>
       </c>
       <c r="B3" s="1" t="n">
@@ -12656,25 +12681,25 @@
         <v>16</v>
       </c>
       <c r="D3" s="8" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="E3" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!B:B,D3)</f>
         <v>9</v>
       </c>
-      <c r="G3" s="12" t="s">
-        <v>73</v>
+      <c r="G3" s="15" t="s">
+        <v>76</v>
       </c>
       <c r="H3" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!C:C,G3)</f>
         <v>11</v>
       </c>
-      <c r="J3" s="11" t="s">
-        <v>71</v>
+      <c r="J3" s="21" t="s">
+        <v>83</v>
       </c>
       <c r="K3" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!B:B,J3)*2+COUNTIF(Tatjes!C:C,J3)</f>
-        <v>26</v>
+        <v>23</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12685,22 +12710,22 @@
         <f aca="false">COUNTIF(Tatjes!A:A,A4)</f>
         <v>12</v>
       </c>
-      <c r="D4" s="21" t="s">
-        <v>83</v>
+      <c r="D4" s="11" t="s">
+        <v>71</v>
       </c>
       <c r="E4" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!B:B,D4)</f>
         <v>9</v>
       </c>
-      <c r="G4" s="15" t="s">
-        <v>76</v>
+      <c r="G4" s="12" t="s">
+        <v>72</v>
       </c>
       <c r="H4" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!C:C,G4)</f>
         <v>8</v>
       </c>
-      <c r="J4" s="15" t="s">
-        <v>76</v>
+      <c r="J4" s="12" t="s">
+        <v>72</v>
       </c>
       <c r="K4" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!B:B,J4)*2+COUNTIF(Tatjes!C:C,J4)</f>
@@ -12716,21 +12741,21 @@
         <v>11</v>
       </c>
       <c r="D5" s="14" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="E5" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!B:B,D5)</f>
-        <v>9</v>
-      </c>
-      <c r="G5" s="11" t="s">
-        <v>71</v>
+        <v>8</v>
+      </c>
+      <c r="G5" s="17" t="s">
+        <v>78</v>
       </c>
       <c r="H5" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!C:C,G5)</f>
         <v>6</v>
       </c>
-      <c r="J5" s="21" t="s">
-        <v>83</v>
+      <c r="J5" s="11" t="s">
+        <v>71</v>
       </c>
       <c r="K5" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!B:B,J5)*2+COUNTIF(Tatjes!C:C,J5)</f>
@@ -12738,7 +12763,7 @@
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="15" t="s">
+      <c r="A6" s="12" t="s">
         <v>89</v>
       </c>
       <c r="B6" s="1" t="n">
@@ -12752,19 +12777,19 @@
         <f aca="false">COUNTIF(Tatjes!B:B,D6)</f>
         <v>8</v>
       </c>
-      <c r="G6" s="17" t="s">
-        <v>78</v>
+      <c r="G6" s="13" t="s">
+        <v>73</v>
       </c>
       <c r="H6" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!C:C,G6)</f>
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="J6" s="14" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="K6" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!B:B,J6)*2+COUNTIF(Tatjes!C:C,J6)</f>
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12805,19 +12830,19 @@
         <f aca="false">COUNTIF(Tatjes!A:A,A8)</f>
         <v>6</v>
       </c>
-      <c r="D8" s="15" t="s">
-        <v>76</v>
+      <c r="D8" s="12" t="s">
+        <v>72</v>
       </c>
       <c r="E8" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!B:B,D8)</f>
         <v>7</v>
       </c>
-      <c r="G8" s="19" t="s">
-        <v>81</v>
+      <c r="G8" s="14" t="s">
+        <v>74</v>
       </c>
       <c r="H8" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!C:C,G8)</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J8" s="22" t="s">
         <v>84</v>
@@ -12842,8 +12867,8 @@
         <f aca="false">COUNTIF(Tatjes!B:B,D9)</f>
         <v>7</v>
       </c>
-      <c r="G9" s="21" t="s">
-        <v>83</v>
+      <c r="G9" s="19" t="s">
+        <v>81</v>
       </c>
       <c r="H9" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!C:C,G9)</f>
@@ -12872,8 +12897,8 @@
         <f aca="false">COUNTIF(Tatjes!B:B,D10)</f>
         <v>5</v>
       </c>
-      <c r="G10" s="13" t="s">
-        <v>74</v>
+      <c r="G10" s="21" t="s">
+        <v>83</v>
       </c>
       <c r="H10" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!C:C,G10)</f>
@@ -12902,15 +12927,15 @@
         <f aca="false">COUNTIF(Tatjes!B:B,D11)</f>
         <v>5</v>
       </c>
-      <c r="G11" s="14" t="s">
-        <v>75</v>
+      <c r="G11" s="11" t="s">
+        <v>71</v>
       </c>
       <c r="H11" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!C:C,G11)</f>
         <v>3</v>
       </c>
-      <c r="J11" s="12" t="s">
-        <v>73</v>
+      <c r="J11" s="15" t="s">
+        <v>76</v>
       </c>
       <c r="K11" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!B:B,J11)*2+COUNTIF(Tatjes!C:C,J11)</f>
@@ -12948,19 +12973,19 @@
       </c>
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="16" t="s">
+      <c r="A13" s="18" t="s">
         <v>98</v>
       </c>
       <c r="B13" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!A:A,A13)</f>
         <v>1</v>
       </c>
-      <c r="D13" s="12" t="s">
+      <c r="D13" s="13" t="s">
         <v>73</v>
       </c>
       <c r="E13" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!B:B,D13)</f>
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G13" s="16" t="s">
         <v>77</v>
@@ -12969,17 +12994,24 @@
         <f aca="false">COUNTIF(Tatjes!C:C,G13)</f>
         <v>2</v>
       </c>
-      <c r="J13" s="20" t="s">
-        <v>82</v>
+      <c r="J13" s="13" t="s">
+        <v>73</v>
       </c>
       <c r="K13" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!B:B,J13)*2+COUNTIF(Tatjes!C:C,J13)</f>
-        <v>11</v>
+        <v>13</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D14" s="27" t="s">
-        <v>96</v>
+      <c r="A14" s="16" t="s">
+        <v>99</v>
+      </c>
+      <c r="B14" s="1" t="n">
+        <f aca="false">COUNTIF(Tatjes!A:A,A14)</f>
+        <v>1</v>
+      </c>
+      <c r="D14" s="15" t="s">
+        <v>76</v>
       </c>
       <c r="E14" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!B:B,D14)</f>
@@ -12992,24 +13024,18 @@
         <f aca="false">COUNTIF(Tatjes!C:C,G14)</f>
         <v>1</v>
       </c>
-      <c r="J14" s="13" t="s">
-        <v>74</v>
+      <c r="J14" s="20" t="s">
+        <v>82</v>
       </c>
       <c r="K14" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!B:B,J14)*2+COUNTIF(Tatjes!C:C,J14)</f>
-        <v>7</v>
+        <v>11</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="9" t="s">
-        <v>18</v>
-      </c>
-      <c r="B15" s="3" t="n">
-        <f aca="false">COUNTA(Tatjes!A:A)-1</f>
-        <v>92</v>
-      </c>
-      <c r="D15" s="13" t="s">
-        <v>74</v>
+      <c r="B15" s="0"/>
+      <c r="D15" s="27" t="s">
+        <v>96</v>
       </c>
       <c r="E15" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!B:B,D15)</f>
@@ -13031,6 +13057,13 @@
       </c>
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="B16" s="3" t="n">
+        <f aca="false">COUNTA(Tatjes!A:A)-1</f>
+        <v>93</v>
+      </c>
       <c r="D16" s="24" t="s">
         <v>87</v>
       </c>
@@ -13146,7 +13179,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B13"/>
+  <autoFilter ref="A1:B14"/>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
   <pageSetup paperSize="9" scale="100" firstPageNumber="0" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" useFirstPageNumber="false" horizontalDpi="300" verticalDpi="300" copies="1"/>

</xml_diff>

<commit_message>
Sync from vault 2026-06-05 17:04:06
</commit_message>
<xml_diff>
--- a/content/Archief/0. PDFs & docs/Obol docs & forms/Irmijn Inc/Irma backup log.xlsx
+++ b/content/Archief/0. PDFs & docs/Obol docs & forms/Irmijn Inc/Irma backup log.xlsx
@@ -15,13 +15,14 @@
   </sheets>
   <definedNames>
     <definedName function="false" hidden="true" localSheetId="3" name="_xlnm._FilterDatabase" vbProcedure="false">Tatdata!$A$1:$B$14</definedName>
-    <definedName function="false" hidden="true" localSheetId="2" name="_xlnm._FilterDatabase" vbProcedure="false">Tatjes!$A$1:$F$94</definedName>
-    <definedName function="false" hidden="false" localSheetId="2" name="_xlnm._FilterDatabase" vbProcedure="false">Tatjes!$A$1:$F$93</definedName>
-    <definedName function="false" hidden="false" localSheetId="2" name="_xlnm._FilterDatabase_0" vbProcedure="false">Tatjes!$A$1:$F$92</definedName>
-    <definedName function="false" hidden="false" localSheetId="2" name="_xlnm._FilterDatabase_0_0" vbProcedure="false">Tatjes!$A$1:$F$91</definedName>
-    <definedName function="false" hidden="false" localSheetId="2" name="_xlnm._FilterDatabase_0_0_0" vbProcedure="false">Tatjes!$A$1:$F$90</definedName>
-    <definedName function="false" hidden="false" localSheetId="2" name="_xlnm._FilterDatabase_0_0_0_0" vbProcedure="false">Tatjes!$A$1:$F$88</definedName>
-    <definedName function="false" hidden="false" localSheetId="3" name="_xlnm._FilterDatabase" vbProcedure="false">Tatdata!$A$1:$B$13</definedName>
+    <definedName function="false" hidden="true" localSheetId="2" name="_xlnm._FilterDatabase" vbProcedure="false">Tatjes!$A$1:$F$95</definedName>
+    <definedName function="false" hidden="false" localSheetId="2" name="_xlnm._FilterDatabase" vbProcedure="false">Tatjes!$A$1:$F$1</definedName>
+    <definedName function="false" hidden="false" localSheetId="2" name="_xlnm._FilterDatabase_0" vbProcedure="false">Tatjes!$A$1:$F$1</definedName>
+    <definedName function="false" hidden="false" localSheetId="2" name="_xlnm._FilterDatabase_0_0" vbProcedure="false">Tatjes!$A$1:$F$1</definedName>
+    <definedName function="false" hidden="false" localSheetId="2" name="_xlnm._FilterDatabase_0_0_0" vbProcedure="false">Tatjes!$A$1:$F$1</definedName>
+    <definedName function="false" hidden="false" localSheetId="2" name="_xlnm._FilterDatabase_0_0_0_0" vbProcedure="false">Tatjes!$A$1:$F$1</definedName>
+    <definedName function="false" hidden="false" localSheetId="2" name="_xlnm._FilterDatabase_0_0_0_0_0" vbProcedure="false">Tatjes!$A$1:$F$1</definedName>
+    <definedName function="false" hidden="false" localSheetId="3" name="_xlnm._FilterDatabase_0" vbProcedure="false">Tatdata!$A$1:$B$13</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.001"/>
   <extLst>
@@ -33,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="496" uniqueCount="102">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="502" uniqueCount="102">
   <si>
     <t xml:space="preserve">Pagina</t>
   </si>
@@ -162,6 +163,9 @@
   </si>
   <si>
     <t xml:space="preserve">Zwarte kubus</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mier</t>
   </si>
   <si>
     <t xml:space="preserve">Jaar</t>
@@ -327,9 +331,6 @@
   </si>
   <si>
     <t xml:space="preserve">Grijs</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Mier</t>
   </si>
   <si>
     <t xml:space="preserve">Molentje</t>
@@ -807,7 +808,7 @@
 </styleSheet>
 </file>
 
-<file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <c:lang val="en-US"/>
   <c:roundedCorners val="0"/>
@@ -854,7 +855,7 @@
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>Omschrijving Kaft Zonnebloem Koperen ei Ruitje Pimpelmees Mijnvogel in Mineur Vlinderbeest Scheepswiel Vondst Tala Vlinder Wolkendroom Kanarie Kopernest Klaver Irmijn Inc logo Obol Boyz Vuurmot Vrijer dan wij Lege kooi In de urn Apenweegschaal Puzzel Groene steen Libel Gift van de Moeders Heks met klauw Bijtje Hoeders Lieveheersbeestje Diep. Diep. Diep. Paal etc Blaadje Zwarte kubus</c:v>
+                  <c:v>Omschrijving Kaft Zonnebloem Koperen ei Ruitje Pimpelmees Mijnvogel in Mineur Vlinderbeest Scheepswiel Vondst Tala Vlinder Wolkendroom Kanarie Kopernest Klaver Irmijn Inc logo Obol Boyz Vuurmot Vrijer dan wij Lege kooi In de urn Apenweegschaal Puzzel Groene steen Libel Gift van de Moeders Heks met klauw Bijtje Hoeders Lieveheersbeestje Diep. Diep. Diep. Paal etc Blaadje Zwarte kubus Mier</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -1489,16 +1490,16 @@
                   <c:v>130</c:v>
                 </c:pt>
                 <c:pt idx="80">
-                  <c:v>131</c:v>
+                  <c:v>136</c:v>
                 </c:pt>
                 <c:pt idx="81">
-                  <c:v/>
+                  <c:v>142</c:v>
                 </c:pt>
                 <c:pt idx="82">
-                  <c:v/>
+                  <c:v>147</c:v>
                 </c:pt>
                 <c:pt idx="83">
-                  <c:v/>
+                  <c:v>148</c:v>
                 </c:pt>
                 <c:pt idx="84">
                   <c:v/>
@@ -1603,11 +1604,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="74773951"/>
-        <c:axId val="78633205"/>
+        <c:axId val="94588878"/>
+        <c:axId val="27235251"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="74773951"/>
+        <c:axId val="94588878"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1663,14 +1664,14 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="78633205"/>
+        <c:crossAx val="27235251"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
         <c:lblOffset val="100"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="78633205"/>
+        <c:axId val="27235251"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1735,7 +1736,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="74773951"/>
+        <c:crossAx val="94588878"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -1762,7 +1763,7 @@
 </c:chartSpace>
 </file>
 
-<file path=xl/charts/chart5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <c:lang val="en-US"/>
   <c:roundedCorners val="0"/>
@@ -2444,13 +2445,13 @@
                   <c:v>47</c:v>
                 </c:pt>
                 <c:pt idx="80">
-                  <c:v/>
+                  <c:v>48</c:v>
                 </c:pt>
                 <c:pt idx="81">
-                  <c:v/>
+                  <c:v>49</c:v>
                 </c:pt>
                 <c:pt idx="82">
-                  <c:v/>
+                  <c:v>49</c:v>
                 </c:pt>
                 <c:pt idx="83">
                   <c:v/>
@@ -3191,13 +3192,13 @@
                   <c:v>18</c:v>
                 </c:pt>
                 <c:pt idx="80">
-                  <c:v/>
+                  <c:v>18</c:v>
                 </c:pt>
                 <c:pt idx="81">
-                  <c:v/>
+                  <c:v>18</c:v>
                 </c:pt>
                 <c:pt idx="82">
-                  <c:v/>
+                  <c:v>18</c:v>
                 </c:pt>
                 <c:pt idx="83">
                   <c:v/>
@@ -3938,13 +3939,13 @@
                   <c:v>11</c:v>
                 </c:pt>
                 <c:pt idx="80">
-                  <c:v/>
+                  <c:v>11</c:v>
                 </c:pt>
                 <c:pt idx="81">
-                  <c:v/>
+                  <c:v>11</c:v>
                 </c:pt>
                 <c:pt idx="82">
-                  <c:v/>
+                  <c:v>12</c:v>
                 </c:pt>
                 <c:pt idx="83">
                   <c:v/>
@@ -4685,13 +4686,13 @@
                   <c:v>4</c:v>
                 </c:pt>
                 <c:pt idx="80">
-                  <c:v/>
+                  <c:v>4</c:v>
                 </c:pt>
                 <c:pt idx="81">
-                  <c:v/>
+                  <c:v>4</c:v>
                 </c:pt>
                 <c:pt idx="82">
-                  <c:v/>
+                  <c:v>4</c:v>
                 </c:pt>
                 <c:pt idx="83">
                   <c:v/>
@@ -4796,11 +4797,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="94870094"/>
-        <c:axId val="9340594"/>
+        <c:axId val="92545215"/>
+        <c:axId val="22253438"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="94870094"/>
+        <c:axId val="92545215"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -4856,14 +4857,14 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="9340594"/>
+        <c:crossAx val="22253438"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
         <c:lblOffset val="100"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="9340594"/>
+        <c:axId val="22253438"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -4928,7 +4929,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="94870094"/>
+        <c:crossAx val="92545215"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -4976,7 +4977,7 @@
 </c:chartSpace>
 </file>
 
-<file path=xl/charts/chart6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <c:lang val="en-US"/>
   <c:roundedCorners val="0"/>
@@ -5016,10 +5017,10 @@
           <c:layoutTarget val="inner"/>
           <c:xMode val="edge"/>
           <c:yMode val="edge"/>
-          <c:x val="0.0889708640740278"/>
-          <c:y val="0.110962864131643"/>
-          <c:w val="0.845942228335626"/>
-          <c:h val="0.793306648877029"/>
+          <c:x val="0.0889764271868943"/>
+          <c:y val="0.110975202935617"/>
+          <c:w val="0.845870068154818"/>
+          <c:h val="0.793172467474702"/>
         </c:manualLayout>
       </c:layout>
       <c:lineChart>
@@ -5151,11 +5152,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="88120819"/>
-        <c:axId val="38893722"/>
+        <c:axId val="78238978"/>
+        <c:axId val="93720606"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="88120819"/>
+        <c:axId val="78238978"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -5183,14 +5184,14 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="38893722"/>
+        <c:crossAx val="93720606"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
         <c:lblOffset val="100"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="38893722"/>
+        <c:axId val="93720606"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -5255,7 +5256,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="88120819"/>
+        <c:crossAx val="78238978"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -5293,9 +5294,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>178560</xdr:colOff>
+      <xdr:colOff>178200</xdr:colOff>
       <xdr:row>23</xdr:row>
-      <xdr:rowOff>42120</xdr:rowOff>
+      <xdr:rowOff>41760</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -5304,7 +5305,7 @@
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
         <a:off x="6578280" y="543600"/>
-        <a:ext cx="5757120" cy="3237120"/>
+        <a:ext cx="5756760" cy="3236760"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -5323,9 +5324,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>342360</xdr:colOff>
+      <xdr:colOff>342000</xdr:colOff>
       <xdr:row>52</xdr:row>
-      <xdr:rowOff>90360</xdr:rowOff>
+      <xdr:rowOff>90000</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -5334,7 +5335,7 @@
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
         <a:off x="6741360" y="5305320"/>
-        <a:ext cx="5757840" cy="3237840"/>
+        <a:ext cx="5757480" cy="3237480"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -5358,9 +5359,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>12</xdr:col>
-      <xdr:colOff>461880</xdr:colOff>
+      <xdr:colOff>461520</xdr:colOff>
       <xdr:row>21</xdr:row>
-      <xdr:rowOff>70560</xdr:rowOff>
+      <xdr:rowOff>70200</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -5369,7 +5370,7 @@
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
         <a:off x="2646720" y="246600"/>
-        <a:ext cx="5757480" cy="3237480"/>
+        <a:ext cx="5757120" cy="3237120"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -6164,11 +6165,11 @@
       </c>
       <c r="K27" s="0" t="n">
         <f aca="false">COUNTIF($D$1:$D$121,$J27)</f>
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="L27" s="6" t="n">
         <f aca="false">$K27/$K$31</f>
-        <v>0.580246913580247</v>
+        <v>0.583333333333333</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6206,7 +6207,7 @@
       </c>
       <c r="L28" s="6" t="n">
         <f aca="false">$K28/$K$31</f>
-        <v>0.222222222222222</v>
+        <v>0.214285714285714</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6244,11 +6245,11 @@
       </c>
       <c r="K29" s="0" t="n">
         <f aca="false">COUNTIF($D$1:$D$121,$J29)</f>
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="L29" s="6" t="n">
         <f aca="false">$K29/$K$31</f>
-        <v>0.135802469135802</v>
+        <v>0.142857142857143</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6290,7 +6291,7 @@
       </c>
       <c r="L30" s="6" t="n">
         <f aca="false">$K30/$K$31</f>
-        <v>0.0493827160493827</v>
+        <v>0.0476190476190476</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6328,7 +6329,7 @@
       </c>
       <c r="K31" s="0" t="n">
         <f aca="false">COUNTA($D$1:$D$121)</f>
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="L31" s="6" t="n">
         <f aca="false">$K31/$K$31</f>
@@ -7738,7 +7739,7 @@
       </c>
       <c r="B81" s="1" t="n">
         <f aca="false">IF(COUNTA(B82)&gt;0,ROUNDDOWN((B82+B80)/2,0),B80+1)</f>
-        <v>131</v>
+        <v>136</v>
       </c>
       <c r="C81" s="2" t="s">
         <v>42</v>
@@ -7767,66 +7768,85 @@
       <c r="A82" s="1" t="n">
         <v>80</v>
       </c>
-      <c r="D82" s="5"/>
-      <c r="E82" s="5" t="str">
+      <c r="B82" s="1" t="n">
+        <v>142</v>
+      </c>
+      <c r="D82" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="E82" s="5" t="n">
         <f aca="false">IF(COUNTA($D82)&gt;0,COUNTIF($D$2:$D82,E$1),"")</f>
-        <v/>
-      </c>
-      <c r="F82" s="5" t="str">
+        <v>18</v>
+      </c>
+      <c r="F82" s="5" t="n">
         <f aca="false">IF(COUNTA($D82)&gt;0,COUNTIF($D$2:$D82,F$1),"")</f>
-        <v/>
-      </c>
-      <c r="G82" s="5" t="str">
+        <v>48</v>
+      </c>
+      <c r="G82" s="5" t="n">
         <f aca="false">IF(COUNTA($D82)&gt;0,COUNTIF($D$2:$D82,G$1),"")</f>
-        <v/>
-      </c>
-      <c r="H82" s="5" t="str">
+        <v>11</v>
+      </c>
+      <c r="H82" s="5" t="n">
         <f aca="false">IF(COUNTA($D82)&gt;0,COUNTIF($D$2:$D82,H$1),"")</f>
-        <v/>
+        <v>4</v>
       </c>
     </row>
     <row r="83" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A83" s="1" t="n">
         <v>81</v>
       </c>
-      <c r="D83" s="5"/>
-      <c r="E83" s="5" t="str">
+      <c r="B83" s="1" t="n">
+        <v>147</v>
+      </c>
+      <c r="D83" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="E83" s="5" t="n">
         <f aca="false">IF(COUNTA($D83)&gt;0,COUNTIF($D$2:$D83,E$1),"")</f>
-        <v/>
-      </c>
-      <c r="F83" s="5" t="str">
+        <v>18</v>
+      </c>
+      <c r="F83" s="5" t="n">
         <f aca="false">IF(COUNTA($D83)&gt;0,COUNTIF($D$2:$D83,F$1),"")</f>
-        <v/>
-      </c>
-      <c r="G83" s="5" t="str">
+        <v>49</v>
+      </c>
+      <c r="G83" s="5" t="n">
         <f aca="false">IF(COUNTA($D83)&gt;0,COUNTIF($D$2:$D83,G$1),"")</f>
-        <v/>
-      </c>
-      <c r="H83" s="5" t="str">
+        <v>11</v>
+      </c>
+      <c r="H83" s="5" t="n">
         <f aca="false">IF(COUNTA($D83)&gt;0,COUNTIF($D$2:$D83,H$1),"")</f>
-        <v/>
+        <v>4</v>
       </c>
     </row>
     <row r="84" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A84" s="1" t="n">
         <v>82</v>
       </c>
-      <c r="D84" s="5"/>
-      <c r="E84" s="5" t="str">
+      <c r="B84" s="1" t="n">
+        <f aca="false">IF(COUNTA(B85)&gt;0,ROUNDDOWN((B85+B83)/2,0),B83+1)</f>
+        <v>148</v>
+      </c>
+      <c r="C84" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="D84" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="E84" s="5" t="n">
         <f aca="false">IF(COUNTA($D84)&gt;0,COUNTIF($D$2:$D84,E$1),"")</f>
-        <v/>
-      </c>
-      <c r="F84" s="5" t="str">
+        <v>18</v>
+      </c>
+      <c r="F84" s="5" t="n">
         <f aca="false">IF(COUNTA($D84)&gt;0,COUNTIF($D$2:$D84,F$1),"")</f>
-        <v/>
-      </c>
-      <c r="G84" s="5" t="str">
+        <v>49</v>
+      </c>
+      <c r="G84" s="5" t="n">
         <f aca="false">IF(COUNTA($D84)&gt;0,COUNTIF($D$2:$D84,G$1),"")</f>
-        <v/>
-      </c>
-      <c r="H84" s="5" t="str">
+        <v>12</v>
+      </c>
+      <c r="H84" s="5" t="n">
         <f aca="false">IF(COUNTA($D84)&gt;0,COUNTIF($D$2:$D84,H$1),"")</f>
-        <v/>
+        <v>4</v>
       </c>
     </row>
     <row r="85" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10093,13 +10113,13 @@
   <sheetData>
     <row r="1" s="4" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="4" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="E1" s="4" t="s">
         <v>2</v>
@@ -10121,7 +10141,7 @@
         <v>429.419178082192</v>
       </c>
       <c r="E2" s="0" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10140,7 +10160,7 @@
         <v>429.419178082192</v>
       </c>
       <c r="E3" s="0" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10159,7 +10179,7 @@
         <v>432.419178082192</v>
       </c>
       <c r="E4" s="0" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10178,7 +10198,7 @@
         <v>433.419178082192</v>
       </c>
       <c r="E5" s="8" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10197,7 +10217,7 @@
         <v>436.419178082192</v>
       </c>
       <c r="E6" s="0" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10216,7 +10236,7 @@
         <v>436.419178082192</v>
       </c>
       <c r="E7" s="0" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10235,7 +10255,7 @@
         <v>437.419178082192</v>
       </c>
       <c r="E8" s="0" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10254,7 +10274,7 @@
         <v>439.419178082192</v>
       </c>
       <c r="E9" s="0" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10273,7 +10293,7 @@
         <v>440.419178082192</v>
       </c>
       <c r="E10" s="0" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10292,7 +10312,7 @@
         <v>443.419178082192</v>
       </c>
       <c r="E11" s="0" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10311,7 +10331,7 @@
         <v>446.419178082192</v>
       </c>
       <c r="E12" s="0" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10330,7 +10350,7 @@
         <v>447.419178082192</v>
       </c>
       <c r="E13" s="0" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10349,7 +10369,7 @@
         <v>447.419178082192</v>
       </c>
       <c r="E14" s="8" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10368,7 +10388,7 @@
         <v>448.419178082192</v>
       </c>
       <c r="E15" s="0" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10387,7 +10407,7 @@
         <v>449.419178082192</v>
       </c>
       <c r="E16" s="8" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10406,7 +10426,7 @@
         <v>449.419178082192</v>
       </c>
       <c r="E17" s="0" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10425,7 +10445,7 @@
         <v>450.419178082192</v>
       </c>
       <c r="E18" s="0" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10444,7 +10464,7 @@
         <v>450.419178082192</v>
       </c>
       <c r="E19" s="0" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
     </row>
   </sheetData>
@@ -10464,7 +10484,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F94"/>
+  <dimension ref="A1:F95"/>
   <sheetFormatPr defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="9.63"/>
@@ -10476,33 +10496,33 @@
   <sheetData>
     <row r="1" s="9" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="9" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="B1" s="9" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C1" s="9" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="D1" s="9" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E1" s="9" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="F1" s="9" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="10" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B2" s="11" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C2" s="12" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="D2" s="0" t="n">
         <f aca="false">IF(ISBLANK(A2),"",COUNTIF(A:A,A2))</f>
@@ -10519,13 +10539,13 @@
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="10" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B3" s="11" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C3" s="12" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="D3" s="0" t="n">
         <f aca="false">IF(ISBLANK(A3),"",COUNTIF(A:A,A3))</f>
@@ -10542,13 +10562,13 @@
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="10" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B4" s="11" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C4" s="13" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="D4" s="0" t="n">
         <f aca="false">IF(ISBLANK(A4),"",COUNTIF(A:A,A4))</f>
@@ -10565,13 +10585,13 @@
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="10" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B5" s="14" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="D5" s="0" t="n">
         <f aca="false">IF(ISBLANK(A5),"",COUNTIF(A:A,A5))</f>
@@ -10588,13 +10608,13 @@
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="10" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B6" s="14" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="C6" s="15" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="D6" s="0" t="n">
         <f aca="false">IF(ISBLANK(A6),"",COUNTIF(A:A,A6))</f>
@@ -10611,13 +10631,13 @@
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="10" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B7" s="14" t="s">
+        <v>75</v>
+      </c>
+      <c r="C7" s="13" t="s">
         <v>74</v>
-      </c>
-      <c r="C7" s="13" t="s">
-        <v>73</v>
       </c>
       <c r="D7" s="0" t="n">
         <f aca="false">IF(ISBLANK(A7),"",COUNTIF(A:A,A7))</f>
@@ -10634,13 +10654,13 @@
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="10" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B8" s="16" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="C8" s="17" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="D8" s="0" t="n">
         <f aca="false">IF(ISBLANK(A8),"",COUNTIF(A:A,A8))</f>
@@ -10657,13 +10677,13 @@
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="10" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B9" s="16" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="C9" s="10" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="D9" s="0" t="n">
         <f aca="false">IF(ISBLANK(A9),"",COUNTIF(A:A,A9))</f>
@@ -10680,13 +10700,13 @@
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="10" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B10" s="12" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="C10" s="10" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="D10" s="0" t="n">
         <f aca="false">IF(ISBLANK(A10),"",COUNTIF(A:A,A10))</f>
@@ -10703,13 +10723,13 @@
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="10" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B11" s="18" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="C11" s="11" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="D11" s="0" t="n">
         <f aca="false">IF(ISBLANK(A11),"",COUNTIF(A:A,A11))</f>
@@ -10726,13 +10746,13 @@
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="10" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B12" s="19" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="C12" s="8" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="D12" s="0" t="n">
         <f aca="false">IF(ISBLANK(A12),"",COUNTIF(A:A,A12))</f>
@@ -10749,13 +10769,13 @@
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="10" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B13" s="19" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="C13" s="10" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="D13" s="0" t="n">
         <f aca="false">IF(ISBLANK(A13),"",COUNTIF(A:A,A13))</f>
@@ -10772,13 +10792,13 @@
     </row>
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="10" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B14" s="20" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="C14" s="8" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="D14" s="0" t="n">
         <f aca="false">IF(ISBLANK(A14),"",COUNTIF(A:A,A14))</f>
@@ -10795,13 +10815,13 @@
     </row>
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="10" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B15" s="20" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="C15" s="8" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="D15" s="0" t="n">
         <f aca="false">IF(ISBLANK(A15),"",COUNTIF(A:A,A15))</f>
@@ -10818,13 +10838,13 @@
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="10" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B16" s="13" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="C16" s="14" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="D16" s="0" t="n">
         <f aca="false">IF(ISBLANK(A16),"",COUNTIF(A:A,A16))</f>
@@ -10841,13 +10861,13 @@
     </row>
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="10" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B17" s="13" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="C17" s="14" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="D17" s="0" t="n">
         <f aca="false">IF(ISBLANK(A17),"",COUNTIF(A:A,A17))</f>
@@ -10867,10 +10887,10 @@
         <v>33</v>
       </c>
       <c r="B18" s="21" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="C18" s="8" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="D18" s="0" t="n">
         <f aca="false">IF(ISBLANK(A18),"",COUNTIF(A:A,A18))</f>
@@ -10890,10 +10910,10 @@
         <v>33</v>
       </c>
       <c r="B19" s="21" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="C19" s="15" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="D19" s="0" t="n">
         <f aca="false">IF(ISBLANK(A19),"",COUNTIF(A:A,A19))</f>
@@ -10913,10 +10933,10 @@
         <v>33</v>
       </c>
       <c r="B20" s="21" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="C20" s="17" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="D20" s="0" t="n">
         <f aca="false">IF(ISBLANK(A20),"",COUNTIF(A:A,A20))</f>
@@ -10936,10 +10956,10 @@
         <v>33</v>
       </c>
       <c r="B21" s="8" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C21" s="17" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="D21" s="0" t="n">
         <f aca="false">IF(ISBLANK(A21),"",COUNTIF(A:A,A21))</f>
@@ -10959,10 +10979,10 @@
         <v>33</v>
       </c>
       <c r="B22" s="14" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="C22" s="15" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="D22" s="0" t="n">
         <f aca="false">IF(ISBLANK(A22),"",COUNTIF(A:A,A22))</f>
@@ -10982,10 +11002,10 @@
         <v>33</v>
       </c>
       <c r="B23" s="14" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="C23" s="15" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="D23" s="0" t="n">
         <f aca="false">IF(ISBLANK(A23),"",COUNTIF(A:A,A23))</f>
@@ -11005,10 +11025,10 @@
         <v>33</v>
       </c>
       <c r="B24" s="14" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="C24" s="15" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="D24" s="0" t="n">
         <f aca="false">IF(ISBLANK(A24),"",COUNTIF(A:A,A24))</f>
@@ -11028,10 +11048,10 @@
         <v>33</v>
       </c>
       <c r="B25" s="22" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="C25" s="15" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="D25" s="0" t="n">
         <f aca="false">IF(ISBLANK(A25),"",COUNTIF(A:A,A25))</f>
@@ -11051,10 +11071,10 @@
         <v>33</v>
       </c>
       <c r="B26" s="22" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="C26" s="14" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="D26" s="0" t="n">
         <f aca="false">IF(ISBLANK(A26),"",COUNTIF(A:A,A26))</f>
@@ -11074,10 +11094,10 @@
         <v>33</v>
       </c>
       <c r="B27" s="22" t="s">
+        <v>85</v>
+      </c>
+      <c r="C27" s="21" t="s">
         <v>84</v>
-      </c>
-      <c r="C27" s="21" t="s">
-        <v>83</v>
       </c>
       <c r="D27" s="0" t="n">
         <f aca="false">IF(ISBLANK(A27),"",COUNTIF(A:A,A27))</f>
@@ -11097,10 +11117,10 @@
         <v>33</v>
       </c>
       <c r="B28" s="16" t="s">
+        <v>78</v>
+      </c>
+      <c r="C28" s="15" t="s">
         <v>77</v>
-      </c>
-      <c r="C28" s="15" t="s">
-        <v>76</v>
       </c>
       <c r="D28" s="0" t="n">
         <f aca="false">IF(ISBLANK(A28),"",COUNTIF(A:A,A28))</f>
@@ -11120,10 +11140,10 @@
         <v>33</v>
       </c>
       <c r="B29" s="16" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="C29" s="23" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="D29" s="0" t="n">
         <f aca="false">IF(ISBLANK(A29),"",COUNTIF(A:A,A29))</f>
@@ -11143,10 +11163,10 @@
         <v>33</v>
       </c>
       <c r="B30" s="12" t="s">
+        <v>73</v>
+      </c>
+      <c r="C30" s="11" t="s">
         <v>72</v>
-      </c>
-      <c r="C30" s="11" t="s">
-        <v>71</v>
       </c>
       <c r="D30" s="0" t="n">
         <f aca="false">IF(ISBLANK(A30),"",COUNTIF(A:A,A30))</f>
@@ -11166,10 +11186,10 @@
         <v>33</v>
       </c>
       <c r="B31" s="12" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="C31" s="16" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="D31" s="0" t="n">
         <f aca="false">IF(ISBLANK(A31),"",COUNTIF(A:A,A31))</f>
@@ -11189,10 +11209,10 @@
         <v>33</v>
       </c>
       <c r="B32" s="20" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="C32" s="8" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="D32" s="0" t="n">
         <f aca="false">IF(ISBLANK(A32),"",COUNTIF(A:A,A32))</f>
@@ -11212,10 +11232,10 @@
         <v>33</v>
       </c>
       <c r="B33" s="15" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="C33" s="17" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="D33" s="0" t="n">
         <f aca="false">IF(ISBLANK(A33),"",COUNTIF(A:A,A33))</f>
@@ -11232,10 +11252,10 @@
     </row>
     <row r="34" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="22" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="B34" s="21" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="D34" s="0" t="n">
         <f aca="false">IF(ISBLANK(A34),"",COUNTIF(A:A,A34))</f>
@@ -11252,10 +11272,10 @@
     </row>
     <row r="35" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="22" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="B35" s="21" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="D35" s="0" t="n">
         <f aca="false">IF(ISBLANK(A35),"",COUNTIF(A:A,A35))</f>
@@ -11272,10 +11292,10 @@
     </row>
     <row r="36" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="22" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="B36" s="8" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="D36" s="0" t="n">
         <f aca="false">IF(ISBLANK(A36),"",COUNTIF(A:A,A36))</f>
@@ -11292,10 +11312,10 @@
     </row>
     <row r="37" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="22" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="B37" s="8" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="D37" s="0" t="n">
         <f aca="false">IF(ISBLANK(A37),"",COUNTIF(A:A,A37))</f>
@@ -11312,10 +11332,10 @@
     </row>
     <row r="38" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="22" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="B38" s="8" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="D38" s="0" t="n">
         <f aca="false">IF(ISBLANK(A38),"",COUNTIF(A:A,A38))</f>
@@ -11332,10 +11352,10 @@
     </row>
     <row r="39" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="22" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="B39" s="8" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="D39" s="0" t="n">
         <f aca="false">IF(ISBLANK(A39),"",COUNTIF(A:A,A39))</f>
@@ -11352,10 +11372,10 @@
     </row>
     <row r="40" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="22" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="B40" s="22" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="D40" s="0" t="n">
         <f aca="false">IF(ISBLANK(A40),"",COUNTIF(A:A,A40))</f>
@@ -11372,10 +11392,10 @@
     </row>
     <row r="41" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="22" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="B41" s="17" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="D41" s="0" t="n">
         <f aca="false">IF(ISBLANK(A41),"",COUNTIF(A:A,A41))</f>
@@ -11392,10 +11412,10 @@
     </row>
     <row r="42" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="22" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="B42" s="17" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="D42" s="0" t="n">
         <f aca="false">IF(ISBLANK(A42),"",COUNTIF(A:A,A42))</f>
@@ -11412,10 +11432,10 @@
     </row>
     <row r="43" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="22" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="B43" s="17" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="D43" s="0" t="n">
         <f aca="false">IF(ISBLANK(A43),"",COUNTIF(A:A,A43))</f>
@@ -11432,10 +11452,10 @@
     </row>
     <row r="44" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="22" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="B44" s="24" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="D44" s="0" t="n">
         <f aca="false">IF(ISBLANK(A44),"",COUNTIF(A:A,A44))</f>
@@ -11452,10 +11472,10 @@
     </row>
     <row r="45" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="22" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="B45" s="24" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="D45" s="0" t="n">
         <f aca="false">IF(ISBLANK(A45),"",COUNTIF(A:A,A45))</f>
@@ -11475,10 +11495,10 @@
         <v>19</v>
       </c>
       <c r="B46" s="21" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="C46" s="13" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="D46" s="0" t="n">
         <f aca="false">IF(ISBLANK(A46),"",COUNTIF(A:A,A46))</f>
@@ -11498,10 +11518,10 @@
         <v>19</v>
       </c>
       <c r="B47" s="21" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="C47" s="13" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="D47" s="0" t="n">
         <f aca="false">IF(ISBLANK(A47),"",COUNTIF(A:A,A47))</f>
@@ -11521,10 +11541,10 @@
         <v>19</v>
       </c>
       <c r="B48" s="8" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C48" s="20" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="D48" s="0" t="n">
         <f aca="false">IF(ISBLANK(A48),"",COUNTIF(A:A,A48))</f>
@@ -11544,10 +11564,10 @@
         <v>19</v>
       </c>
       <c r="B49" s="14" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="C49" s="15" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="D49" s="0" t="n">
         <f aca="false">IF(ISBLANK(A49),"",COUNTIF(A:A,A49))</f>
@@ -11567,10 +11587,10 @@
         <v>19</v>
       </c>
       <c r="B50" s="16" t="s">
+        <v>78</v>
+      </c>
+      <c r="C50" s="15" t="s">
         <v>77</v>
-      </c>
-      <c r="C50" s="15" t="s">
-        <v>76</v>
       </c>
       <c r="D50" s="0" t="n">
         <f aca="false">IF(ISBLANK(A50),"",COUNTIF(A:A,A50))</f>
@@ -11590,10 +11610,10 @@
         <v>19</v>
       </c>
       <c r="B51" s="16" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="C51" s="12" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="D51" s="0" t="n">
         <f aca="false">IF(ISBLANK(A51),"",COUNTIF(A:A,A51))</f>
@@ -11613,10 +11633,10 @@
         <v>19</v>
       </c>
       <c r="B52" s="12" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="C52" s="19" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="D52" s="0" t="n">
         <f aca="false">IF(ISBLANK(A52),"",COUNTIF(A:A,A52))</f>
@@ -11636,10 +11656,10 @@
         <v>19</v>
       </c>
       <c r="B53" s="20" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="C53" s="8" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="D53" s="0" t="n">
         <f aca="false">IF(ISBLANK(A53),"",COUNTIF(A:A,A53))</f>
@@ -11659,10 +11679,10 @@
         <v>19</v>
       </c>
       <c r="B54" s="13" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="C54" s="15" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="D54" s="0" t="n">
         <f aca="false">IF(ISBLANK(A54),"",COUNTIF(A:A,A54))</f>
@@ -11682,10 +11702,10 @@
         <v>19</v>
       </c>
       <c r="B55" s="13" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="C55" s="21" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="D55" s="0" t="n">
         <f aca="false">IF(ISBLANK(A55),"",COUNTIF(A:A,A55))</f>
@@ -11705,10 +11725,10 @@
         <v>19</v>
       </c>
       <c r="B56" s="25" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="C56" s="8" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="D56" s="0" t="n">
         <f aca="false">IF(ISBLANK(A56),"",COUNTIF(A:A,A56))</f>
@@ -11725,13 +11745,13 @@
     </row>
     <row r="57" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="12" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="B57" s="11" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C57" s="12" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="D57" s="0" t="n">
         <f aca="false">IF(ISBLANK(A57),"",COUNTIF(A:A,A57))</f>
@@ -11748,13 +11768,13 @@
     </row>
     <row r="58" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="12" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="B58" s="11" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C58" s="12" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="D58" s="0" t="n">
         <f aca="false">IF(ISBLANK(A58),"",COUNTIF(A:A,A58))</f>
@@ -11771,13 +11791,13 @@
     </row>
     <row r="59" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="12" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="B59" s="11" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C59" s="12" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="D59" s="0" t="n">
         <f aca="false">IF(ISBLANK(A59),"",COUNTIF(A:A,A59))</f>
@@ -11794,13 +11814,13 @@
     </row>
     <row r="60" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="12" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="B60" s="11" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C60" s="13" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="D60" s="0" t="n">
         <f aca="false">IF(ISBLANK(A60),"",COUNTIF(A:A,A60))</f>
@@ -11817,13 +11837,13 @@
     </row>
     <row r="61" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="12" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="B61" s="16" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="C61" s="12" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="D61" s="0" t="n">
         <f aca="false">IF(ISBLANK(A61),"",COUNTIF(A:A,A61))</f>
@@ -11840,13 +11860,13 @@
     </row>
     <row r="62" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="12" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="B62" s="12" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="C62" s="19" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="D62" s="0" t="n">
         <f aca="false">IF(ISBLANK(A62),"",COUNTIF(A:A,A62))</f>
@@ -11863,13 +11883,13 @@
     </row>
     <row r="63" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="12" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="B63" s="19" t="s">
+        <v>82</v>
+      </c>
+      <c r="C63" s="18" t="s">
         <v>81</v>
-      </c>
-      <c r="C63" s="18" t="s">
-        <v>80</v>
       </c>
       <c r="D63" s="0" t="n">
         <f aca="false">IF(ISBLANK(A63),"",COUNTIF(A:A,A63))</f>
@@ -11886,13 +11906,13 @@
     </row>
     <row r="64" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="12" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="B64" s="19" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="C64" s="10" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="D64" s="0" t="n">
         <f aca="false">IF(ISBLANK(A64),"",COUNTIF(A:A,A64))</f>
@@ -11909,13 +11929,13 @@
     </row>
     <row r="65" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="12" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="B65" s="17" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="C65" s="8" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="D65" s="0" t="n">
         <f aca="false">IF(ISBLANK(A65),"",COUNTIF(A:A,A65))</f>
@@ -11932,13 +11952,13 @@
     </row>
     <row r="66" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="12" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="B66" s="15" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="C66" s="14" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="D66" s="0" t="n">
         <f aca="false">IF(ISBLANK(A66),"",COUNTIF(A:A,A66))</f>
@@ -11955,13 +11975,13 @@
     </row>
     <row r="67" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="21" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="B67" s="21" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="C67" s="8" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="D67" s="0" t="n">
         <f aca="false">IF(ISBLANK(A67),"",COUNTIF(A:A,A67))</f>
@@ -11978,13 +11998,13 @@
     </row>
     <row r="68" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="21" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="B68" s="21" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="C68" s="17" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="D68" s="0" t="n">
         <f aca="false">IF(ISBLANK(A68),"",COUNTIF(A:A,A68))</f>
@@ -12001,13 +12021,13 @@
     </row>
     <row r="69" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A69" s="21" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="B69" s="8" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C69" s="17" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="D69" s="0" t="n">
         <f aca="false">IF(ISBLANK(A69),"",COUNTIF(A:A,A69))</f>
@@ -12024,13 +12044,13 @@
     </row>
     <row r="70" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A70" s="21" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="B70" s="14" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="C70" s="15" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="D70" s="0" t="n">
         <f aca="false">IF(ISBLANK(A70),"",COUNTIF(A:A,A70))</f>
@@ -12047,13 +12067,13 @@
     </row>
     <row r="71" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A71" s="21" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="B71" s="22" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="C71" s="8" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="D71" s="0" t="n">
         <f aca="false">IF(ISBLANK(A71),"",COUNTIF(A:A,A71))</f>
@@ -12070,13 +12090,13 @@
     </row>
     <row r="72" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A72" s="21" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="B72" s="22" t="s">
+        <v>85</v>
+      </c>
+      <c r="C72" s="21" t="s">
         <v>84</v>
-      </c>
-      <c r="C72" s="21" t="s">
-        <v>83</v>
       </c>
       <c r="D72" s="0" t="n">
         <f aca="false">IF(ISBLANK(A72),"",COUNTIF(A:A,A72))</f>
@@ -12093,13 +12113,13 @@
     </row>
     <row r="73" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A73" s="21" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="B73" s="26" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="C73" s="8" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="D73" s="0" t="n">
         <f aca="false">IF(ISBLANK(A73),"",COUNTIF(A:A,A73))</f>
@@ -12119,10 +12139,10 @@
         <v>36</v>
       </c>
       <c r="B74" s="18" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="C74" s="8" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="D74" s="0" t="n">
         <f aca="false">IF(ISBLANK(A74),"",COUNTIF(A:A,A74))</f>
@@ -12142,10 +12162,10 @@
         <v>36</v>
       </c>
       <c r="B75" s="18" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="C75" s="8" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="D75" s="0" t="n">
         <f aca="false">IF(ISBLANK(A75),"",COUNTIF(A:A,A75))</f>
@@ -12165,10 +12185,10 @@
         <v>36</v>
       </c>
       <c r="B76" s="18" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="C76" s="8" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="D76" s="0" t="n">
         <f aca="false">IF(ISBLANK(A76),"",COUNTIF(A:A,A76))</f>
@@ -12188,10 +12208,10 @@
         <v>36</v>
       </c>
       <c r="B77" s="18" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="C77" s="8" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="D77" s="0" t="n">
         <f aca="false">IF(ISBLANK(A77),"",COUNTIF(A:A,A77))</f>
@@ -12211,10 +12231,10 @@
         <v>36</v>
       </c>
       <c r="B78" s="18" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="C78" s="8" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="D78" s="0" t="n">
         <f aca="false">IF(ISBLANK(A78),"",COUNTIF(A:A,A78))</f>
@@ -12234,10 +12254,10 @@
         <v>36</v>
       </c>
       <c r="B79" s="18" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="C79" s="8" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="D79" s="0" t="n">
         <f aca="false">IF(ISBLANK(A79),"",COUNTIF(A:A,A79))</f>
@@ -12254,10 +12274,10 @@
     </row>
     <row r="80" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A80" s="22" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="B80" s="8" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="D80" s="0" t="n">
         <f aca="false">IF(ISBLANK(A80),"",COUNTIF(A:A,A80))</f>
@@ -12274,10 +12294,10 @@
     </row>
     <row r="81" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A81" s="22" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="B81" s="22" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="D81" s="0" t="n">
         <f aca="false">IF(ISBLANK(A81),"",COUNTIF(A:A,A81))</f>
@@ -12294,10 +12314,10 @@
     </row>
     <row r="82" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A82" s="22" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="B82" s="22" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="D82" s="0" t="n">
         <f aca="false">IF(ISBLANK(A82),"",COUNTIF(A:A,A82))</f>
@@ -12314,10 +12334,10 @@
     </row>
     <row r="83" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A83" s="22" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="B83" s="17" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="D83" s="0" t="n">
         <f aca="false">IF(ISBLANK(A83),"",COUNTIF(A:A,A83))</f>
@@ -12334,13 +12354,13 @@
     </row>
     <row r="84" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A84" s="25" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="B84" s="8" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C84" s="18" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="D84" s="0" t="n">
         <f aca="false">IF(ISBLANK(A84),"",COUNTIF(A:A,A84))</f>
@@ -12357,13 +12377,13 @@
     </row>
     <row r="85" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A85" s="25" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="B85" s="20" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="C85" s="18" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="D85" s="0" t="n">
         <f aca="false">IF(ISBLANK(A85),"",COUNTIF(A:A,A85))</f>
@@ -12380,13 +12400,13 @@
     </row>
     <row r="86" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A86" s="25" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="B86" s="25" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="C86" s="18" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="D86" s="0" t="n">
         <f aca="false">IF(ISBLANK(A86),"",COUNTIF(A:A,A86))</f>
@@ -12403,13 +12423,13 @@
     </row>
     <row r="87" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A87" s="19" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="B87" s="11" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C87" s="18" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="D87" s="0" t="n">
         <f aca="false">IF(ISBLANK(A87),"",COUNTIF(A:A,A87))</f>
@@ -12426,13 +12446,13 @@
     </row>
     <row r="88" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A88" s="19" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="B88" s="12" t="s">
+        <v>73</v>
+      </c>
+      <c r="C88" s="11" t="s">
         <v>72</v>
-      </c>
-      <c r="C88" s="11" t="s">
-        <v>71</v>
       </c>
       <c r="D88" s="0" t="n">
         <f aca="false">IF(ISBLANK(A88),"",COUNTIF(A:A,A88))</f>
@@ -12449,13 +12469,13 @@
     </row>
     <row r="89" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A89" s="19" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="B89" s="19" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="C89" s="19" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="D89" s="0" t="n">
         <f aca="false">IF(ISBLANK(A89),"",COUNTIF(A:A,A89))</f>
@@ -12472,13 +12492,13 @@
     </row>
     <row r="90" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A90" s="27" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="B90" s="11" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C90" s="12" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="D90" s="0" t="n">
         <f aca="false">IF(ISBLANK(A90),"",COUNTIF(A:A,A90))</f>
@@ -12495,13 +12515,13 @@
     </row>
     <row r="91" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A91" s="27" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="B91" s="27" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="C91" s="28" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="D91" s="0" t="n">
         <f aca="false">IF(ISBLANK(A91),"",COUNTIF(A:A,A91))</f>
@@ -12518,13 +12538,13 @@
     </row>
     <row r="92" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A92" s="27" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="B92" s="27" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="C92" s="28" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="D92" s="0" t="n">
         <f aca="false">IF(ISBLANK(A92),"",COUNTIF(A:A,A92))</f>
@@ -12541,14 +12561,14 @@
     </row>
     <row r="93" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A93" s="18" t="s">
-        <v>98</v>
+        <v>43</v>
       </c>
       <c r="B93" s="21" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="D93" s="0" t="n">
         <f aca="false">IF(ISBLANK(A93),"",COUNTIF(A:A,A93))</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E93" s="0" t="n">
         <f aca="false">IF(ISBLANK(B93),"",COUNTIF(B:B,B93))</f>
@@ -12560,30 +12580,50 @@
       </c>
     </row>
     <row r="94" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A94" s="16" t="s">
-        <v>99</v>
-      </c>
-      <c r="B94" s="12" t="s">
-        <v>72</v>
-      </c>
-      <c r="C94" s="16" t="s">
-        <v>77</v>
+      <c r="A94" s="18" t="s">
+        <v>43</v>
+      </c>
+      <c r="B94" s="28" t="s">
+        <v>98</v>
       </c>
       <c r="D94" s="0" t="n">
         <f aca="false">IF(ISBLANK(A94),"",COUNTIF(A:A,A94))</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E94" s="0" t="n">
         <f aca="false">IF(ISBLANK(B94),"",COUNTIF(B:B,B94))</f>
+        <v>1</v>
+      </c>
+      <c r="F94" s="0" t="str">
+        <f aca="false">IF(ISBLANK(C94),"",COUNTIF(C:C,C94))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="95" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A95" s="16" t="s">
+        <v>99</v>
+      </c>
+      <c r="B95" s="12" t="s">
+        <v>73</v>
+      </c>
+      <c r="C95" s="16" t="s">
+        <v>78</v>
+      </c>
+      <c r="D95" s="0" t="n">
+        <f aca="false">IF(ISBLANK(A95),"",COUNTIF(A:A,A95))</f>
+        <v>1</v>
+      </c>
+      <c r="E95" s="0" t="n">
+        <f aca="false">IF(ISBLANK(B95),"",COUNTIF(B:B,B95))</f>
         <v>7</v>
       </c>
-      <c r="F94" s="0" t="n">
-        <f aca="false">IF(ISBLANK(C94),"",COUNTIF(C:C,C94))</f>
+      <c r="F95" s="0" t="n">
+        <f aca="false">IF(ISBLANK(C95),"",COUNTIF(C:C,C95))</f>
         <v>2</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F94"/>
+  <autoFilter ref="A1:F95"/>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
   <pageSetup paperSize="9" scale="100" firstPageNumber="0" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" useFirstPageNumber="false" horizontalDpi="300" verticalDpi="300" copies="1"/>
@@ -12618,19 +12658,19 @@
   <sheetData>
     <row r="1" s="9" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="9" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>100</v>
       </c>
       <c r="D1" s="9" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="E1" s="3" t="s">
         <v>100</v>
       </c>
       <c r="G1" s="9" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="H1" s="3" t="s">
         <v>100</v>
@@ -12644,28 +12684,28 @@
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="10" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B2" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!A:A,A2)</f>
         <v>16</v>
       </c>
       <c r="D2" s="21" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="E2" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!B:B,D2)</f>
         <v>10</v>
       </c>
       <c r="G2" s="8" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="H2" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!C:C,G2)</f>
         <v>18</v>
       </c>
       <c r="J2" s="8" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="K2" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!B:B,J2)*2+COUNTIF(Tatjes!C:C,J2)</f>
@@ -12681,21 +12721,21 @@
         <v>16</v>
       </c>
       <c r="D3" s="8" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="E3" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!B:B,D3)</f>
         <v>9</v>
       </c>
       <c r="G3" s="15" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="H3" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!C:C,G3)</f>
         <v>11</v>
       </c>
       <c r="J3" s="21" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="K3" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!B:B,J3)*2+COUNTIF(Tatjes!C:C,J3)</f>
@@ -12704,28 +12744,28 @@
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="22" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="B4" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!A:A,A4)</f>
         <v>12</v>
       </c>
       <c r="D4" s="11" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="E4" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!B:B,D4)</f>
         <v>9</v>
       </c>
       <c r="G4" s="12" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="H4" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!C:C,G4)</f>
         <v>8</v>
       </c>
       <c r="J4" s="12" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="K4" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!B:B,J4)*2+COUNTIF(Tatjes!C:C,J4)</f>
@@ -12741,21 +12781,21 @@
         <v>11</v>
       </c>
       <c r="D5" s="14" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="E5" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!B:B,D5)</f>
         <v>8</v>
       </c>
       <c r="G5" s="17" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="H5" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!C:C,G5)</f>
         <v>6</v>
       </c>
       <c r="J5" s="11" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="K5" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!B:B,J5)*2+COUNTIF(Tatjes!C:C,J5)</f>
@@ -12764,28 +12804,28 @@
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="12" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="B6" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!A:A,A6)</f>
         <v>10</v>
       </c>
       <c r="D6" s="22" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="E6" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!B:B,D6)</f>
         <v>8</v>
       </c>
       <c r="G6" s="13" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="H6" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!C:C,G6)</f>
         <v>5</v>
       </c>
       <c r="J6" s="14" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="K6" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!B:B,J6)*2+COUNTIF(Tatjes!C:C,J6)</f>
@@ -12794,28 +12834,28 @@
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="21" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="B7" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!A:A,A7)</f>
         <v>7</v>
       </c>
       <c r="D7" s="16" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="E7" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!B:B,D7)</f>
         <v>7</v>
       </c>
       <c r="G7" s="18" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="H7" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!C:C,G7)</f>
         <v>5</v>
       </c>
       <c r="J7" s="18" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="K7" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!B:B,J7)*2+COUNTIF(Tatjes!C:C,J7)</f>
@@ -12831,21 +12871,21 @@
         <v>6</v>
       </c>
       <c r="D8" s="12" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="E8" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!B:B,D8)</f>
         <v>7</v>
       </c>
       <c r="G8" s="14" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="H8" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!C:C,G8)</f>
         <v>4</v>
       </c>
       <c r="J8" s="22" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="K8" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!B:B,J8)*2+COUNTIF(Tatjes!C:C,J8)</f>
@@ -12854,28 +12894,28 @@
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="22" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="B9" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!A:A,A9)</f>
         <v>4</v>
       </c>
       <c r="D9" s="18" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="E9" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!B:B,D9)</f>
         <v>7</v>
       </c>
       <c r="G9" s="19" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="H9" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!C:C,G9)</f>
         <v>3</v>
       </c>
       <c r="J9" s="17" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="K9" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!B:B,J9)*2+COUNTIF(Tatjes!C:C,J9)</f>
@@ -12884,28 +12924,28 @@
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="25" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="B10" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!A:A,A10)</f>
         <v>3</v>
       </c>
       <c r="D10" s="19" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="E10" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!B:B,D10)</f>
         <v>5</v>
       </c>
       <c r="G10" s="21" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="H10" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!C:C,G10)</f>
         <v>3</v>
       </c>
       <c r="J10" s="16" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="K10" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!B:B,J10)*2+COUNTIF(Tatjes!C:C,J10)</f>
@@ -12914,28 +12954,28 @@
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="19" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="B11" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!A:A,A11)</f>
         <v>3</v>
       </c>
       <c r="D11" s="17" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="E11" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!B:B,D11)</f>
         <v>5</v>
       </c>
       <c r="G11" s="11" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="H11" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!C:C,G11)</f>
         <v>3</v>
       </c>
       <c r="J11" s="15" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="K11" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!B:B,J11)*2+COUNTIF(Tatjes!C:C,J11)</f>
@@ -12944,28 +12984,28 @@
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="27" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="B12" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!A:A,A12)</f>
         <v>3</v>
       </c>
       <c r="D12" s="20" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="E12" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!B:B,D12)</f>
         <v>5</v>
       </c>
       <c r="G12" s="28" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="H12" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!C:C,G12)</f>
         <v>2</v>
       </c>
       <c r="J12" s="19" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="K12" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!B:B,J12)*2+COUNTIF(Tatjes!C:C,J12)</f>
@@ -12974,28 +13014,28 @@
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="18" t="s">
-        <v>98</v>
+        <v>43</v>
       </c>
       <c r="B13" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!A:A,A13)</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D13" s="13" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="E13" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!B:B,D13)</f>
         <v>4</v>
       </c>
       <c r="G13" s="16" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="H13" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!C:C,G13)</f>
         <v>2</v>
       </c>
       <c r="J13" s="13" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="K13" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!B:B,J13)*2+COUNTIF(Tatjes!C:C,J13)</f>
@@ -13011,21 +13051,21 @@
         <v>1</v>
       </c>
       <c r="D14" s="15" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="E14" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!B:B,D14)</f>
         <v>2</v>
       </c>
       <c r="G14" s="20" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="H14" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!C:C,G14)</f>
         <v>1</v>
       </c>
       <c r="J14" s="20" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="K14" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!B:B,J14)*2+COUNTIF(Tatjes!C:C,J14)</f>
@@ -13035,21 +13075,21 @@
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B15" s="0"/>
       <c r="D15" s="27" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="E15" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!B:B,D15)</f>
         <v>2</v>
       </c>
       <c r="G15" s="23" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="H15" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!C:C,G15)</f>
         <v>1</v>
       </c>
       <c r="J15" s="27" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="K15" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!B:B,J15)*2+COUNTIF(Tatjes!C:C,J15)</f>
@@ -13062,24 +13102,24 @@
       </c>
       <c r="B16" s="3" t="n">
         <f aca="false">COUNTA(Tatjes!A:A)-1</f>
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="D16" s="24" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="E16" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!B:B,D16)</f>
         <v>2</v>
       </c>
       <c r="G16" s="27" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="H16" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!C:C,G16)</f>
         <v>0</v>
       </c>
-      <c r="J16" s="24" t="s">
-        <v>87</v>
+      <c r="J16" s="28" t="s">
+        <v>98</v>
       </c>
       <c r="K16" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!B:B,J16)*2+COUNTIF(Tatjes!C:C,J16)</f>
@@ -13088,20 +13128,20 @@
     </row>
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D17" s="25" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="E17" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!B:B,D17)</f>
         <v>2</v>
       </c>
       <c r="G17" s="22" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="H17" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!C:C,G17)</f>
         <v>0</v>
       </c>
-      <c r="J17" s="25" t="s">
+      <c r="J17" s="24" t="s">
         <v>88</v>
       </c>
       <c r="K17" s="1" t="n">
@@ -13110,45 +13150,45 @@
       </c>
     </row>
     <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D18" s="26" t="s">
-        <v>91</v>
+      <c r="D18" s="28" t="s">
+        <v>98</v>
       </c>
       <c r="E18" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!B:B,D18)</f>
         <v>1</v>
       </c>
       <c r="G18" s="24" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="H18" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!C:C,G18)</f>
         <v>0</v>
       </c>
-      <c r="J18" s="28" t="s">
-        <v>97</v>
+      <c r="J18" s="25" t="s">
+        <v>89</v>
       </c>
       <c r="K18" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!B:B,J18)*2+COUNTIF(Tatjes!C:C,J18)</f>
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D19" s="28" t="s">
-        <v>97</v>
+      <c r="D19" s="26" t="s">
+        <v>92</v>
       </c>
       <c r="E19" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!B:B,D19)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G19" s="26" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="H19" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!C:C,G19)</f>
         <v>0</v>
       </c>
       <c r="J19" s="26" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="K19" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!B:B,J19)*2+COUNTIF(Tatjes!C:C,J19)</f>
@@ -13157,21 +13197,21 @@
     </row>
     <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D20" s="23" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="E20" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!B:B,D20)</f>
         <v>0</v>
       </c>
       <c r="G20" s="25" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="H20" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!C:C,G20)</f>
         <v>0</v>
       </c>
       <c r="J20" s="23" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="K20" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!B:B,J20)*2+COUNTIF(Tatjes!C:C,J20)</f>

</xml_diff>

<commit_message>
Sync from vault 2026-06-06 14:47:36
</commit_message>
<xml_diff>
--- a/content/Archief/0. PDFs & docs/Obol docs & forms/Irmijn Inc/Irma backup log.xlsx
+++ b/content/Archief/0. PDFs & docs/Obol docs & forms/Irmijn Inc/Irma backup log.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="3"/>
   </bookViews>
   <sheets>
     <sheet name="Logboek" sheetId="1" state="visible" r:id="rId2"/>
@@ -15,13 +15,14 @@
   </sheets>
   <definedNames>
     <definedName function="false" hidden="true" localSheetId="3" name="_xlnm._FilterDatabase" vbProcedure="false">Tatdata!$A$1:$B$14</definedName>
-    <definedName function="false" hidden="true" localSheetId="2" name="_xlnm._FilterDatabase" vbProcedure="false">Tatjes!$A$1:$F$95</definedName>
-    <definedName function="false" hidden="false" localSheetId="2" name="_xlnm._FilterDatabase" vbProcedure="false">Tatjes!$A$1:$F$1</definedName>
+    <definedName function="false" hidden="true" localSheetId="2" name="_xlnm._FilterDatabase" vbProcedure="false">Tatjes!$A$1:$F$97</definedName>
+    <definedName function="false" hidden="false" localSheetId="2" name="_xlnm._FilterDatabase" vbProcedure="false">Tatjes!$A$1:$F$95</definedName>
     <definedName function="false" hidden="false" localSheetId="2" name="_xlnm._FilterDatabase_0" vbProcedure="false">Tatjes!$A$1:$F$1</definedName>
     <definedName function="false" hidden="false" localSheetId="2" name="_xlnm._FilterDatabase_0_0" vbProcedure="false">Tatjes!$A$1:$F$1</definedName>
     <definedName function="false" hidden="false" localSheetId="2" name="_xlnm._FilterDatabase_0_0_0" vbProcedure="false">Tatjes!$A$1:$F$1</definedName>
     <definedName function="false" hidden="false" localSheetId="2" name="_xlnm._FilterDatabase_0_0_0_0" vbProcedure="false">Tatjes!$A$1:$F$1</definedName>
     <definedName function="false" hidden="false" localSheetId="2" name="_xlnm._FilterDatabase_0_0_0_0_0" vbProcedure="false">Tatjes!$A$1:$F$1</definedName>
+    <definedName function="false" hidden="false" localSheetId="2" name="_xlnm._FilterDatabase_0_0_0_0_0_0" vbProcedure="false">Tatjes!$A$1:$F$1</definedName>
     <definedName function="false" hidden="false" localSheetId="3" name="_xlnm._FilterDatabase_0" vbProcedure="false">Tatdata!$A$1:$B$13</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.001"/>
@@ -34,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="502" uniqueCount="102">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="506" uniqueCount="102">
   <si>
     <t xml:space="preserve">Pagina</t>
   </si>
@@ -252,22 +253,22 @@
     <t xml:space="preserve">Bloem</t>
   </si>
   <si>
-    <t xml:space="preserve">Zilver</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Paars</t>
-  </si>
-  <si>
     <t xml:space="preserve">Marine</t>
   </si>
   <si>
     <t xml:space="preserve">Blauw</t>
   </si>
   <si>
+    <t xml:space="preserve">Fuchsia</t>
+  </si>
+  <si>
     <t xml:space="preserve">Geel</t>
   </si>
   <si>
-    <t xml:space="preserve">Aqua</t>
+    <t xml:space="preserve">Roze</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Oranje</t>
   </si>
   <si>
     <t xml:space="preserve">Lila</t>
@@ -276,25 +277,25 @@
     <t xml:space="preserve">Lichtgeel</t>
   </si>
   <si>
-    <t xml:space="preserve">Roze</t>
+    <t xml:space="preserve">Paars</t>
   </si>
   <si>
     <t xml:space="preserve">Zwart</t>
   </si>
   <si>
-    <t xml:space="preserve">Fuchsia</t>
+    <t xml:space="preserve">Zilver</t>
   </si>
   <si>
-    <t xml:space="preserve">Oranje</t>
+    <t xml:space="preserve">Aqua</t>
   </si>
   <si>
-    <t xml:space="preserve">Gras</t>
+    <t xml:space="preserve">Wit</t>
   </si>
   <si>
     <t xml:space="preserve">Groen</t>
   </si>
   <si>
-    <t xml:space="preserve">Wit</t>
+    <t xml:space="preserve">Gras</t>
   </si>
   <si>
     <t xml:space="preserve">Klaver4</t>
@@ -318,6 +319,9 @@
     <t xml:space="preserve">Klaver3</t>
   </si>
   <si>
+    <t xml:space="preserve">Grijs</t>
+  </si>
+  <si>
     <t xml:space="preserve">Lieveheer</t>
   </si>
   <si>
@@ -328,9 +332,6 @@
   </si>
   <si>
     <t xml:space="preserve">Bruin</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Grijs</t>
   </si>
   <si>
     <t xml:space="preserve">Molentje</t>
@@ -424,18 +425,6 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFDDDDDD"/>
-        <bgColor rgb="FFFFCCCC"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF800080"/>
-        <bgColor rgb="FF800080"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="FF2A6099"/>
         <bgColor rgb="FF004586"/>
       </patternFill>
@@ -448,8 +437,14 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF9BE2F6"/>
-        <bgColor rgb="FFCCFFFF"/>
+        <fgColor rgb="FFFF56F8"/>
+        <bgColor rgb="FFFF00FF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFBF00"/>
+        <bgColor rgb="FFFF9900"/>
       </patternFill>
     </fill>
     <fill>
@@ -466,26 +461,32 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="FF800080"/>
+        <bgColor rgb="FF800080"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="FF000000"/>
         <bgColor rgb="FF003300"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFF56F8"/>
-        <bgColor rgb="FFFF00FF"/>
+        <fgColor rgb="FFDDDDDD"/>
+        <bgColor rgb="FFFFCCCC"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFBF00"/>
-        <bgColor rgb="FFFF9900"/>
+        <fgColor rgb="FF9BE2F6"/>
+        <bgColor rgb="FFCCFFFF"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFBBE33D"/>
-        <bgColor rgb="FFACB20C"/>
+        <fgColor rgb="FFFFFFFF"/>
+        <bgColor rgb="FFFFFFD7"/>
       </patternFill>
     </fill>
     <fill>
@@ -496,8 +497,8 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFFF"/>
-        <bgColor rgb="FFFFFFD7"/>
+        <fgColor rgb="FFBBE33D"/>
+        <bgColor rgb="FFACB20C"/>
       </patternFill>
     </fill>
     <fill>
@@ -520,14 +521,14 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF813709"/>
-        <bgColor rgb="FF993366"/>
+        <fgColor rgb="FF808080"/>
+        <bgColor rgb="FF969696"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF808080"/>
-        <bgColor rgb="FF969696"/>
+        <fgColor rgb="FF813709"/>
+        <bgColor rgb="FF993366"/>
       </patternFill>
     </fill>
   </fills>
@@ -610,15 +611,15 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -634,7 +635,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="10" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="10" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1604,11 +1605,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="94588878"/>
-        <c:axId val="27235251"/>
+        <c:axId val="35948083"/>
+        <c:axId val="22270167"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="94588878"/>
+        <c:axId val="35948083"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1664,14 +1665,14 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="27235251"/>
+        <c:crossAx val="22270167"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
         <c:lblOffset val="100"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="27235251"/>
+        <c:axId val="22270167"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1736,7 +1737,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="94588878"/>
+        <c:crossAx val="35948083"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -4797,11 +4798,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="92545215"/>
-        <c:axId val="22253438"/>
+        <c:axId val="55703045"/>
+        <c:axId val="19932584"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="92545215"/>
+        <c:axId val="55703045"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -4857,14 +4858,14 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="22253438"/>
+        <c:crossAx val="19932584"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
         <c:lblOffset val="100"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="22253438"/>
+        <c:axId val="19932584"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -4929,7 +4930,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="92545215"/>
+        <c:crossAx val="55703045"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -5017,10 +5018,10 @@
           <c:layoutTarget val="inner"/>
           <c:xMode val="edge"/>
           <c:yMode val="edge"/>
-          <c:x val="0.0889764271868943"/>
-          <c:y val="0.110975202935617"/>
-          <c:w val="0.845870068154818"/>
-          <c:h val="0.793172467474702"/>
+          <c:x val="0.0889819909954977"/>
+          <c:y val="0.110987544483986"/>
+          <c:w val="0.845797898949475"/>
+          <c:h val="0.793038256227758"/>
         </c:manualLayout>
       </c:layout>
       <c:lineChart>
@@ -5152,11 +5153,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="78238978"/>
-        <c:axId val="93720606"/>
+        <c:axId val="12659909"/>
+        <c:axId val="36983749"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="78238978"/>
+        <c:axId val="12659909"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -5184,14 +5185,14 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="93720606"/>
+        <c:crossAx val="36983749"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
         <c:lblOffset val="100"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="93720606"/>
+        <c:axId val="36983749"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -5256,7 +5257,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="78238978"/>
+        <c:crossAx val="12659909"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -5294,9 +5295,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>178200</xdr:colOff>
+      <xdr:colOff>177840</xdr:colOff>
       <xdr:row>23</xdr:row>
-      <xdr:rowOff>41760</xdr:rowOff>
+      <xdr:rowOff>41400</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -5305,7 +5306,7 @@
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
         <a:off x="6578280" y="543600"/>
-        <a:ext cx="5756760" cy="3236760"/>
+        <a:ext cx="5756400" cy="3236400"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -5324,9 +5325,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>342000</xdr:colOff>
+      <xdr:colOff>341640</xdr:colOff>
       <xdr:row>52</xdr:row>
-      <xdr:rowOff>90000</xdr:rowOff>
+      <xdr:rowOff>89640</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -5335,7 +5336,7 @@
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
         <a:off x="6741360" y="5305320"/>
-        <a:ext cx="5757480" cy="3237480"/>
+        <a:ext cx="5757120" cy="3237120"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -5359,9 +5360,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>12</xdr:col>
-      <xdr:colOff>461520</xdr:colOff>
+      <xdr:colOff>461160</xdr:colOff>
       <xdr:row>21</xdr:row>
-      <xdr:rowOff>70200</xdr:rowOff>
+      <xdr:rowOff>69840</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -5370,7 +5371,7 @@
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
         <a:off x="2646720" y="246600"/>
-        <a:ext cx="5757120" cy="3237120"/>
+        <a:ext cx="5756760" cy="3236760"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -10484,7 +10485,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F95"/>
+  <dimension ref="A1:F97"/>
   <sheetFormatPr defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="9.63"/>
@@ -10530,11 +10531,11 @@
       </c>
       <c r="E2" s="0" t="n">
         <f aca="false">IF(ISBLANK(B2),"",COUNTIF(B:B,B2))</f>
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="F2" s="0" t="n">
         <f aca="false">IF(ISBLANK(C2),"",COUNTIF(C:C,C2))</f>
-        <v>8</v>
+        <v>4</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10553,22 +10554,22 @@
       </c>
       <c r="E3" s="0" t="n">
         <f aca="false">IF(ISBLANK(B3),"",COUNTIF(B:B,B3))</f>
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="F3" s="0" t="n">
         <f aca="false">IF(ISBLANK(C3),"",COUNTIF(C:C,C3))</f>
-        <v>8</v>
+        <v>4</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="10" t="s">
         <v>71</v>
       </c>
-      <c r="B4" s="11" t="s">
-        <v>72</v>
-      </c>
-      <c r="C4" s="13" t="s">
+      <c r="B4" s="13" t="s">
         <v>74</v>
+      </c>
+      <c r="C4" s="8" t="s">
+        <v>75</v>
       </c>
       <c r="D4" s="0" t="n">
         <f aca="false">IF(ISBLANK(A4),"",COUNTIF(A:A,A4))</f>
@@ -10576,21 +10577,21 @@
       </c>
       <c r="E4" s="0" t="n">
         <f aca="false">IF(ISBLANK(B4),"",COUNTIF(B:B,B4))</f>
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="F4" s="0" t="n">
         <f aca="false">IF(ISBLANK(C4),"",COUNTIF(C:C,C4))</f>
-        <v>5</v>
+        <v>18</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="10" t="s">
         <v>71</v>
       </c>
-      <c r="B5" s="14" t="s">
-        <v>75</v>
-      </c>
-      <c r="C5" s="8" t="s">
+      <c r="B5" s="13" t="s">
+        <v>74</v>
+      </c>
+      <c r="C5" s="10" t="s">
         <v>76</v>
       </c>
       <c r="D5" s="0" t="n">
@@ -10599,11 +10600,11 @@
       </c>
       <c r="E5" s="0" t="n">
         <f aca="false">IF(ISBLANK(B5),"",COUNTIF(B:B,B5))</f>
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="F5" s="0" t="n">
         <f aca="false">IF(ISBLANK(C5),"",COUNTIF(C:C,C5))</f>
-        <v>18</v>
+        <v>4</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10611,10 +10612,10 @@
         <v>71</v>
       </c>
       <c r="B6" s="14" t="s">
+        <v>77</v>
+      </c>
+      <c r="C6" s="8" t="s">
         <v>75</v>
-      </c>
-      <c r="C6" s="15" t="s">
-        <v>77</v>
       </c>
       <c r="D6" s="0" t="n">
         <f aca="false">IF(ISBLANK(A6),"",COUNTIF(A:A,A6))</f>
@@ -10622,11 +10623,11 @@
       </c>
       <c r="E6" s="0" t="n">
         <f aca="false">IF(ISBLANK(B6),"",COUNTIF(B:B,B6))</f>
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="F6" s="0" t="n">
         <f aca="false">IF(ISBLANK(C6),"",COUNTIF(C:C,C6))</f>
-        <v>11</v>
+        <v>18</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10634,10 +10635,10 @@
         <v>71</v>
       </c>
       <c r="B7" s="14" t="s">
+        <v>77</v>
+      </c>
+      <c r="C7" s="8" t="s">
         <v>75</v>
-      </c>
-      <c r="C7" s="13" t="s">
-        <v>74</v>
       </c>
       <c r="D7" s="0" t="n">
         <f aca="false">IF(ISBLANK(A7),"",COUNTIF(A:A,A7))</f>
@@ -10645,21 +10646,21 @@
       </c>
       <c r="E7" s="0" t="n">
         <f aca="false">IF(ISBLANK(B7),"",COUNTIF(B:B,B7))</f>
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="F7" s="0" t="n">
         <f aca="false">IF(ISBLANK(C7),"",COUNTIF(C:C,C7))</f>
-        <v>5</v>
+        <v>18</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="10" t="s">
         <v>71</v>
       </c>
-      <c r="B8" s="16" t="s">
+      <c r="B8" s="15" t="s">
         <v>78</v>
       </c>
-      <c r="C8" s="17" t="s">
+      <c r="C8" s="16" t="s">
         <v>79</v>
       </c>
       <c r="D8" s="0" t="n">
@@ -10679,11 +10680,11 @@
       <c r="A9" s="10" t="s">
         <v>71</v>
       </c>
-      <c r="B9" s="16" t="s">
+      <c r="B9" s="15" t="s">
         <v>78</v>
       </c>
       <c r="C9" s="10" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="D9" s="0" t="n">
         <f aca="false">IF(ISBLANK(A9),"",COUNTIF(A:A,A9))</f>
@@ -10702,11 +10703,11 @@
       <c r="A10" s="10" t="s">
         <v>71</v>
       </c>
-      <c r="B10" s="12" t="s">
-        <v>73</v>
+      <c r="B10" s="17" t="s">
+        <v>80</v>
       </c>
       <c r="C10" s="10" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="D10" s="0" t="n">
         <f aca="false">IF(ISBLANK(A10),"",COUNTIF(A:A,A10))</f>
@@ -10728,8 +10729,8 @@
       <c r="B11" s="18" t="s">
         <v>81</v>
       </c>
-      <c r="C11" s="11" t="s">
-        <v>72</v>
+      <c r="C11" s="19" t="s">
+        <v>82</v>
       </c>
       <c r="D11" s="0" t="n">
         <f aca="false">IF(ISBLANK(A11),"",COUNTIF(A:A,A11))</f>
@@ -10748,11 +10749,11 @@
       <c r="A12" s="10" t="s">
         <v>71</v>
       </c>
-      <c r="B12" s="19" t="s">
-        <v>82</v>
+      <c r="B12" s="12" t="s">
+        <v>73</v>
       </c>
       <c r="C12" s="8" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D12" s="0" t="n">
         <f aca="false">IF(ISBLANK(A12),"",COUNTIF(A:A,A12))</f>
@@ -10760,7 +10761,7 @@
       </c>
       <c r="E12" s="0" t="n">
         <f aca="false">IF(ISBLANK(B12),"",COUNTIF(B:B,B12))</f>
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="F12" s="0" t="n">
         <f aca="false">IF(ISBLANK(C12),"",COUNTIF(C:C,C12))</f>
@@ -10771,11 +10772,11 @@
       <c r="A13" s="10" t="s">
         <v>71</v>
       </c>
-      <c r="B13" s="19" t="s">
-        <v>82</v>
-      </c>
-      <c r="C13" s="10" t="s">
-        <v>80</v>
+      <c r="B13" s="12" t="s">
+        <v>73</v>
+      </c>
+      <c r="C13" s="20" t="s">
+        <v>83</v>
       </c>
       <c r="D13" s="0" t="n">
         <f aca="false">IF(ISBLANK(A13),"",COUNTIF(A:A,A13))</f>
@@ -10783,22 +10784,22 @@
       </c>
       <c r="E13" s="0" t="n">
         <f aca="false">IF(ISBLANK(B13),"",COUNTIF(B:B,B13))</f>
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="F13" s="0" t="n">
         <f aca="false">IF(ISBLANK(C13),"",COUNTIF(C:C,C13))</f>
-        <v>4</v>
+        <v>11</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="10" t="s">
         <v>71</v>
       </c>
-      <c r="B14" s="20" t="s">
-        <v>83</v>
-      </c>
-      <c r="C14" s="8" t="s">
-        <v>76</v>
+      <c r="B14" s="12" t="s">
+        <v>73</v>
+      </c>
+      <c r="C14" s="11" t="s">
+        <v>72</v>
       </c>
       <c r="D14" s="0" t="n">
         <f aca="false">IF(ISBLANK(A14),"",COUNTIF(A:A,A14))</f>
@@ -10806,22 +10807,22 @@
       </c>
       <c r="E14" s="0" t="n">
         <f aca="false">IF(ISBLANK(B14),"",COUNTIF(B:B,B14))</f>
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="F14" s="0" t="n">
         <f aca="false">IF(ISBLANK(C14),"",COUNTIF(C:C,C14))</f>
-        <v>18</v>
+        <v>5</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="10" t="s">
         <v>71</v>
       </c>
-      <c r="B15" s="20" t="s">
-        <v>83</v>
-      </c>
-      <c r="C15" s="8" t="s">
-        <v>76</v>
+      <c r="B15" s="19" t="s">
+        <v>82</v>
+      </c>
+      <c r="C15" s="17" t="s">
+        <v>80</v>
       </c>
       <c r="D15" s="0" t="n">
         <f aca="false">IF(ISBLANK(A15),"",COUNTIF(A:A,A15))</f>
@@ -10829,22 +10830,22 @@
       </c>
       <c r="E15" s="0" t="n">
         <f aca="false">IF(ISBLANK(B15),"",COUNTIF(B:B,B15))</f>
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="F15" s="0" t="n">
         <f aca="false">IF(ISBLANK(C15),"",COUNTIF(C:C,C15))</f>
-        <v>18</v>
+        <v>8</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="10" t="s">
         <v>71</v>
       </c>
-      <c r="B16" s="13" t="s">
-        <v>74</v>
-      </c>
-      <c r="C16" s="14" t="s">
-        <v>75</v>
+      <c r="B16" s="19" t="s">
+        <v>82</v>
+      </c>
+      <c r="C16" s="17" t="s">
+        <v>80</v>
       </c>
       <c r="D16" s="0" t="n">
         <f aca="false">IF(ISBLANK(A16),"",COUNTIF(A:A,A16))</f>
@@ -10852,22 +10853,22 @@
       </c>
       <c r="E16" s="0" t="n">
         <f aca="false">IF(ISBLANK(B16),"",COUNTIF(B:B,B16))</f>
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="F16" s="0" t="n">
         <f aca="false">IF(ISBLANK(C16),"",COUNTIF(C:C,C16))</f>
-        <v>4</v>
+        <v>8</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="10" t="s">
         <v>71</v>
       </c>
-      <c r="B17" s="13" t="s">
-        <v>74</v>
-      </c>
-      <c r="C17" s="14" t="s">
-        <v>75</v>
+      <c r="B17" s="19" t="s">
+        <v>82</v>
+      </c>
+      <c r="C17" s="11" t="s">
+        <v>72</v>
       </c>
       <c r="D17" s="0" t="n">
         <f aca="false">IF(ISBLANK(A17),"",COUNTIF(A:A,A17))</f>
@@ -10875,22 +10876,22 @@
       </c>
       <c r="E17" s="0" t="n">
         <f aca="false">IF(ISBLANK(B17),"",COUNTIF(B:B,B17))</f>
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="F17" s="0" t="n">
         <f aca="false">IF(ISBLANK(C17),"",COUNTIF(C:C,C17))</f>
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="14" t="s">
+      <c r="A18" s="12" t="s">
         <v>33</v>
       </c>
-      <c r="B18" s="21" t="s">
-        <v>84</v>
-      </c>
-      <c r="C18" s="8" t="s">
-        <v>76</v>
+      <c r="B18" s="20" t="s">
+        <v>83</v>
+      </c>
+      <c r="C18" s="16" t="s">
+        <v>79</v>
       </c>
       <c r="D18" s="0" t="n">
         <f aca="false">IF(ISBLANK(A18),"",COUNTIF(A:A,A18))</f>
@@ -10898,22 +10899,22 @@
       </c>
       <c r="E18" s="0" t="n">
         <f aca="false">IF(ISBLANK(B18),"",COUNTIF(B:B,B18))</f>
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="F18" s="0" t="n">
         <f aca="false">IF(ISBLANK(C18),"",COUNTIF(C:C,C18))</f>
-        <v>18</v>
+        <v>6</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="14" t="s">
+      <c r="A19" s="12" t="s">
         <v>33</v>
       </c>
-      <c r="B19" s="21" t="s">
-        <v>84</v>
-      </c>
-      <c r="C19" s="15" t="s">
+      <c r="B19" s="14" t="s">
         <v>77</v>
+      </c>
+      <c r="C19" s="8" t="s">
+        <v>75</v>
       </c>
       <c r="D19" s="0" t="n">
         <f aca="false">IF(ISBLANK(A19),"",COUNTIF(A:A,A19))</f>
@@ -10921,22 +10922,22 @@
       </c>
       <c r="E19" s="0" t="n">
         <f aca="false">IF(ISBLANK(B19),"",COUNTIF(B:B,B19))</f>
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="F19" s="0" t="n">
         <f aca="false">IF(ISBLANK(C19),"",COUNTIF(C:C,C19))</f>
-        <v>11</v>
+        <v>18</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="14" t="s">
+      <c r="A20" s="12" t="s">
         <v>33</v>
       </c>
-      <c r="B20" s="21" t="s">
-        <v>84</v>
-      </c>
-      <c r="C20" s="17" t="s">
-        <v>79</v>
+      <c r="B20" s="15" t="s">
+        <v>78</v>
+      </c>
+      <c r="C20" s="20" t="s">
+        <v>83</v>
       </c>
       <c r="D20" s="0" t="n">
         <f aca="false">IF(ISBLANK(A20),"",COUNTIF(A:A,A20))</f>
@@ -10944,22 +10945,22 @@
       </c>
       <c r="E20" s="0" t="n">
         <f aca="false">IF(ISBLANK(B20),"",COUNTIF(B:B,B20))</f>
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="F20" s="0" t="n">
         <f aca="false">IF(ISBLANK(C20),"",COUNTIF(C:C,C20))</f>
-        <v>6</v>
+        <v>11</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="14" t="s">
+      <c r="A21" s="12" t="s">
         <v>33</v>
       </c>
-      <c r="B21" s="8" t="s">
-        <v>76</v>
-      </c>
-      <c r="C21" s="17" t="s">
-        <v>79</v>
+      <c r="B21" s="15" t="s">
+        <v>78</v>
+      </c>
+      <c r="C21" s="21" t="s">
+        <v>84</v>
       </c>
       <c r="D21" s="0" t="n">
         <f aca="false">IF(ISBLANK(A21),"",COUNTIF(A:A,A21))</f>
@@ -10967,22 +10968,22 @@
       </c>
       <c r="E21" s="0" t="n">
         <f aca="false">IF(ISBLANK(B21),"",COUNTIF(B:B,B21))</f>
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="F21" s="0" t="n">
         <f aca="false">IF(ISBLANK(C21),"",COUNTIF(C:C,C21))</f>
-        <v>6</v>
+        <v>1</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="14" t="s">
+      <c r="A22" s="12" t="s">
         <v>33</v>
       </c>
-      <c r="B22" s="14" t="s">
-        <v>75</v>
-      </c>
-      <c r="C22" s="15" t="s">
-        <v>77</v>
+      <c r="B22" s="17" t="s">
+        <v>80</v>
+      </c>
+      <c r="C22" s="19" t="s">
+        <v>82</v>
       </c>
       <c r="D22" s="0" t="n">
         <f aca="false">IF(ISBLANK(A22),"",COUNTIF(A:A,A22))</f>
@@ -10990,22 +10991,22 @@
       </c>
       <c r="E22" s="0" t="n">
         <f aca="false">IF(ISBLANK(B22),"",COUNTIF(B:B,B22))</f>
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F22" s="0" t="n">
         <f aca="false">IF(ISBLANK(C22),"",COUNTIF(C:C,C22))</f>
-        <v>11</v>
+        <v>3</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="14" t="s">
+      <c r="A23" s="12" t="s">
         <v>33</v>
       </c>
-      <c r="B23" s="14" t="s">
-        <v>75</v>
+      <c r="B23" s="17" t="s">
+        <v>80</v>
       </c>
       <c r="C23" s="15" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="D23" s="0" t="n">
         <f aca="false">IF(ISBLANK(A23),"",COUNTIF(A:A,A23))</f>
@@ -11013,22 +11014,22 @@
       </c>
       <c r="E23" s="0" t="n">
         <f aca="false">IF(ISBLANK(B23),"",COUNTIF(B:B,B23))</f>
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F23" s="0" t="n">
         <f aca="false">IF(ISBLANK(C23),"",COUNTIF(C:C,C23))</f>
-        <v>11</v>
+        <v>2</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="14" t="s">
+      <c r="A24" s="12" t="s">
         <v>33</v>
       </c>
-      <c r="B24" s="14" t="s">
-        <v>75</v>
-      </c>
-      <c r="C24" s="15" t="s">
-        <v>77</v>
+      <c r="B24" s="12" t="s">
+        <v>73</v>
+      </c>
+      <c r="C24" s="20" t="s">
+        <v>83</v>
       </c>
       <c r="D24" s="0" t="n">
         <f aca="false">IF(ISBLANK(A24),"",COUNTIF(A:A,A24))</f>
@@ -11044,14 +11045,14 @@
       </c>
     </row>
     <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="14" t="s">
+      <c r="A25" s="12" t="s">
         <v>33</v>
       </c>
-      <c r="B25" s="22" t="s">
-        <v>85</v>
-      </c>
-      <c r="C25" s="15" t="s">
-        <v>77</v>
+      <c r="B25" s="12" t="s">
+        <v>73</v>
+      </c>
+      <c r="C25" s="20" t="s">
+        <v>83</v>
       </c>
       <c r="D25" s="0" t="n">
         <f aca="false">IF(ISBLANK(A25),"",COUNTIF(A:A,A25))</f>
@@ -11067,14 +11068,14 @@
       </c>
     </row>
     <row r="26" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="14" t="s">
+      <c r="A26" s="12" t="s">
         <v>33</v>
       </c>
-      <c r="B26" s="22" t="s">
-        <v>85</v>
-      </c>
-      <c r="C26" s="14" t="s">
-        <v>75</v>
+      <c r="B26" s="12" t="s">
+        <v>73</v>
+      </c>
+      <c r="C26" s="20" t="s">
+        <v>83</v>
       </c>
       <c r="D26" s="0" t="n">
         <f aca="false">IF(ISBLANK(A26),"",COUNTIF(A:A,A26))</f>
@@ -11086,18 +11087,18 @@
       </c>
       <c r="F26" s="0" t="n">
         <f aca="false">IF(ISBLANK(C26),"",COUNTIF(C:C,C26))</f>
-        <v>4</v>
+        <v>11</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="14" t="s">
+      <c r="A27" s="12" t="s">
         <v>33</v>
       </c>
       <c r="B27" s="22" t="s">
         <v>85</v>
       </c>
-      <c r="C27" s="21" t="s">
-        <v>84</v>
+      <c r="C27" s="20" t="s">
+        <v>83</v>
       </c>
       <c r="D27" s="0" t="n">
         <f aca="false">IF(ISBLANK(A27),"",COUNTIF(A:A,A27))</f>
@@ -11109,18 +11110,18 @@
       </c>
       <c r="F27" s="0" t="n">
         <f aca="false">IF(ISBLANK(C27),"",COUNTIF(C:C,C27))</f>
-        <v>3</v>
+        <v>11</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="14" t="s">
+      <c r="A28" s="12" t="s">
         <v>33</v>
       </c>
-      <c r="B28" s="16" t="s">
-        <v>78</v>
-      </c>
-      <c r="C28" s="15" t="s">
-        <v>77</v>
+      <c r="B28" s="22" t="s">
+        <v>85</v>
+      </c>
+      <c r="C28" s="12" t="s">
+        <v>73</v>
       </c>
       <c r="D28" s="0" t="n">
         <f aca="false">IF(ISBLANK(A28),"",COUNTIF(A:A,A28))</f>
@@ -11128,19 +11129,19 @@
       </c>
       <c r="E28" s="0" t="n">
         <f aca="false">IF(ISBLANK(B28),"",COUNTIF(B:B,B28))</f>
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F28" s="0" t="n">
         <f aca="false">IF(ISBLANK(C28),"",COUNTIF(C:C,C28))</f>
-        <v>11</v>
+        <v>4</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="14" t="s">
+      <c r="A29" s="12" t="s">
         <v>33</v>
       </c>
-      <c r="B29" s="16" t="s">
-        <v>78</v>
+      <c r="B29" s="22" t="s">
+        <v>85</v>
       </c>
       <c r="C29" s="23" t="s">
         <v>86</v>
@@ -11151,22 +11152,22 @@
       </c>
       <c r="E29" s="0" t="n">
         <f aca="false">IF(ISBLANK(B29),"",COUNTIF(B:B,B29))</f>
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F29" s="0" t="n">
         <f aca="false">IF(ISBLANK(C29),"",COUNTIF(C:C,C29))</f>
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="14" t="s">
+      <c r="A30" s="12" t="s">
         <v>33</v>
       </c>
-      <c r="B30" s="12" t="s">
-        <v>73</v>
-      </c>
-      <c r="C30" s="11" t="s">
-        <v>72</v>
+      <c r="B30" s="8" t="s">
+        <v>75</v>
+      </c>
+      <c r="C30" s="16" t="s">
+        <v>79</v>
       </c>
       <c r="D30" s="0" t="n">
         <f aca="false">IF(ISBLANK(A30),"",COUNTIF(A:A,A30))</f>
@@ -11174,22 +11175,22 @@
       </c>
       <c r="E30" s="0" t="n">
         <f aca="false">IF(ISBLANK(B30),"",COUNTIF(B:B,B30))</f>
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="F30" s="0" t="n">
         <f aca="false">IF(ISBLANK(C30),"",COUNTIF(C:C,C30))</f>
-        <v>3</v>
+        <v>6</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="14" t="s">
+      <c r="A31" s="12" t="s">
         <v>33</v>
       </c>
-      <c r="B31" s="12" t="s">
-        <v>73</v>
-      </c>
-      <c r="C31" s="16" t="s">
-        <v>78</v>
+      <c r="B31" s="23" t="s">
+        <v>86</v>
+      </c>
+      <c r="C31" s="8" t="s">
+        <v>75</v>
       </c>
       <c r="D31" s="0" t="n">
         <f aca="false">IF(ISBLANK(A31),"",COUNTIF(A:A,A31))</f>
@@ -11197,22 +11198,22 @@
       </c>
       <c r="E31" s="0" t="n">
         <f aca="false">IF(ISBLANK(B31),"",COUNTIF(B:B,B31))</f>
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="F31" s="0" t="n">
         <f aca="false">IF(ISBLANK(C31),"",COUNTIF(C:C,C31))</f>
-        <v>2</v>
+        <v>18</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="14" t="s">
+      <c r="A32" s="12" t="s">
         <v>33</v>
       </c>
-      <c r="B32" s="20" t="s">
+      <c r="B32" s="23" t="s">
+        <v>86</v>
+      </c>
+      <c r="C32" s="20" t="s">
         <v>83</v>
-      </c>
-      <c r="C32" s="8" t="s">
-        <v>76</v>
       </c>
       <c r="D32" s="0" t="n">
         <f aca="false">IF(ISBLANK(A32),"",COUNTIF(A:A,A32))</f>
@@ -11220,21 +11221,21 @@
       </c>
       <c r="E32" s="0" t="n">
         <f aca="false">IF(ISBLANK(B32),"",COUNTIF(B:B,B32))</f>
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="F32" s="0" t="n">
         <f aca="false">IF(ISBLANK(C32),"",COUNTIF(C:C,C32))</f>
-        <v>18</v>
+        <v>11</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="14" t="s">
+      <c r="A33" s="12" t="s">
         <v>33</v>
       </c>
-      <c r="B33" s="15" t="s">
-        <v>77</v>
-      </c>
-      <c r="C33" s="17" t="s">
+      <c r="B33" s="23" t="s">
+        <v>86</v>
+      </c>
+      <c r="C33" s="16" t="s">
         <v>79</v>
       </c>
       <c r="D33" s="0" t="n">
@@ -11243,7 +11244,7 @@
       </c>
       <c r="E33" s="0" t="n">
         <f aca="false">IF(ISBLANK(B33),"",COUNTIF(B:B,B33))</f>
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="F33" s="0" t="n">
         <f aca="false">IF(ISBLANK(C33),"",COUNTIF(C:C,C33))</f>
@@ -11254,8 +11255,8 @@
       <c r="A34" s="22" t="s">
         <v>87</v>
       </c>
-      <c r="B34" s="21" t="s">
-        <v>84</v>
+      <c r="B34" s="24" t="s">
+        <v>88</v>
       </c>
       <c r="D34" s="0" t="n">
         <f aca="false">IF(ISBLANK(A34),"",COUNTIF(A:A,A34))</f>
@@ -11263,7 +11264,7 @@
       </c>
       <c r="E34" s="0" t="n">
         <f aca="false">IF(ISBLANK(B34),"",COUNTIF(B:B,B34))</f>
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="F34" s="0" t="str">
         <f aca="false">IF(ISBLANK(C34),"",COUNTIF(C:C,C34))</f>
@@ -11274,8 +11275,8 @@
       <c r="A35" s="22" t="s">
         <v>87</v>
       </c>
-      <c r="B35" s="21" t="s">
-        <v>84</v>
+      <c r="B35" s="24" t="s">
+        <v>88</v>
       </c>
       <c r="D35" s="0" t="n">
         <f aca="false">IF(ISBLANK(A35),"",COUNTIF(A:A,A35))</f>
@@ -11283,7 +11284,7 @@
       </c>
       <c r="E35" s="0" t="n">
         <f aca="false">IF(ISBLANK(B35),"",COUNTIF(B:B,B35))</f>
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="F35" s="0" t="str">
         <f aca="false">IF(ISBLANK(C35),"",COUNTIF(C:C,C35))</f>
@@ -11294,8 +11295,8 @@
       <c r="A36" s="22" t="s">
         <v>87</v>
       </c>
-      <c r="B36" s="8" t="s">
-        <v>76</v>
+      <c r="B36" s="16" t="s">
+        <v>79</v>
       </c>
       <c r="D36" s="0" t="n">
         <f aca="false">IF(ISBLANK(A36),"",COUNTIF(A:A,A36))</f>
@@ -11303,7 +11304,7 @@
       </c>
       <c r="E36" s="0" t="n">
         <f aca="false">IF(ISBLANK(B36),"",COUNTIF(B:B,B36))</f>
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="F36" s="0" t="str">
         <f aca="false">IF(ISBLANK(C36),"",COUNTIF(C:C,C36))</f>
@@ -11314,8 +11315,8 @@
       <c r="A37" s="22" t="s">
         <v>87</v>
       </c>
-      <c r="B37" s="8" t="s">
-        <v>76</v>
+      <c r="B37" s="16" t="s">
+        <v>79</v>
       </c>
       <c r="D37" s="0" t="n">
         <f aca="false">IF(ISBLANK(A37),"",COUNTIF(A:A,A37))</f>
@@ -11323,7 +11324,7 @@
       </c>
       <c r="E37" s="0" t="n">
         <f aca="false">IF(ISBLANK(B37),"",COUNTIF(B:B,B37))</f>
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="F37" s="0" t="str">
         <f aca="false">IF(ISBLANK(C37),"",COUNTIF(C:C,C37))</f>
@@ -11334,8 +11335,8 @@
       <c r="A38" s="22" t="s">
         <v>87</v>
       </c>
-      <c r="B38" s="8" t="s">
-        <v>76</v>
+      <c r="B38" s="16" t="s">
+        <v>79</v>
       </c>
       <c r="D38" s="0" t="n">
         <f aca="false">IF(ISBLANK(A38),"",COUNTIF(A:A,A38))</f>
@@ -11343,7 +11344,7 @@
       </c>
       <c r="E38" s="0" t="n">
         <f aca="false">IF(ISBLANK(B38),"",COUNTIF(B:B,B38))</f>
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="F38" s="0" t="str">
         <f aca="false">IF(ISBLANK(C38),"",COUNTIF(C:C,C38))</f>
@@ -11354,8 +11355,8 @@
       <c r="A39" s="22" t="s">
         <v>87</v>
       </c>
-      <c r="B39" s="8" t="s">
-        <v>76</v>
+      <c r="B39" s="22" t="s">
+        <v>85</v>
       </c>
       <c r="D39" s="0" t="n">
         <f aca="false">IF(ISBLANK(A39),"",COUNTIF(A:A,A39))</f>
@@ -11363,7 +11364,7 @@
       </c>
       <c r="E39" s="0" t="n">
         <f aca="false">IF(ISBLANK(B39),"",COUNTIF(B:B,B39))</f>
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F39" s="0" t="str">
         <f aca="false">IF(ISBLANK(C39),"",COUNTIF(C:C,C39))</f>
@@ -11374,8 +11375,8 @@
       <c r="A40" s="22" t="s">
         <v>87</v>
       </c>
-      <c r="B40" s="22" t="s">
-        <v>85</v>
+      <c r="B40" s="8" t="s">
+        <v>75</v>
       </c>
       <c r="D40" s="0" t="n">
         <f aca="false">IF(ISBLANK(A40),"",COUNTIF(A:A,A40))</f>
@@ -11383,7 +11384,7 @@
       </c>
       <c r="E40" s="0" t="n">
         <f aca="false">IF(ISBLANK(B40),"",COUNTIF(B:B,B40))</f>
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="F40" s="0" t="str">
         <f aca="false">IF(ISBLANK(C40),"",COUNTIF(C:C,C40))</f>
@@ -11394,8 +11395,8 @@
       <c r="A41" s="22" t="s">
         <v>87</v>
       </c>
-      <c r="B41" s="17" t="s">
-        <v>79</v>
+      <c r="B41" s="8" t="s">
+        <v>75</v>
       </c>
       <c r="D41" s="0" t="n">
         <f aca="false">IF(ISBLANK(A41),"",COUNTIF(A:A,A41))</f>
@@ -11403,7 +11404,7 @@
       </c>
       <c r="E41" s="0" t="n">
         <f aca="false">IF(ISBLANK(B41),"",COUNTIF(B:B,B41))</f>
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="F41" s="0" t="str">
         <f aca="false">IF(ISBLANK(C41),"",COUNTIF(C:C,C41))</f>
@@ -11414,8 +11415,8 @@
       <c r="A42" s="22" t="s">
         <v>87</v>
       </c>
-      <c r="B42" s="17" t="s">
-        <v>79</v>
+      <c r="B42" s="8" t="s">
+        <v>75</v>
       </c>
       <c r="D42" s="0" t="n">
         <f aca="false">IF(ISBLANK(A42),"",COUNTIF(A:A,A42))</f>
@@ -11423,7 +11424,7 @@
       </c>
       <c r="E42" s="0" t="n">
         <f aca="false">IF(ISBLANK(B42),"",COUNTIF(B:B,B42))</f>
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="F42" s="0" t="str">
         <f aca="false">IF(ISBLANK(C42),"",COUNTIF(C:C,C42))</f>
@@ -11434,8 +11435,8 @@
       <c r="A43" s="22" t="s">
         <v>87</v>
       </c>
-      <c r="B43" s="17" t="s">
-        <v>79</v>
+      <c r="B43" s="8" t="s">
+        <v>75</v>
       </c>
       <c r="D43" s="0" t="n">
         <f aca="false">IF(ISBLANK(A43),"",COUNTIF(A:A,A43))</f>
@@ -11443,7 +11444,7 @@
       </c>
       <c r="E43" s="0" t="n">
         <f aca="false">IF(ISBLANK(B43),"",COUNTIF(B:B,B43))</f>
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="F43" s="0" t="str">
         <f aca="false">IF(ISBLANK(C43),"",COUNTIF(C:C,C43))</f>
@@ -11454,8 +11455,8 @@
       <c r="A44" s="22" t="s">
         <v>87</v>
       </c>
-      <c r="B44" s="24" t="s">
-        <v>88</v>
+      <c r="B44" s="23" t="s">
+        <v>86</v>
       </c>
       <c r="D44" s="0" t="n">
         <f aca="false">IF(ISBLANK(A44),"",COUNTIF(A:A,A44))</f>
@@ -11463,7 +11464,7 @@
       </c>
       <c r="E44" s="0" t="n">
         <f aca="false">IF(ISBLANK(B44),"",COUNTIF(B:B,B44))</f>
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="F44" s="0" t="str">
         <f aca="false">IF(ISBLANK(C44),"",COUNTIF(C:C,C44))</f>
@@ -11474,8 +11475,8 @@
       <c r="A45" s="22" t="s">
         <v>87</v>
       </c>
-      <c r="B45" s="24" t="s">
-        <v>88</v>
+      <c r="B45" s="23" t="s">
+        <v>86</v>
       </c>
       <c r="D45" s="0" t="n">
         <f aca="false">IF(ISBLANK(A45),"",COUNTIF(A:A,A45))</f>
@@ -11483,7 +11484,7 @@
       </c>
       <c r="E45" s="0" t="n">
         <f aca="false">IF(ISBLANK(B45),"",COUNTIF(B:B,B45))</f>
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="F45" s="0" t="str">
         <f aca="false">IF(ISBLANK(C45),"",COUNTIF(C:C,C45))</f>
@@ -11491,14 +11492,14 @@
       </c>
     </row>
     <row r="46" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A46" s="20" t="s">
+      <c r="A46" s="14" t="s">
         <v>19</v>
       </c>
-      <c r="B46" s="21" t="s">
-        <v>84</v>
-      </c>
-      <c r="C46" s="13" t="s">
-        <v>74</v>
+      <c r="B46" s="18" t="s">
+        <v>43</v>
+      </c>
+      <c r="C46" s="23" t="s">
+        <v>86</v>
       </c>
       <c r="D46" s="0" t="n">
         <f aca="false">IF(ISBLANK(A46),"",COUNTIF(A:A,A46))</f>
@@ -11506,22 +11507,22 @@
       </c>
       <c r="E46" s="0" t="n">
         <f aca="false">IF(ISBLANK(B46),"",COUNTIF(B:B,B46))</f>
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="F46" s="0" t="n">
         <f aca="false">IF(ISBLANK(C46),"",COUNTIF(C:C,C46))</f>
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A47" s="20" t="s">
+      <c r="A47" s="14" t="s">
         <v>19</v>
       </c>
-      <c r="B47" s="21" t="s">
-        <v>84</v>
-      </c>
-      <c r="C47" s="13" t="s">
-        <v>74</v>
+      <c r="B47" s="25" t="s">
+        <v>89</v>
+      </c>
+      <c r="C47" s="8" t="s">
+        <v>75</v>
       </c>
       <c r="D47" s="0" t="n">
         <f aca="false">IF(ISBLANK(A47),"",COUNTIF(A:A,A47))</f>
@@ -11529,19 +11530,19 @@
       </c>
       <c r="E47" s="0" t="n">
         <f aca="false">IF(ISBLANK(B47),"",COUNTIF(B:B,B47))</f>
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="F47" s="0" t="n">
         <f aca="false">IF(ISBLANK(C47),"",COUNTIF(C:C,C47))</f>
-        <v>5</v>
+        <v>18</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A48" s="20" t="s">
+      <c r="A48" s="14" t="s">
         <v>19</v>
       </c>
-      <c r="B48" s="8" t="s">
-        <v>76</v>
+      <c r="B48" s="11" t="s">
+        <v>72</v>
       </c>
       <c r="C48" s="20" t="s">
         <v>83</v>
@@ -11552,22 +11553,22 @@
       </c>
       <c r="E48" s="0" t="n">
         <f aca="false">IF(ISBLANK(B48),"",COUNTIF(B:B,B48))</f>
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="F48" s="0" t="n">
         <f aca="false">IF(ISBLANK(C48),"",COUNTIF(C:C,C48))</f>
-        <v>1</v>
+        <v>11</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A49" s="20" t="s">
+      <c r="A49" s="14" t="s">
         <v>19</v>
       </c>
       <c r="B49" s="14" t="s">
+        <v>77</v>
+      </c>
+      <c r="C49" s="8" t="s">
         <v>75</v>
-      </c>
-      <c r="C49" s="15" t="s">
-        <v>77</v>
       </c>
       <c r="D49" s="0" t="n">
         <f aca="false">IF(ISBLANK(A49),"",COUNTIF(A:A,A49))</f>
@@ -11575,22 +11576,22 @@
       </c>
       <c r="E49" s="0" t="n">
         <f aca="false">IF(ISBLANK(B49),"",COUNTIF(B:B,B49))</f>
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="F49" s="0" t="n">
         <f aca="false">IF(ISBLANK(C49),"",COUNTIF(C:C,C49))</f>
-        <v>11</v>
+        <v>18</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A50" s="20" t="s">
+      <c r="A50" s="14" t="s">
         <v>19</v>
       </c>
-      <c r="B50" s="16" t="s">
+      <c r="B50" s="15" t="s">
         <v>78</v>
       </c>
-      <c r="C50" s="15" t="s">
-        <v>77</v>
+      <c r="C50" s="20" t="s">
+        <v>83</v>
       </c>
       <c r="D50" s="0" t="n">
         <f aca="false">IF(ISBLANK(A50),"",COUNTIF(A:A,A50))</f>
@@ -11606,14 +11607,14 @@
       </c>
     </row>
     <row r="51" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A51" s="20" t="s">
+      <c r="A51" s="14" t="s">
         <v>19</v>
       </c>
-      <c r="B51" s="16" t="s">
+      <c r="B51" s="15" t="s">
         <v>78</v>
       </c>
-      <c r="C51" s="12" t="s">
-        <v>73</v>
+      <c r="C51" s="17" t="s">
+        <v>80</v>
       </c>
       <c r="D51" s="0" t="n">
         <f aca="false">IF(ISBLANK(A51),"",COUNTIF(A:A,A51))</f>
@@ -11629,14 +11630,14 @@
       </c>
     </row>
     <row r="52" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A52" s="20" t="s">
+      <c r="A52" s="14" t="s">
         <v>19</v>
       </c>
-      <c r="B52" s="12" t="s">
-        <v>73</v>
-      </c>
-      <c r="C52" s="19" t="s">
-        <v>82</v>
+      <c r="B52" s="17" t="s">
+        <v>80</v>
+      </c>
+      <c r="C52" s="13" t="s">
+        <v>74</v>
       </c>
       <c r="D52" s="0" t="n">
         <f aca="false">IF(ISBLANK(A52),"",COUNTIF(A:A,A52))</f>
@@ -11652,14 +11653,14 @@
       </c>
     </row>
     <row r="53" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A53" s="20" t="s">
+      <c r="A53" s="14" t="s">
         <v>19</v>
       </c>
-      <c r="B53" s="20" t="s">
+      <c r="B53" s="12" t="s">
+        <v>73</v>
+      </c>
+      <c r="C53" s="20" t="s">
         <v>83</v>
-      </c>
-      <c r="C53" s="8" t="s">
-        <v>76</v>
       </c>
       <c r="D53" s="0" t="n">
         <f aca="false">IF(ISBLANK(A53),"",COUNTIF(A:A,A53))</f>
@@ -11667,21 +11668,21 @@
       </c>
       <c r="E53" s="0" t="n">
         <f aca="false">IF(ISBLANK(B53),"",COUNTIF(B:B,B53))</f>
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="F53" s="0" t="n">
         <f aca="false">IF(ISBLANK(C53),"",COUNTIF(C:C,C53))</f>
-        <v>18</v>
+        <v>11</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A54" s="20" t="s">
+      <c r="A54" s="14" t="s">
         <v>19</v>
       </c>
-      <c r="B54" s="13" t="s">
-        <v>74</v>
-      </c>
-      <c r="C54" s="15" t="s">
+      <c r="B54" s="8" t="s">
+        <v>75</v>
+      </c>
+      <c r="C54" s="14" t="s">
         <v>77</v>
       </c>
       <c r="D54" s="0" t="n">
@@ -11690,22 +11691,22 @@
       </c>
       <c r="E54" s="0" t="n">
         <f aca="false">IF(ISBLANK(B54),"",COUNTIF(B:B,B54))</f>
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="F54" s="0" t="n">
         <f aca="false">IF(ISBLANK(C54),"",COUNTIF(C:C,C54))</f>
-        <v>11</v>
+        <v>1</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A55" s="20" t="s">
+      <c r="A55" s="14" t="s">
         <v>19</v>
       </c>
-      <c r="B55" s="13" t="s">
-        <v>74</v>
-      </c>
-      <c r="C55" s="21" t="s">
-        <v>84</v>
+      <c r="B55" s="23" t="s">
+        <v>86</v>
+      </c>
+      <c r="C55" s="11" t="s">
+        <v>72</v>
       </c>
       <c r="D55" s="0" t="n">
         <f aca="false">IF(ISBLANK(A55),"",COUNTIF(A:A,A55))</f>
@@ -11713,22 +11714,22 @@
       </c>
       <c r="E55" s="0" t="n">
         <f aca="false">IF(ISBLANK(B55),"",COUNTIF(B:B,B55))</f>
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="F55" s="0" t="n">
         <f aca="false">IF(ISBLANK(C55),"",COUNTIF(C:C,C55))</f>
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A56" s="20" t="s">
+      <c r="A56" s="14" t="s">
         <v>19</v>
       </c>
-      <c r="B56" s="25" t="s">
-        <v>89</v>
-      </c>
-      <c r="C56" s="8" t="s">
-        <v>76</v>
+      <c r="B56" s="23" t="s">
+        <v>86</v>
+      </c>
+      <c r="C56" s="11" t="s">
+        <v>72</v>
       </c>
       <c r="D56" s="0" t="n">
         <f aca="false">IF(ISBLANK(A56),"",COUNTIF(A:A,A56))</f>
@@ -11736,19 +11737,19 @@
       </c>
       <c r="E56" s="0" t="n">
         <f aca="false">IF(ISBLANK(B56),"",COUNTIF(B:B,B56))</f>
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="F56" s="0" t="n">
         <f aca="false">IF(ISBLANK(C56),"",COUNTIF(C:C,C56))</f>
-        <v>18</v>
+        <v>5</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A57" s="12" t="s">
+      <c r="A57" s="17" t="s">
         <v>90</v>
       </c>
-      <c r="B57" s="11" t="s">
-        <v>72</v>
+      <c r="B57" s="20" t="s">
+        <v>83</v>
       </c>
       <c r="C57" s="12" t="s">
         <v>73</v>
@@ -11759,22 +11760,22 @@
       </c>
       <c r="E57" s="0" t="n">
         <f aca="false">IF(ISBLANK(B57),"",COUNTIF(B:B,B57))</f>
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="F57" s="0" t="n">
         <f aca="false">IF(ISBLANK(C57),"",COUNTIF(C:C,C57))</f>
-        <v>8</v>
+        <v>4</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A58" s="12" t="s">
+      <c r="A58" s="17" t="s">
         <v>90</v>
       </c>
-      <c r="B58" s="11" t="s">
-        <v>72</v>
-      </c>
-      <c r="C58" s="12" t="s">
-        <v>73</v>
+      <c r="B58" s="13" t="s">
+        <v>74</v>
+      </c>
+      <c r="C58" s="18" t="s">
+        <v>81</v>
       </c>
       <c r="D58" s="0" t="n">
         <f aca="false">IF(ISBLANK(A58),"",COUNTIF(A:A,A58))</f>
@@ -11782,22 +11783,22 @@
       </c>
       <c r="E58" s="0" t="n">
         <f aca="false">IF(ISBLANK(B58),"",COUNTIF(B:B,B58))</f>
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="F58" s="0" t="n">
         <f aca="false">IF(ISBLANK(C58),"",COUNTIF(C:C,C58))</f>
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A59" s="12" t="s">
+      <c r="A59" s="17" t="s">
         <v>90</v>
       </c>
-      <c r="B59" s="11" t="s">
-        <v>72</v>
-      </c>
-      <c r="C59" s="12" t="s">
-        <v>73</v>
+      <c r="B59" s="13" t="s">
+        <v>74</v>
+      </c>
+      <c r="C59" s="10" t="s">
+        <v>76</v>
       </c>
       <c r="D59" s="0" t="n">
         <f aca="false">IF(ISBLANK(A59),"",COUNTIF(A:A,A59))</f>
@@ -11805,22 +11806,22 @@
       </c>
       <c r="E59" s="0" t="n">
         <f aca="false">IF(ISBLANK(B59),"",COUNTIF(B:B,B59))</f>
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="F59" s="0" t="n">
         <f aca="false">IF(ISBLANK(C59),"",COUNTIF(C:C,C59))</f>
-        <v>8</v>
+        <v>4</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A60" s="12" t="s">
+      <c r="A60" s="17" t="s">
         <v>90</v>
       </c>
-      <c r="B60" s="11" t="s">
-        <v>72</v>
-      </c>
-      <c r="C60" s="13" t="s">
-        <v>74</v>
+      <c r="B60" s="16" t="s">
+        <v>79</v>
+      </c>
+      <c r="C60" s="8" t="s">
+        <v>75</v>
       </c>
       <c r="D60" s="0" t="n">
         <f aca="false">IF(ISBLANK(A60),"",COUNTIF(A:A,A60))</f>
@@ -11828,22 +11829,22 @@
       </c>
       <c r="E60" s="0" t="n">
         <f aca="false">IF(ISBLANK(B60),"",COUNTIF(B:B,B60))</f>
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="F60" s="0" t="n">
         <f aca="false">IF(ISBLANK(C60),"",COUNTIF(C:C,C60))</f>
-        <v>5</v>
+        <v>18</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A61" s="12" t="s">
+      <c r="A61" s="17" t="s">
         <v>90</v>
       </c>
-      <c r="B61" s="16" t="s">
+      <c r="B61" s="15" t="s">
         <v>78</v>
       </c>
-      <c r="C61" s="12" t="s">
-        <v>73</v>
+      <c r="C61" s="17" t="s">
+        <v>80</v>
       </c>
       <c r="D61" s="0" t="n">
         <f aca="false">IF(ISBLANK(A61),"",COUNTIF(A:A,A61))</f>
@@ -11859,14 +11860,14 @@
       </c>
     </row>
     <row r="62" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A62" s="12" t="s">
+      <c r="A62" s="17" t="s">
         <v>90</v>
       </c>
-      <c r="B62" s="12" t="s">
-        <v>73</v>
-      </c>
-      <c r="C62" s="19" t="s">
-        <v>82</v>
+      <c r="B62" s="17" t="s">
+        <v>80</v>
+      </c>
+      <c r="C62" s="13" t="s">
+        <v>74</v>
       </c>
       <c r="D62" s="0" t="n">
         <f aca="false">IF(ISBLANK(A62),"",COUNTIF(A:A,A62))</f>
@@ -11882,14 +11883,14 @@
       </c>
     </row>
     <row r="63" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A63" s="12" t="s">
+      <c r="A63" s="17" t="s">
         <v>90</v>
       </c>
       <c r="B63" s="19" t="s">
         <v>82</v>
       </c>
-      <c r="C63" s="18" t="s">
-        <v>81</v>
+      <c r="C63" s="17" t="s">
+        <v>80</v>
       </c>
       <c r="D63" s="0" t="n">
         <f aca="false">IF(ISBLANK(A63),"",COUNTIF(A:A,A63))</f>
@@ -11897,21 +11898,21 @@
       </c>
       <c r="E63" s="0" t="n">
         <f aca="false">IF(ISBLANK(B63),"",COUNTIF(B:B,B63))</f>
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="F63" s="0" t="n">
         <f aca="false">IF(ISBLANK(C63),"",COUNTIF(C:C,C63))</f>
-        <v>5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A64" s="12" t="s">
+      <c r="A64" s="17" t="s">
         <v>90</v>
       </c>
       <c r="B64" s="19" t="s">
         <v>82</v>
       </c>
-      <c r="C64" s="10" t="s">
+      <c r="C64" s="17" t="s">
         <v>80</v>
       </c>
       <c r="D64" s="0" t="n">
@@ -11920,22 +11921,22 @@
       </c>
       <c r="E64" s="0" t="n">
         <f aca="false">IF(ISBLANK(B64),"",COUNTIF(B:B,B64))</f>
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="F64" s="0" t="n">
         <f aca="false">IF(ISBLANK(C64),"",COUNTIF(C:C,C64))</f>
-        <v>4</v>
+        <v>8</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A65" s="12" t="s">
+      <c r="A65" s="17" t="s">
         <v>90</v>
       </c>
-      <c r="B65" s="17" t="s">
-        <v>79</v>
-      </c>
-      <c r="C65" s="8" t="s">
-        <v>76</v>
+      <c r="B65" s="19" t="s">
+        <v>82</v>
+      </c>
+      <c r="C65" s="17" t="s">
+        <v>80</v>
       </c>
       <c r="D65" s="0" t="n">
         <f aca="false">IF(ISBLANK(A65),"",COUNTIF(A:A,A65))</f>
@@ -11943,22 +11944,22 @@
       </c>
       <c r="E65" s="0" t="n">
         <f aca="false">IF(ISBLANK(B65),"",COUNTIF(B:B,B65))</f>
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="F65" s="0" t="n">
         <f aca="false">IF(ISBLANK(C65),"",COUNTIF(C:C,C65))</f>
-        <v>18</v>
+        <v>8</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A66" s="12" t="s">
+      <c r="A66" s="17" t="s">
         <v>90</v>
       </c>
-      <c r="B66" s="15" t="s">
-        <v>77</v>
-      </c>
-      <c r="C66" s="14" t="s">
-        <v>75</v>
+      <c r="B66" s="19" t="s">
+        <v>82</v>
+      </c>
+      <c r="C66" s="11" t="s">
+        <v>72</v>
       </c>
       <c r="D66" s="0" t="n">
         <f aca="false">IF(ISBLANK(A66),"",COUNTIF(A:A,A66))</f>
@@ -11966,22 +11967,22 @@
       </c>
       <c r="E66" s="0" t="n">
         <f aca="false">IF(ISBLANK(B66),"",COUNTIF(B:B,B66))</f>
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="F66" s="0" t="n">
         <f aca="false">IF(ISBLANK(C66),"",COUNTIF(C:C,C66))</f>
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A67" s="21" t="s">
+      <c r="A67" s="23" t="s">
         <v>91</v>
       </c>
-      <c r="B67" s="21" t="s">
-        <v>84</v>
+      <c r="B67" s="26" t="s">
+        <v>92</v>
       </c>
       <c r="C67" s="8" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D67" s="0" t="n">
         <f aca="false">IF(ISBLANK(A67),"",COUNTIF(A:A,A67))</f>
@@ -11989,7 +11990,7 @@
       </c>
       <c r="E67" s="0" t="n">
         <f aca="false">IF(ISBLANK(B67),"",COUNTIF(B:B,B67))</f>
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="F67" s="0" t="n">
         <f aca="false">IF(ISBLANK(C67),"",COUNTIF(C:C,C67))</f>
@@ -11997,14 +11998,14 @@
       </c>
     </row>
     <row r="68" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A68" s="21" t="s">
+      <c r="A68" s="23" t="s">
         <v>91</v>
       </c>
-      <c r="B68" s="21" t="s">
-        <v>84</v>
-      </c>
-      <c r="C68" s="17" t="s">
-        <v>79</v>
+      <c r="B68" s="12" t="s">
+        <v>73</v>
+      </c>
+      <c r="C68" s="20" t="s">
+        <v>83</v>
       </c>
       <c r="D68" s="0" t="n">
         <f aca="false">IF(ISBLANK(A68),"",COUNTIF(A:A,A68))</f>
@@ -12012,22 +12013,22 @@
       </c>
       <c r="E68" s="0" t="n">
         <f aca="false">IF(ISBLANK(B68),"",COUNTIF(B:B,B68))</f>
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="F68" s="0" t="n">
         <f aca="false">IF(ISBLANK(C68),"",COUNTIF(C:C,C68))</f>
-        <v>6</v>
+        <v>11</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A69" s="21" t="s">
+      <c r="A69" s="23" t="s">
         <v>91</v>
       </c>
-      <c r="B69" s="8" t="s">
-        <v>76</v>
-      </c>
-      <c r="C69" s="17" t="s">
-        <v>79</v>
+      <c r="B69" s="22" t="s">
+        <v>85</v>
+      </c>
+      <c r="C69" s="8" t="s">
+        <v>75</v>
       </c>
       <c r="D69" s="0" t="n">
         <f aca="false">IF(ISBLANK(A69),"",COUNTIF(A:A,A69))</f>
@@ -12035,22 +12036,22 @@
       </c>
       <c r="E69" s="0" t="n">
         <f aca="false">IF(ISBLANK(B69),"",COUNTIF(B:B,B69))</f>
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F69" s="0" t="n">
         <f aca="false">IF(ISBLANK(C69),"",COUNTIF(C:C,C69))</f>
-        <v>6</v>
+        <v>18</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A70" s="21" t="s">
+      <c r="A70" s="23" t="s">
         <v>91</v>
       </c>
-      <c r="B70" s="14" t="s">
-        <v>75</v>
-      </c>
-      <c r="C70" s="15" t="s">
-        <v>77</v>
+      <c r="B70" s="22" t="s">
+        <v>85</v>
+      </c>
+      <c r="C70" s="23" t="s">
+        <v>86</v>
       </c>
       <c r="D70" s="0" t="n">
         <f aca="false">IF(ISBLANK(A70),"",COUNTIF(A:A,A70))</f>
@@ -12062,18 +12063,18 @@
       </c>
       <c r="F70" s="0" t="n">
         <f aca="false">IF(ISBLANK(C70),"",COUNTIF(C:C,C70))</f>
-        <v>11</v>
+        <v>3</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A71" s="21" t="s">
+      <c r="A71" s="23" t="s">
         <v>91</v>
       </c>
-      <c r="B71" s="22" t="s">
-        <v>85</v>
-      </c>
-      <c r="C71" s="8" t="s">
-        <v>76</v>
+      <c r="B71" s="8" t="s">
+        <v>75</v>
+      </c>
+      <c r="C71" s="16" t="s">
+        <v>79</v>
       </c>
       <c r="D71" s="0" t="n">
         <f aca="false">IF(ISBLANK(A71),"",COUNTIF(A:A,A71))</f>
@@ -12081,22 +12082,22 @@
       </c>
       <c r="E71" s="0" t="n">
         <f aca="false">IF(ISBLANK(B71),"",COUNTIF(B:B,B71))</f>
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="F71" s="0" t="n">
         <f aca="false">IF(ISBLANK(C71),"",COUNTIF(C:C,C71))</f>
-        <v>18</v>
+        <v>6</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A72" s="21" t="s">
+      <c r="A72" s="23" t="s">
         <v>91</v>
       </c>
-      <c r="B72" s="22" t="s">
-        <v>85</v>
-      </c>
-      <c r="C72" s="21" t="s">
-        <v>84</v>
+      <c r="B72" s="23" t="s">
+        <v>86</v>
+      </c>
+      <c r="C72" s="8" t="s">
+        <v>75</v>
       </c>
       <c r="D72" s="0" t="n">
         <f aca="false">IF(ISBLANK(A72),"",COUNTIF(A:A,A72))</f>
@@ -12104,22 +12105,22 @@
       </c>
       <c r="E72" s="0" t="n">
         <f aca="false">IF(ISBLANK(B72),"",COUNTIF(B:B,B72))</f>
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F72" s="0" t="n">
         <f aca="false">IF(ISBLANK(C72),"",COUNTIF(C:C,C72))</f>
-        <v>3</v>
+        <v>18</v>
       </c>
     </row>
     <row r="73" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A73" s="21" t="s">
+      <c r="A73" s="23" t="s">
         <v>91</v>
       </c>
-      <c r="B73" s="26" t="s">
-        <v>92</v>
-      </c>
-      <c r="C73" s="8" t="s">
-        <v>76</v>
+      <c r="B73" s="23" t="s">
+        <v>86</v>
+      </c>
+      <c r="C73" s="16" t="s">
+        <v>79</v>
       </c>
       <c r="D73" s="0" t="n">
         <f aca="false">IF(ISBLANK(A73),"",COUNTIF(A:A,A73))</f>
@@ -12127,11 +12128,11 @@
       </c>
       <c r="E73" s="0" t="n">
         <f aca="false">IF(ISBLANK(B73),"",COUNTIF(B:B,B73))</f>
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F73" s="0" t="n">
         <f aca="false">IF(ISBLANK(C73),"",COUNTIF(C:C,C73))</f>
-        <v>18</v>
+        <v>6</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12142,7 +12143,7 @@
         <v>81</v>
       </c>
       <c r="C74" s="8" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D74" s="0" t="n">
         <f aca="false">IF(ISBLANK(A74),"",COUNTIF(A:A,A74))</f>
@@ -12165,7 +12166,7 @@
         <v>81</v>
       </c>
       <c r="C75" s="8" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D75" s="0" t="n">
         <f aca="false">IF(ISBLANK(A75),"",COUNTIF(A:A,A75))</f>
@@ -12188,7 +12189,7 @@
         <v>81</v>
       </c>
       <c r="C76" s="8" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D76" s="0" t="n">
         <f aca="false">IF(ISBLANK(A76),"",COUNTIF(A:A,A76))</f>
@@ -12211,7 +12212,7 @@
         <v>81</v>
       </c>
       <c r="C77" s="8" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D77" s="0" t="n">
         <f aca="false">IF(ISBLANK(A77),"",COUNTIF(A:A,A77))</f>
@@ -12234,7 +12235,7 @@
         <v>81</v>
       </c>
       <c r="C78" s="8" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D78" s="0" t="n">
         <f aca="false">IF(ISBLANK(A78),"",COUNTIF(A:A,A78))</f>
@@ -12257,7 +12258,7 @@
         <v>81</v>
       </c>
       <c r="C79" s="8" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D79" s="0" t="n">
         <f aca="false">IF(ISBLANK(A79),"",COUNTIF(A:A,A79))</f>
@@ -12276,8 +12277,8 @@
       <c r="A80" s="22" t="s">
         <v>93</v>
       </c>
-      <c r="B80" s="8" t="s">
-        <v>76</v>
+      <c r="B80" s="16" t="s">
+        <v>79</v>
       </c>
       <c r="D80" s="0" t="n">
         <f aca="false">IF(ISBLANK(A80),"",COUNTIF(A:A,A80))</f>
@@ -12285,7 +12286,7 @@
       </c>
       <c r="E80" s="0" t="n">
         <f aca="false">IF(ISBLANK(B80),"",COUNTIF(B:B,B80))</f>
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="F80" s="0" t="str">
         <f aca="false">IF(ISBLANK(C80),"",COUNTIF(C:C,C80))</f>
@@ -12336,8 +12337,8 @@
       <c r="A83" s="22" t="s">
         <v>93</v>
       </c>
-      <c r="B83" s="17" t="s">
-        <v>79</v>
+      <c r="B83" s="8" t="s">
+        <v>75</v>
       </c>
       <c r="D83" s="0" t="n">
         <f aca="false">IF(ISBLANK(A83),"",COUNTIF(A:A,A83))</f>
@@ -12345,7 +12346,7 @@
       </c>
       <c r="E83" s="0" t="n">
         <f aca="false">IF(ISBLANK(B83),"",COUNTIF(B:B,B83))</f>
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="F83" s="0" t="str">
         <f aca="false">IF(ISBLANK(C83),"",COUNTIF(C:C,C83))</f>
@@ -12353,106 +12354,94 @@
       </c>
     </row>
     <row r="84" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A84" s="25" t="s">
+      <c r="A84" s="18" t="s">
+        <v>43</v>
+      </c>
+      <c r="B84" s="27" t="s">
         <v>94</v>
-      </c>
-      <c r="B84" s="8" t="s">
-        <v>76</v>
-      </c>
-      <c r="C84" s="18" t="s">
-        <v>81</v>
       </c>
       <c r="D84" s="0" t="n">
         <f aca="false">IF(ISBLANK(A84),"",COUNTIF(A:A,A84))</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E84" s="0" t="n">
         <f aca="false">IF(ISBLANK(B84),"",COUNTIF(B:B,B84))</f>
-        <v>9</v>
-      </c>
-      <c r="F84" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="F84" s="0" t="str">
         <f aca="false">IF(ISBLANK(C84),"",COUNTIF(C:C,C84))</f>
-        <v>5</v>
+        <v/>
       </c>
     </row>
     <row r="85" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A85" s="25" t="s">
+      <c r="A85" s="18" t="s">
+        <v>43</v>
+      </c>
+      <c r="B85" s="27" t="s">
         <v>94</v>
-      </c>
-      <c r="B85" s="20" t="s">
-        <v>83</v>
-      </c>
-      <c r="C85" s="18" t="s">
-        <v>81</v>
       </c>
       <c r="D85" s="0" t="n">
         <f aca="false">IF(ISBLANK(A85),"",COUNTIF(A:A,A85))</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E85" s="0" t="n">
         <f aca="false">IF(ISBLANK(B85),"",COUNTIF(B:B,B85))</f>
-        <v>5</v>
-      </c>
-      <c r="F85" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="F85" s="0" t="str">
         <f aca="false">IF(ISBLANK(C85),"",COUNTIF(C:C,C85))</f>
-        <v>5</v>
+        <v/>
       </c>
     </row>
     <row r="86" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A86" s="25" t="s">
-        <v>94</v>
-      </c>
-      <c r="B86" s="25" t="s">
-        <v>89</v>
-      </c>
-      <c r="C86" s="18" t="s">
-        <v>81</v>
+      <c r="A86" s="18" t="s">
+        <v>43</v>
+      </c>
+      <c r="B86" s="11" t="s">
+        <v>72</v>
       </c>
       <c r="D86" s="0" t="n">
         <f aca="false">IF(ISBLANK(A86),"",COUNTIF(A:A,A86))</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E86" s="0" t="n">
         <f aca="false">IF(ISBLANK(B86),"",COUNTIF(B:B,B86))</f>
-        <v>2</v>
-      </c>
-      <c r="F86" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="F86" s="0" t="str">
         <f aca="false">IF(ISBLANK(C86),"",COUNTIF(C:C,C86))</f>
-        <v>5</v>
+        <v/>
       </c>
     </row>
     <row r="87" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A87" s="19" t="s">
-        <v>95</v>
-      </c>
-      <c r="B87" s="11" t="s">
-        <v>72</v>
-      </c>
-      <c r="C87" s="18" t="s">
-        <v>81</v>
+      <c r="A87" s="18" t="s">
+        <v>43</v>
+      </c>
+      <c r="B87" s="23" t="s">
+        <v>86</v>
       </c>
       <c r="D87" s="0" t="n">
         <f aca="false">IF(ISBLANK(A87),"",COUNTIF(A:A,A87))</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E87" s="0" t="n">
         <f aca="false">IF(ISBLANK(B87),"",COUNTIF(B:B,B87))</f>
-        <v>9</v>
-      </c>
-      <c r="F87" s="0" t="n">
+        <v>10</v>
+      </c>
+      <c r="F87" s="0" t="str">
         <f aca="false">IF(ISBLANK(C87),"",COUNTIF(C:C,C87))</f>
-        <v>5</v>
+        <v/>
       </c>
     </row>
     <row r="88" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A88" s="19" t="s">
+      <c r="A88" s="25" t="s">
         <v>95</v>
       </c>
-      <c r="B88" s="12" t="s">
-        <v>73</v>
-      </c>
-      <c r="C88" s="11" t="s">
-        <v>72</v>
+      <c r="B88" s="25" t="s">
+        <v>89</v>
+      </c>
+      <c r="C88" s="18" t="s">
+        <v>81</v>
       </c>
       <c r="D88" s="0" t="n">
         <f aca="false">IF(ISBLANK(A88),"",COUNTIF(A:A,A88))</f>
@@ -12460,22 +12449,22 @@
       </c>
       <c r="E88" s="0" t="n">
         <f aca="false">IF(ISBLANK(B88),"",COUNTIF(B:B,B88))</f>
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="F88" s="0" t="n">
         <f aca="false">IF(ISBLANK(C88),"",COUNTIF(C:C,C88))</f>
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="89" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A89" s="19" t="s">
+      <c r="A89" s="25" t="s">
         <v>95</v>
       </c>
-      <c r="B89" s="19" t="s">
-        <v>82</v>
-      </c>
-      <c r="C89" s="19" t="s">
-        <v>82</v>
+      <c r="B89" s="14" t="s">
+        <v>77</v>
+      </c>
+      <c r="C89" s="18" t="s">
+        <v>81</v>
       </c>
       <c r="D89" s="0" t="n">
         <f aca="false">IF(ISBLANK(A89),"",COUNTIF(A:A,A89))</f>
@@ -12487,18 +12476,18 @@
       </c>
       <c r="F89" s="0" t="n">
         <f aca="false">IF(ISBLANK(C89),"",COUNTIF(C:C,C89))</f>
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="90" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A90" s="27" t="s">
-        <v>96</v>
-      </c>
-      <c r="B90" s="11" t="s">
-        <v>72</v>
-      </c>
-      <c r="C90" s="12" t="s">
-        <v>73</v>
+      <c r="A90" s="25" t="s">
+        <v>95</v>
+      </c>
+      <c r="B90" s="8" t="s">
+        <v>75</v>
+      </c>
+      <c r="C90" s="18" t="s">
+        <v>81</v>
       </c>
       <c r="D90" s="0" t="n">
         <f aca="false">IF(ISBLANK(A90),"",COUNTIF(A:A,A90))</f>
@@ -12510,18 +12499,18 @@
       </c>
       <c r="F90" s="0" t="n">
         <f aca="false">IF(ISBLANK(C90),"",COUNTIF(C:C,C90))</f>
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="91" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A91" s="27" t="s">
+      <c r="A91" s="13" t="s">
         <v>96</v>
       </c>
-      <c r="B91" s="27" t="s">
-        <v>97</v>
-      </c>
-      <c r="C91" s="28" t="s">
-        <v>98</v>
+      <c r="B91" s="13" t="s">
+        <v>74</v>
+      </c>
+      <c r="C91" s="13" t="s">
+        <v>74</v>
       </c>
       <c r="D91" s="0" t="n">
         <f aca="false">IF(ISBLANK(A91),"",COUNTIF(A:A,A91))</f>
@@ -12529,22 +12518,22 @@
       </c>
       <c r="E91" s="0" t="n">
         <f aca="false">IF(ISBLANK(B91),"",COUNTIF(B:B,B91))</f>
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="F91" s="0" t="n">
         <f aca="false">IF(ISBLANK(C91),"",COUNTIF(C:C,C91))</f>
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="92" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A92" s="27" t="s">
+      <c r="A92" s="13" t="s">
         <v>96</v>
       </c>
-      <c r="B92" s="27" t="s">
-        <v>97</v>
-      </c>
-      <c r="C92" s="28" t="s">
-        <v>98</v>
+      <c r="B92" s="17" t="s">
+        <v>80</v>
+      </c>
+      <c r="C92" s="19" t="s">
+        <v>82</v>
       </c>
       <c r="D92" s="0" t="n">
         <f aca="false">IF(ISBLANK(A92),"",COUNTIF(A:A,A92))</f>
@@ -12552,78 +12541,130 @@
       </c>
       <c r="E92" s="0" t="n">
         <f aca="false">IF(ISBLANK(B92),"",COUNTIF(B:B,B92))</f>
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="F92" s="0" t="n">
         <f aca="false">IF(ISBLANK(C92),"",COUNTIF(C:C,C92))</f>
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="93" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A93" s="18" t="s">
-        <v>43</v>
-      </c>
-      <c r="B93" s="21" t="s">
-        <v>84</v>
+      <c r="A93" s="13" t="s">
+        <v>96</v>
+      </c>
+      <c r="B93" s="19" t="s">
+        <v>82</v>
+      </c>
+      <c r="C93" s="18" t="s">
+        <v>81</v>
       </c>
       <c r="D93" s="0" t="n">
         <f aca="false">IF(ISBLANK(A93),"",COUNTIF(A:A,A93))</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E93" s="0" t="n">
         <f aca="false">IF(ISBLANK(B93),"",COUNTIF(B:B,B93))</f>
-        <v>10</v>
-      </c>
-      <c r="F93" s="0" t="str">
+        <v>9</v>
+      </c>
+      <c r="F93" s="0" t="n">
         <f aca="false">IF(ISBLANK(C93),"",COUNTIF(C:C,C93))</f>
-        <v/>
+        <v>5</v>
       </c>
     </row>
     <row r="94" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A94" s="18" t="s">
-        <v>43</v>
+      <c r="A94" s="28" t="s">
+        <v>97</v>
       </c>
       <c r="B94" s="28" t="s">
         <v>98</v>
       </c>
+      <c r="C94" s="27" t="s">
+        <v>94</v>
+      </c>
       <c r="D94" s="0" t="n">
         <f aca="false">IF(ISBLANK(A94),"",COUNTIF(A:A,A94))</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E94" s="0" t="n">
         <f aca="false">IF(ISBLANK(B94),"",COUNTIF(B:B,B94))</f>
-        <v>1</v>
-      </c>
-      <c r="F94" s="0" t="str">
+        <v>2</v>
+      </c>
+      <c r="F94" s="0" t="n">
         <f aca="false">IF(ISBLANK(C94),"",COUNTIF(C:C,C94))</f>
-        <v/>
+        <v>2</v>
       </c>
     </row>
     <row r="95" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A95" s="16" t="s">
-        <v>99</v>
-      </c>
-      <c r="B95" s="12" t="s">
-        <v>73</v>
-      </c>
-      <c r="C95" s="16" t="s">
-        <v>78</v>
+      <c r="A95" s="28" t="s">
+        <v>97</v>
+      </c>
+      <c r="B95" s="28" t="s">
+        <v>98</v>
+      </c>
+      <c r="C95" s="27" t="s">
+        <v>94</v>
       </c>
       <c r="D95" s="0" t="n">
         <f aca="false">IF(ISBLANK(A95),"",COUNTIF(A:A,A95))</f>
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E95" s="0" t="n">
         <f aca="false">IF(ISBLANK(B95),"",COUNTIF(B:B,B95))</f>
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="F95" s="0" t="n">
         <f aca="false">IF(ISBLANK(C95),"",COUNTIF(C:C,C95))</f>
         <v>2</v>
       </c>
     </row>
+    <row r="96" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A96" s="28" t="s">
+        <v>97</v>
+      </c>
+      <c r="B96" s="19" t="s">
+        <v>82</v>
+      </c>
+      <c r="C96" s="17" t="s">
+        <v>80</v>
+      </c>
+      <c r="D96" s="0" t="n">
+        <f aca="false">IF(ISBLANK(A96),"",COUNTIF(A:A,A96))</f>
+        <v>3</v>
+      </c>
+      <c r="E96" s="0" t="n">
+        <f aca="false">IF(ISBLANK(B96),"",COUNTIF(B:B,B96))</f>
+        <v>9</v>
+      </c>
+      <c r="F96" s="0" t="n">
+        <f aca="false">IF(ISBLANK(C96),"",COUNTIF(C:C,C96))</f>
+        <v>8</v>
+      </c>
+    </row>
+    <row r="97" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A97" s="15" t="s">
+        <v>99</v>
+      </c>
+      <c r="B97" s="17" t="s">
+        <v>80</v>
+      </c>
+      <c r="C97" s="15" t="s">
+        <v>78</v>
+      </c>
+      <c r="D97" s="0" t="n">
+        <f aca="false">IF(ISBLANK(A97),"",COUNTIF(A:A,A97))</f>
+        <v>1</v>
+      </c>
+      <c r="E97" s="0" t="n">
+        <f aca="false">IF(ISBLANK(B97),"",COUNTIF(B:B,B97))</f>
+        <v>7</v>
+      </c>
+      <c r="F97" s="0" t="n">
+        <f aca="false">IF(ISBLANK(C97),"",COUNTIF(C:C,C97))</f>
+        <v>2</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:F95"/>
+  <autoFilter ref="A1:F97"/>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
   <pageSetup paperSize="9" scale="100" firstPageNumber="0" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" useFirstPageNumber="false" horizontalDpi="300" verticalDpi="300" copies="1"/>
@@ -12690,22 +12731,22 @@
         <f aca="false">COUNTIF(Tatjes!A:A,A2)</f>
         <v>16</v>
       </c>
-      <c r="D2" s="21" t="s">
-        <v>84</v>
+      <c r="D2" s="23" t="s">
+        <v>86</v>
       </c>
       <c r="E2" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!B:B,D2)</f>
         <v>10</v>
       </c>
       <c r="G2" s="8" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="H2" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!C:C,G2)</f>
         <v>18</v>
       </c>
       <c r="J2" s="8" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="K2" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!B:B,J2)*2+COUNTIF(Tatjes!C:C,J2)</f>
@@ -12713,7 +12754,7 @@
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="14" t="s">
+      <c r="A3" s="12" t="s">
         <v>33</v>
       </c>
       <c r="B3" s="1" t="n">
@@ -12721,21 +12762,21 @@
         <v>16</v>
       </c>
       <c r="D3" s="8" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="E3" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!B:B,D3)</f>
         <v>9</v>
       </c>
-      <c r="G3" s="15" t="s">
-        <v>77</v>
+      <c r="G3" s="20" t="s">
+        <v>83</v>
       </c>
       <c r="H3" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!C:C,G3)</f>
         <v>11</v>
       </c>
-      <c r="J3" s="21" t="s">
-        <v>84</v>
+      <c r="J3" s="23" t="s">
+        <v>86</v>
       </c>
       <c r="K3" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!B:B,J3)*2+COUNTIF(Tatjes!C:C,J3)</f>
@@ -12750,22 +12791,22 @@
         <f aca="false">COUNTIF(Tatjes!A:A,A4)</f>
         <v>12</v>
       </c>
-      <c r="D4" s="11" t="s">
-        <v>72</v>
+      <c r="D4" s="19" t="s">
+        <v>82</v>
       </c>
       <c r="E4" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!B:B,D4)</f>
         <v>9</v>
       </c>
-      <c r="G4" s="12" t="s">
-        <v>73</v>
+      <c r="G4" s="17" t="s">
+        <v>80</v>
       </c>
       <c r="H4" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!C:C,G4)</f>
         <v>8</v>
       </c>
-      <c r="J4" s="12" t="s">
-        <v>73</v>
+      <c r="J4" s="17" t="s">
+        <v>80</v>
       </c>
       <c r="K4" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!B:B,J4)*2+COUNTIF(Tatjes!C:C,J4)</f>
@@ -12773,29 +12814,29 @@
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="20" t="s">
+      <c r="A5" s="14" t="s">
         <v>19</v>
       </c>
       <c r="B5" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!A:A,A5)</f>
         <v>11</v>
       </c>
-      <c r="D5" s="14" t="s">
-        <v>75</v>
+      <c r="D5" s="12" t="s">
+        <v>73</v>
       </c>
       <c r="E5" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!B:B,D5)</f>
         <v>8</v>
       </c>
-      <c r="G5" s="17" t="s">
+      <c r="G5" s="16" t="s">
         <v>79</v>
       </c>
       <c r="H5" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!C:C,G5)</f>
         <v>6</v>
       </c>
-      <c r="J5" s="11" t="s">
-        <v>72</v>
+      <c r="J5" s="19" t="s">
+        <v>82</v>
       </c>
       <c r="K5" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!B:B,J5)*2+COUNTIF(Tatjes!C:C,J5)</f>
@@ -12803,7 +12844,7 @@
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="12" t="s">
+      <c r="A6" s="17" t="s">
         <v>90</v>
       </c>
       <c r="B6" s="1" t="n">
@@ -12817,15 +12858,15 @@
         <f aca="false">COUNTIF(Tatjes!B:B,D6)</f>
         <v>8</v>
       </c>
-      <c r="G6" s="13" t="s">
-        <v>74</v>
+      <c r="G6" s="11" t="s">
+        <v>72</v>
       </c>
       <c r="H6" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!C:C,G6)</f>
         <v>5</v>
       </c>
-      <c r="J6" s="14" t="s">
-        <v>75</v>
+      <c r="J6" s="12" t="s">
+        <v>73</v>
       </c>
       <c r="K6" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!B:B,J6)*2+COUNTIF(Tatjes!C:C,J6)</f>
@@ -12833,14 +12874,14 @@
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="21" t="s">
+      <c r="A7" s="23" t="s">
         <v>91</v>
       </c>
       <c r="B7" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!A:A,A7)</f>
         <v>7</v>
       </c>
-      <c r="D7" s="16" t="s">
+      <c r="D7" s="15" t="s">
         <v>78</v>
       </c>
       <c r="E7" s="1" t="n">
@@ -12870,15 +12911,15 @@
         <f aca="false">COUNTIF(Tatjes!A:A,A8)</f>
         <v>6</v>
       </c>
-      <c r="D8" s="12" t="s">
-        <v>73</v>
+      <c r="D8" s="17" t="s">
+        <v>80</v>
       </c>
       <c r="E8" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!B:B,D8)</f>
         <v>7</v>
       </c>
-      <c r="G8" s="14" t="s">
-        <v>75</v>
+      <c r="G8" s="12" t="s">
+        <v>73</v>
       </c>
       <c r="H8" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!C:C,G8)</f>
@@ -12907,14 +12948,14 @@
         <f aca="false">COUNTIF(Tatjes!B:B,D9)</f>
         <v>7</v>
       </c>
-      <c r="G9" s="19" t="s">
-        <v>82</v>
+      <c r="G9" s="13" t="s">
+        <v>74</v>
       </c>
       <c r="H9" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!C:C,G9)</f>
         <v>3</v>
       </c>
-      <c r="J9" s="17" t="s">
+      <c r="J9" s="16" t="s">
         <v>79</v>
       </c>
       <c r="K9" s="1" t="n">
@@ -12923,28 +12964,28 @@
       </c>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="25" t="s">
-        <v>94</v>
+      <c r="A10" s="18" t="s">
+        <v>43</v>
       </c>
       <c r="B10" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!A:A,A10)</f>
-        <v>3</v>
-      </c>
-      <c r="D10" s="19" t="s">
-        <v>82</v>
+        <v>4</v>
+      </c>
+      <c r="D10" s="13" t="s">
+        <v>74</v>
       </c>
       <c r="E10" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!B:B,D10)</f>
         <v>5</v>
       </c>
-      <c r="G10" s="21" t="s">
-        <v>84</v>
+      <c r="G10" s="23" t="s">
+        <v>86</v>
       </c>
       <c r="H10" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!C:C,G10)</f>
         <v>3</v>
       </c>
-      <c r="J10" s="16" t="s">
+      <c r="J10" s="15" t="s">
         <v>78</v>
       </c>
       <c r="K10" s="1" t="n">
@@ -12953,29 +12994,29 @@
       </c>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="19" t="s">
+      <c r="A11" s="25" t="s">
         <v>95</v>
       </c>
       <c r="B11" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!A:A,A11)</f>
         <v>3</v>
       </c>
-      <c r="D11" s="17" t="s">
+      <c r="D11" s="16" t="s">
         <v>79</v>
       </c>
       <c r="E11" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!B:B,D11)</f>
         <v>5</v>
       </c>
-      <c r="G11" s="11" t="s">
-        <v>72</v>
+      <c r="G11" s="19" t="s">
+        <v>82</v>
       </c>
       <c r="H11" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!C:C,G11)</f>
         <v>3</v>
       </c>
-      <c r="J11" s="15" t="s">
-        <v>77</v>
+      <c r="J11" s="20" t="s">
+        <v>83</v>
       </c>
       <c r="K11" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!B:B,J11)*2+COUNTIF(Tatjes!C:C,J11)</f>
@@ -12983,29 +13024,29 @@
       </c>
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="27" t="s">
+      <c r="A12" s="13" t="s">
         <v>96</v>
       </c>
       <c r="B12" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!A:A,A12)</f>
         <v>3</v>
       </c>
-      <c r="D12" s="20" t="s">
-        <v>83</v>
+      <c r="D12" s="14" t="s">
+        <v>77</v>
       </c>
       <c r="E12" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!B:B,D12)</f>
         <v>5</v>
       </c>
-      <c r="G12" s="28" t="s">
-        <v>98</v>
+      <c r="G12" s="27" t="s">
+        <v>94</v>
       </c>
       <c r="H12" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!C:C,G12)</f>
         <v>2</v>
       </c>
-      <c r="J12" s="19" t="s">
-        <v>82</v>
+      <c r="J12" s="13" t="s">
+        <v>74</v>
       </c>
       <c r="K12" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!B:B,J12)*2+COUNTIF(Tatjes!C:C,J12)</f>
@@ -13013,29 +13054,29 @@
       </c>
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="18" t="s">
-        <v>43</v>
+      <c r="A13" s="28" t="s">
+        <v>97</v>
       </c>
       <c r="B13" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!A:A,A13)</f>
-        <v>2</v>
-      </c>
-      <c r="D13" s="13" t="s">
-        <v>74</v>
+        <v>3</v>
+      </c>
+      <c r="D13" s="11" t="s">
+        <v>72</v>
       </c>
       <c r="E13" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!B:B,D13)</f>
         <v>4</v>
       </c>
-      <c r="G13" s="16" t="s">
+      <c r="G13" s="15" t="s">
         <v>78</v>
       </c>
       <c r="H13" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!C:C,G13)</f>
         <v>2</v>
       </c>
-      <c r="J13" s="13" t="s">
-        <v>74</v>
+      <c r="J13" s="11" t="s">
+        <v>72</v>
       </c>
       <c r="K13" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!B:B,J13)*2+COUNTIF(Tatjes!C:C,J13)</f>
@@ -13043,29 +13084,29 @@
       </c>
     </row>
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="16" t="s">
+      <c r="A14" s="15" t="s">
         <v>99</v>
       </c>
       <c r="B14" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!A:A,A14)</f>
         <v>1</v>
       </c>
-      <c r="D14" s="15" t="s">
-        <v>77</v>
+      <c r="D14" s="20" t="s">
+        <v>83</v>
       </c>
       <c r="E14" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!B:B,D14)</f>
         <v>2</v>
       </c>
-      <c r="G14" s="20" t="s">
-        <v>83</v>
+      <c r="G14" s="14" t="s">
+        <v>77</v>
       </c>
       <c r="H14" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!C:C,G14)</f>
         <v>1</v>
       </c>
-      <c r="J14" s="20" t="s">
-        <v>83</v>
+      <c r="J14" s="14" t="s">
+        <v>77</v>
       </c>
       <c r="K14" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!B:B,J14)*2+COUNTIF(Tatjes!C:C,J14)</f>
@@ -13074,26 +13115,26 @@
     </row>
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B15" s="0"/>
-      <c r="D15" s="27" t="s">
-        <v>97</v>
+      <c r="D15" s="28" t="s">
+        <v>98</v>
       </c>
       <c r="E15" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!B:B,D15)</f>
         <v>2</v>
       </c>
-      <c r="G15" s="23" t="s">
-        <v>86</v>
+      <c r="G15" s="21" t="s">
+        <v>84</v>
       </c>
       <c r="H15" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!C:C,G15)</f>
         <v>1</v>
       </c>
       <c r="J15" s="27" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="K15" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!B:B,J15)*2+COUNTIF(Tatjes!C:C,J15)</f>
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13102,17 +13143,17 @@
       </c>
       <c r="B16" s="3" t="n">
         <f aca="false">COUNTA(Tatjes!A:A)-1</f>
+        <v>96</v>
+      </c>
+      <c r="D16" s="27" t="s">
         <v>94</v>
-      </c>
-      <c r="D16" s="24" t="s">
-        <v>88</v>
       </c>
       <c r="E16" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!B:B,D16)</f>
         <v>2</v>
       </c>
-      <c r="G16" s="27" t="s">
-        <v>97</v>
+      <c r="G16" s="28" t="s">
+        <v>98</v>
       </c>
       <c r="H16" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!C:C,G16)</f>
@@ -13127,8 +13168,8 @@
       </c>
     </row>
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D17" s="25" t="s">
-        <v>89</v>
+      <c r="D17" s="24" t="s">
+        <v>88</v>
       </c>
       <c r="E17" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!B:B,D17)</f>
@@ -13150,12 +13191,12 @@
       </c>
     </row>
     <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D18" s="28" t="s">
-        <v>98</v>
+      <c r="D18" s="25" t="s">
+        <v>89</v>
       </c>
       <c r="E18" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!B:B,D18)</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G18" s="24" t="s">
         <v>88</v>
@@ -13196,8 +13237,8 @@
       </c>
     </row>
     <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D20" s="23" t="s">
-        <v>86</v>
+      <c r="D20" s="21" t="s">
+        <v>84</v>
       </c>
       <c r="E20" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!B:B,D20)</f>
@@ -13210,8 +13251,8 @@
         <f aca="false">COUNTIF(Tatjes!C:C,G20)</f>
         <v>0</v>
       </c>
-      <c r="J20" s="23" t="s">
-        <v>86</v>
+      <c r="J20" s="21" t="s">
+        <v>84</v>
       </c>
       <c r="K20" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!B:B,J20)*2+COUNTIF(Tatjes!C:C,J20)</f>

</xml_diff>

<commit_message>
Sync from vault 2026-06-10 00:59:09
</commit_message>
<xml_diff>
--- a/content/Archief/0. PDFs & docs/Obol docs & forms/Irmijn Inc/Irma backup log.xlsx
+++ b/content/Archief/0. PDFs & docs/Obol docs & forms/Irmijn Inc/Irma backup log.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="3"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="Logboek" sheetId="1" state="visible" r:id="rId2"/>
@@ -15,14 +15,14 @@
   </sheets>
   <definedNames>
     <definedName function="false" hidden="true" localSheetId="3" name="_xlnm._FilterDatabase" vbProcedure="false">Tatdata!$A$1:$B$14</definedName>
-    <definedName function="false" hidden="true" localSheetId="2" name="_xlnm._FilterDatabase" vbProcedure="false">Tatjes!$A$1:$F$97</definedName>
-    <definedName function="false" hidden="false" localSheetId="2" name="_xlnm._FilterDatabase" vbProcedure="false">Tatjes!$A$1:$F$95</definedName>
-    <definedName function="false" hidden="false" localSheetId="2" name="_xlnm._FilterDatabase_0" vbProcedure="false">Tatjes!$A$1:$F$1</definedName>
+    <definedName function="false" hidden="true" localSheetId="2" name="_xlnm._FilterDatabase" vbProcedure="false">Tatjes!$A$1:$F$95</definedName>
+    <definedName function="false" hidden="false" localSheetId="2" name="_xlnm._FilterDatabase" vbProcedure="false">Tatjes!$A$1:$F$97</definedName>
     <definedName function="false" hidden="false" localSheetId="2" name="_xlnm._FilterDatabase_0_0" vbProcedure="false">Tatjes!$A$1:$F$1</definedName>
     <definedName function="false" hidden="false" localSheetId="2" name="_xlnm._FilterDatabase_0_0_0" vbProcedure="false">Tatjes!$A$1:$F$1</definedName>
     <definedName function="false" hidden="false" localSheetId="2" name="_xlnm._FilterDatabase_0_0_0_0" vbProcedure="false">Tatjes!$A$1:$F$1</definedName>
     <definedName function="false" hidden="false" localSheetId="2" name="_xlnm._FilterDatabase_0_0_0_0_0" vbProcedure="false">Tatjes!$A$1:$F$1</definedName>
     <definedName function="false" hidden="false" localSheetId="2" name="_xlnm._FilterDatabase_0_0_0_0_0_0" vbProcedure="false">Tatjes!$A$1:$F$1</definedName>
+    <definedName function="false" hidden="false" localSheetId="2" name="_xlnm._FilterDatabase_0_0_0_0_0_0_0" vbProcedure="false">Tatjes!$A$1:$F$1</definedName>
     <definedName function="false" hidden="false" localSheetId="3" name="_xlnm._FilterDatabase_0" vbProcedure="false">Tatdata!$A$1:$B$13</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.001"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="506" uniqueCount="102">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="510" uniqueCount="102">
   <si>
     <t xml:space="preserve">Pagina</t>
   </si>
@@ -1500,19 +1500,19 @@
                   <c:v>147</c:v>
                 </c:pt>
                 <c:pt idx="83">
-                  <c:v>148</c:v>
+                  <c:v>153</c:v>
                 </c:pt>
                 <c:pt idx="84">
-                  <c:v/>
+                  <c:v>159</c:v>
                 </c:pt>
                 <c:pt idx="85">
-                  <c:v/>
+                  <c:v>164</c:v>
                 </c:pt>
                 <c:pt idx="86">
-                  <c:v/>
+                  <c:v>166</c:v>
                 </c:pt>
                 <c:pt idx="87">
-                  <c:v/>
+                  <c:v>167</c:v>
                 </c:pt>
                 <c:pt idx="88">
                   <c:v/>
@@ -1605,11 +1605,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="35948083"/>
-        <c:axId val="22270167"/>
+        <c:axId val="11680434"/>
+        <c:axId val="44658088"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="35948083"/>
+        <c:axId val="11680434"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1665,14 +1665,14 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="22270167"/>
+        <c:crossAx val="44658088"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
         <c:lblOffset val="100"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="22270167"/>
+        <c:axId val="44658088"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1737,7 +1737,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="35948083"/>
+        <c:crossAx val="11680434"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -2455,16 +2455,16 @@
                   <c:v>49</c:v>
                 </c:pt>
                 <c:pt idx="83">
-                  <c:v/>
+                  <c:v>50</c:v>
                 </c:pt>
                 <c:pt idx="84">
-                  <c:v/>
+                  <c:v>51</c:v>
                 </c:pt>
                 <c:pt idx="85">
-                  <c:v/>
+                  <c:v>52</c:v>
                 </c:pt>
                 <c:pt idx="86">
-                  <c:v/>
+                  <c:v>52</c:v>
                 </c:pt>
                 <c:pt idx="87">
                   <c:v/>
@@ -3202,16 +3202,16 @@
                   <c:v>18</c:v>
                 </c:pt>
                 <c:pt idx="83">
-                  <c:v/>
+                  <c:v>18</c:v>
                 </c:pt>
                 <c:pt idx="84">
-                  <c:v/>
+                  <c:v>18</c:v>
                 </c:pt>
                 <c:pt idx="85">
-                  <c:v/>
+                  <c:v>18</c:v>
                 </c:pt>
                 <c:pt idx="86">
-                  <c:v/>
+                  <c:v>18</c:v>
                 </c:pt>
                 <c:pt idx="87">
                   <c:v/>
@@ -3949,16 +3949,16 @@
                   <c:v>12</c:v>
                 </c:pt>
                 <c:pt idx="83">
-                  <c:v/>
+                  <c:v>12</c:v>
                 </c:pt>
                 <c:pt idx="84">
-                  <c:v/>
+                  <c:v>12</c:v>
                 </c:pt>
                 <c:pt idx="85">
-                  <c:v/>
+                  <c:v>12</c:v>
                 </c:pt>
                 <c:pt idx="86">
-                  <c:v/>
+                  <c:v>12</c:v>
                 </c:pt>
                 <c:pt idx="87">
                   <c:v/>
@@ -4696,16 +4696,16 @@
                   <c:v>4</c:v>
                 </c:pt>
                 <c:pt idx="83">
-                  <c:v/>
+                  <c:v>4</c:v>
                 </c:pt>
                 <c:pt idx="84">
-                  <c:v/>
+                  <c:v>4</c:v>
                 </c:pt>
                 <c:pt idx="85">
-                  <c:v/>
+                  <c:v>4</c:v>
                 </c:pt>
                 <c:pt idx="86">
-                  <c:v/>
+                  <c:v>5</c:v>
                 </c:pt>
                 <c:pt idx="87">
                   <c:v/>
@@ -4798,11 +4798,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="55703045"/>
-        <c:axId val="19932584"/>
+        <c:axId val="49364643"/>
+        <c:axId val="20403298"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="55703045"/>
+        <c:axId val="49364643"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -4858,14 +4858,14 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="19932584"/>
+        <c:crossAx val="20403298"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
         <c:lblOffset val="100"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="19932584"/>
+        <c:axId val="20403298"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -4930,7 +4930,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="55703045"/>
+        <c:crossAx val="49364643"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -5018,10 +5018,10 @@
           <c:layoutTarget val="inner"/>
           <c:xMode val="edge"/>
           <c:yMode val="edge"/>
-          <c:x val="0.0889819909954977"/>
-          <c:y val="0.110987544483986"/>
-          <c:w val="0.845797898949475"/>
-          <c:h val="0.793038256227758"/>
+          <c:x val="0.0889875554999687"/>
+          <c:y val="0.110999888777667"/>
+          <c:w val="0.845725720717904"/>
+          <c:h val="0.792904015126237"/>
         </c:manualLayout>
       </c:layout>
       <c:lineChart>
@@ -5153,11 +5153,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="12659909"/>
-        <c:axId val="36983749"/>
+        <c:axId val="85835509"/>
+        <c:axId val="83753811"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="12659909"/>
+        <c:axId val="85835509"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -5185,14 +5185,14 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="36983749"/>
+        <c:crossAx val="83753811"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
         <c:lblOffset val="100"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="36983749"/>
+        <c:axId val="83753811"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -5257,7 +5257,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="12659909"/>
+        <c:crossAx val="85835509"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -5295,9 +5295,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>177840</xdr:colOff>
+      <xdr:colOff>177480</xdr:colOff>
       <xdr:row>23</xdr:row>
-      <xdr:rowOff>41400</xdr:rowOff>
+      <xdr:rowOff>41040</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -5306,7 +5306,7 @@
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
         <a:off x="6578280" y="543600"/>
-        <a:ext cx="5756400" cy="3236400"/>
+        <a:ext cx="5756040" cy="3236040"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -5325,9 +5325,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>341640</xdr:colOff>
+      <xdr:colOff>341280</xdr:colOff>
       <xdr:row>52</xdr:row>
-      <xdr:rowOff>89640</xdr:rowOff>
+      <xdr:rowOff>89280</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -5336,7 +5336,7 @@
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
         <a:off x="6741360" y="5305320"/>
-        <a:ext cx="5757120" cy="3237120"/>
+        <a:ext cx="5756760" cy="3236760"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -5360,9 +5360,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>12</xdr:col>
-      <xdr:colOff>461160</xdr:colOff>
+      <xdr:colOff>460800</xdr:colOff>
       <xdr:row>21</xdr:row>
-      <xdr:rowOff>69840</xdr:rowOff>
+      <xdr:rowOff>69480</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -5371,7 +5371,7 @@
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
         <a:off x="2646720" y="246600"/>
-        <a:ext cx="5756760" cy="3236760"/>
+        <a:ext cx="5756400" cy="3236400"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -6166,11 +6166,11 @@
       </c>
       <c r="K27" s="0" t="n">
         <f aca="false">COUNTIF($D$1:$D$121,$J27)</f>
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="L27" s="6" t="n">
         <f aca="false">$K27/$K$31</f>
-        <v>0.583333333333333</v>
+        <v>0.590909090909091</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6208,7 +6208,7 @@
       </c>
       <c r="L28" s="6" t="n">
         <f aca="false">$K28/$K$31</f>
-        <v>0.214285714285714</v>
+        <v>0.204545454545455</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6250,7 +6250,7 @@
       </c>
       <c r="L29" s="6" t="n">
         <f aca="false">$K29/$K$31</f>
-        <v>0.142857142857143</v>
+        <v>0.136363636363636</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6288,11 +6288,11 @@
       </c>
       <c r="K30" s="0" t="n">
         <f aca="false">COUNTIF($D$1:$D$121,$J30)</f>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L30" s="6" t="n">
         <f aca="false">$K30/$K$31</f>
-        <v>0.0476190476190476</v>
+        <v>0.0568181818181818</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6330,7 +6330,7 @@
       </c>
       <c r="K31" s="0" t="n">
         <f aca="false">COUNTA($D$1:$D$121)</f>
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="L31" s="6" t="n">
         <f aca="false">$K31/$K$31</f>
@@ -7825,7 +7825,7 @@
       </c>
       <c r="B84" s="1" t="n">
         <f aca="false">IF(COUNTA(B85)&gt;0,ROUNDDOWN((B85+B83)/2,0),B83+1)</f>
-        <v>148</v>
+        <v>153</v>
       </c>
       <c r="C84" s="2" t="s">
         <v>43</v>
@@ -7854,88 +7854,109 @@
       <c r="A85" s="1" t="n">
         <v>83</v>
       </c>
-      <c r="D85" s="5"/>
-      <c r="E85" s="5" t="str">
+      <c r="B85" s="1" t="n">
+        <v>159</v>
+      </c>
+      <c r="D85" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="E85" s="5" t="n">
         <f aca="false">IF(COUNTA($D85)&gt;0,COUNTIF($D$2:$D85,E$1),"")</f>
-        <v/>
-      </c>
-      <c r="F85" s="5" t="str">
+        <v>18</v>
+      </c>
+      <c r="F85" s="5" t="n">
         <f aca="false">IF(COUNTA($D85)&gt;0,COUNTIF($D$2:$D85,F$1),"")</f>
-        <v/>
-      </c>
-      <c r="G85" s="5" t="str">
+        <v>50</v>
+      </c>
+      <c r="G85" s="5" t="n">
         <f aca="false">IF(COUNTA($D85)&gt;0,COUNTIF($D$2:$D85,G$1),"")</f>
-        <v/>
-      </c>
-      <c r="H85" s="5" t="str">
+        <v>12</v>
+      </c>
+      <c r="H85" s="5" t="n">
         <f aca="false">IF(COUNTA($D85)&gt;0,COUNTIF($D$2:$D85,H$1),"")</f>
-        <v/>
+        <v>4</v>
       </c>
     </row>
     <row r="86" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A86" s="1" t="n">
         <v>84</v>
       </c>
-      <c r="D86" s="5"/>
-      <c r="E86" s="5" t="str">
+      <c r="B86" s="1" t="n">
+        <v>164</v>
+      </c>
+      <c r="D86" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="E86" s="5" t="n">
         <f aca="false">IF(COUNTA($D86)&gt;0,COUNTIF($D$2:$D86,E$1),"")</f>
-        <v/>
-      </c>
-      <c r="F86" s="5" t="str">
+        <v>18</v>
+      </c>
+      <c r="F86" s="5" t="n">
         <f aca="false">IF(COUNTA($D86)&gt;0,COUNTIF($D$2:$D86,F$1),"")</f>
-        <v/>
-      </c>
-      <c r="G86" s="5" t="str">
+        <v>51</v>
+      </c>
+      <c r="G86" s="5" t="n">
         <f aca="false">IF(COUNTA($D86)&gt;0,COUNTIF($D$2:$D86,G$1),"")</f>
-        <v/>
-      </c>
-      <c r="H86" s="5" t="str">
+        <v>12</v>
+      </c>
+      <c r="H86" s="5" t="n">
         <f aca="false">IF(COUNTA($D86)&gt;0,COUNTIF($D$2:$D86,H$1),"")</f>
-        <v/>
+        <v>4</v>
       </c>
     </row>
     <row r="87" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A87" s="1" t="n">
         <v>85</v>
       </c>
-      <c r="D87" s="5"/>
-      <c r="E87" s="5" t="str">
+      <c r="B87" s="1" t="n">
+        <v>166</v>
+      </c>
+      <c r="D87" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="E87" s="5" t="n">
         <f aca="false">IF(COUNTA($D87)&gt;0,COUNTIF($D$2:$D87,E$1),"")</f>
-        <v/>
-      </c>
-      <c r="F87" s="5" t="str">
+        <v>18</v>
+      </c>
+      <c r="F87" s="5" t="n">
         <f aca="false">IF(COUNTA($D87)&gt;0,COUNTIF($D$2:$D87,F$1),"")</f>
-        <v/>
-      </c>
-      <c r="G87" s="5" t="str">
+        <v>52</v>
+      </c>
+      <c r="G87" s="5" t="n">
         <f aca="false">IF(COUNTA($D87)&gt;0,COUNTIF($D$2:$D87,G$1),"")</f>
-        <v/>
-      </c>
-      <c r="H87" s="5" t="str">
+        <v>12</v>
+      </c>
+      <c r="H87" s="5" t="n">
         <f aca="false">IF(COUNTA($D87)&gt;0,COUNTIF($D$2:$D87,H$1),"")</f>
-        <v/>
+        <v>4</v>
       </c>
     </row>
     <row r="88" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A88" s="1" t="n">
         <v>86</v>
       </c>
-      <c r="D88" s="5"/>
-      <c r="E88" s="5" t="str">
+      <c r="B88" s="1" t="n">
+        <f aca="false">IF(COUNTA(B89)&gt;0,ROUNDDOWN((B89+B87)/2,0),B87+1)</f>
+        <v>167</v>
+      </c>
+      <c r="D88" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="E88" s="5" t="n">
         <f aca="false">IF(COUNTA($D88)&gt;0,COUNTIF($D$2:$D88,E$1),"")</f>
-        <v/>
-      </c>
-      <c r="F88" s="5" t="str">
+        <v>18</v>
+      </c>
+      <c r="F88" s="5" t="n">
         <f aca="false">IF(COUNTA($D88)&gt;0,COUNTIF($D$2:$D88,F$1),"")</f>
-        <v/>
-      </c>
-      <c r="G88" s="5" t="str">
+        <v>52</v>
+      </c>
+      <c r="G88" s="5" t="n">
         <f aca="false">IF(COUNTA($D88)&gt;0,COUNTIF($D$2:$D88,G$1),"")</f>
-        <v/>
-      </c>
-      <c r="H88" s="5" t="str">
+        <v>12</v>
+      </c>
+      <c r="H88" s="5" t="n">
         <f aca="false">IF(COUNTA($D88)&gt;0,COUNTIF($D$2:$D88,H$1),"")</f>
-        <v/>
+        <v>5</v>
       </c>
     </row>
     <row r="89" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12664,7 +12685,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F97"/>
+  <autoFilter ref="A1:F95"/>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
   <pageSetup paperSize="9" scale="100" firstPageNumber="0" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" useFirstPageNumber="false" horizontalDpi="300" verticalDpi="300" copies="1"/>

</xml_diff>

<commit_message>
Sync from vault 2026-06-10 01:09:42
</commit_message>
<xml_diff>
--- a/content/Archief/0. PDFs & docs/Obol docs & forms/Irmijn Inc/Irma backup log.xlsx
+++ b/content/Archief/0. PDFs & docs/Obol docs & forms/Irmijn Inc/Irma backup log.xlsx
@@ -809,7 +809,7 @@
 </styleSheet>
 </file>
 
-<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/charts/chart7.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <c:lang val="en-US"/>
   <c:roundedCorners val="0"/>
@@ -1605,11 +1605,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="11680434"/>
-        <c:axId val="44658088"/>
+        <c:axId val="94763605"/>
+        <c:axId val="58235698"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="11680434"/>
+        <c:axId val="94763605"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1665,14 +1665,14 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="44658088"/>
+        <c:crossAx val="58235698"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
         <c:lblOffset val="100"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="44658088"/>
+        <c:axId val="58235698"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1737,7 +1737,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="11680434"/>
+        <c:crossAx val="94763605"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -1764,7 +1764,7 @@
 </c:chartSpace>
 </file>
 
-<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/charts/chart8.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <c:lang val="en-US"/>
   <c:roundedCorners val="0"/>
@@ -4798,11 +4798,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="49364643"/>
-        <c:axId val="20403298"/>
+        <c:axId val="98412282"/>
+        <c:axId val="54528503"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="49364643"/>
+        <c:axId val="98412282"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -4858,14 +4858,14 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="20403298"/>
+        <c:crossAx val="54528503"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
         <c:lblOffset val="100"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="20403298"/>
+        <c:axId val="54528503"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -4930,7 +4930,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="49364643"/>
+        <c:crossAx val="98412282"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -4978,7 +4978,7 @@
 </c:chartSpace>
 </file>
 
-<file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/charts/chart9.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <c:lang val="en-US"/>
   <c:roundedCorners val="0"/>
@@ -5153,11 +5153,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="85835509"/>
-        <c:axId val="83753811"/>
+        <c:axId val="40895745"/>
+        <c:axId val="75326003"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="85835509"/>
+        <c:axId val="40895745"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -5185,14 +5185,14 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="83753811"/>
+        <c:crossAx val="75326003"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
         <c:lblOffset val="100"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="83753811"/>
+        <c:axId val="75326003"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -5257,7 +5257,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="85835509"/>
+        <c:crossAx val="40895745"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>

</xml_diff>

<commit_message>
Sync from vault 2026-06-13 14:22:58
</commit_message>
<xml_diff>
--- a/content/Archief/0. PDFs & docs/Obol docs & forms/Irmijn Inc/Irma backup log.xlsx
+++ b/content/Archief/0. PDFs & docs/Obol docs & forms/Irmijn Inc/Irma backup log.xlsx
@@ -15,8 +15,9 @@
   </sheets>
   <definedNames>
     <definedName function="false" hidden="true" localSheetId="3" name="_xlnm._FilterDatabase" vbProcedure="false">Tatdata!$A$1:$B$14</definedName>
-    <definedName function="false" hidden="true" localSheetId="2" name="_xlnm._FilterDatabase" vbProcedure="false">Tatjes!$A$1:$F$95</definedName>
-    <definedName function="false" hidden="false" localSheetId="2" name="_xlnm._FilterDatabase" vbProcedure="false">Tatjes!$A$1:$F$97</definedName>
+    <definedName function="false" hidden="true" localSheetId="2" name="_xlnm._FilterDatabase" vbProcedure="false">Tatjes!$A$1:$F$98</definedName>
+    <definedName function="false" hidden="false" localSheetId="2" name="_xlnm._FilterDatabase" vbProcedure="false">Tatjes!$A$1:$F$95</definedName>
+    <definedName function="false" hidden="false" localSheetId="2" name="_xlnm._FilterDatabase_0" vbProcedure="false">Tatjes!$A$1:$F$97</definedName>
     <definedName function="false" hidden="false" localSheetId="2" name="_xlnm._FilterDatabase_0_0" vbProcedure="false">Tatjes!$A$1:$F$1</definedName>
     <definedName function="false" hidden="false" localSheetId="2" name="_xlnm._FilterDatabase_0_0_0" vbProcedure="false">Tatjes!$A$1:$F$1</definedName>
     <definedName function="false" hidden="false" localSheetId="2" name="_xlnm._FilterDatabase_0_0_0_0" vbProcedure="false">Tatjes!$A$1:$F$1</definedName>
@@ -35,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="510" uniqueCount="102">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="513" uniqueCount="102">
   <si>
     <t xml:space="preserve">Pagina</t>
   </si>
@@ -280,13 +281,13 @@
     <t xml:space="preserve">Paars</t>
   </si>
   <si>
+    <t xml:space="preserve">Aqua</t>
+  </si>
+  <si>
     <t xml:space="preserve">Zwart</t>
   </si>
   <si>
     <t xml:space="preserve">Zilver</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Aqua</t>
   </si>
   <si>
     <t xml:space="preserve">Wit</t>
@@ -304,10 +305,10 @@
     <t xml:space="preserve">Olijf</t>
   </si>
   <si>
-    <t xml:space="preserve">Rood</t>
+    <t xml:space="preserve">Ruit</t>
   </si>
   <si>
-    <t xml:space="preserve">Ruit</t>
+    <t xml:space="preserve">Rood</t>
   </si>
   <si>
     <t xml:space="preserve">Blad</t>
@@ -467,6 +468,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="FF9BE2F6"/>
+        <bgColor rgb="FFCCFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="FF000000"/>
         <bgColor rgb="FF003300"/>
       </patternFill>
@@ -475,12 +482,6 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFDDDDDD"/>
         <bgColor rgb="FFFFCCCC"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF9BE2F6"/>
-        <bgColor rgb="FFCCFFFF"/>
       </patternFill>
     </fill>
     <fill>
@@ -639,11 +640,11 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="11" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="11" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="12" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="12" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -809,7 +810,7 @@
 </styleSheet>
 </file>
 
-<file path=xl/charts/chart7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <c:lang val="en-US"/>
   <c:roundedCorners val="0"/>
@@ -1605,11 +1606,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="94763605"/>
-        <c:axId val="58235698"/>
+        <c:axId val="21405630"/>
+        <c:axId val="45281978"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="94763605"/>
+        <c:axId val="21405630"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1665,14 +1666,14 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="58235698"/>
+        <c:crossAx val="45281978"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
         <c:lblOffset val="100"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="58235698"/>
+        <c:axId val="45281978"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1737,7 +1738,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="94763605"/>
+        <c:crossAx val="21405630"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -1764,7 +1765,7 @@
 </c:chartSpace>
 </file>
 
-<file path=xl/charts/chart8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <c:lang val="en-US"/>
   <c:roundedCorners val="0"/>
@@ -4798,11 +4799,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="98412282"/>
-        <c:axId val="54528503"/>
+        <c:axId val="62624546"/>
+        <c:axId val="54897483"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="98412282"/>
+        <c:axId val="62624546"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -4858,14 +4859,14 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="54528503"/>
+        <c:crossAx val="54897483"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
         <c:lblOffset val="100"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="54528503"/>
+        <c:axId val="54897483"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -4930,7 +4931,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="98412282"/>
+        <c:crossAx val="62624546"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -4978,7 +4979,7 @@
 </c:chartSpace>
 </file>
 
-<file path=xl/charts/chart9.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <c:lang val="en-US"/>
   <c:roundedCorners val="0"/>
@@ -5018,10 +5019,10 @@
           <c:layoutTarget val="inner"/>
           <c:xMode val="edge"/>
           <c:yMode val="edge"/>
-          <c:x val="0.0889875554999687"/>
-          <c:y val="0.110999888777667"/>
-          <c:w val="0.845725720717904"/>
-          <c:h val="0.792904015126237"/>
+          <c:x val="0.0889931207004378"/>
+          <c:y val="0.111012235817575"/>
+          <c:w val="0.845653533458412"/>
+          <c:h val="0.792769744160178"/>
         </c:manualLayout>
       </c:layout>
       <c:lineChart>
@@ -5153,11 +5154,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="40895745"/>
-        <c:axId val="75326003"/>
+        <c:axId val="79621647"/>
+        <c:axId val="25400266"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="40895745"/>
+        <c:axId val="79621647"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -5185,14 +5186,14 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="75326003"/>
+        <c:crossAx val="25400266"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
         <c:lblOffset val="100"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="75326003"/>
+        <c:axId val="25400266"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -5257,7 +5258,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="40895745"/>
+        <c:crossAx val="79621647"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -5295,9 +5296,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>177480</xdr:colOff>
+      <xdr:colOff>177120</xdr:colOff>
       <xdr:row>23</xdr:row>
-      <xdr:rowOff>41040</xdr:rowOff>
+      <xdr:rowOff>40680</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -5306,7 +5307,7 @@
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
         <a:off x="6578280" y="543600"/>
-        <a:ext cx="5756040" cy="3236040"/>
+        <a:ext cx="5755680" cy="3235680"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -5325,9 +5326,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>341280</xdr:colOff>
+      <xdr:colOff>340920</xdr:colOff>
       <xdr:row>52</xdr:row>
-      <xdr:rowOff>89280</xdr:rowOff>
+      <xdr:rowOff>88920</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -5336,7 +5337,7 @@
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
         <a:off x="6741360" y="5305320"/>
-        <a:ext cx="5756760" cy="3236760"/>
+        <a:ext cx="5756400" cy="3236400"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -5360,9 +5361,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>12</xdr:col>
-      <xdr:colOff>460800</xdr:colOff>
+      <xdr:colOff>460440</xdr:colOff>
       <xdr:row>21</xdr:row>
-      <xdr:rowOff>69480</xdr:rowOff>
+      <xdr:rowOff>69120</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -5371,7 +5372,7 @@
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
         <a:off x="2646720" y="246600"/>
-        <a:ext cx="5756400" cy="3236400"/>
+        <a:ext cx="5756040" cy="3236040"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -10506,7 +10507,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F97"/>
+  <dimension ref="A1:F98"/>
   <sheetFormatPr defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="9.63"/>
@@ -10747,11 +10748,11 @@
       <c r="A11" s="10" t="s">
         <v>71</v>
       </c>
-      <c r="B11" s="18" t="s">
-        <v>81</v>
-      </c>
-      <c r="C11" s="19" t="s">
-        <v>82</v>
+      <c r="B11" s="12" t="s">
+        <v>73</v>
+      </c>
+      <c r="C11" s="8" t="s">
+        <v>75</v>
       </c>
       <c r="D11" s="0" t="n">
         <f aca="false">IF(ISBLANK(A11),"",COUNTIF(A:A,A11))</f>
@@ -10759,11 +10760,11 @@
       </c>
       <c r="E11" s="0" t="n">
         <f aca="false">IF(ISBLANK(B11),"",COUNTIF(B:B,B11))</f>
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F11" s="0" t="n">
         <f aca="false">IF(ISBLANK(C11),"",COUNTIF(C:C,C11))</f>
-        <v>3</v>
+        <v>18</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10773,8 +10774,8 @@
       <c r="B12" s="12" t="s">
         <v>73</v>
       </c>
-      <c r="C12" s="8" t="s">
-        <v>75</v>
+      <c r="C12" s="18" t="s">
+        <v>81</v>
       </c>
       <c r="D12" s="0" t="n">
         <f aca="false">IF(ISBLANK(A12),"",COUNTIF(A:A,A12))</f>
@@ -10786,7 +10787,7 @@
       </c>
       <c r="F12" s="0" t="n">
         <f aca="false">IF(ISBLANK(C12),"",COUNTIF(C:C,C12))</f>
-        <v>18</v>
+        <v>11</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10796,8 +10797,8 @@
       <c r="B13" s="12" t="s">
         <v>73</v>
       </c>
-      <c r="C13" s="20" t="s">
-        <v>83</v>
+      <c r="C13" s="11" t="s">
+        <v>72</v>
       </c>
       <c r="D13" s="0" t="n">
         <f aca="false">IF(ISBLANK(A13),"",COUNTIF(A:A,A13))</f>
@@ -10809,18 +10810,18 @@
       </c>
       <c r="F13" s="0" t="n">
         <f aca="false">IF(ISBLANK(C13),"",COUNTIF(C:C,C13))</f>
-        <v>11</v>
+        <v>5</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="10" t="s">
         <v>71</v>
       </c>
-      <c r="B14" s="12" t="s">
-        <v>73</v>
-      </c>
-      <c r="C14" s="11" t="s">
-        <v>72</v>
+      <c r="B14" s="19" t="s">
+        <v>82</v>
+      </c>
+      <c r="C14" s="20" t="s">
+        <v>83</v>
       </c>
       <c r="D14" s="0" t="n">
         <f aca="false">IF(ISBLANK(A14),"",COUNTIF(A:A,A14))</f>
@@ -10832,15 +10833,15 @@
       </c>
       <c r="F14" s="0" t="n">
         <f aca="false">IF(ISBLANK(C14),"",COUNTIF(C:C,C14))</f>
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="10" t="s">
         <v>71</v>
       </c>
-      <c r="B15" s="19" t="s">
-        <v>82</v>
+      <c r="B15" s="20" t="s">
+        <v>83</v>
       </c>
       <c r="C15" s="17" t="s">
         <v>80</v>
@@ -10862,8 +10863,8 @@
       <c r="A16" s="10" t="s">
         <v>71</v>
       </c>
-      <c r="B16" s="19" t="s">
-        <v>82</v>
+      <c r="B16" s="20" t="s">
+        <v>83</v>
       </c>
       <c r="C16" s="17" t="s">
         <v>80</v>
@@ -10885,8 +10886,8 @@
       <c r="A17" s="10" t="s">
         <v>71</v>
       </c>
-      <c r="B17" s="19" t="s">
-        <v>82</v>
+      <c r="B17" s="20" t="s">
+        <v>83</v>
       </c>
       <c r="C17" s="11" t="s">
         <v>72</v>
@@ -10908,8 +10909,8 @@
       <c r="A18" s="12" t="s">
         <v>33</v>
       </c>
-      <c r="B18" s="20" t="s">
-        <v>83</v>
+      <c r="B18" s="18" t="s">
+        <v>81</v>
       </c>
       <c r="C18" s="16" t="s">
         <v>79</v>
@@ -10957,8 +10958,8 @@
       <c r="B20" s="15" t="s">
         <v>78</v>
       </c>
-      <c r="C20" s="20" t="s">
-        <v>83</v>
+      <c r="C20" s="18" t="s">
+        <v>81</v>
       </c>
       <c r="D20" s="0" t="n">
         <f aca="false">IF(ISBLANK(A20),"",COUNTIF(A:A,A20))</f>
@@ -11003,8 +11004,8 @@
       <c r="B22" s="17" t="s">
         <v>80</v>
       </c>
-      <c r="C22" s="19" t="s">
-        <v>82</v>
+      <c r="C22" s="20" t="s">
+        <v>83</v>
       </c>
       <c r="D22" s="0" t="n">
         <f aca="false">IF(ISBLANK(A22),"",COUNTIF(A:A,A22))</f>
@@ -11049,8 +11050,8 @@
       <c r="B24" s="12" t="s">
         <v>73</v>
       </c>
-      <c r="C24" s="20" t="s">
-        <v>83</v>
+      <c r="C24" s="18" t="s">
+        <v>81</v>
       </c>
       <c r="D24" s="0" t="n">
         <f aca="false">IF(ISBLANK(A24),"",COUNTIF(A:A,A24))</f>
@@ -11072,8 +11073,8 @@
       <c r="B25" s="12" t="s">
         <v>73</v>
       </c>
-      <c r="C25" s="20" t="s">
-        <v>83</v>
+      <c r="C25" s="18" t="s">
+        <v>81</v>
       </c>
       <c r="D25" s="0" t="n">
         <f aca="false">IF(ISBLANK(A25),"",COUNTIF(A:A,A25))</f>
@@ -11095,8 +11096,8 @@
       <c r="B26" s="12" t="s">
         <v>73</v>
       </c>
-      <c r="C26" s="20" t="s">
-        <v>83</v>
+      <c r="C26" s="18" t="s">
+        <v>81</v>
       </c>
       <c r="D26" s="0" t="n">
         <f aca="false">IF(ISBLANK(A26),"",COUNTIF(A:A,A26))</f>
@@ -11118,8 +11119,8 @@
       <c r="B27" s="22" t="s">
         <v>85</v>
       </c>
-      <c r="C27" s="20" t="s">
-        <v>83</v>
+      <c r="C27" s="18" t="s">
+        <v>81</v>
       </c>
       <c r="D27" s="0" t="n">
         <f aca="false">IF(ISBLANK(A27),"",COUNTIF(A:A,A27))</f>
@@ -11177,7 +11178,7 @@
       </c>
       <c r="F29" s="0" t="n">
         <f aca="false">IF(ISBLANK(C29),"",COUNTIF(C:C,C29))</f>
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11233,8 +11234,8 @@
       <c r="B32" s="23" t="s">
         <v>86</v>
       </c>
-      <c r="C32" s="20" t="s">
-        <v>83</v>
+      <c r="C32" s="18" t="s">
+        <v>81</v>
       </c>
       <c r="D32" s="0" t="n">
         <f aca="false">IF(ISBLANK(A32),"",COUNTIF(A:A,A32))</f>
@@ -11513,14 +11514,14 @@
       </c>
     </row>
     <row r="46" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A46" s="14" t="s">
-        <v>19</v>
+      <c r="A46" s="17" t="s">
+        <v>89</v>
       </c>
       <c r="B46" s="18" t="s">
-        <v>43</v>
-      </c>
-      <c r="C46" s="23" t="s">
-        <v>86</v>
+        <v>81</v>
+      </c>
+      <c r="C46" s="12" t="s">
+        <v>73</v>
       </c>
       <c r="D46" s="0" t="n">
         <f aca="false">IF(ISBLANK(A46),"",COUNTIF(A:A,A46))</f>
@@ -11528,22 +11529,22 @@
       </c>
       <c r="E46" s="0" t="n">
         <f aca="false">IF(ISBLANK(B46),"",COUNTIF(B:B,B46))</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F46" s="0" t="n">
         <f aca="false">IF(ISBLANK(C46),"",COUNTIF(C:C,C46))</f>
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A47" s="14" t="s">
-        <v>19</v>
-      </c>
-      <c r="B47" s="25" t="s">
+      <c r="A47" s="17" t="s">
         <v>89</v>
       </c>
-      <c r="C47" s="8" t="s">
-        <v>75</v>
+      <c r="B47" s="13" t="s">
+        <v>74</v>
+      </c>
+      <c r="C47" s="19" t="s">
+        <v>82</v>
       </c>
       <c r="D47" s="0" t="n">
         <f aca="false">IF(ISBLANK(A47),"",COUNTIF(A:A,A47))</f>
@@ -11551,22 +11552,22 @@
       </c>
       <c r="E47" s="0" t="n">
         <f aca="false">IF(ISBLANK(B47),"",COUNTIF(B:B,B47))</f>
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="F47" s="0" t="n">
         <f aca="false">IF(ISBLANK(C47),"",COUNTIF(C:C,C47))</f>
-        <v>18</v>
+        <v>5</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A48" s="14" t="s">
-        <v>19</v>
-      </c>
-      <c r="B48" s="11" t="s">
-        <v>72</v>
-      </c>
-      <c r="C48" s="20" t="s">
-        <v>83</v>
+      <c r="A48" s="17" t="s">
+        <v>89</v>
+      </c>
+      <c r="B48" s="13" t="s">
+        <v>74</v>
+      </c>
+      <c r="C48" s="10" t="s">
+        <v>76</v>
       </c>
       <c r="D48" s="0" t="n">
         <f aca="false">IF(ISBLANK(A48),"",COUNTIF(A:A,A48))</f>
@@ -11574,19 +11575,19 @@
       </c>
       <c r="E48" s="0" t="n">
         <f aca="false">IF(ISBLANK(B48),"",COUNTIF(B:B,B48))</f>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F48" s="0" t="n">
         <f aca="false">IF(ISBLANK(C48),"",COUNTIF(C:C,C48))</f>
-        <v>11</v>
+        <v>4</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A49" s="14" t="s">
-        <v>19</v>
-      </c>
-      <c r="B49" s="14" t="s">
-        <v>77</v>
+      <c r="A49" s="17" t="s">
+        <v>89</v>
+      </c>
+      <c r="B49" s="16" t="s">
+        <v>79</v>
       </c>
       <c r="C49" s="8" t="s">
         <v>75</v>
@@ -11605,14 +11606,14 @@
       </c>
     </row>
     <row r="50" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A50" s="14" t="s">
-        <v>19</v>
+      <c r="A50" s="17" t="s">
+        <v>89</v>
       </c>
       <c r="B50" s="15" t="s">
         <v>78</v>
       </c>
-      <c r="C50" s="20" t="s">
-        <v>83</v>
+      <c r="C50" s="17" t="s">
+        <v>80</v>
       </c>
       <c r="D50" s="0" t="n">
         <f aca="false">IF(ISBLANK(A50),"",COUNTIF(A:A,A50))</f>
@@ -11624,18 +11625,18 @@
       </c>
       <c r="F50" s="0" t="n">
         <f aca="false">IF(ISBLANK(C50),"",COUNTIF(C:C,C50))</f>
-        <v>11</v>
+        <v>8</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A51" s="14" t="s">
-        <v>19</v>
-      </c>
-      <c r="B51" s="15" t="s">
-        <v>78</v>
-      </c>
-      <c r="C51" s="17" t="s">
+      <c r="A51" s="17" t="s">
+        <v>89</v>
+      </c>
+      <c r="B51" s="17" t="s">
         <v>80</v>
+      </c>
+      <c r="C51" s="13" t="s">
+        <v>74</v>
       </c>
       <c r="D51" s="0" t="n">
         <f aca="false">IF(ISBLANK(A51),"",COUNTIF(A:A,A51))</f>
@@ -11647,18 +11648,18 @@
       </c>
       <c r="F51" s="0" t="n">
         <f aca="false">IF(ISBLANK(C51),"",COUNTIF(C:C,C51))</f>
-        <v>8</v>
+        <v>3</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A52" s="14" t="s">
-        <v>19</v>
-      </c>
-      <c r="B52" s="17" t="s">
-        <v>80</v>
-      </c>
-      <c r="C52" s="13" t="s">
-        <v>74</v>
+      <c r="A52" s="17" t="s">
+        <v>89</v>
+      </c>
+      <c r="B52" s="19" t="s">
+        <v>82</v>
+      </c>
+      <c r="C52" s="23" t="s">
+        <v>86</v>
       </c>
       <c r="D52" s="0" t="n">
         <f aca="false">IF(ISBLANK(A52),"",COUNTIF(A:A,A52))</f>
@@ -11666,22 +11667,22 @@
       </c>
       <c r="E52" s="0" t="n">
         <f aca="false">IF(ISBLANK(B52),"",COUNTIF(B:B,B52))</f>
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F52" s="0" t="n">
         <f aca="false">IF(ISBLANK(C52),"",COUNTIF(C:C,C52))</f>
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A53" s="14" t="s">
-        <v>19</v>
-      </c>
-      <c r="B53" s="12" t="s">
-        <v>73</v>
-      </c>
-      <c r="C53" s="20" t="s">
+      <c r="A53" s="17" t="s">
+        <v>89</v>
+      </c>
+      <c r="B53" s="20" t="s">
         <v>83</v>
+      </c>
+      <c r="C53" s="17" t="s">
+        <v>80</v>
       </c>
       <c r="D53" s="0" t="n">
         <f aca="false">IF(ISBLANK(A53),"",COUNTIF(A:A,A53))</f>
@@ -11689,22 +11690,22 @@
       </c>
       <c r="E53" s="0" t="n">
         <f aca="false">IF(ISBLANK(B53),"",COUNTIF(B:B,B53))</f>
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="F53" s="0" t="n">
         <f aca="false">IF(ISBLANK(C53),"",COUNTIF(C:C,C53))</f>
-        <v>11</v>
+        <v>8</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A54" s="14" t="s">
-        <v>19</v>
-      </c>
-      <c r="B54" s="8" t="s">
-        <v>75</v>
-      </c>
-      <c r="C54" s="14" t="s">
-        <v>77</v>
+      <c r="A54" s="17" t="s">
+        <v>89</v>
+      </c>
+      <c r="B54" s="20" t="s">
+        <v>83</v>
+      </c>
+      <c r="C54" s="17" t="s">
+        <v>80</v>
       </c>
       <c r="D54" s="0" t="n">
         <f aca="false">IF(ISBLANK(A54),"",COUNTIF(A:A,A54))</f>
@@ -11716,18 +11717,18 @@
       </c>
       <c r="F54" s="0" t="n">
         <f aca="false">IF(ISBLANK(C54),"",COUNTIF(C:C,C54))</f>
-        <v>1</v>
+        <v>8</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A55" s="14" t="s">
-        <v>19</v>
-      </c>
-      <c r="B55" s="23" t="s">
-        <v>86</v>
-      </c>
-      <c r="C55" s="11" t="s">
-        <v>72</v>
+      <c r="A55" s="17" t="s">
+        <v>89</v>
+      </c>
+      <c r="B55" s="20" t="s">
+        <v>83</v>
+      </c>
+      <c r="C55" s="17" t="s">
+        <v>80</v>
       </c>
       <c r="D55" s="0" t="n">
         <f aca="false">IF(ISBLANK(A55),"",COUNTIF(A:A,A55))</f>
@@ -11735,19 +11736,19 @@
       </c>
       <c r="E55" s="0" t="n">
         <f aca="false">IF(ISBLANK(B55),"",COUNTIF(B:B,B55))</f>
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F55" s="0" t="n">
         <f aca="false">IF(ISBLANK(C55),"",COUNTIF(C:C,C55))</f>
-        <v>5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A56" s="14" t="s">
-        <v>19</v>
-      </c>
-      <c r="B56" s="23" t="s">
-        <v>86</v>
+      <c r="A56" s="17" t="s">
+        <v>89</v>
+      </c>
+      <c r="B56" s="20" t="s">
+        <v>83</v>
       </c>
       <c r="C56" s="11" t="s">
         <v>72</v>
@@ -11758,7 +11759,7 @@
       </c>
       <c r="E56" s="0" t="n">
         <f aca="false">IF(ISBLANK(B56),"",COUNTIF(B:B,B56))</f>
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F56" s="0" t="n">
         <f aca="false">IF(ISBLANK(C56),"",COUNTIF(C:C,C56))</f>
@@ -11766,22 +11767,22 @@
       </c>
     </row>
     <row r="57" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A57" s="17" t="s">
-        <v>90</v>
-      </c>
-      <c r="B57" s="20" t="s">
-        <v>83</v>
-      </c>
-      <c r="C57" s="12" t="s">
-        <v>73</v>
+      <c r="A57" s="14" t="s">
+        <v>19</v>
+      </c>
+      <c r="B57" s="19" t="s">
+        <v>43</v>
+      </c>
+      <c r="C57" s="23" t="s">
+        <v>86</v>
       </c>
       <c r="D57" s="0" t="n">
         <f aca="false">IF(ISBLANK(A57),"",COUNTIF(A:A,A57))</f>
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="E57" s="0" t="n">
         <f aca="false">IF(ISBLANK(B57),"",COUNTIF(B:B,B57))</f>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F57" s="0" t="n">
         <f aca="false">IF(ISBLANK(C57),"",COUNTIF(C:C,C57))</f>
@@ -11789,64 +11790,64 @@
       </c>
     </row>
     <row r="58" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A58" s="17" t="s">
+      <c r="A58" s="14" t="s">
+        <v>19</v>
+      </c>
+      <c r="B58" s="25" t="s">
         <v>90</v>
       </c>
-      <c r="B58" s="13" t="s">
-        <v>74</v>
-      </c>
-      <c r="C58" s="18" t="s">
-        <v>81</v>
+      <c r="C58" s="8" t="s">
+        <v>75</v>
       </c>
       <c r="D58" s="0" t="n">
         <f aca="false">IF(ISBLANK(A58),"",COUNTIF(A:A,A58))</f>
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="E58" s="0" t="n">
         <f aca="false">IF(ISBLANK(B58),"",COUNTIF(B:B,B58))</f>
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="F58" s="0" t="n">
         <f aca="false">IF(ISBLANK(C58),"",COUNTIF(C:C,C58))</f>
-        <v>5</v>
+        <v>18</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A59" s="17" t="s">
-        <v>90</v>
-      </c>
-      <c r="B59" s="13" t="s">
-        <v>74</v>
-      </c>
-      <c r="C59" s="10" t="s">
-        <v>76</v>
+      <c r="A59" s="14" t="s">
+        <v>19</v>
+      </c>
+      <c r="B59" s="11" t="s">
+        <v>72</v>
+      </c>
+      <c r="C59" s="18" t="s">
+        <v>81</v>
       </c>
       <c r="D59" s="0" t="n">
         <f aca="false">IF(ISBLANK(A59),"",COUNTIF(A:A,A59))</f>
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="E59" s="0" t="n">
         <f aca="false">IF(ISBLANK(B59),"",COUNTIF(B:B,B59))</f>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F59" s="0" t="n">
         <f aca="false">IF(ISBLANK(C59),"",COUNTIF(C:C,C59))</f>
-        <v>4</v>
+        <v>11</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A60" s="17" t="s">
-        <v>90</v>
-      </c>
-      <c r="B60" s="16" t="s">
-        <v>79</v>
+      <c r="A60" s="14" t="s">
+        <v>19</v>
+      </c>
+      <c r="B60" s="14" t="s">
+        <v>77</v>
       </c>
       <c r="C60" s="8" t="s">
         <v>75</v>
       </c>
       <c r="D60" s="0" t="n">
         <f aca="false">IF(ISBLANK(A60),"",COUNTIF(A:A,A60))</f>
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="E60" s="0" t="n">
         <f aca="false">IF(ISBLANK(B60),"",COUNTIF(B:B,B60))</f>
@@ -11858,18 +11859,18 @@
       </c>
     </row>
     <row r="61" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A61" s="17" t="s">
-        <v>90</v>
+      <c r="A61" s="14" t="s">
+        <v>19</v>
       </c>
       <c r="B61" s="15" t="s">
         <v>78</v>
       </c>
-      <c r="C61" s="17" t="s">
-        <v>80</v>
+      <c r="C61" s="18" t="s">
+        <v>81</v>
       </c>
       <c r="D61" s="0" t="n">
         <f aca="false">IF(ISBLANK(A61),"",COUNTIF(A:A,A61))</f>
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="E61" s="0" t="n">
         <f aca="false">IF(ISBLANK(B61),"",COUNTIF(B:B,B61))</f>
@@ -11877,22 +11878,22 @@
       </c>
       <c r="F61" s="0" t="n">
         <f aca="false">IF(ISBLANK(C61),"",COUNTIF(C:C,C61))</f>
-        <v>8</v>
+        <v>11</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A62" s="17" t="s">
-        <v>90</v>
-      </c>
-      <c r="B62" s="17" t="s">
+      <c r="A62" s="14" t="s">
+        <v>19</v>
+      </c>
+      <c r="B62" s="15" t="s">
+        <v>78</v>
+      </c>
+      <c r="C62" s="17" t="s">
         <v>80</v>
-      </c>
-      <c r="C62" s="13" t="s">
-        <v>74</v>
       </c>
       <c r="D62" s="0" t="n">
         <f aca="false">IF(ISBLANK(A62),"",COUNTIF(A:A,A62))</f>
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="E62" s="0" t="n">
         <f aca="false">IF(ISBLANK(B62),"",COUNTIF(B:B,B62))</f>
@@ -11900,68 +11901,68 @@
       </c>
       <c r="F62" s="0" t="n">
         <f aca="false">IF(ISBLANK(C62),"",COUNTIF(C:C,C62))</f>
-        <v>3</v>
+        <v>8</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A63" s="17" t="s">
-        <v>90</v>
-      </c>
-      <c r="B63" s="19" t="s">
-        <v>82</v>
-      </c>
-      <c r="C63" s="17" t="s">
+      <c r="A63" s="14" t="s">
+        <v>19</v>
+      </c>
+      <c r="B63" s="17" t="s">
         <v>80</v>
+      </c>
+      <c r="C63" s="13" t="s">
+        <v>74</v>
       </c>
       <c r="D63" s="0" t="n">
         <f aca="false">IF(ISBLANK(A63),"",COUNTIF(A:A,A63))</f>
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="E63" s="0" t="n">
         <f aca="false">IF(ISBLANK(B63),"",COUNTIF(B:B,B63))</f>
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="F63" s="0" t="n">
         <f aca="false">IF(ISBLANK(C63),"",COUNTIF(C:C,C63))</f>
-        <v>8</v>
+        <v>3</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A64" s="17" t="s">
-        <v>90</v>
-      </c>
-      <c r="B64" s="19" t="s">
-        <v>82</v>
-      </c>
-      <c r="C64" s="17" t="s">
-        <v>80</v>
+      <c r="A64" s="14" t="s">
+        <v>19</v>
+      </c>
+      <c r="B64" s="12" t="s">
+        <v>73</v>
+      </c>
+      <c r="C64" s="18" t="s">
+        <v>81</v>
       </c>
       <c r="D64" s="0" t="n">
         <f aca="false">IF(ISBLANK(A64),"",COUNTIF(A:A,A64))</f>
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="E64" s="0" t="n">
         <f aca="false">IF(ISBLANK(B64),"",COUNTIF(B:B,B64))</f>
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F64" s="0" t="n">
         <f aca="false">IF(ISBLANK(C64),"",COUNTIF(C:C,C64))</f>
-        <v>8</v>
+        <v>11</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A65" s="17" t="s">
-        <v>90</v>
-      </c>
-      <c r="B65" s="19" t="s">
-        <v>82</v>
-      </c>
-      <c r="C65" s="17" t="s">
-        <v>80</v>
+      <c r="A65" s="14" t="s">
+        <v>19</v>
+      </c>
+      <c r="B65" s="8" t="s">
+        <v>75</v>
+      </c>
+      <c r="C65" s="14" t="s">
+        <v>77</v>
       </c>
       <c r="D65" s="0" t="n">
         <f aca="false">IF(ISBLANK(A65),"",COUNTIF(A:A,A65))</f>
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="E65" s="0" t="n">
         <f aca="false">IF(ISBLANK(B65),"",COUNTIF(B:B,B65))</f>
@@ -11969,26 +11970,26 @@
       </c>
       <c r="F65" s="0" t="n">
         <f aca="false">IF(ISBLANK(C65),"",COUNTIF(C:C,C65))</f>
-        <v>8</v>
+        <v>1</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A66" s="17" t="s">
-        <v>90</v>
-      </c>
-      <c r="B66" s="19" t="s">
-        <v>82</v>
+      <c r="A66" s="14" t="s">
+        <v>19</v>
+      </c>
+      <c r="B66" s="23" t="s">
+        <v>86</v>
       </c>
       <c r="C66" s="11" t="s">
         <v>72</v>
       </c>
       <c r="D66" s="0" t="n">
         <f aca="false">IF(ISBLANK(A66),"",COUNTIF(A:A,A66))</f>
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="E66" s="0" t="n">
         <f aca="false">IF(ISBLANK(B66),"",COUNTIF(B:B,B66))</f>
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F66" s="0" t="n">
         <f aca="false">IF(ISBLANK(C66),"",COUNTIF(C:C,C66))</f>
@@ -11996,37 +11997,37 @@
       </c>
     </row>
     <row r="67" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A67" s="23" t="s">
-        <v>91</v>
-      </c>
-      <c r="B67" s="26" t="s">
-        <v>92</v>
-      </c>
-      <c r="C67" s="8" t="s">
-        <v>75</v>
+      <c r="A67" s="14" t="s">
+        <v>19</v>
+      </c>
+      <c r="B67" s="23" t="s">
+        <v>86</v>
+      </c>
+      <c r="C67" s="11" t="s">
+        <v>72</v>
       </c>
       <c r="D67" s="0" t="n">
         <f aca="false">IF(ISBLANK(A67),"",COUNTIF(A:A,A67))</f>
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="E67" s="0" t="n">
         <f aca="false">IF(ISBLANK(B67),"",COUNTIF(B:B,B67))</f>
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F67" s="0" t="n">
         <f aca="false">IF(ISBLANK(C67),"",COUNTIF(C:C,C67))</f>
-        <v>18</v>
+        <v>5</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="23" t="s">
         <v>91</v>
       </c>
-      <c r="B68" s="12" t="s">
-        <v>73</v>
-      </c>
-      <c r="C68" s="20" t="s">
-        <v>83</v>
+      <c r="B68" s="26" t="s">
+        <v>92</v>
+      </c>
+      <c r="C68" s="8" t="s">
+        <v>75</v>
       </c>
       <c r="D68" s="0" t="n">
         <f aca="false">IF(ISBLANK(A68),"",COUNTIF(A:A,A68))</f>
@@ -12034,22 +12035,22 @@
       </c>
       <c r="E68" s="0" t="n">
         <f aca="false">IF(ISBLANK(B68),"",COUNTIF(B:B,B68))</f>
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="F68" s="0" t="n">
         <f aca="false">IF(ISBLANK(C68),"",COUNTIF(C:C,C68))</f>
-        <v>11</v>
+        <v>18</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A69" s="23" t="s">
         <v>91</v>
       </c>
-      <c r="B69" s="22" t="s">
-        <v>85</v>
-      </c>
-      <c r="C69" s="8" t="s">
-        <v>75</v>
+      <c r="B69" s="12" t="s">
+        <v>73</v>
+      </c>
+      <c r="C69" s="18" t="s">
+        <v>81</v>
       </c>
       <c r="D69" s="0" t="n">
         <f aca="false">IF(ISBLANK(A69),"",COUNTIF(A:A,A69))</f>
@@ -12061,7 +12062,7 @@
       </c>
       <c r="F69" s="0" t="n">
         <f aca="false">IF(ISBLANK(C69),"",COUNTIF(C:C,C69))</f>
-        <v>18</v>
+        <v>11</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12071,8 +12072,8 @@
       <c r="B70" s="22" t="s">
         <v>85</v>
       </c>
-      <c r="C70" s="23" t="s">
-        <v>86</v>
+      <c r="C70" s="8" t="s">
+        <v>75</v>
       </c>
       <c r="D70" s="0" t="n">
         <f aca="false">IF(ISBLANK(A70),"",COUNTIF(A:A,A70))</f>
@@ -12084,18 +12085,18 @@
       </c>
       <c r="F70" s="0" t="n">
         <f aca="false">IF(ISBLANK(C70),"",COUNTIF(C:C,C70))</f>
-        <v>3</v>
+        <v>18</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A71" s="23" t="s">
         <v>91</v>
       </c>
-      <c r="B71" s="8" t="s">
-        <v>75</v>
-      </c>
-      <c r="C71" s="16" t="s">
-        <v>79</v>
+      <c r="B71" s="22" t="s">
+        <v>85</v>
+      </c>
+      <c r="C71" s="23" t="s">
+        <v>86</v>
       </c>
       <c r="D71" s="0" t="n">
         <f aca="false">IF(ISBLANK(A71),"",COUNTIF(A:A,A71))</f>
@@ -12103,22 +12104,22 @@
       </c>
       <c r="E71" s="0" t="n">
         <f aca="false">IF(ISBLANK(B71),"",COUNTIF(B:B,B71))</f>
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F71" s="0" t="n">
         <f aca="false">IF(ISBLANK(C71),"",COUNTIF(C:C,C71))</f>
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A72" s="23" t="s">
         <v>91</v>
       </c>
-      <c r="B72" s="23" t="s">
-        <v>86</v>
-      </c>
-      <c r="C72" s="8" t="s">
+      <c r="B72" s="8" t="s">
         <v>75</v>
+      </c>
+      <c r="C72" s="16" t="s">
+        <v>79</v>
       </c>
       <c r="D72" s="0" t="n">
         <f aca="false">IF(ISBLANK(A72),"",COUNTIF(A:A,A72))</f>
@@ -12126,11 +12127,11 @@
       </c>
       <c r="E72" s="0" t="n">
         <f aca="false">IF(ISBLANK(B72),"",COUNTIF(B:B,B72))</f>
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F72" s="0" t="n">
         <f aca="false">IF(ISBLANK(C72),"",COUNTIF(C:C,C72))</f>
-        <v>18</v>
+        <v>6</v>
       </c>
     </row>
     <row r="73" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12140,8 +12141,8 @@
       <c r="B73" s="23" t="s">
         <v>86</v>
       </c>
-      <c r="C73" s="16" t="s">
-        <v>79</v>
+      <c r="C73" s="8" t="s">
+        <v>75</v>
       </c>
       <c r="D73" s="0" t="n">
         <f aca="false">IF(ISBLANK(A73),"",COUNTIF(A:A,A73))</f>
@@ -12153,38 +12154,38 @@
       </c>
       <c r="F73" s="0" t="n">
         <f aca="false">IF(ISBLANK(C73),"",COUNTIF(C:C,C73))</f>
-        <v>6</v>
+        <v>18</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A74" s="8" t="s">
-        <v>36</v>
-      </c>
-      <c r="B74" s="18" t="s">
-        <v>81</v>
-      </c>
-      <c r="C74" s="8" t="s">
-        <v>75</v>
+      <c r="A74" s="23" t="s">
+        <v>91</v>
+      </c>
+      <c r="B74" s="23" t="s">
+        <v>86</v>
+      </c>
+      <c r="C74" s="16" t="s">
+        <v>79</v>
       </c>
       <c r="D74" s="0" t="n">
         <f aca="false">IF(ISBLANK(A74),"",COUNTIF(A:A,A74))</f>
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E74" s="0" t="n">
         <f aca="false">IF(ISBLANK(B74),"",COUNTIF(B:B,B74))</f>
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="F74" s="0" t="n">
         <f aca="false">IF(ISBLANK(C74),"",COUNTIF(C:C,C74))</f>
-        <v>18</v>
+        <v>6</v>
       </c>
     </row>
     <row r="75" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A75" s="8" t="s">
         <v>36</v>
       </c>
-      <c r="B75" s="18" t="s">
-        <v>81</v>
+      <c r="B75" s="19" t="s">
+        <v>82</v>
       </c>
       <c r="C75" s="8" t="s">
         <v>75</v>
@@ -12195,7 +12196,7 @@
       </c>
       <c r="E75" s="0" t="n">
         <f aca="false">IF(ISBLANK(B75),"",COUNTIF(B:B,B75))</f>
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F75" s="0" t="n">
         <f aca="false">IF(ISBLANK(C75),"",COUNTIF(C:C,C75))</f>
@@ -12206,8 +12207,8 @@
       <c r="A76" s="8" t="s">
         <v>36</v>
       </c>
-      <c r="B76" s="18" t="s">
-        <v>81</v>
+      <c r="B76" s="19" t="s">
+        <v>82</v>
       </c>
       <c r="C76" s="8" t="s">
         <v>75</v>
@@ -12218,7 +12219,7 @@
       </c>
       <c r="E76" s="0" t="n">
         <f aca="false">IF(ISBLANK(B76),"",COUNTIF(B:B,B76))</f>
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F76" s="0" t="n">
         <f aca="false">IF(ISBLANK(C76),"",COUNTIF(C:C,C76))</f>
@@ -12229,8 +12230,8 @@
       <c r="A77" s="8" t="s">
         <v>36</v>
       </c>
-      <c r="B77" s="18" t="s">
-        <v>81</v>
+      <c r="B77" s="19" t="s">
+        <v>82</v>
       </c>
       <c r="C77" s="8" t="s">
         <v>75</v>
@@ -12241,7 +12242,7 @@
       </c>
       <c r="E77" s="0" t="n">
         <f aca="false">IF(ISBLANK(B77),"",COUNTIF(B:B,B77))</f>
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F77" s="0" t="n">
         <f aca="false">IF(ISBLANK(C77),"",COUNTIF(C:C,C77))</f>
@@ -12252,8 +12253,8 @@
       <c r="A78" s="8" t="s">
         <v>36</v>
       </c>
-      <c r="B78" s="18" t="s">
-        <v>81</v>
+      <c r="B78" s="19" t="s">
+        <v>82</v>
       </c>
       <c r="C78" s="8" t="s">
         <v>75</v>
@@ -12264,7 +12265,7 @@
       </c>
       <c r="E78" s="0" t="n">
         <f aca="false">IF(ISBLANK(B78),"",COUNTIF(B:B,B78))</f>
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F78" s="0" t="n">
         <f aca="false">IF(ISBLANK(C78),"",COUNTIF(C:C,C78))</f>
@@ -12275,8 +12276,8 @@
       <c r="A79" s="8" t="s">
         <v>36</v>
       </c>
-      <c r="B79" s="18" t="s">
-        <v>81</v>
+      <c r="B79" s="19" t="s">
+        <v>82</v>
       </c>
       <c r="C79" s="8" t="s">
         <v>75</v>
@@ -12287,7 +12288,7 @@
       </c>
       <c r="E79" s="0" t="n">
         <f aca="false">IF(ISBLANK(B79),"",COUNTIF(B:B,B79))</f>
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F79" s="0" t="n">
         <f aca="false">IF(ISBLANK(C79),"",COUNTIF(C:C,C79))</f>
@@ -12295,31 +12296,34 @@
       </c>
     </row>
     <row r="80" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A80" s="22" t="s">
-        <v>93</v>
-      </c>
-      <c r="B80" s="16" t="s">
-        <v>79</v>
+      <c r="A80" s="8" t="s">
+        <v>36</v>
+      </c>
+      <c r="B80" s="19" t="s">
+        <v>82</v>
+      </c>
+      <c r="C80" s="8" t="s">
+        <v>75</v>
       </c>
       <c r="D80" s="0" t="n">
         <f aca="false">IF(ISBLANK(A80),"",COUNTIF(A:A,A80))</f>
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="E80" s="0" t="n">
         <f aca="false">IF(ISBLANK(B80),"",COUNTIF(B:B,B80))</f>
-        <v>5</v>
-      </c>
-      <c r="F80" s="0" t="str">
+        <v>8</v>
+      </c>
+      <c r="F80" s="0" t="n">
         <f aca="false">IF(ISBLANK(C80),"",COUNTIF(C:C,C80))</f>
-        <v/>
+        <v>18</v>
       </c>
     </row>
     <row r="81" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A81" s="22" t="s">
         <v>93</v>
       </c>
-      <c r="B81" s="22" t="s">
-        <v>85</v>
+      <c r="B81" s="16" t="s">
+        <v>79</v>
       </c>
       <c r="D81" s="0" t="n">
         <f aca="false">IF(ISBLANK(A81),"",COUNTIF(A:A,A81))</f>
@@ -12327,7 +12331,7 @@
       </c>
       <c r="E81" s="0" t="n">
         <f aca="false">IF(ISBLANK(B81),"",COUNTIF(B:B,B81))</f>
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="F81" s="0" t="str">
         <f aca="false">IF(ISBLANK(C81),"",COUNTIF(C:C,C81))</f>
@@ -12358,8 +12362,8 @@
       <c r="A83" s="22" t="s">
         <v>93</v>
       </c>
-      <c r="B83" s="8" t="s">
-        <v>75</v>
+      <c r="B83" s="22" t="s">
+        <v>85</v>
       </c>
       <c r="D83" s="0" t="n">
         <f aca="false">IF(ISBLANK(A83),"",COUNTIF(A:A,A83))</f>
@@ -12367,7 +12371,7 @@
       </c>
       <c r="E83" s="0" t="n">
         <f aca="false">IF(ISBLANK(B83),"",COUNTIF(B:B,B83))</f>
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F83" s="0" t="str">
         <f aca="false">IF(ISBLANK(C83),"",COUNTIF(C:C,C83))</f>
@@ -12375,11 +12379,11 @@
       </c>
     </row>
     <row r="84" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A84" s="18" t="s">
-        <v>43</v>
-      </c>
-      <c r="B84" s="27" t="s">
-        <v>94</v>
+      <c r="A84" s="22" t="s">
+        <v>93</v>
+      </c>
+      <c r="B84" s="8" t="s">
+        <v>75</v>
       </c>
       <c r="D84" s="0" t="n">
         <f aca="false">IF(ISBLANK(A84),"",COUNTIF(A:A,A84))</f>
@@ -12387,7 +12391,7 @@
       </c>
       <c r="E84" s="0" t="n">
         <f aca="false">IF(ISBLANK(B84),"",COUNTIF(B:B,B84))</f>
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="F84" s="0" t="str">
         <f aca="false">IF(ISBLANK(C84),"",COUNTIF(C:C,C84))</f>
@@ -12395,7 +12399,7 @@
       </c>
     </row>
     <row r="85" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A85" s="18" t="s">
+      <c r="A85" s="19" t="s">
         <v>43</v>
       </c>
       <c r="B85" s="27" t="s">
@@ -12415,11 +12419,11 @@
       </c>
     </row>
     <row r="86" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A86" s="18" t="s">
+      <c r="A86" s="19" t="s">
         <v>43</v>
       </c>
-      <c r="B86" s="11" t="s">
-        <v>72</v>
+      <c r="B86" s="27" t="s">
+        <v>94</v>
       </c>
       <c r="D86" s="0" t="n">
         <f aca="false">IF(ISBLANK(A86),"",COUNTIF(A:A,A86))</f>
@@ -12427,7 +12431,7 @@
       </c>
       <c r="E86" s="0" t="n">
         <f aca="false">IF(ISBLANK(B86),"",COUNTIF(B:B,B86))</f>
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F86" s="0" t="str">
         <f aca="false">IF(ISBLANK(C86),"",COUNTIF(C:C,C86))</f>
@@ -12435,11 +12439,11 @@
       </c>
     </row>
     <row r="87" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A87" s="18" t="s">
+      <c r="A87" s="19" t="s">
         <v>43</v>
       </c>
-      <c r="B87" s="23" t="s">
-        <v>86</v>
+      <c r="B87" s="11" t="s">
+        <v>72</v>
       </c>
       <c r="D87" s="0" t="n">
         <f aca="false">IF(ISBLANK(A87),"",COUNTIF(A:A,A87))</f>
@@ -12447,7 +12451,7 @@
       </c>
       <c r="E87" s="0" t="n">
         <f aca="false">IF(ISBLANK(B87),"",COUNTIF(B:B,B87))</f>
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="F87" s="0" t="str">
         <f aca="false">IF(ISBLANK(C87),"",COUNTIF(C:C,C87))</f>
@@ -12455,37 +12459,34 @@
       </c>
     </row>
     <row r="88" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A88" s="25" t="s">
-        <v>95</v>
-      </c>
-      <c r="B88" s="25" t="s">
-        <v>89</v>
-      </c>
-      <c r="C88" s="18" t="s">
-        <v>81</v>
+      <c r="A88" s="19" t="s">
+        <v>43</v>
+      </c>
+      <c r="B88" s="23" t="s">
+        <v>86</v>
       </c>
       <c r="D88" s="0" t="n">
         <f aca="false">IF(ISBLANK(A88),"",COUNTIF(A:A,A88))</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E88" s="0" t="n">
         <f aca="false">IF(ISBLANK(B88),"",COUNTIF(B:B,B88))</f>
-        <v>2</v>
-      </c>
-      <c r="F88" s="0" t="n">
+        <v>10</v>
+      </c>
+      <c r="F88" s="0" t="str">
         <f aca="false">IF(ISBLANK(C88),"",COUNTIF(C:C,C88))</f>
-        <v>5</v>
+        <v/>
       </c>
     </row>
     <row r="89" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A89" s="25" t="s">
         <v>95</v>
       </c>
-      <c r="B89" s="14" t="s">
-        <v>77</v>
-      </c>
-      <c r="C89" s="18" t="s">
-        <v>81</v>
+      <c r="B89" s="25" t="s">
+        <v>90</v>
+      </c>
+      <c r="C89" s="19" t="s">
+        <v>82</v>
       </c>
       <c r="D89" s="0" t="n">
         <f aca="false">IF(ISBLANK(A89),"",COUNTIF(A:A,A89))</f>
@@ -12493,7 +12494,7 @@
       </c>
       <c r="E89" s="0" t="n">
         <f aca="false">IF(ISBLANK(B89),"",COUNTIF(B:B,B89))</f>
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="F89" s="0" t="n">
         <f aca="false">IF(ISBLANK(C89),"",COUNTIF(C:C,C89))</f>
@@ -12504,11 +12505,11 @@
       <c r="A90" s="25" t="s">
         <v>95</v>
       </c>
-      <c r="B90" s="8" t="s">
-        <v>75</v>
-      </c>
-      <c r="C90" s="18" t="s">
-        <v>81</v>
+      <c r="B90" s="14" t="s">
+        <v>77</v>
+      </c>
+      <c r="C90" s="19" t="s">
+        <v>82</v>
       </c>
       <c r="D90" s="0" t="n">
         <f aca="false">IF(ISBLANK(A90),"",COUNTIF(A:A,A90))</f>
@@ -12516,7 +12517,7 @@
       </c>
       <c r="E90" s="0" t="n">
         <f aca="false">IF(ISBLANK(B90),"",COUNTIF(B:B,B90))</f>
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="F90" s="0" t="n">
         <f aca="false">IF(ISBLANK(C90),"",COUNTIF(C:C,C90))</f>
@@ -12524,14 +12525,14 @@
       </c>
     </row>
     <row r="91" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A91" s="13" t="s">
-        <v>96</v>
-      </c>
-      <c r="B91" s="13" t="s">
-        <v>74</v>
-      </c>
-      <c r="C91" s="13" t="s">
-        <v>74</v>
+      <c r="A91" s="25" t="s">
+        <v>95</v>
+      </c>
+      <c r="B91" s="8" t="s">
+        <v>75</v>
+      </c>
+      <c r="C91" s="19" t="s">
+        <v>82</v>
       </c>
       <c r="D91" s="0" t="n">
         <f aca="false">IF(ISBLANK(A91),"",COUNTIF(A:A,A91))</f>
@@ -12539,22 +12540,22 @@
       </c>
       <c r="E91" s="0" t="n">
         <f aca="false">IF(ISBLANK(B91),"",COUNTIF(B:B,B91))</f>
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="F91" s="0" t="n">
         <f aca="false">IF(ISBLANK(C91),"",COUNTIF(C:C,C91))</f>
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="92" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A92" s="13" t="s">
         <v>96</v>
       </c>
-      <c r="B92" s="17" t="s">
-        <v>80</v>
-      </c>
-      <c r="C92" s="19" t="s">
-        <v>82</v>
+      <c r="B92" s="13" t="s">
+        <v>74</v>
+      </c>
+      <c r="C92" s="13" t="s">
+        <v>74</v>
       </c>
       <c r="D92" s="0" t="n">
         <f aca="false">IF(ISBLANK(A92),"",COUNTIF(A:A,A92))</f>
@@ -12562,7 +12563,7 @@
       </c>
       <c r="E92" s="0" t="n">
         <f aca="false">IF(ISBLANK(B92),"",COUNTIF(B:B,B92))</f>
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="F92" s="0" t="n">
         <f aca="false">IF(ISBLANK(C92),"",COUNTIF(C:C,C92))</f>
@@ -12573,11 +12574,11 @@
       <c r="A93" s="13" t="s">
         <v>96</v>
       </c>
-      <c r="B93" s="19" t="s">
-        <v>82</v>
-      </c>
-      <c r="C93" s="18" t="s">
-        <v>81</v>
+      <c r="B93" s="17" t="s">
+        <v>80</v>
+      </c>
+      <c r="C93" s="20" t="s">
+        <v>83</v>
       </c>
       <c r="D93" s="0" t="n">
         <f aca="false">IF(ISBLANK(A93),"",COUNTIF(A:A,A93))</f>
@@ -12585,22 +12586,22 @@
       </c>
       <c r="E93" s="0" t="n">
         <f aca="false">IF(ISBLANK(B93),"",COUNTIF(B:B,B93))</f>
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="F93" s="0" t="n">
         <f aca="false">IF(ISBLANK(C93),"",COUNTIF(C:C,C93))</f>
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="94" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A94" s="28" t="s">
-        <v>97</v>
-      </c>
-      <c r="B94" s="28" t="s">
-        <v>98</v>
-      </c>
-      <c r="C94" s="27" t="s">
-        <v>94</v>
+      <c r="A94" s="13" t="s">
+        <v>96</v>
+      </c>
+      <c r="B94" s="20" t="s">
+        <v>83</v>
+      </c>
+      <c r="C94" s="19" t="s">
+        <v>82</v>
       </c>
       <c r="D94" s="0" t="n">
         <f aca="false">IF(ISBLANK(A94),"",COUNTIF(A:A,A94))</f>
@@ -12608,11 +12609,11 @@
       </c>
       <c r="E94" s="0" t="n">
         <f aca="false">IF(ISBLANK(B94),"",COUNTIF(B:B,B94))</f>
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="F94" s="0" t="n">
         <f aca="false">IF(ISBLANK(C94),"",COUNTIF(C:C,C94))</f>
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="95" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12642,11 +12643,11 @@
       <c r="A96" s="28" t="s">
         <v>97</v>
       </c>
-      <c r="B96" s="19" t="s">
-        <v>82</v>
-      </c>
-      <c r="C96" s="17" t="s">
-        <v>80</v>
+      <c r="B96" s="28" t="s">
+        <v>98</v>
+      </c>
+      <c r="C96" s="27" t="s">
+        <v>94</v>
       </c>
       <c r="D96" s="0" t="n">
         <f aca="false">IF(ISBLANK(A96),"",COUNTIF(A:A,A96))</f>
@@ -12654,38 +12655,61 @@
       </c>
       <c r="E96" s="0" t="n">
         <f aca="false">IF(ISBLANK(B96),"",COUNTIF(B:B,B96))</f>
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="F96" s="0" t="n">
         <f aca="false">IF(ISBLANK(C96),"",COUNTIF(C:C,C96))</f>
-        <v>8</v>
+        <v>2</v>
       </c>
     </row>
     <row r="97" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A97" s="15" t="s">
-        <v>99</v>
-      </c>
-      <c r="B97" s="17" t="s">
+      <c r="A97" s="28" t="s">
+        <v>97</v>
+      </c>
+      <c r="B97" s="20" t="s">
+        <v>83</v>
+      </c>
+      <c r="C97" s="17" t="s">
         <v>80</v>
-      </c>
-      <c r="C97" s="15" t="s">
-        <v>78</v>
       </c>
       <c r="D97" s="0" t="n">
         <f aca="false">IF(ISBLANK(A97),"",COUNTIF(A:A,A97))</f>
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E97" s="0" t="n">
         <f aca="false">IF(ISBLANK(B97),"",COUNTIF(B:B,B97))</f>
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="F97" s="0" t="n">
         <f aca="false">IF(ISBLANK(C97),"",COUNTIF(C:C,C97))</f>
+        <v>8</v>
+      </c>
+    </row>
+    <row r="98" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A98" s="15" t="s">
+        <v>99</v>
+      </c>
+      <c r="B98" s="17" t="s">
+        <v>80</v>
+      </c>
+      <c r="C98" s="15" t="s">
+        <v>78</v>
+      </c>
+      <c r="D98" s="0" t="n">
+        <f aca="false">IF(ISBLANK(A98),"",COUNTIF(A:A,A98))</f>
+        <v>1</v>
+      </c>
+      <c r="E98" s="0" t="n">
+        <f aca="false">IF(ISBLANK(B98),"",COUNTIF(B:B,B98))</f>
+        <v>7</v>
+      </c>
+      <c r="F98" s="0" t="n">
+        <f aca="false">IF(ISBLANK(C98),"",COUNTIF(C:C,C98))</f>
         <v>2</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F95"/>
+  <autoFilter ref="A1:F98"/>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
   <pageSetup paperSize="9" scale="100" firstPageNumber="0" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" useFirstPageNumber="false" horizontalDpi="300" verticalDpi="300" copies="1"/>
@@ -12789,8 +12813,8 @@
         <f aca="false">COUNTIF(Tatjes!B:B,D3)</f>
         <v>9</v>
       </c>
-      <c r="G3" s="20" t="s">
-        <v>83</v>
+      <c r="G3" s="18" t="s">
+        <v>81</v>
       </c>
       <c r="H3" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!C:C,G3)</f>
@@ -12801,7 +12825,7 @@
       </c>
       <c r="K3" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!B:B,J3)*2+COUNTIF(Tatjes!C:C,J3)</f>
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12812,8 +12836,8 @@
         <f aca="false">COUNTIF(Tatjes!A:A,A4)</f>
         <v>12</v>
       </c>
-      <c r="D4" s="19" t="s">
-        <v>82</v>
+      <c r="D4" s="20" t="s">
+        <v>83</v>
       </c>
       <c r="E4" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!B:B,D4)</f>
@@ -12835,8 +12859,8 @@
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="14" t="s">
-        <v>19</v>
+      <c r="A5" s="17" t="s">
+        <v>89</v>
       </c>
       <c r="B5" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!A:A,A5)</f>
@@ -12856,8 +12880,8 @@
         <f aca="false">COUNTIF(Tatjes!C:C,G5)</f>
         <v>6</v>
       </c>
-      <c r="J5" s="19" t="s">
-        <v>82</v>
+      <c r="J5" s="20" t="s">
+        <v>83</v>
       </c>
       <c r="K5" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!B:B,J5)*2+COUNTIF(Tatjes!C:C,J5)</f>
@@ -12865,12 +12889,12 @@
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="17" t="s">
-        <v>90</v>
+      <c r="A6" s="14" t="s">
+        <v>19</v>
       </c>
       <c r="B6" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!A:A,A6)</f>
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D6" s="22" t="s">
         <v>85</v>
@@ -12886,12 +12910,12 @@
         <f aca="false">COUNTIF(Tatjes!C:C,G6)</f>
         <v>5</v>
       </c>
-      <c r="J6" s="12" t="s">
-        <v>73</v>
+      <c r="J6" s="19" t="s">
+        <v>82</v>
       </c>
       <c r="K6" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!B:B,J6)*2+COUNTIF(Tatjes!C:C,J6)</f>
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12902,26 +12926,26 @@
         <f aca="false">COUNTIF(Tatjes!A:A,A7)</f>
         <v>7</v>
       </c>
-      <c r="D7" s="15" t="s">
-        <v>78</v>
+      <c r="D7" s="19" t="s">
+        <v>82</v>
       </c>
       <c r="E7" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!B:B,D7)</f>
-        <v>7</v>
-      </c>
-      <c r="G7" s="18" t="s">
-        <v>81</v>
+        <v>8</v>
+      </c>
+      <c r="G7" s="19" t="s">
+        <v>82</v>
       </c>
       <c r="H7" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!C:C,G7)</f>
         <v>5</v>
       </c>
-      <c r="J7" s="18" t="s">
-        <v>81</v>
+      <c r="J7" s="12" t="s">
+        <v>73</v>
       </c>
       <c r="K7" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!B:B,J7)*2+COUNTIF(Tatjes!C:C,J7)</f>
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12932,8 +12956,8 @@
         <f aca="false">COUNTIF(Tatjes!A:A,A8)</f>
         <v>6</v>
       </c>
-      <c r="D8" s="17" t="s">
-        <v>80</v>
+      <c r="D8" s="15" t="s">
+        <v>78</v>
       </c>
       <c r="E8" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!B:B,D8)</f>
@@ -12962,19 +12986,19 @@
         <f aca="false">COUNTIF(Tatjes!A:A,A9)</f>
         <v>4</v>
       </c>
-      <c r="D9" s="18" t="s">
-        <v>81</v>
+      <c r="D9" s="17" t="s">
+        <v>80</v>
       </c>
       <c r="E9" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!B:B,D9)</f>
         <v>7</v>
       </c>
-      <c r="G9" s="13" t="s">
-        <v>74</v>
+      <c r="G9" s="23" t="s">
+        <v>86</v>
       </c>
       <c r="H9" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!C:C,G9)</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J9" s="16" t="s">
         <v>79</v>
@@ -12985,7 +13009,7 @@
       </c>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="18" t="s">
+      <c r="A10" s="19" t="s">
         <v>43</v>
       </c>
       <c r="B10" s="1" t="n">
@@ -12999,8 +13023,8 @@
         <f aca="false">COUNTIF(Tatjes!B:B,D10)</f>
         <v>5</v>
       </c>
-      <c r="G10" s="23" t="s">
-        <v>86</v>
+      <c r="G10" s="13" t="s">
+        <v>74</v>
       </c>
       <c r="H10" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!C:C,G10)</f>
@@ -13029,15 +13053,15 @@
         <f aca="false">COUNTIF(Tatjes!B:B,D11)</f>
         <v>5</v>
       </c>
-      <c r="G11" s="19" t="s">
-        <v>82</v>
+      <c r="G11" s="20" t="s">
+        <v>83</v>
       </c>
       <c r="H11" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!C:C,G11)</f>
         <v>3</v>
       </c>
-      <c r="J11" s="20" t="s">
-        <v>83</v>
+      <c r="J11" s="18" t="s">
+        <v>81</v>
       </c>
       <c r="K11" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!B:B,J11)*2+COUNTIF(Tatjes!C:C,J11)</f>
@@ -13112,8 +13136,8 @@
         <f aca="false">COUNTIF(Tatjes!A:A,A14)</f>
         <v>1</v>
       </c>
-      <c r="D14" s="20" t="s">
-        <v>83</v>
+      <c r="D14" s="18" t="s">
+        <v>81</v>
       </c>
       <c r="E14" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!B:B,D14)</f>
@@ -13164,7 +13188,7 @@
       </c>
       <c r="B16" s="3" t="n">
         <f aca="false">COUNTA(Tatjes!A:A)-1</f>
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="D16" s="27" t="s">
         <v>94</v>
@@ -13213,7 +13237,7 @@
     </row>
     <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D18" s="25" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="E18" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!B:B,D18)</f>
@@ -13227,7 +13251,7 @@
         <v>0</v>
       </c>
       <c r="J18" s="25" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="K18" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!B:B,J18)*2+COUNTIF(Tatjes!C:C,J18)</f>
@@ -13266,7 +13290,7 @@
         <v>0</v>
       </c>
       <c r="G20" s="25" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="H20" s="1" t="n">
         <f aca="false">COUNTIF(Tatjes!C:C,G20)</f>

</xml_diff>